<commit_message>
Mise à jour d'Évolution
Copie du fichier `yarn.lock` d'Evolution

Rouler `yarn generateSurvey`

Les libellés de question utilisent le nom de la question comme clé au
lieu du path.

Changements dans l'excel:
- Les colonnes section et path de l'onglet "Labels" ont été renommés à
  namespace et key

À noter que certains custom widgets auront peut-être encore des anciens
libellés qui ne seront pas trouvés. Certains ont été corrigés pour les
tests UI, mais ce pourra être fait plus méthodiquement en révisant
chaque section.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2353" uniqueCount="1390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2353" uniqueCount="1392">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -3841,6 +3841,12 @@
   </si>
   <si>
     <t xml:space="preserve">Very burdensome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">namespace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">key</t>
   </si>
   <si>
     <t xml:space="preserve">addGroupedObject</t>
@@ -15619,10 +15625,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>3</v>
+        <v>1039</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>1040</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>6</v>
@@ -15642,13 +15648,13 @@
         <v>107</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -15658,13 +15664,13 @@
         <v>107</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
@@ -15674,13 +15680,13 @@
         <v>415</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1046</v>
+        <v>1048</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>1047</v>
+        <v>1049</v>
       </c>
       <c r="E4" s="10"/>
     </row>
@@ -15689,13 +15695,13 @@
         <v>415</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1048</v>
+        <v>1050</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1049</v>
+        <v>1051</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>1050</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15703,13 +15709,13 @@
         <v>415</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1051</v>
+        <v>1053</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1052</v>
+        <v>1054</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>1053</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15717,13 +15723,13 @@
         <v>415</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1054</v>
+        <v>1056</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1055</v>
+        <v>1057</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>1056</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15731,13 +15737,13 @@
         <v>415</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1057</v>
+        <v>1059</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>1058</v>
+        <v>1060</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>1059</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15745,13 +15751,13 @@
         <v>415</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1060</v>
+        <v>1062</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>1061</v>
+        <v>1063</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>1062</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15759,13 +15765,13 @@
         <v>415</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1063</v>
+        <v>1065</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>1064</v>
+        <v>1066</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>1065</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15773,13 +15779,13 @@
         <v>415</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1066</v>
+        <v>1068</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>1067</v>
+        <v>1069</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>1068</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15787,13 +15793,13 @@
         <v>415</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1069</v>
+        <v>1071</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>1070</v>
+        <v>1072</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>1071</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15801,13 +15807,13 @@
         <v>415</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1072</v>
+        <v>1074</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>1073</v>
+        <v>1075</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15815,7 +15821,7 @@
         <v>415</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1075</v>
+        <v>1077</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>747</v>
@@ -15829,13 +15835,13 @@
         <v>415</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1076</v>
+        <v>1078</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>1077</v>
+        <v>1079</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>1078</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15843,19 +15849,19 @@
         <v>328</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>1079</v>
+        <v>1081</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>1080</v>
+        <v>1082</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>1081</v>
+        <v>1083</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>1082</v>
+        <v>1084</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>1083</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15863,19 +15869,19 @@
         <v>328</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>1084</v>
+        <v>1086</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>1086</v>
+        <v>1088</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>1087</v>
+        <v>1089</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>1088</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15883,19 +15889,19 @@
         <v>328</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>1090</v>
+        <v>1092</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15903,19 +15909,19 @@
         <v>328</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>1094</v>
+        <v>1096</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>1096</v>
+        <v>1098</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>1097</v>
+        <v>1099</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>1098</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15923,19 +15929,19 @@
         <v>328</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1099</v>
+        <v>1101</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>1100</v>
+        <v>1102</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>1101</v>
+        <v>1103</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>1102</v>
+        <v>1104</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>1103</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15943,19 +15949,19 @@
         <v>328</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>1104</v>
+        <v>1106</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>1105</v>
+        <v>1107</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>1106</v>
+        <v>1108</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>1107</v>
+        <v>1109</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>1108</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15963,13 +15969,13 @@
         <v>328</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>1109</v>
+        <v>1111</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>1110</v>
+        <v>1112</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>1111</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15977,13 +15983,13 @@
         <v>328</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>1112</v>
+        <v>1114</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>1113</v>
+        <v>1115</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>1114</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -15991,13 +15997,13 @@
         <v>328</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>1115</v>
+        <v>1117</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>1116</v>
+        <v>1118</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>1117</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16005,13 +16011,13 @@
         <v>328</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>1118</v>
+        <v>1120</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>1119</v>
+        <v>1121</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>1120</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16019,19 +16025,19 @@
         <v>328</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>1122</v>
+        <v>1124</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>1123</v>
+        <v>1125</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>1124</v>
+        <v>1126</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>1125</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16039,13 +16045,13 @@
         <v>328</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>1126</v>
+        <v>1128</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>1127</v>
+        <v>1129</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>1128</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16053,13 +16059,13 @@
         <v>328</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>1129</v>
+        <v>1131</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>1130</v>
+        <v>1132</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>1131</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16067,13 +16073,13 @@
         <v>328</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>1132</v>
+        <v>1134</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>1133</v>
+        <v>1135</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>1134</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16081,13 +16087,13 @@
         <v>328</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1135</v>
+        <v>1137</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>1136</v>
+        <v>1138</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>1137</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16095,13 +16101,13 @@
         <v>328</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>1138</v>
+        <v>1140</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>1139</v>
+        <v>1141</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>1140</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16109,13 +16115,13 @@
         <v>328</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>1141</v>
+        <v>1143</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>1142</v>
+        <v>1144</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>1143</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16123,13 +16129,13 @@
         <v>328</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>1144</v>
+        <v>1146</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>1145</v>
+        <v>1147</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>1146</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16137,13 +16143,13 @@
         <v>328</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>1147</v>
+        <v>1149</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>1148</v>
+        <v>1150</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>1149</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16151,13 +16157,13 @@
         <v>328</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>1150</v>
+        <v>1152</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>1151</v>
+        <v>1153</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>1152</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16165,13 +16171,13 @@
         <v>328</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>1153</v>
+        <v>1155</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>1154</v>
+        <v>1156</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>1155</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16179,13 +16185,13 @@
         <v>328</v>
       </c>
       <c r="B37" s="10" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C37" s="10" t="s">
         <v>1156</v>
       </c>
-      <c r="C37" s="10" t="s">
-        <v>1154</v>
-      </c>
       <c r="D37" s="10" t="s">
-        <v>1155</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16193,13 +16199,13 @@
         <v>328</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>1158</v>
+        <v>1160</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>1159</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16207,13 +16213,13 @@
         <v>328</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>1160</v>
+        <v>1162</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>1161</v>
+        <v>1163</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>1162</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16221,13 +16227,13 @@
         <v>328</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>1163</v>
+        <v>1165</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>1164</v>
+        <v>1166</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16235,13 +16241,13 @@
         <v>328</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>1166</v>
+        <v>1168</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>1167</v>
+        <v>1169</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>1168</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16249,13 +16255,13 @@
         <v>328</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>1169</v>
+        <v>1171</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>1170</v>
+        <v>1172</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>1171</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16263,13 +16269,13 @@
         <v>328</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>1172</v>
+        <v>1174</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>1173</v>
+        <v>1175</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>1174</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16277,13 +16283,13 @@
         <v>328</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>1175</v>
+        <v>1177</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>1176</v>
+        <v>1178</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>1177</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16291,13 +16297,13 @@
         <v>328</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>1178</v>
+        <v>1180</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>1179</v>
+        <v>1181</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>1180</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16305,13 +16311,13 @@
         <v>328</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>1181</v>
+        <v>1183</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>1182</v>
+        <v>1184</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>1183</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16319,13 +16325,13 @@
         <v>328</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>1184</v>
+        <v>1186</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>1185</v>
+        <v>1187</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>1186</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16333,19 +16339,19 @@
         <v>328</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>1187</v>
+        <v>1189</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>1188</v>
+        <v>1190</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>1189</v>
+        <v>1191</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>1190</v>
+        <v>1192</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>1191</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16353,19 +16359,19 @@
         <v>328</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>1192</v>
+        <v>1194</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>1193</v>
+        <v>1195</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>1194</v>
+        <v>1196</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>1195</v>
+        <v>1197</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>1196</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16373,19 +16379,19 @@
         <v>328</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>1197</v>
+        <v>1199</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>1198</v>
+        <v>1200</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>1199</v>
+        <v>1201</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>1200</v>
+        <v>1202</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>1201</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16393,19 +16399,19 @@
         <v>328</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>1202</v>
+        <v>1204</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>1203</v>
+        <v>1205</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>1204</v>
+        <v>1206</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>1205</v>
+        <v>1207</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16413,19 +16419,19 @@
         <v>328</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>1207</v>
+        <v>1209</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>1208</v>
+        <v>1210</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>1209</v>
+        <v>1211</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>1210</v>
+        <v>1212</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>1211</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16433,19 +16439,19 @@
         <v>328</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>1212</v>
+        <v>1214</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>1213</v>
+        <v>1215</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>1214</v>
+        <v>1216</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>1215</v>
+        <v>1217</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>1216</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16453,19 +16459,19 @@
         <v>328</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>1217</v>
+        <v>1219</v>
       </c>
       <c r="C54" s="10" t="s">
-        <v>1218</v>
+        <v>1220</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>1219</v>
+        <v>1221</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>1220</v>
+        <v>1222</v>
       </c>
       <c r="F54" s="10" t="s">
-        <v>1221</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16473,19 +16479,19 @@
         <v>328</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>1222</v>
+        <v>1224</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>1223</v>
+        <v>1225</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>1224</v>
+        <v>1226</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>1225</v>
+        <v>1227</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>1226</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16493,13 +16499,13 @@
         <v>107</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>1227</v>
+        <v>1229</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>1228</v>
+        <v>1230</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>1229</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16507,13 +16513,13 @@
         <v>107</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>1230</v>
+        <v>1232</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>1231</v>
+        <v>1233</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>1232</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16521,13 +16527,13 @@
         <v>107</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>1233</v>
+        <v>1235</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>1234</v>
+        <v>1236</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>1235</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16535,13 +16541,13 @@
         <v>107</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>1236</v>
+        <v>1238</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>1237</v>
+        <v>1239</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>1238</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16549,13 +16555,13 @@
         <v>107</v>
       </c>
       <c r="B60" s="75" t="s">
-        <v>1239</v>
+        <v>1241</v>
       </c>
       <c r="C60" s="10" t="s">
-        <v>1240</v>
+        <v>1242</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>1241</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16563,13 +16569,13 @@
         <v>107</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>1242</v>
+        <v>1244</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>1243</v>
+        <v>1245</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>1244</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16577,13 +16583,13 @@
         <v>107</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>1245</v>
+        <v>1247</v>
       </c>
       <c r="C62" s="10" t="s">
-        <v>1246</v>
+        <v>1248</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>1247</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16591,19 +16597,19 @@
         <v>107</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>1248</v>
+        <v>1250</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>1249</v>
+        <v>1251</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>1250</v>
+        <v>1252</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>1251</v>
+        <v>1253</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16611,13 +16617,13 @@
         <v>107</v>
       </c>
       <c r="B64" s="34" t="s">
-        <v>1253</v>
+        <v>1255</v>
       </c>
       <c r="C64" s="34" t="s">
-        <v>1254</v>
+        <v>1256</v>
       </c>
       <c r="D64" s="75" t="s">
-        <v>1255</v>
+        <v>1257</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
@@ -16627,13 +16633,13 @@
         <v>107</v>
       </c>
       <c r="B65" s="34" t="s">
-        <v>1256</v>
+        <v>1258</v>
       </c>
       <c r="C65" s="34" t="s">
-        <v>1257</v>
+        <v>1259</v>
       </c>
       <c r="D65" s="75" t="s">
-        <v>1258</v>
+        <v>1260</v>
       </c>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
@@ -16643,7 +16649,7 @@
         <v>328</v>
       </c>
       <c r="B66" s="59" t="s">
-        <v>1259</v>
+        <v>1261</v>
       </c>
       <c r="C66" s="59" t="s">
         <v>703</v>
@@ -16659,7 +16665,7 @@
         <v>328</v>
       </c>
       <c r="B67" s="59" t="s">
-        <v>1260</v>
+        <v>1262</v>
       </c>
       <c r="C67" s="59" t="s">
         <v>921</v>
@@ -16675,7 +16681,7 @@
         <v>328</v>
       </c>
       <c r="B68" s="59" t="s">
-        <v>1261</v>
+        <v>1263</v>
       </c>
       <c r="C68" s="59" t="s">
         <v>923</v>
@@ -16691,7 +16697,7 @@
         <v>328</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>1262</v>
+        <v>1264</v>
       </c>
       <c r="C69" s="10" t="s">
         <v>926</v>
@@ -16711,7 +16717,7 @@
         <v>415</v>
       </c>
       <c r="B70" s="59" t="s">
-        <v>1263</v>
+        <v>1265</v>
       </c>
       <c r="C70" s="10" t="s">
         <v>933</v>
@@ -16731,7 +16737,7 @@
         <v>415</v>
       </c>
       <c r="B71" s="59" t="s">
-        <v>1264</v>
+        <v>1266</v>
       </c>
       <c r="C71" s="10" t="s">
         <v>938</v>
@@ -16751,13 +16757,13 @@
         <v>415</v>
       </c>
       <c r="B72" s="59" t="s">
-        <v>1265</v>
+        <v>1267</v>
       </c>
       <c r="C72" s="10" t="s">
-        <v>1266</v>
+        <v>1268</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>1267</v>
+        <v>1269</v>
       </c>
       <c r="E72" s="10"/>
       <c r="F72" s="10"/>
@@ -16767,13 +16773,13 @@
         <v>415</v>
       </c>
       <c r="B73" s="59" t="s">
-        <v>1268</v>
+        <v>1270</v>
       </c>
       <c r="C73" s="10" t="s">
-        <v>1269</v>
+        <v>1271</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>1270</v>
+        <v>1272</v>
       </c>
       <c r="E73" s="10"/>
       <c r="F73" s="10"/>
@@ -16783,13 +16789,13 @@
         <v>415</v>
       </c>
       <c r="B74" s="59" t="s">
-        <v>1271</v>
+        <v>1273</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>1272</v>
+        <v>1274</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>1273</v>
+        <v>1275</v>
       </c>
       <c r="E74" s="10"/>
       <c r="F74" s="10"/>
@@ -16799,13 +16805,13 @@
         <v>415</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>1274</v>
+        <v>1276</v>
       </c>
       <c r="C75" s="10" t="s">
-        <v>1275</v>
+        <v>1277</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>1276</v>
+        <v>1278</v>
       </c>
       <c r="E75" s="10"/>
       <c r="F75" s="10"/>
@@ -16815,13 +16821,13 @@
         <v>328</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>1277</v>
+        <v>1279</v>
       </c>
       <c r="C76" s="10" t="s">
-        <v>1278</v>
+        <v>1280</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>1279</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16829,13 +16835,13 @@
         <v>328</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>1280</v>
+        <v>1282</v>
       </c>
       <c r="C77" s="10" t="s">
-        <v>1281</v>
+        <v>1283</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>1282</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16843,13 +16849,13 @@
         <v>328</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>1283</v>
+        <v>1285</v>
       </c>
       <c r="C78" s="10" t="s">
-        <v>1284</v>
+        <v>1286</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>1285</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16857,13 +16863,13 @@
         <v>328</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>1286</v>
+        <v>1288</v>
       </c>
       <c r="C79" s="10" t="s">
-        <v>1287</v>
+        <v>1289</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>1288</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16871,7 +16877,7 @@
         <v>107</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>1289</v>
+        <v>1291</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>982</v>
@@ -16891,7 +16897,7 @@
         <v>107</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>1290</v>
+        <v>1292</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>986</v>
@@ -16911,7 +16917,7 @@
         <v>107</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>1291</v>
+        <v>1293</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>990</v>
@@ -16931,7 +16937,7 @@
         <v>107</v>
       </c>
       <c r="B83" s="20" t="s">
-        <v>1292</v>
+        <v>1294</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>994</v>
@@ -16951,7 +16957,7 @@
         <v>107</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>1293</v>
+        <v>1295</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>998</v>
@@ -16971,19 +16977,19 @@
         <v>277</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>1294</v>
+        <v>1296</v>
       </c>
       <c r="C85" s="10" t="s">
-        <v>1295</v>
+        <v>1297</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>1296</v>
+        <v>1298</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>1297</v>
+        <v>1299</v>
       </c>
       <c r="F85" s="10" t="s">
-        <v>1298</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16991,19 +16997,19 @@
         <v>277</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>1299</v>
+        <v>1301</v>
       </c>
       <c r="C86" s="10" t="s">
-        <v>1300</v>
+        <v>1302</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>1301</v>
+        <v>1303</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>1302</v>
+        <v>1304</v>
       </c>
       <c r="F86" s="10" t="s">
-        <v>1303</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17011,13 +17017,13 @@
         <v>572</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>1304</v>
+        <v>1306</v>
       </c>
       <c r="C87" s="10" t="s">
-        <v>1305</v>
+        <v>1307</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>1306</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17025,13 +17031,13 @@
         <v>415</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>1307</v>
+        <v>1309</v>
       </c>
       <c r="C88" s="10" t="s">
-        <v>1308</v>
+        <v>1310</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>1309</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17039,13 +17045,13 @@
         <v>415</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>1310</v>
+        <v>1312</v>
       </c>
       <c r="C89" s="10" t="s">
-        <v>1311</v>
+        <v>1313</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>1312</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17053,13 +17059,13 @@
         <v>415</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>1313</v>
+        <v>1315</v>
       </c>
       <c r="C90" s="10" t="s">
-        <v>1314</v>
+        <v>1316</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>1315</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17067,13 +17073,13 @@
         <v>415</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>1316</v>
+        <v>1318</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>1317</v>
+        <v>1319</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>1318</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17081,13 +17087,13 @@
         <v>415</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>1319</v>
+        <v>1321</v>
       </c>
       <c r="C92" s="10" t="s">
-        <v>1320</v>
+        <v>1322</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>1321</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17095,13 +17101,13 @@
         <v>415</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>1322</v>
+        <v>1324</v>
       </c>
       <c r="C93" s="10" t="s">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17109,13 +17115,13 @@
         <v>415</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>1325</v>
+        <v>1327</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>1326</v>
+        <v>1328</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>1327</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17123,13 +17129,13 @@
         <v>415</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>1328</v>
+        <v>1330</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>1329</v>
+        <v>1331</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>1329</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17137,13 +17143,13 @@
         <v>415</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>1330</v>
+        <v>1332</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>1331</v>
+        <v>1333</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>1332</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17151,13 +17157,13 @@
         <v>415</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>1333</v>
+        <v>1335</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>1334</v>
+        <v>1336</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>1335</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17165,13 +17171,13 @@
         <v>415</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>1336</v>
+        <v>1338</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>1337</v>
+        <v>1339</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>1338</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17179,13 +17185,13 @@
         <v>415</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>1339</v>
+        <v>1341</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>1340</v>
+        <v>1342</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>1341</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17193,13 +17199,13 @@
         <v>415</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>1342</v>
+        <v>1344</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>1343</v>
+        <v>1345</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>1344</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17207,13 +17213,13 @@
         <v>415</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>1345</v>
+        <v>1347</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>1346</v>
+        <v>1348</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17221,13 +17227,13 @@
         <v>415</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>1350</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17235,13 +17241,13 @@
         <v>415</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>1351</v>
+        <v>1353</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>1352</v>
+        <v>1354</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>1353</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17249,13 +17255,13 @@
         <v>415</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>1354</v>
+        <v>1356</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>1355</v>
+        <v>1357</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>1356</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17263,13 +17269,13 @@
         <v>415</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>1357</v>
+        <v>1359</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>1358</v>
+        <v>1360</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>1359</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17277,13 +17283,13 @@
         <v>415</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>1360</v>
+        <v>1362</v>
       </c>
       <c r="C106" s="2" t="s">
-        <v>1361</v>
+        <v>1363</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>1362</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17291,13 +17297,13 @@
         <v>415</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>1363</v>
+        <v>1365</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>1364</v>
+        <v>1366</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>1365</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17305,13 +17311,13 @@
         <v>415</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>1367</v>
+        <v>1369</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>1368</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17319,13 +17325,13 @@
         <v>415</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>1369</v>
+        <v>1371</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>1370</v>
+        <v>1372</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>1371</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17333,13 +17339,13 @@
         <v>415</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>1372</v>
+        <v>1374</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>1373</v>
+        <v>1375</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>1374</v>
+        <v>1376</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17347,13 +17353,13 @@
         <v>415</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>1375</v>
+        <v>1377</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>1376</v>
+        <v>1378</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>1377</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17361,13 +17367,13 @@
         <v>415</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>1378</v>
+        <v>1380</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>1379</v>
+        <v>1381</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>1380</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17375,13 +17381,13 @@
         <v>415</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>1381</v>
+        <v>1383</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>1382</v>
+        <v>1384</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>1383</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17389,13 +17395,13 @@
         <v>415</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>1384</v>
+        <v>1386</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>1385</v>
+        <v>1387</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>1386</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17403,13 +17409,13 @@
         <v>415</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>1387</v>
+        <v>1389</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>1388</v>
+        <v>1390</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>1389</v>
+        <v>1391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nav: ajout des sections pré-fin sous la section fin
Le parent de la section omissions est maintenant "end", de même que
celui de longue distance.

Fixe en partie #132 en ayant une seule section "Fin" et en omettant les
autres sections.

Par contre, la section n'est pas activée par défaut et, donc, les tests
UI ont été désactivés pour cette section. La navigation correcte dans le
cas d'une section parent avec enfants invisibles sera fixé dans
Evolution avec l'issue https://github.com/chairemobilite/evolution/issues/1634
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -53,15 +53,15 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>33</xdr:colOff>
+                <xdr:colOff>18</xdr:colOff>
                 <xdr:row>42</xdr:row>
-                <xdr:rowOff>10</xdr:rowOff>
+                <xdr:rowOff>5</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>18</xdr:col>
-                <xdr:colOff>4</xdr:colOff>
+                <xdr:colOff>2</xdr:colOff>
                 <xdr:row>60</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
+                <xdr:rowOff>4</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4244" uniqueCount="2358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4245" uniqueCount="2358">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -19392,7 +19392,7 @@
         <v>1</v>
       </c>
       <c r="T169" s="11"/>
-      <c r="U169" s="0"/>
+      <c r="U169" s="2"/>
       <c r="V169" s="11"/>
       <c r="W169" s="11"/>
       <c r="X169" s="11"/>
@@ -19452,7 +19452,7 @@
         <v>1</v>
       </c>
       <c r="T170" s="11"/>
-      <c r="U170" s="0"/>
+      <c r="U170" s="2"/>
       <c r="V170" s="11"/>
       <c r="W170" s="11"/>
       <c r="X170" s="11"/>
@@ -21293,7 +21293,6 @@
       <c r="F65" s="10" t="s">
         <v>1064</v>
       </c>
-      <c r="G65" s="0"/>
       <c r="H65" s="2" t="s">
         <v>1075</v>
       </c>
@@ -22536,7 +22535,6 @@
         <v>906</v>
       </c>
       <c r="F130" s="78"/>
-      <c r="G130" s="0"/>
     </row>
     <row r="131" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
@@ -22590,7 +22588,7 @@
         <v>1078</v>
       </c>
       <c r="F133" s="78"/>
-      <c r="G133" s="0"/>
+      <c r="G133" s="2"/>
       <c r="H133" s="78" t="s">
         <v>1114</v>
       </c>
@@ -22904,8 +22902,8 @@
         <v>1146</v>
       </c>
       <c r="E10" s="84" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="F10" s="84" t="n">
         <f aca="false">FALSE()</f>
@@ -22914,6 +22912,9 @@
       <c r="G10" s="84" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>907</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
visitedPlaces: Adaptation du libellé pour `school` selon âge
fixes #149

pour la catégorie d'activité `school`, le libellé utilise l'interval
selon l'âge de la personne pour mettre "École" ou "Études" selon les
besoins.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -53,7 +53,7 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>11</xdr:col>
-                <xdr:colOff>3</xdr:colOff>
+                <xdr:colOff>2</xdr:colOff>
                 <xdr:row>42</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:from>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4622" uniqueCount="2535">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4618" uniqueCount="2535">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -5910,271 +5910,271 @@
     <t xml:space="preserve">Work</t>
   </si>
   <si>
-    <t xml:space="preserve">activityCategories.school</t>
-  </si>
-  <si>
-    <t xml:space="preserve">École</t>
-  </si>
-  <si>
-    <t xml:space="preserve">School</t>
+    <t xml:space="preserve">activityCategories.schoolStudies_interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1-15)[École];(15-inf)[Études];</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1-15)[School];(15-inf)[Studies];</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activityCategories.shoppingServiceRestaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magasinage, Service ou Restauration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopping, Services or Restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activityCategories.dropFetchSomeone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reconduire ou Aller chercher quelqu'un</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drop someone off or Pick someone up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activityCategories.leisure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loisirs (sport, arts, promenade, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leisure (sport, arts, stroll, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activityCategories.other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activityCategories.otherParentHome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Domicile de l'autre parent ou tuteur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home of the other parent or guardian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activityCategories.home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.workUsual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travail au lieu habituel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work (out-of-home fixed location)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.workNotUsual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travail dans un autre lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work (other place)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.workOnTheRoad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travail sur la route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Work on the road</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.volunteering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bénévolat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volunteering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.schoolUsual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Études au lieu principal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Studies ([établissement scolaire]/high school, college, university)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.schoolNotUsual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Études dans un autre lieu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Studies (different location)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.shopping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magasinage (achats, station-service, épicerie, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopping (store, gas station, grocery)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restaurant, café, bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restaurant, coffee shop, bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service (coiffeur, réparations, avocat, banque, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service (hairdresser, repairs, lawyer, bank)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.medical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santé (hôpital, clinique, physiothérapie, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical (clinic, hospital, physiotherapy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.veterinarian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vétérinaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veterinary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.worship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lieu de culte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Place of worship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.pickClassifiedPurchase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Récupérer un achat chez un particulier (petites annonces)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick up an item from a private seller (online marketplace/classifieds)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.dropSomeone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reconduire quelqu'un</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drop someone off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.fetchSomeone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aller chercher quelqu'un</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick someone up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.accompanySomeone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accompagner quelqu'un</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accompany someone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.leisureStroll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promenade sans destination fixe (ex. : aller courir, promener le chien)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stroll with no fixed destination (ex: go running/jogging, walk with pet, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.leisureSports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sport, entrainement, aller au parc (destination fixe)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sport, training, park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.leisureArtsMusicCulture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arts, Musique ou culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arts, Music ou culture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.leisureTourism</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vacances, tourisme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vacation, tourism</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.visiting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visite chez ami.e.s, copain.e ou famille</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visiting friends, partner or family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.secondaryHome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résidence secondaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secondary residence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">activities.schoolNotStudent</t>
   </si>
   <si>
     <t xml:space="preserve">Études</t>
   </si>
   <si>
     <t xml:space="preserve">Studies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activityCategories.shoppingServiceRestaurant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magasinage, Service ou Restauration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopping, Services or Restaurant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activityCategories.dropFetchSomeone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reconduire ou Aller chercher quelqu'un</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drop someone off or Pick someone up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activityCategories.leisure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Loisirs (sport, arts, promenade, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leisure (sport, arts, stroll, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activityCategories.other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activityCategories.otherParentHome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Domicile de l'autre parent ou tuteur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home of the other parent or guardian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activityCategories.home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.workUsual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travail au lieu habituel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work (out-of-home fixed location)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.workNotUsual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travail dans un autre lieu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work (other place)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.workOnTheRoad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travail sur la route</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Work on the road</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.volunteering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bénévolat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volunteering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.schoolUsual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Études au lieu principal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Studies ([établissement scolaire]/high school, college, university)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.schoolNotUsual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Études dans un autre lieu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Studies (different location)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.shopping</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Magasinage (achats, station-service, épicerie, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopping (store, gas station, grocery)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.restaurant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restaurant, café, bar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restaurant, coffee shop, bar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service (coiffeur, réparations, avocat, banque, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Service (hairdresser, repairs, lawyer, bank)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.medical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Santé (hôpital, clinique, physiothérapie, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medical (clinic, hospital, physiotherapy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.veterinarian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vétérinaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Veterinary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.worship</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lieu de culte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Place of worship</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.pickClassifiedPurchase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Récupérer un achat chez un particulier (petites annonces)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pick up an item from a private seller (online marketplace/classifieds)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.dropSomeone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reconduire quelqu'un</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drop someone off</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.fetchSomeone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aller chercher quelqu'un</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pick someone up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.accompanySomeone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accompagner quelqu'un</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accompany someone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.leisureStroll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Promenade sans destination fixe (ex. : aller courir, promener le chien)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stroll with no fixed destination (ex: go running/jogging, walk with pet, etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.leisureSports</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sport, entrainement, aller au parc (destination fixe)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sport, training, park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.leisureArtsMusicCulture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arts, Musique ou culture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arts, Music ou culture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.leisureTourism</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vacances, tourisme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vacation, tourism</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.visiting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visite chez ami.e.s, copain.e ou famille</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visiting friends, partner or family</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.secondaryHome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Résidence secondaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Secondary residence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">activities.schoolNotStudent</t>
   </si>
   <si>
     <t xml:space="preserve">onTheRoadNextPlaceCategoryChoices.wentBackHome</t>
@@ -9356,7 +9356,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="107">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -9714,6 +9714,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -14547,7 +14551,7 @@
       <c r="V75" s="18"/>
       <c r="W75" s="18"/>
     </row>
-    <row r="76" s="2" customFormat="true" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" s="2" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="28" t="s">
         <v>449</v>
       </c>
@@ -24136,7 +24140,7 @@
         <v>1142</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="77" t="s">
         <v>385</v>
       </c>
@@ -24152,6 +24156,10 @@
       <c r="E75" s="65" t="s">
         <v>1142</v>
       </c>
+      <c r="F75" s="65"/>
+      <c r="G75" s="65"/>
+      <c r="H75" s="65"/>
+      <c r="I75" s="65"/>
     </row>
     <row r="76" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="11" t="s">
@@ -24314,11 +24322,10 @@
       <c r="F84" s="65"/>
       <c r="G84" s="65"/>
     </row>
-    <row r="85" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="65" t="s">
         <v>659</v>
       </c>
-      <c r="B85" s="65"/>
       <c r="C85" s="65" t="s">
         <v>1211</v>
       </c>
@@ -24328,8 +24335,8 @@
       <c r="E85" s="35" t="s">
         <v>1212</v>
       </c>
-      <c r="F85" s="65"/>
-      <c r="G85" s="65"/>
+      <c r="H85" s="2"/>
+      <c r="I85" s="2"/>
     </row>
     <row r="86" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="65" t="s">
@@ -24694,7 +24701,7 @@
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
     </row>
-    <row r="104" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" s="2" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="11" t="s">
         <v>111</v>
       </c>
@@ -24714,8 +24721,6 @@
         <v>1184</v>
       </c>
       <c r="G104" s="10"/>
-      <c r="H104" s="2"/>
-      <c r="I104" s="2"/>
     </row>
     <row r="105" s="2" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
@@ -24875,11 +24880,10 @@
       <c r="F112" s="65"/>
       <c r="G112" s="65"/>
     </row>
-    <row r="113" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="65" t="s">
         <v>123</v>
       </c>
-      <c r="B113" s="65"/>
       <c r="C113" s="28" t="s">
         <v>85</v>
       </c>
@@ -24889,12 +24893,13 @@
       <c r="E113" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="F113" s="65"/>
       <c r="G113" s="65" t="s">
         <v>1200</v>
       </c>
-    </row>
-    <row r="114" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H113" s="2"/>
+      <c r="I113" s="2"/>
+    </row>
+    <row r="114" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="65" t="s">
         <v>123</v>
       </c>
@@ -24910,8 +24915,8 @@
       <c r="E114" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="H114" s="2"/>
-      <c r="I114" s="2"/>
+      <c r="F114" s="65"/>
+      <c r="G114" s="65"/>
     </row>
     <row r="115" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="65" t="s">
@@ -24950,7 +24955,7 @@
       </c>
       <c r="G116" s="65"/>
     </row>
-    <row r="117" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="65" t="s">
         <v>183</v>
       </c>
@@ -24966,8 +24971,8 @@
       <c r="E117" s="35" t="n">
         <v>6</v>
       </c>
-      <c r="F117" s="65"/>
-      <c r="G117" s="65"/>
+      <c r="H117" s="2"/>
+      <c r="I117" s="2"/>
     </row>
     <row r="118" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="65" t="s">
@@ -25008,7 +25013,7 @@
       <c r="H119" s="2"/>
       <c r="I119" s="2"/>
     </row>
-    <row r="120" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="65" t="s">
         <v>188</v>
       </c>
@@ -25027,8 +25032,7 @@
       <c r="F120" s="65" t="s">
         <v>1183</v>
       </c>
-      <c r="H120" s="2"/>
-      <c r="I120" s="2"/>
+      <c r="G120" s="65"/>
     </row>
     <row r="121" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="65" t="s">
@@ -25104,7 +25108,7 @@
       <c r="F124" s="65"/>
       <c r="G124" s="65"/>
     </row>
-    <row r="125" s="2" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
         <v>202</v>
       </c>
@@ -25120,8 +25124,8 @@
       <c r="E125" s="35" t="s">
         <v>1142</v>
       </c>
-      <c r="F125" s="65"/>
-      <c r="G125" s="65"/>
+      <c r="H125" s="2"/>
+      <c r="I125" s="2"/>
     </row>
     <row r="126" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="65" t="s">
@@ -26048,7 +26052,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F227"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="16.72"/>
@@ -27134,34 +27138,32 @@
       <c r="E68" s="28"/>
       <c r="F68" s="28"/>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="22" t="s">
+    <row r="69" s="90" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="90" t="s">
         <v>431</v>
       </c>
-      <c r="B69" s="10" t="s">
+      <c r="B69" s="90" t="s">
         <v>1552</v>
       </c>
-      <c r="C69" s="28" t="s">
+      <c r="C69" s="90" t="s">
         <v>1553</v>
       </c>
-      <c r="D69" s="28" t="s">
+      <c r="D69" s="90" t="s">
         <v>1554</v>
       </c>
-      <c r="E69" s="28"/>
-      <c r="F69" s="28"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="22" t="s">
         <v>431</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>1552</v>
+        <v>1555</v>
       </c>
       <c r="C70" s="28" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="D70" s="28" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="E70" s="28"/>
       <c r="F70" s="28"/>
@@ -27171,13 +27173,13 @@
         <v>431</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="C71" s="28" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="D71" s="28" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="E71" s="28"/>
       <c r="F71" s="28"/>
@@ -27187,13 +27189,13 @@
         <v>431</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="C72" s="28" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="D72" s="28" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="E72" s="28"/>
       <c r="F72" s="28"/>
@@ -27203,13 +27205,13 @@
         <v>431</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="C73" s="28" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="D73" s="28" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="E73" s="28"/>
       <c r="F73" s="28"/>
@@ -27219,13 +27221,13 @@
         <v>431</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="C74" s="28" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="D74" s="28" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="E74" s="28"/>
       <c r="F74" s="28"/>
@@ -27235,13 +27237,13 @@
         <v>431</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="C75" s="28" t="s">
-        <v>1570</v>
+        <v>1245</v>
       </c>
       <c r="D75" s="28" t="s">
-        <v>1571</v>
+        <v>1246</v>
       </c>
       <c r="E75" s="28"/>
       <c r="F75" s="28"/>
@@ -27251,13 +27253,13 @@
         <v>431</v>
       </c>
       <c r="B76" s="10" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C76" s="28" t="s">
         <v>1572</v>
       </c>
-      <c r="C76" s="28" t="s">
-        <v>1245</v>
-      </c>
       <c r="D76" s="28" t="s">
-        <v>1246</v>
+        <v>1573</v>
       </c>
       <c r="E76" s="28"/>
       <c r="F76" s="28"/>
@@ -27267,13 +27269,13 @@
         <v>431</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="C77" s="28" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="D77" s="28" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="E77" s="28"/>
       <c r="F77" s="28"/>
@@ -27283,13 +27285,13 @@
         <v>431</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
       <c r="C78" s="28" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="D78" s="28" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="E78" s="28"/>
       <c r="F78" s="28"/>
@@ -27299,13 +27301,13 @@
         <v>431</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="C79" s="28" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="D79" s="28" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="E79" s="28"/>
       <c r="F79" s="28"/>
@@ -27315,13 +27317,13 @@
         <v>431</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="C80" s="28" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="D80" s="28" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="E80" s="28"/>
       <c r="F80" s="28"/>
@@ -27331,13 +27333,13 @@
         <v>431</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="C81" s="28" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="D81" s="28" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="E81" s="28"/>
       <c r="F81" s="28"/>
@@ -27347,13 +27349,13 @@
         <v>431</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="C82" s="28" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="D82" s="28" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="E82" s="28"/>
       <c r="F82" s="28"/>
@@ -27363,13 +27365,13 @@
         <v>431</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="C83" s="28" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
       <c r="D83" s="28" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="E83" s="28"/>
       <c r="F83" s="28"/>
@@ -27379,13 +27381,13 @@
         <v>431</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="C84" s="28" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="D84" s="28" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
       <c r="E84" s="28"/>
       <c r="F84" s="28"/>
@@ -27395,13 +27397,13 @@
         <v>431</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="C85" s="28" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="D85" s="28" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="E85" s="28"/>
       <c r="F85" s="28"/>
@@ -27411,13 +27413,13 @@
         <v>431</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="C86" s="28" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="D86" s="28" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="E86" s="28"/>
       <c r="F86" s="28"/>
@@ -27427,13 +27429,13 @@
         <v>431</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="C87" s="28" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="D87" s="28" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="E87" s="28"/>
       <c r="F87" s="28"/>
@@ -27443,13 +27445,13 @@
         <v>431</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="C88" s="28" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="D88" s="28" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="E88" s="28"/>
       <c r="F88" s="28"/>
@@ -27459,13 +27461,13 @@
         <v>431</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="C89" s="28" t="s">
-        <v>1610</v>
+        <v>1565</v>
       </c>
       <c r="D89" s="28" t="s">
-        <v>1611</v>
+        <v>1566</v>
       </c>
       <c r="E89" s="28"/>
       <c r="F89" s="28"/>
@@ -27475,13 +27477,13 @@
         <v>431</v>
       </c>
       <c r="B90" s="10" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C90" s="28" t="s">
         <v>1612</v>
       </c>
-      <c r="C90" s="28" t="s">
-        <v>1567</v>
-      </c>
       <c r="D90" s="28" t="s">
-        <v>1568</v>
+        <v>1613</v>
       </c>
       <c r="E90" s="28"/>
       <c r="F90" s="28"/>
@@ -27491,13 +27493,13 @@
         <v>431</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="D91" s="28" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="E91" s="28"/>
       <c r="F91" s="28"/>
@@ -27507,13 +27509,13 @@
         <v>431</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="D92" s="28" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="E92" s="28"/>
       <c r="F92" s="28"/>
@@ -27523,13 +27525,13 @@
         <v>431</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="D93" s="28" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="E93" s="28"/>
       <c r="F93" s="28"/>
@@ -27539,13 +27541,13 @@
         <v>431</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="D94" s="28" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="E94" s="28"/>
       <c r="F94" s="28"/>
@@ -27555,13 +27557,13 @@
         <v>431</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="D95" s="28" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="E95" s="28"/>
       <c r="F95" s="28"/>
@@ -27571,13 +27573,13 @@
         <v>431</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="D96" s="28" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="E96" s="28"/>
       <c r="F96" s="28"/>
@@ -27587,13 +27589,13 @@
         <v>431</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="D97" s="28" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="E97" s="28"/>
       <c r="F97" s="28"/>
@@ -27603,13 +27605,13 @@
         <v>431</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>1634</v>
+        <v>1580</v>
       </c>
       <c r="C98" s="28" t="s">
-        <v>1635</v>
+        <v>1581</v>
       </c>
       <c r="D98" s="28" t="s">
-        <v>1636</v>
+        <v>1582</v>
       </c>
       <c r="E98" s="28"/>
       <c r="F98" s="28"/>
@@ -27619,13 +27621,13 @@
         <v>431</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>1582</v>
+        <v>1635</v>
       </c>
       <c r="C99" s="28" t="s">
-        <v>1583</v>
+        <v>1636</v>
       </c>
       <c r="D99" s="28" t="s">
-        <v>1584</v>
+        <v>1637</v>
       </c>
       <c r="E99" s="28"/>
       <c r="F99" s="28"/>
@@ -27635,99 +27637,91 @@
         <v>431</v>
       </c>
       <c r="B100" s="10" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="C100" s="28" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="D100" s="28" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
       <c r="E100" s="28"/>
       <c r="F100" s="28"/>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A101" s="22" t="s">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="B101" s="10" t="s">
-        <v>1640</v>
-      </c>
-      <c r="C101" s="28" t="s">
-        <v>1555</v>
-      </c>
-      <c r="D101" s="28" t="s">
-        <v>1556</v>
-      </c>
-      <c r="E101" s="28"/>
-      <c r="F101" s="28"/>
+      <c r="B101" s="2" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>1245</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>1246</v>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="0" t="s">
+      <c r="A102" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="B102" s="0" t="s">
-        <v>1641</v>
-      </c>
-      <c r="C102" s="0" t="s">
-        <v>1245</v>
-      </c>
-      <c r="D102" s="0" t="s">
-        <v>1246</v>
-      </c>
-      <c r="E102" s="0"/>
-      <c r="F102" s="0"/>
+      <c r="B102" s="2" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>1643</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>1644</v>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0" t="s">
+      <c r="A103" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="B103" s="0" t="s">
-        <v>1642</v>
-      </c>
-      <c r="C103" s="0" t="s">
-        <v>1643</v>
-      </c>
-      <c r="D103" s="0" t="s">
-        <v>1644</v>
-      </c>
-      <c r="E103" s="0"/>
-      <c r="F103" s="0"/>
+      <c r="B103" s="2" t="s">
+        <v>1645</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>1646</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>1647</v>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="0" t="s">
+      <c r="A104" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="B104" s="0" t="s">
-        <v>1645</v>
-      </c>
-      <c r="C104" s="0" t="s">
-        <v>1646</v>
-      </c>
-      <c r="D104" s="0" t="s">
-        <v>1647</v>
-      </c>
-      <c r="E104" s="0"/>
-      <c r="F104" s="0"/>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="0" t="s">
-        <v>431</v>
-      </c>
-      <c r="B105" s="0" t="s">
+      <c r="B104" s="2" t="s">
         <v>1648</v>
       </c>
-      <c r="C105" s="0" t="s">
+      <c r="C104" s="2" t="s">
         <v>1649</v>
       </c>
-      <c r="D105" s="0" t="s">
+      <c r="D104" s="2" t="s">
         <v>1650</v>
       </c>
-      <c r="E105" s="0" t="s">
+      <c r="E104" s="2" t="s">
         <v>1651</v>
       </c>
-      <c r="F105" s="0" t="s">
+      <c r="F104" s="2" t="s">
         <v>1652</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>1653</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>1654</v>
+      </c>
+      <c r="D105" s="10" t="s">
+        <v>1655</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27735,13 +27729,13 @@
         <v>152</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>1653</v>
+        <v>1656</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>1654</v>
+        <v>1657</v>
       </c>
       <c r="D106" s="10" t="s">
-        <v>1655</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27749,13 +27743,13 @@
         <v>152</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>1656</v>
+        <v>1659</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>1657</v>
+        <v>1660</v>
       </c>
       <c r="D107" s="10" t="s">
-        <v>1658</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27763,13 +27757,13 @@
         <v>152</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>1659</v>
+        <v>1662</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>1660</v>
+        <v>1663</v>
       </c>
       <c r="D108" s="10" t="s">
-        <v>1661</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27777,41 +27771,41 @@
         <v>152</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>1662</v>
+        <v>1665</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>1663</v>
+        <v>1666</v>
       </c>
       <c r="D109" s="10" t="s">
-        <v>1664</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1667</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B110" s="2" t="s">
-        <v>1665</v>
+      <c r="B110" s="91" t="s">
+        <v>1668</v>
       </c>
       <c r="C110" s="10" t="s">
-        <v>1666</v>
+        <v>1669</v>
       </c>
       <c r="D110" s="10" t="s">
-        <v>1667</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B111" s="90" t="s">
-        <v>1668</v>
+      <c r="B111" s="10" t="s">
+        <v>1671</v>
       </c>
       <c r="C111" s="10" t="s">
-        <v>1669</v>
+        <v>1672</v>
       </c>
       <c r="D111" s="10" t="s">
-        <v>1670</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27819,13 +27813,13 @@
         <v>152</v>
       </c>
       <c r="B112" s="10" t="s">
-        <v>1671</v>
+        <v>1674</v>
       </c>
       <c r="C112" s="10" t="s">
-        <v>1672</v>
+        <v>1675</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>1673</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27833,33 +27827,33 @@
         <v>152</v>
       </c>
       <c r="B113" s="10" t="s">
-        <v>1674</v>
+        <v>1677</v>
       </c>
       <c r="C113" s="10" t="s">
-        <v>1675</v>
-      </c>
-      <c r="D113" s="10" t="s">
-        <v>1676</v>
-      </c>
-    </row>
-    <row r="114" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1678</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>1679</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>1680</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>1681</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B114" s="10" t="s">
-        <v>1677</v>
-      </c>
-      <c r="C114" s="10" t="s">
-        <v>1678</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>1679</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>1680</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>1681</v>
+      <c r="B114" s="45" t="s">
+        <v>1682</v>
+      </c>
+      <c r="C114" s="45" t="s">
+        <v>1683</v>
+      </c>
+      <c r="D114" s="91" t="s">
+        <v>1684</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27867,27 +27861,27 @@
         <v>152</v>
       </c>
       <c r="B115" s="45" t="s">
-        <v>1682</v>
+        <v>1685</v>
       </c>
       <c r="C115" s="45" t="s">
-        <v>1683</v>
-      </c>
-      <c r="D115" s="90" t="s">
-        <v>1684</v>
-      </c>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1686</v>
+      </c>
+      <c r="D115" s="91" t="s">
+        <v>1687</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B116" s="45" t="s">
-        <v>1685</v>
+      <c r="B116" s="10" t="s">
+        <v>1688</v>
       </c>
       <c r="C116" s="45" t="s">
-        <v>1686</v>
-      </c>
-      <c r="D116" s="90" t="s">
-        <v>1687</v>
+        <v>1689</v>
+      </c>
+      <c r="D116" s="91" t="s">
+        <v>1690</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27895,13 +27889,13 @@
         <v>152</v>
       </c>
       <c r="B117" s="10" t="s">
-        <v>1688</v>
-      </c>
-      <c r="C117" s="45" t="s">
-        <v>1689</v>
-      </c>
-      <c r="D117" s="90" t="s">
-        <v>1690</v>
+        <v>1691</v>
+      </c>
+      <c r="C117" s="28" t="s">
+        <v>1692</v>
+      </c>
+      <c r="D117" s="28" t="s">
+        <v>1693</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27909,41 +27903,43 @@
         <v>152</v>
       </c>
       <c r="B118" s="10" t="s">
-        <v>1691</v>
-      </c>
-      <c r="C118" s="28" t="s">
-        <v>1692</v>
-      </c>
-      <c r="D118" s="28" t="s">
-        <v>1693</v>
+        <v>1694</v>
+      </c>
+      <c r="C118" s="92" t="s">
+        <v>1695</v>
+      </c>
+      <c r="D118" s="92" t="s">
+        <v>1695</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B119" s="10" t="s">
-        <v>1694</v>
-      </c>
-      <c r="C119" s="91" t="s">
-        <v>1695</v>
-      </c>
-      <c r="D119" s="91" t="s">
-        <v>1695</v>
-      </c>
+      <c r="A119" s="18" t="s">
+        <v>431</v>
+      </c>
+      <c r="B119" s="35" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C119" s="35" t="s">
+        <v>1245</v>
+      </c>
+      <c r="D119" s="35" t="s">
+        <v>1246</v>
+      </c>
+      <c r="E119" s="35"/>
+      <c r="F119" s="35"/>
     </row>
     <row r="120" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="18" t="s">
         <v>431</v>
       </c>
       <c r="B120" s="35" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="C120" s="35" t="s">
-        <v>1245</v>
+        <v>1643</v>
       </c>
       <c r="D120" s="35" t="s">
-        <v>1246</v>
+        <v>1644</v>
       </c>
       <c r="E120" s="35"/>
       <c r="F120" s="35"/>
@@ -27953,51 +27949,49 @@
         <v>431</v>
       </c>
       <c r="B121" s="35" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="C121" s="35" t="s">
-        <v>1643</v>
+        <v>1646</v>
       </c>
       <c r="D121" s="35" t="s">
-        <v>1644</v>
+        <v>1647</v>
       </c>
       <c r="E121" s="35"/>
       <c r="F121" s="35"/>
     </row>
-    <row r="122" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="18" t="s">
         <v>431</v>
       </c>
-      <c r="B122" s="35" t="s">
-        <v>1698</v>
-      </c>
-      <c r="C122" s="35" t="s">
-        <v>1646</v>
-      </c>
-      <c r="D122" s="35" t="s">
-        <v>1647</v>
-      </c>
-      <c r="E122" s="35"/>
-      <c r="F122" s="35"/>
-    </row>
-    <row r="123" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="18" t="s">
+      <c r="B122" s="10" t="s">
+        <v>1699</v>
+      </c>
+      <c r="C122" s="10" t="s">
+        <v>1649</v>
+      </c>
+      <c r="D122" s="10" t="s">
+        <v>1650</v>
+      </c>
+      <c r="E122" s="10" t="s">
+        <v>1651</v>
+      </c>
+      <c r="F122" s="10" t="s">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="2" t="s">
         <v>431</v>
       </c>
       <c r="B123" s="10" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
       <c r="C123" s="10" t="s">
-        <v>1649</v>
+        <v>1701</v>
       </c>
       <c r="D123" s="10" t="s">
-        <v>1650</v>
-      </c>
-      <c r="E123" s="10" t="s">
-        <v>1651</v>
-      </c>
-      <c r="F123" s="10" t="s">
-        <v>1652</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28005,27 +27999,27 @@
         <v>431</v>
       </c>
       <c r="B124" s="10" t="s">
-        <v>1700</v>
+        <v>1703</v>
       </c>
       <c r="C124" s="10" t="s">
-        <v>1701</v>
+        <v>1704</v>
       </c>
       <c r="D124" s="10" t="s">
-        <v>1702</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1705</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="2" t="s">
         <v>431</v>
       </c>
       <c r="B125" s="10" t="s">
-        <v>1703</v>
+        <v>1706</v>
       </c>
       <c r="C125" s="10" t="s">
-        <v>1704</v>
+        <v>1707</v>
       </c>
       <c r="D125" s="10" t="s">
-        <v>1705</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28033,47 +28027,53 @@
         <v>431</v>
       </c>
       <c r="B126" s="10" t="s">
-        <v>1706</v>
+        <v>1709</v>
       </c>
       <c r="C126" s="10" t="s">
-        <v>1707</v>
+        <v>1710</v>
       </c>
       <c r="D126" s="10" t="s">
-        <v>1708</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="B127" s="10" t="s">
-        <v>1709</v>
+      <c r="A127" s="18" t="s">
+        <v>526</v>
+      </c>
+      <c r="B127" s="35" t="s">
+        <v>1712</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>1710</v>
+        <v>1713</v>
       </c>
       <c r="D127" s="10" t="s">
-        <v>1711</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1714</v>
+      </c>
+      <c r="E127" s="10" t="s">
+        <v>1715</v>
+      </c>
+      <c r="F127" s="10" t="s">
+        <v>1716</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="18" t="s">
         <v>526</v>
       </c>
       <c r="B128" s="35" t="s">
-        <v>1712</v>
+        <v>1717</v>
       </c>
       <c r="C128" s="10" t="s">
-        <v>1713</v>
+        <v>1718</v>
       </c>
       <c r="D128" s="10" t="s">
-        <v>1714</v>
+        <v>1719</v>
       </c>
       <c r="E128" s="10" t="s">
-        <v>1715</v>
+        <v>1720</v>
       </c>
       <c r="F128" s="10" t="s">
-        <v>1716</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28081,33 +28081,29 @@
         <v>526</v>
       </c>
       <c r="B129" s="35" t="s">
-        <v>1717</v>
+        <v>1722</v>
       </c>
       <c r="C129" s="10" t="s">
-        <v>1718</v>
+        <v>1723</v>
       </c>
       <c r="D129" s="10" t="s">
-        <v>1719</v>
-      </c>
-      <c r="E129" s="10" t="s">
-        <v>1720</v>
-      </c>
-      <c r="F129" s="10" t="s">
-        <v>1721</v>
-      </c>
+        <v>1724</v>
+      </c>
+      <c r="E129" s="10"/>
+      <c r="F129" s="10"/>
     </row>
     <row r="130" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="18" t="s">
         <v>526</v>
       </c>
       <c r="B130" s="35" t="s">
-        <v>1722</v>
+        <v>1725</v>
       </c>
       <c r="C130" s="10" t="s">
-        <v>1723</v>
+        <v>1726</v>
       </c>
       <c r="D130" s="10" t="s">
-        <v>1724</v>
+        <v>1727</v>
       </c>
       <c r="E130" s="10"/>
       <c r="F130" s="10"/>
@@ -28117,29 +28113,29 @@
         <v>526</v>
       </c>
       <c r="B131" s="35" t="s">
-        <v>1725</v>
+        <v>1728</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>1726</v>
+        <v>1729</v>
       </c>
       <c r="D131" s="10" t="s">
-        <v>1727</v>
+        <v>1730</v>
       </c>
       <c r="E131" s="10"/>
       <c r="F131" s="10"/>
     </row>
-    <row r="132" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="18" t="s">
         <v>526</v>
       </c>
-      <c r="B132" s="35" t="s">
-        <v>1728</v>
+      <c r="B132" s="10" t="s">
+        <v>1731</v>
       </c>
       <c r="C132" s="10" t="s">
-        <v>1729</v>
+        <v>1732</v>
       </c>
       <c r="D132" s="10" t="s">
-        <v>1730</v>
+        <v>1733</v>
       </c>
       <c r="E132" s="10"/>
       <c r="F132" s="10"/>
@@ -28149,13 +28145,13 @@
         <v>526</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>1731</v>
-      </c>
-      <c r="C133" s="10" t="s">
-        <v>1732</v>
-      </c>
-      <c r="D133" s="10" t="s">
-        <v>1733</v>
+        <v>1734</v>
+      </c>
+      <c r="C133" s="11" t="s">
+        <v>1735</v>
+      </c>
+      <c r="D133" s="11" t="s">
+        <v>1736</v>
       </c>
       <c r="E133" s="10"/>
       <c r="F133" s="10"/>
@@ -28165,13 +28161,13 @@
         <v>526</v>
       </c>
       <c r="B134" s="10" t="s">
-        <v>1734</v>
+        <v>1737</v>
       </c>
       <c r="C134" s="11" t="s">
-        <v>1735</v>
+        <v>1738</v>
       </c>
       <c r="D134" s="11" t="s">
-        <v>1736</v>
+        <v>1739</v>
       </c>
       <c r="E134" s="10"/>
       <c r="F134" s="10"/>
@@ -28181,29 +28177,29 @@
         <v>526</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>1737</v>
+        <v>1740</v>
       </c>
       <c r="C135" s="11" t="s">
-        <v>1738</v>
+        <v>1741</v>
       </c>
       <c r="D135" s="11" t="s">
-        <v>1739</v>
+        <v>1742</v>
       </c>
       <c r="E135" s="10"/>
       <c r="F135" s="10"/>
     </row>
-    <row r="136" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="18" t="s">
         <v>526</v>
       </c>
       <c r="B136" s="10" t="s">
-        <v>1740</v>
+        <v>1743</v>
       </c>
       <c r="C136" s="11" t="s">
-        <v>1741</v>
+        <v>1744</v>
       </c>
       <c r="D136" s="11" t="s">
-        <v>1742</v>
+        <v>1745</v>
       </c>
       <c r="E136" s="10"/>
       <c r="F136" s="10"/>
@@ -28212,14 +28208,14 @@
       <c r="A137" s="18" t="s">
         <v>526</v>
       </c>
-      <c r="B137" s="10" t="s">
-        <v>1743</v>
+      <c r="B137" s="45" t="s">
+        <v>1746</v>
       </c>
       <c r="C137" s="11" t="s">
-        <v>1744</v>
+        <v>1747</v>
       </c>
       <c r="D137" s="11" t="s">
-        <v>1745</v>
+        <v>1748</v>
       </c>
       <c r="E137" s="10"/>
       <c r="F137" s="10"/>
@@ -28229,13 +28225,13 @@
         <v>526</v>
       </c>
       <c r="B138" s="45" t="s">
-        <v>1746</v>
+        <v>1749</v>
       </c>
       <c r="C138" s="11" t="s">
-        <v>1747</v>
+        <v>1750</v>
       </c>
       <c r="D138" s="11" t="s">
-        <v>1748</v>
+        <v>1751</v>
       </c>
       <c r="E138" s="10"/>
       <c r="F138" s="10"/>
@@ -28245,13 +28241,13 @@
         <v>526</v>
       </c>
       <c r="B139" s="45" t="s">
-        <v>1749</v>
+        <v>1752</v>
       </c>
       <c r="C139" s="11" t="s">
-        <v>1750</v>
+        <v>1753</v>
       </c>
       <c r="D139" s="11" t="s">
-        <v>1751</v>
+        <v>1754</v>
       </c>
       <c r="E139" s="10"/>
       <c r="F139" s="10"/>
@@ -28261,13 +28257,13 @@
         <v>526</v>
       </c>
       <c r="B140" s="45" t="s">
-        <v>1752</v>
+        <v>1755</v>
       </c>
       <c r="C140" s="11" t="s">
-        <v>1753</v>
+        <v>1756</v>
       </c>
       <c r="D140" s="11" t="s">
-        <v>1754</v>
+        <v>1757</v>
       </c>
       <c r="E140" s="10"/>
       <c r="F140" s="10"/>
@@ -28277,13 +28273,13 @@
         <v>526</v>
       </c>
       <c r="B141" s="45" t="s">
-        <v>1755</v>
+        <v>1758</v>
       </c>
       <c r="C141" s="11" t="s">
-        <v>1756</v>
+        <v>1759</v>
       </c>
       <c r="D141" s="11" t="s">
-        <v>1757</v>
+        <v>1760</v>
       </c>
       <c r="E141" s="10"/>
       <c r="F141" s="10"/>
@@ -28293,13 +28289,13 @@
         <v>526</v>
       </c>
       <c r="B142" s="45" t="s">
-        <v>1758</v>
+        <v>1761</v>
       </c>
       <c r="C142" s="11" t="s">
-        <v>1759</v>
+        <v>1762</v>
       </c>
       <c r="D142" s="11" t="s">
-        <v>1760</v>
+        <v>1763</v>
       </c>
       <c r="E142" s="10"/>
       <c r="F142" s="10"/>
@@ -28309,13 +28305,13 @@
         <v>526</v>
       </c>
       <c r="B143" s="45" t="s">
-        <v>1761</v>
+        <v>1764</v>
       </c>
       <c r="C143" s="11" t="s">
-        <v>1762</v>
+        <v>1765</v>
       </c>
       <c r="D143" s="11" t="s">
-        <v>1763</v>
+        <v>1766</v>
       </c>
       <c r="E143" s="10"/>
       <c r="F143" s="10"/>
@@ -28325,13 +28321,13 @@
         <v>526</v>
       </c>
       <c r="B144" s="45" t="s">
-        <v>1764</v>
+        <v>1767</v>
       </c>
       <c r="C144" s="11" t="s">
-        <v>1765</v>
+        <v>1756</v>
       </c>
       <c r="D144" s="11" t="s">
-        <v>1766</v>
+        <v>1757</v>
       </c>
       <c r="E144" s="10"/>
       <c r="F144" s="10"/>
@@ -28341,13 +28337,13 @@
         <v>526</v>
       </c>
       <c r="B145" s="45" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
       <c r="C145" s="11" t="s">
-        <v>1756</v>
+        <v>1769</v>
       </c>
       <c r="D145" s="11" t="s">
-        <v>1757</v>
+        <v>1770</v>
       </c>
       <c r="E145" s="10"/>
       <c r="F145" s="10"/>
@@ -28357,13 +28353,13 @@
         <v>526</v>
       </c>
       <c r="B146" s="45" t="s">
-        <v>1768</v>
+        <v>1771</v>
       </c>
       <c r="C146" s="11" t="s">
-        <v>1769</v>
+        <v>1772</v>
       </c>
       <c r="D146" s="11" t="s">
-        <v>1770</v>
+        <v>1773</v>
       </c>
       <c r="E146" s="10"/>
       <c r="F146" s="10"/>
@@ -28373,13 +28369,13 @@
         <v>526</v>
       </c>
       <c r="B147" s="45" t="s">
-        <v>1771</v>
+        <v>1774</v>
       </c>
       <c r="C147" s="11" t="s">
-        <v>1772</v>
+        <v>1775</v>
       </c>
       <c r="D147" s="11" t="s">
-        <v>1773</v>
+        <v>1776</v>
       </c>
       <c r="E147" s="10"/>
       <c r="F147" s="10"/>
@@ -28389,13 +28385,13 @@
         <v>526</v>
       </c>
       <c r="B148" s="45" t="s">
-        <v>1774</v>
+        <v>1777</v>
       </c>
       <c r="C148" s="11" t="s">
-        <v>1775</v>
+        <v>1778</v>
       </c>
       <c r="D148" s="11" t="s">
-        <v>1776</v>
+        <v>1779</v>
       </c>
       <c r="E148" s="10"/>
       <c r="F148" s="10"/>
@@ -28405,13 +28401,13 @@
         <v>526</v>
       </c>
       <c r="B149" s="45" t="s">
-        <v>1777</v>
+        <v>1780</v>
       </c>
       <c r="C149" s="11" t="s">
-        <v>1778</v>
+        <v>1781</v>
       </c>
       <c r="D149" s="11" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
       <c r="E149" s="10"/>
       <c r="F149" s="10"/>
@@ -28421,13 +28417,13 @@
         <v>526</v>
       </c>
       <c r="B150" s="45" t="s">
-        <v>1780</v>
+        <v>1783</v>
       </c>
       <c r="C150" s="11" t="s">
-        <v>1781</v>
+        <v>1784</v>
       </c>
       <c r="D150" s="11" t="s">
-        <v>1782</v>
+        <v>1785</v>
       </c>
       <c r="E150" s="10"/>
       <c r="F150" s="10"/>
@@ -28437,13 +28433,13 @@
         <v>526</v>
       </c>
       <c r="B151" s="45" t="s">
-        <v>1783</v>
+        <v>1786</v>
       </c>
       <c r="C151" s="11" t="s">
-        <v>1784</v>
+        <v>1787</v>
       </c>
       <c r="D151" s="11" t="s">
-        <v>1785</v>
+        <v>1788</v>
       </c>
       <c r="E151" s="10"/>
       <c r="F151" s="10"/>
@@ -28453,13 +28449,13 @@
         <v>526</v>
       </c>
       <c r="B152" s="45" t="s">
-        <v>1786</v>
+        <v>1789</v>
       </c>
       <c r="C152" s="11" t="s">
-        <v>1787</v>
+        <v>1790</v>
       </c>
       <c r="D152" s="11" t="s">
-        <v>1788</v>
+        <v>1791</v>
       </c>
       <c r="E152" s="10"/>
       <c r="F152" s="10"/>
@@ -28469,13 +28465,13 @@
         <v>526</v>
       </c>
       <c r="B153" s="45" t="s">
-        <v>1789</v>
+        <v>1792</v>
       </c>
       <c r="C153" s="11" t="s">
-        <v>1790</v>
+        <v>1793</v>
       </c>
       <c r="D153" s="11" t="s">
-        <v>1791</v>
+        <v>1794</v>
       </c>
       <c r="E153" s="10"/>
       <c r="F153" s="10"/>
@@ -28485,13 +28481,13 @@
         <v>526</v>
       </c>
       <c r="B154" s="45" t="s">
-        <v>1792</v>
+        <v>1795</v>
       </c>
       <c r="C154" s="11" t="s">
-        <v>1793</v>
+        <v>1784</v>
       </c>
       <c r="D154" s="11" t="s">
-        <v>1794</v>
+        <v>1785</v>
       </c>
       <c r="E154" s="10"/>
       <c r="F154" s="10"/>
@@ -28501,13 +28497,13 @@
         <v>526</v>
       </c>
       <c r="B155" s="45" t="s">
-        <v>1795</v>
+        <v>1796</v>
       </c>
       <c r="C155" s="11" t="s">
-        <v>1784</v>
+        <v>1797</v>
       </c>
       <c r="D155" s="11" t="s">
-        <v>1785</v>
+        <v>1798</v>
       </c>
       <c r="E155" s="10"/>
       <c r="F155" s="10"/>
@@ -28517,183 +28513,187 @@
         <v>526</v>
       </c>
       <c r="B156" s="45" t="s">
-        <v>1796</v>
+        <v>1799</v>
       </c>
       <c r="C156" s="11" t="s">
-        <v>1797</v>
+        <v>1800</v>
       </c>
       <c r="D156" s="11" t="s">
-        <v>1798</v>
+        <v>1801</v>
       </c>
       <c r="E156" s="10"/>
       <c r="F156" s="10"/>
     </row>
-    <row r="157" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="18" t="s">
-        <v>526</v>
-      </c>
-      <c r="B157" s="45" t="s">
-        <v>1799</v>
-      </c>
-      <c r="C157" s="11" t="s">
-        <v>1800</v>
-      </c>
-      <c r="D157" s="11" t="s">
-        <v>1801</v>
-      </c>
-      <c r="E157" s="10"/>
-      <c r="F157" s="10"/>
-    </row>
-    <row r="158" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B157" s="1" t="s">
+        <v>1802</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>1803</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>1804</v>
+      </c>
+      <c r="E157" s="1" t="s">
+        <v>1805</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>1806</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="2" t="s">
         <v>152</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>1802</v>
+        <v>1807</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>1803</v>
+        <v>1808</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>1804</v>
+        <v>1809</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>1805</v>
+        <v>1810</v>
       </c>
       <c r="F158" s="1" t="s">
-        <v>1806</v>
-      </c>
-    </row>
-    <row r="159" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1811</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B159" s="1" t="s">
-        <v>1807</v>
+      <c r="B159" s="93" t="s">
+        <v>1812</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>1808</v>
+        <v>1813</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>1809</v>
+        <v>1814</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>1810</v>
+        <v>1815</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>1811</v>
-      </c>
-    </row>
-    <row r="160" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1816</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B160" s="92" t="s">
-        <v>1812</v>
+      <c r="B160" s="93" t="s">
+        <v>1817</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>1813</v>
+        <v>1818</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>1814</v>
+        <v>1819</v>
       </c>
       <c r="E160" s="1" t="s">
-        <v>1815</v>
+        <v>1820</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>1816</v>
+        <v>1821</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B161" s="92" t="s">
-        <v>1817</v>
+      <c r="B161" s="93" t="s">
+        <v>1822</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>1818</v>
+        <v>1823</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>1819</v>
+        <v>1824</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>1820</v>
+        <v>1825</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="162" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="B162" s="92" t="s">
-        <v>1822</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>1823</v>
-      </c>
-      <c r="D162" s="1" t="s">
-        <v>1824</v>
-      </c>
-      <c r="E162" s="1" t="s">
-        <v>1825</v>
-      </c>
-      <c r="F162" s="1" t="s">
-        <v>1826</v>
-      </c>
+        <v>342</v>
+      </c>
+      <c r="B162" s="94" t="s">
+        <v>1827</v>
+      </c>
+      <c r="C162" s="65" t="s">
+        <v>1828</v>
+      </c>
+      <c r="D162" s="28" t="s">
+        <v>1829</v>
+      </c>
+      <c r="E162" s="10"/>
+      <c r="F162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="B163" s="93" t="s">
-        <v>1827</v>
-      </c>
-      <c r="C163" s="65" t="s">
-        <v>1828</v>
-      </c>
-      <c r="D163" s="28" t="s">
-        <v>1829</v>
+      <c r="B163" s="10" t="s">
+        <v>1830</v>
+      </c>
+      <c r="C163" s="10" t="s">
+        <v>1831</v>
+      </c>
+      <c r="D163" s="10" t="s">
+        <v>1832</v>
       </c>
       <c r="E163" s="10"/>
       <c r="F163" s="10"/>
     </row>
-    <row r="164" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="B164" s="10" t="s">
-        <v>1830</v>
+      <c r="B164" s="2" t="s">
+        <v>1833</v>
       </c>
       <c r="C164" s="10" t="s">
-        <v>1831</v>
+        <v>1834</v>
       </c>
       <c r="D164" s="10" t="s">
-        <v>1832</v>
-      </c>
-      <c r="E164" s="10"/>
-      <c r="F164" s="10"/>
+        <v>1835</v>
+      </c>
+      <c r="E164" s="10" t="s">
+        <v>1836</v>
+      </c>
+      <c r="F164" s="10" t="s">
+        <v>1837</v>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="2" t="s">
         <v>342</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>1833</v>
+        <v>1838</v>
       </c>
       <c r="C165" s="10" t="s">
-        <v>1834</v>
+        <v>1839</v>
       </c>
       <c r="D165" s="10" t="s">
-        <v>1835</v>
+        <v>1840</v>
       </c>
       <c r="E165" s="10" t="s">
-        <v>1836</v>
+        <v>1841</v>
       </c>
       <c r="F165" s="10" t="s">
-        <v>1837</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28701,59 +28701,59 @@
         <v>342</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>1838</v>
-      </c>
-      <c r="C166" s="10" t="s">
-        <v>1839</v>
-      </c>
-      <c r="D166" s="10" t="s">
-        <v>1840</v>
-      </c>
-      <c r="E166" s="10" t="s">
-        <v>1841</v>
-      </c>
-      <c r="F166" s="10" t="s">
-        <v>1842</v>
-      </c>
-    </row>
-    <row r="167" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1843</v>
+      </c>
+      <c r="C166" s="28" t="s">
+        <v>1844</v>
+      </c>
+      <c r="D166" s="28" t="s">
+        <v>1845</v>
+      </c>
+      <c r="E166" s="28" t="s">
+        <v>1846</v>
+      </c>
+      <c r="F166" s="28" t="s">
+        <v>1847</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="2" t="s">
         <v>342</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>1843</v>
+        <v>1848</v>
       </c>
       <c r="C167" s="28" t="s">
-        <v>1844</v>
+        <v>1849</v>
       </c>
       <c r="D167" s="28" t="s">
-        <v>1845</v>
+        <v>1850</v>
       </c>
       <c r="E167" s="28" t="s">
-        <v>1846</v>
+        <v>1851</v>
       </c>
       <c r="F167" s="28" t="s">
-        <v>1847</v>
-      </c>
-    </row>
-    <row r="168" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1852</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="2" t="s">
         <v>342</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>1848</v>
+        <v>1853</v>
       </c>
       <c r="C168" s="28" t="s">
-        <v>1849</v>
+        <v>1854</v>
       </c>
       <c r="D168" s="28" t="s">
-        <v>1850</v>
+        <v>1855</v>
       </c>
       <c r="E168" s="28" t="s">
-        <v>1851</v>
+        <v>1856</v>
       </c>
       <c r="F168" s="28" t="s">
-        <v>1852</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28761,39 +28761,39 @@
         <v>342</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>1853</v>
+        <v>1858</v>
       </c>
       <c r="C169" s="28" t="s">
-        <v>1854</v>
-      </c>
-      <c r="D169" s="28" t="s">
-        <v>1855</v>
+        <v>1859</v>
+      </c>
+      <c r="D169" s="65" t="s">
+        <v>1860</v>
       </c>
       <c r="E169" s="28" t="s">
-        <v>1856</v>
-      </c>
-      <c r="F169" s="28" t="s">
-        <v>1857</v>
-      </c>
-    </row>
-    <row r="170" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1861</v>
+      </c>
+      <c r="F169" s="65" t="s">
+        <v>1862</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="B170" s="2" t="s">
-        <v>1858</v>
+      <c r="B170" s="10" t="s">
+        <v>1863</v>
       </c>
       <c r="C170" s="28" t="s">
-        <v>1859</v>
+        <v>1864</v>
       </c>
       <c r="D170" s="65" t="s">
-        <v>1860</v>
+        <v>1865</v>
       </c>
       <c r="E170" s="28" t="s">
-        <v>1861</v>
+        <v>1866</v>
       </c>
       <c r="F170" s="65" t="s">
-        <v>1862</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28801,65 +28801,59 @@
         <v>342</v>
       </c>
       <c r="B171" s="10" t="s">
-        <v>1863</v>
+        <v>1868</v>
       </c>
       <c r="C171" s="28" t="s">
-        <v>1864</v>
+        <v>1869</v>
       </c>
       <c r="D171" s="65" t="s">
-        <v>1865</v>
-      </c>
-      <c r="E171" s="28" t="s">
-        <v>1866</v>
-      </c>
-      <c r="F171" s="65" t="s">
-        <v>1867</v>
-      </c>
-    </row>
-    <row r="172" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1870</v>
+      </c>
+      <c r="E171" s="28"/>
+      <c r="F171" s="65"/>
+    </row>
+    <row r="172" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="2" t="s">
         <v>342</v>
       </c>
       <c r="B172" s="10" t="s">
-        <v>1868</v>
+        <v>1871</v>
       </c>
       <c r="C172" s="28" t="s">
-        <v>1869</v>
-      </c>
-      <c r="D172" s="65" t="s">
-        <v>1870</v>
+        <v>1872</v>
+      </c>
+      <c r="D172" s="28" t="s">
+        <v>1873</v>
       </c>
       <c r="E172" s="28"/>
       <c r="F172" s="65"/>
     </row>
-    <row r="173" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="B173" s="10" t="s">
-        <v>1871</v>
-      </c>
-      <c r="C173" s="28" t="s">
-        <v>1872</v>
-      </c>
-      <c r="D173" s="28" t="s">
-        <v>1873</v>
-      </c>
-      <c r="E173" s="28"/>
-      <c r="F173" s="65"/>
+        <v>1027</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>1874</v>
+      </c>
+      <c r="C173" s="10" t="s">
+        <v>1875</v>
+      </c>
+      <c r="D173" s="10" t="s">
+        <v>1876</v>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="2" t="s">
-        <v>1027</v>
+        <v>526</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>1874</v>
+        <v>1877</v>
       </c>
       <c r="C174" s="10" t="s">
-        <v>1875</v>
+        <v>1878</v>
       </c>
       <c r="D174" s="10" t="s">
-        <v>1876</v>
+        <v>1879</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28867,13 +28861,13 @@
         <v>526</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>1877</v>
+        <v>1880</v>
       </c>
       <c r="C175" s="10" t="s">
-        <v>1878</v>
+        <v>1881</v>
       </c>
       <c r="D175" s="10" t="s">
-        <v>1879</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28881,13 +28875,13 @@
         <v>526</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>1880</v>
+        <v>1883</v>
       </c>
       <c r="C176" s="10" t="s">
-        <v>1881</v>
+        <v>1884</v>
       </c>
       <c r="D176" s="10" t="s">
-        <v>1882</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28895,13 +28889,13 @@
         <v>526</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>1883</v>
+        <v>1886</v>
       </c>
       <c r="C177" s="10" t="s">
-        <v>1884</v>
+        <v>1887</v>
       </c>
       <c r="D177" s="10" t="s">
-        <v>1885</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28909,13 +28903,13 @@
         <v>526</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>1886</v>
+        <v>1889</v>
       </c>
       <c r="C178" s="10" t="s">
-        <v>1887</v>
+        <v>1890</v>
       </c>
       <c r="D178" s="10" t="s">
-        <v>1888</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28923,27 +28917,27 @@
         <v>526</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>1889</v>
+        <v>1892</v>
       </c>
       <c r="C179" s="10" t="s">
-        <v>1890</v>
+        <v>1893</v>
       </c>
       <c r="D179" s="10" t="s">
-        <v>1891</v>
-      </c>
-    </row>
-    <row r="180" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1894</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="2" t="s">
         <v>526</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>1892</v>
-      </c>
-      <c r="C180" s="10" t="s">
-        <v>1893</v>
-      </c>
-      <c r="D180" s="10" t="s">
-        <v>1894</v>
+        <v>1895</v>
+      </c>
+      <c r="C180" s="2" t="s">
+        <v>1896</v>
+      </c>
+      <c r="D180" s="2" t="s">
+        <v>1897</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28951,13 +28945,13 @@
         <v>526</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>1895</v>
+        <v>1898</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>1896</v>
+        <v>1899</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>1897</v>
+        <v>1899</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28965,13 +28959,13 @@
         <v>526</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>1898</v>
+        <v>1900</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>1899</v>
+        <v>1901</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>1899</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28979,13 +28973,13 @@
         <v>526</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>1900</v>
+        <v>1903</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>1901</v>
+        <v>1904</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>1902</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28993,13 +28987,13 @@
         <v>526</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>1903</v>
+        <v>1906</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>1904</v>
+        <v>1907</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>1905</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29007,13 +29001,13 @@
         <v>526</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>1906</v>
+        <v>1909</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>1907</v>
+        <v>1910</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>1908</v>
+        <v>1911</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29021,13 +29015,13 @@
         <v>526</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>1909</v>
+        <v>1912</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>1910</v>
+        <v>1913</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>1911</v>
+        <v>1914</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29035,13 +29029,13 @@
         <v>526</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>1912</v>
+        <v>1915</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>1913</v>
+        <v>1916</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>1914</v>
+        <v>1917</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29049,13 +29043,13 @@
         <v>526</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>1915</v>
+        <v>1918</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>1916</v>
+        <v>1919</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>1917</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29063,13 +29057,13 @@
         <v>526</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>1918</v>
+        <v>1921</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>1919</v>
+        <v>1922</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>1920</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29077,13 +29071,13 @@
         <v>526</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>1921</v>
+        <v>1924</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>1922</v>
+        <v>1925</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>1923</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29091,13 +29085,13 @@
         <v>526</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>1924</v>
+        <v>1927</v>
       </c>
       <c r="C191" s="2" t="s">
-        <v>1925</v>
+        <v>1928</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>1926</v>
+        <v>1929</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29105,13 +29099,13 @@
         <v>526</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>1927</v>
+        <v>1930</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>1928</v>
+        <v>1931</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>1929</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29119,13 +29113,13 @@
         <v>526</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>1930</v>
+        <v>1933</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>1931</v>
+        <v>1934</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>1932</v>
+        <v>1935</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29133,13 +29127,13 @@
         <v>526</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>1933</v>
+        <v>1936</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>1934</v>
+        <v>1937</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>1935</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29147,13 +29141,13 @@
         <v>526</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>1936</v>
+        <v>1939</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>1937</v>
+        <v>1940</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>1938</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29161,41 +29155,41 @@
         <v>526</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>1939</v>
+        <v>1942</v>
       </c>
       <c r="C196" s="2" t="s">
-        <v>1940</v>
+        <v>1943</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>1941</v>
-      </c>
-    </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B197" s="2" t="s">
-        <v>1942</v>
-      </c>
-      <c r="C197" s="2" t="s">
-        <v>1943</v>
-      </c>
-      <c r="D197" s="2" t="s">
-        <v>1944</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B197" s="29" t="s">
+        <v>1945</v>
+      </c>
+      <c r="C197" s="65" t="s">
+        <v>1946</v>
+      </c>
+      <c r="D197" s="35" t="s">
+        <v>1947</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B198" s="29" t="s">
-        <v>1945</v>
-      </c>
-      <c r="C198" s="65" t="s">
-        <v>1946</v>
-      </c>
-      <c r="D198" s="35" t="s">
-        <v>1947</v>
+      <c r="B198" s="2" t="s">
+        <v>1948</v>
+      </c>
+      <c r="C198" s="2" t="s">
+        <v>1949</v>
+      </c>
+      <c r="D198" s="2" t="s">
+        <v>1950</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29203,13 +29197,13 @@
         <v>526</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>1948</v>
+        <v>1951</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>1949</v>
+        <v>1952</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>1950</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29217,13 +29211,13 @@
         <v>526</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>1951</v>
+        <v>1954</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>1952</v>
+        <v>1955</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>1953</v>
+        <v>1956</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29231,13 +29225,13 @@
         <v>526</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>1954</v>
+        <v>1957</v>
       </c>
       <c r="C201" s="2" t="s">
-        <v>1955</v>
+        <v>1958</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>1956</v>
+        <v>1959</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29245,41 +29239,41 @@
         <v>526</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>1957</v>
+        <v>1960</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>1958</v>
+        <v>1961</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>1959</v>
-      </c>
-    </row>
-    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1962</v>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="2" t="s">
         <v>526</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>1960</v>
-      </c>
-      <c r="C203" s="2" t="s">
-        <v>1961</v>
-      </c>
-      <c r="D203" s="2" t="s">
-        <v>1962</v>
+        <v>1963</v>
+      </c>
+      <c r="C203" s="65" t="s">
+        <v>1964</v>
+      </c>
+      <c r="D203" s="35" t="s">
+        <v>1965</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B204" s="2" t="s">
-        <v>1963</v>
+      <c r="B204" s="29" t="s">
+        <v>1966</v>
       </c>
       <c r="C204" s="65" t="s">
-        <v>1964</v>
+        <v>1967</v>
       </c>
       <c r="D204" s="35" t="s">
-        <v>1965</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29287,13 +29281,13 @@
         <v>526</v>
       </c>
       <c r="B205" s="29" t="s">
-        <v>1966</v>
+        <v>1969</v>
       </c>
       <c r="C205" s="65" t="s">
-        <v>1967</v>
+        <v>1970</v>
       </c>
       <c r="D205" s="35" t="s">
-        <v>1968</v>
+        <v>1971</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29301,13 +29295,13 @@
         <v>526</v>
       </c>
       <c r="B206" s="29" t="s">
-        <v>1969</v>
+        <v>1972</v>
       </c>
       <c r="C206" s="65" t="s">
-        <v>1970</v>
+        <v>1973</v>
       </c>
       <c r="D206" s="35" t="s">
-        <v>1971</v>
+        <v>1974</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29315,13 +29309,13 @@
         <v>526</v>
       </c>
       <c r="B207" s="29" t="s">
-        <v>1972</v>
+        <v>1975</v>
       </c>
       <c r="C207" s="65" t="s">
-        <v>1973</v>
+        <v>1976</v>
       </c>
       <c r="D207" s="35" t="s">
-        <v>1974</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29329,13 +29323,13 @@
         <v>526</v>
       </c>
       <c r="B208" s="29" t="s">
-        <v>1975</v>
+        <v>1978</v>
       </c>
       <c r="C208" s="65" t="s">
-        <v>1976</v>
+        <v>1979</v>
       </c>
       <c r="D208" s="35" t="s">
-        <v>1977</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29343,13 +29337,13 @@
         <v>526</v>
       </c>
       <c r="B209" s="29" t="s">
-        <v>1978</v>
+        <v>1981</v>
       </c>
       <c r="C209" s="65" t="s">
-        <v>1979</v>
+        <v>1976</v>
       </c>
       <c r="D209" s="35" t="s">
-        <v>1980</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29357,13 +29351,13 @@
         <v>526</v>
       </c>
       <c r="B210" s="29" t="s">
-        <v>1981</v>
+        <v>1982</v>
       </c>
       <c r="C210" s="65" t="s">
-        <v>1976</v>
+        <v>1979</v>
       </c>
       <c r="D210" s="35" t="s">
-        <v>1977</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29371,13 +29365,13 @@
         <v>526</v>
       </c>
       <c r="B211" s="29" t="s">
-        <v>1982</v>
+        <v>1983</v>
       </c>
       <c r="C211" s="65" t="s">
-        <v>1979</v>
+        <v>1946</v>
       </c>
       <c r="D211" s="35" t="s">
-        <v>1980</v>
+        <v>1947</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29385,13 +29379,13 @@
         <v>526</v>
       </c>
       <c r="B212" s="29" t="s">
-        <v>1983</v>
+        <v>1984</v>
       </c>
       <c r="C212" s="65" t="s">
-        <v>1946</v>
+        <v>1985</v>
       </c>
       <c r="D212" s="35" t="s">
-        <v>1947</v>
+        <v>1986</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29399,13 +29393,13 @@
         <v>526</v>
       </c>
       <c r="B213" s="29" t="s">
-        <v>1984</v>
+        <v>1987</v>
       </c>
       <c r="C213" s="65" t="s">
-        <v>1985</v>
+        <v>1988</v>
       </c>
       <c r="D213" s="35" t="s">
-        <v>1986</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29413,179 +29407,179 @@
         <v>526</v>
       </c>
       <c r="B214" s="29" t="s">
-        <v>1987</v>
+        <v>1990</v>
       </c>
       <c r="C214" s="65" t="s">
-        <v>1988</v>
+        <v>1991</v>
       </c>
       <c r="D214" s="35" t="s">
-        <v>1989</v>
-      </c>
-    </row>
-    <row r="215" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1992</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="B215" s="29" t="s">
-        <v>1990</v>
-      </c>
-      <c r="C215" s="65" t="s">
-        <v>1991</v>
+      <c r="B215" s="10" t="s">
+        <v>1993</v>
+      </c>
+      <c r="C215" s="10" t="s">
+        <v>1994</v>
       </c>
       <c r="D215" s="35" t="s">
-        <v>1992</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="2" t="s">
-        <v>526</v>
-      </c>
-      <c r="B216" s="10" t="s">
-        <v>1993</v>
+      <c r="A216" s="21" t="s">
+        <v>729</v>
+      </c>
+      <c r="B216" s="11" t="s">
+        <v>1996</v>
       </c>
       <c r="C216" s="10" t="s">
-        <v>1994</v>
-      </c>
-      <c r="D216" s="35" t="s">
-        <v>1995</v>
-      </c>
-    </row>
-    <row r="217" customFormat="false" ht="30.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A217" s="21" t="s">
+        <v>1997</v>
+      </c>
+      <c r="D216" s="95" t="s">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="2" t="s">
         <v>729</v>
       </c>
-      <c r="B217" s="11" t="s">
-        <v>1996</v>
-      </c>
-      <c r="C217" s="10" t="s">
-        <v>1997</v>
-      </c>
-      <c r="D217" s="94" t="s">
-        <v>1998</v>
-      </c>
-    </row>
-    <row r="218" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B217" s="2" t="s">
+        <v>1999</v>
+      </c>
+      <c r="C217" s="21" t="s">
+        <v>1336</v>
+      </c>
+      <c r="D217" s="28" t="s">
+        <v>1337</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="2" t="s">
         <v>729</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>1999</v>
-      </c>
-      <c r="C218" s="21" t="s">
-        <v>1336</v>
+        <v>2000</v>
+      </c>
+      <c r="C218" s="65" t="s">
+        <v>2001</v>
       </c>
       <c r="D218" s="28" t="s">
-        <v>1337</v>
-      </c>
-    </row>
-    <row r="219" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="268.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="2" t="s">
         <v>729</v>
       </c>
-      <c r="B219" s="2" t="s">
-        <v>2000</v>
-      </c>
-      <c r="C219" s="65" t="s">
-        <v>2001</v>
-      </c>
-      <c r="D219" s="28" t="s">
-        <v>2002</v>
-      </c>
-    </row>
-    <row r="220" customFormat="false" ht="268.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B219" s="22" t="s">
+        <v>2003</v>
+      </c>
+      <c r="C219" s="11" t="s">
+        <v>2004</v>
+      </c>
+      <c r="D219" s="11" t="s">
+        <v>2005</v>
+      </c>
+      <c r="E219" s="11" t="s">
+        <v>2006</v>
+      </c>
+      <c r="F219" s="11" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="223.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="2" t="s">
         <v>729</v>
       </c>
       <c r="B220" s="22" t="s">
-        <v>2003</v>
+        <v>2008</v>
       </c>
       <c r="C220" s="11" t="s">
-        <v>2004</v>
+        <v>2009</v>
       </c>
       <c r="D220" s="11" t="s">
-        <v>2005</v>
+        <v>2010</v>
       </c>
       <c r="E220" s="11" t="s">
-        <v>2006</v>
+        <v>2011</v>
       </c>
       <c r="F220" s="11" t="s">
-        <v>2007</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="223.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="B221" s="22" t="s">
-        <v>2008</v>
-      </c>
-      <c r="C221" s="11" t="s">
-        <v>2009</v>
-      </c>
-      <c r="D221" s="11" t="s">
-        <v>2010</v>
-      </c>
-      <c r="E221" s="11" t="s">
-        <v>2011</v>
-      </c>
-      <c r="F221" s="11" t="s">
-        <v>2012</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>816</v>
+      </c>
+      <c r="B221" s="2" t="s">
+        <v>2013</v>
+      </c>
+      <c r="C221" s="21" t="s">
+        <v>1336</v>
+      </c>
+      <c r="D221" s="28" t="s">
+        <v>1337</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="2" t="s">
         <v>816</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>2013</v>
-      </c>
-      <c r="C222" s="21" t="s">
+        <v>2014</v>
+      </c>
+      <c r="C222" s="65" t="s">
+        <v>2015</v>
+      </c>
+      <c r="D222" s="10" t="s">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B223" s="2" t="s">
+        <v>2017</v>
+      </c>
+      <c r="C223" s="21" t="s">
         <v>1336</v>
       </c>
-      <c r="D222" s="28" t="s">
+      <c r="D223" s="28" t="s">
         <v>1337</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="60.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A223" s="2" t="s">
-        <v>816</v>
-      </c>
-      <c r="B223" s="2" t="s">
-        <v>2014</v>
-      </c>
-      <c r="C223" s="65" t="s">
-        <v>2015</v>
-      </c>
-      <c r="D223" s="10" t="s">
-        <v>2016</v>
-      </c>
-    </row>
-    <row r="224" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="75.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="2" t="s">
         <v>1027</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>2017</v>
-      </c>
-      <c r="C224" s="21" t="s">
-        <v>1336</v>
+        <v>2018</v>
+      </c>
+      <c r="C224" s="65" t="s">
+        <v>2019</v>
       </c>
       <c r="D224" s="28" t="s">
-        <v>1337</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="75.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="2" t="s">
-        <v>1027</v>
-      </c>
-      <c r="B225" s="2" t="s">
-        <v>2018</v>
-      </c>
-      <c r="C225" s="65" t="s">
-        <v>2019</v>
-      </c>
-      <c r="D225" s="28" t="s">
-        <v>2020</v>
+        <v>974</v>
+      </c>
+      <c r="B225" s="11" t="s">
+        <v>2021</v>
+      </c>
+      <c r="C225" s="11" t="s">
+        <v>2022</v>
+      </c>
+      <c r="D225" s="11" t="s">
+        <v>2023</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="75.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29593,29 +29587,16 @@
         <v>974</v>
       </c>
       <c r="B226" s="11" t="s">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C226" s="11" t="s">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="D226" s="11" t="s">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="75.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A227" s="2" t="s">
-        <v>974</v>
-      </c>
-      <c r="B227" s="11" t="s">
-        <v>2024</v>
-      </c>
-      <c r="C227" s="11" t="s">
-        <v>2025</v>
-      </c>
-      <c r="D227" s="11" t="s">
         <v>2026</v>
       </c>
     </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -29644,28 +29625,28 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="96" t="s">
         <v>2027</v>
       </c>
-      <c r="B1" s="95" t="s">
+      <c r="B1" s="96" t="s">
         <v>1134</v>
       </c>
-      <c r="C1" s="95" t="s">
+      <c r="C1" s="96" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="95" t="s">
+      <c r="D1" s="96" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="96" t="s">
+      <c r="E1" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="96" t="s">
+      <c r="F1" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="95" t="s">
+      <c r="G1" s="96" t="s">
         <v>2028</v>
       </c>
-      <c r="H1" s="95" t="s">
+      <c r="H1" s="96" t="s">
         <v>12</v>
       </c>
       <c r="I1" s="29" t="s">
@@ -29734,10 +29715,10 @@
         <v>212</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="E5" s="22"/>
       <c r="F5" s="22"/>
@@ -29917,7 +29898,7 @@
       <c r="I16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="97" t="s">
+      <c r="A17" s="98" t="s">
         <v>2044</v>
       </c>
       <c r="B17" s="22" t="s">
@@ -29935,7 +29916,7 @@
       <c r="H17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="97" t="s">
+      <c r="A18" s="98" t="s">
         <v>2044</v>
       </c>
       <c r="B18" s="22" t="s">
@@ -29953,7 +29934,7 @@
       <c r="H18" s="22"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="97" t="s">
+      <c r="A19" s="98" t="s">
         <v>2044</v>
       </c>
       <c r="B19" s="22"/>
@@ -29967,7 +29948,7 @@
       <c r="H19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="97" t="s">
+      <c r="A20" s="98" t="s">
         <v>170</v>
       </c>
       <c r="B20" s="22" t="s">
@@ -29985,7 +29966,7 @@
       <c r="H20" s="22"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="97" t="s">
+      <c r="A21" s="98" t="s">
         <v>170</v>
       </c>
       <c r="B21" s="22" t="s">
@@ -30003,7 +29984,7 @@
       <c r="H21" s="22"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="97" t="s">
+      <c r="A22" s="98" t="s">
         <v>170</v>
       </c>
       <c r="B22" s="22" t="s">
@@ -30021,7 +30002,7 @@
       <c r="H22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="97" t="s">
+      <c r="A23" s="98" t="s">
         <v>170</v>
       </c>
       <c r="B23" s="22"/>
@@ -30151,7 +30132,7 @@
       <c r="F30" s="22"/>
       <c r="G30" s="22"/>
       <c r="H30" s="22"/>
-      <c r="I30" s="98" t="n">
+      <c r="I30" s="99" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -30173,7 +30154,7 @@
       <c r="F31" s="22"/>
       <c r="G31" s="22"/>
       <c r="H31" s="22"/>
-      <c r="I31" s="98" t="n">
+      <c r="I31" s="99" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -30195,7 +30176,7 @@
       <c r="F32" s="22"/>
       <c r="G32" s="22"/>
       <c r="H32" s="22"/>
-      <c r="I32" s="98" t="n">
+      <c r="I32" s="99" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -30217,7 +30198,7 @@
       <c r="F33" s="22"/>
       <c r="G33" s="22"/>
       <c r="H33" s="22"/>
-      <c r="I33" s="98" t="n">
+      <c r="I33" s="99" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -30239,7 +30220,7 @@
       <c r="F34" s="22"/>
       <c r="G34" s="22"/>
       <c r="H34" s="22"/>
-      <c r="I34" s="98" t="n">
+      <c r="I34" s="99" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -30797,7 +30778,7 @@
       <c r="I64" s="22"/>
     </row>
     <row r="65" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="97" t="s">
+      <c r="A65" s="98" t="s">
         <v>303</v>
       </c>
       <c r="B65" s="22" t="s">
@@ -30816,7 +30797,7 @@
       <c r="I65" s="29"/>
     </row>
     <row r="66" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="97" t="s">
+      <c r="A66" s="98" t="s">
         <v>303</v>
       </c>
       <c r="B66" s="22" t="s">
@@ -30835,7 +30816,7 @@
       <c r="I66" s="29"/>
     </row>
     <row r="67" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="97" t="s">
+      <c r="A67" s="98" t="s">
         <v>303</v>
       </c>
       <c r="B67" s="22" t="s">
@@ -30854,7 +30835,7 @@
       <c r="I67" s="29"/>
     </row>
     <row r="68" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="97" t="s">
+      <c r="A68" s="98" t="s">
         <v>303</v>
       </c>
       <c r="B68" s="22" t="s">
@@ -30873,7 +30854,7 @@
       <c r="I68" s="29"/>
     </row>
     <row r="69" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="97" t="s">
+      <c r="A69" s="98" t="s">
         <v>303</v>
       </c>
       <c r="B69" s="22" t="s">
@@ -30892,7 +30873,7 @@
       <c r="I69" s="29"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="97" t="s">
+      <c r="A70" s="98" t="s">
         <v>878</v>
       </c>
       <c r="B70" s="29" t="s">
@@ -30906,7 +30887,7 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="97" t="s">
+      <c r="A71" s="98" t="s">
         <v>878</v>
       </c>
       <c r="B71" s="29" t="s">
@@ -30920,7 +30901,7 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="97" t="s">
+      <c r="A72" s="98" t="s">
         <v>878</v>
       </c>
       <c r="B72" s="29" t="s">
@@ -30933,8 +30914,8 @@
         <v>2162</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="97" t="s">
+    <row r="73" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="98" t="s">
         <v>878</v>
       </c>
       <c r="B73" s="29" t="s">
@@ -30946,6 +30927,11 @@
       <c r="D73" s="29" t="s">
         <v>2165</v>
       </c>
+      <c r="E73" s="29"/>
+      <c r="F73" s="29"/>
+      <c r="G73" s="29"/>
+      <c r="H73" s="29"/>
+      <c r="I73" s="29"/>
     </row>
     <row r="74" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="29" t="s">
@@ -31213,7 +31199,7 @@
       <c r="H87" s="29"/>
       <c r="I87" s="29"/>
     </row>
-    <row r="88" s="2" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="29" t="s">
         <v>1055</v>
       </c>
@@ -31226,14 +31212,9 @@
       <c r="D88" s="29" t="s">
         <v>2206</v>
       </c>
-      <c r="E88" s="29"/>
-      <c r="F88" s="29"/>
-      <c r="G88" s="29"/>
-      <c r="H88" s="29"/>
-      <c r="I88" s="29"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="99" t="s">
+      <c r="A89" s="100" t="s">
         <v>81</v>
       </c>
       <c r="B89" s="60" t="s">
@@ -31247,7 +31228,7 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="99" t="s">
+      <c r="A90" s="100" t="s">
         <v>81</v>
       </c>
       <c r="B90" s="29" t="s">
@@ -31261,21 +31242,21 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="99" t="s">
+      <c r="A91" s="100" t="s">
         <v>81</v>
       </c>
       <c r="B91" s="29" t="s">
         <v>212</v>
       </c>
       <c r="C91" s="29" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="99" t="s">
+      <c r="A92" s="100" t="s">
         <v>81</v>
       </c>
       <c r="B92" s="29" t="s">
@@ -31291,7 +31272,7 @@
       <c r="F92" s="60"/>
     </row>
     <row r="93" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="100" t="s">
+      <c r="A93" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B93" s="22" t="s">
@@ -31312,7 +31293,7 @@
       <c r="I93" s="22"/>
     </row>
     <row r="94" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="100" t="s">
+      <c r="A94" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B94" s="22" t="s">
@@ -31333,7 +31314,7 @@
       <c r="I94" s="22"/>
     </row>
     <row r="95" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="100" t="s">
+      <c r="A95" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B95" s="22" t="s">
@@ -31352,7 +31333,7 @@
       <c r="I95" s="22"/>
     </row>
     <row r="96" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="100" t="s">
+      <c r="A96" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B96" s="22" t="s">
@@ -31371,7 +31352,7 @@
       <c r="I96" s="22"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="100" t="s">
+      <c r="A97" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B97" s="22" t="s">
@@ -31390,7 +31371,7 @@
       <c r="I97" s="22"/>
     </row>
     <row r="98" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="100" t="s">
+      <c r="A98" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B98" s="22" t="s">
@@ -31411,7 +31392,7 @@
       <c r="I98" s="22"/>
     </row>
     <row r="99" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="100" t="s">
+      <c r="A99" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B99" s="22" t="s">
@@ -31430,7 +31411,7 @@
       <c r="I99" s="22"/>
     </row>
     <row r="100" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="100" t="s">
+      <c r="A100" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B100" s="22" t="s">
@@ -31451,17 +31432,17 @@
       <c r="I100" s="22"/>
     </row>
     <row r="101" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="100" t="s">
+      <c r="A101" s="101" t="s">
         <v>403</v>
       </c>
       <c r="B101" s="22" t="s">
         <v>212</v>
       </c>
       <c r="C101" s="28" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
       <c r="D101" s="65" t="s">
-        <v>1568</v>
+        <v>1566</v>
       </c>
       <c r="E101" s="28"/>
       <c r="F101" s="28"/>
@@ -31470,7 +31451,7 @@
       <c r="I101" s="22"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="101" t="s">
+      <c r="A102" s="102" t="s">
         <v>2235</v>
       </c>
       <c r="B102" s="29" t="s">
@@ -31490,7 +31471,7 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="101" t="s">
+      <c r="A103" s="102" t="s">
         <v>2235</v>
       </c>
       <c r="B103" s="29" t="s">
@@ -31510,7 +31491,7 @@
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="101" t="s">
+      <c r="A104" s="102" t="s">
         <v>2235</v>
       </c>
       <c r="B104" s="29" t="s">
@@ -31524,7 +31505,7 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="101" t="s">
+      <c r="A105" s="102" t="s">
         <v>744</v>
       </c>
       <c r="B105" s="60" t="s">
@@ -31538,7 +31519,7 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="101" t="s">
+      <c r="A106" s="102" t="s">
         <v>744</v>
       </c>
       <c r="B106" s="60" t="s">
@@ -31552,7 +31533,7 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="101" t="s">
+      <c r="A107" s="102" t="s">
         <v>744</v>
       </c>
       <c r="B107" s="60" t="s">
@@ -31566,7 +31547,7 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="101" t="s">
+      <c r="A108" s="102" t="s">
         <v>744</v>
       </c>
       <c r="B108" s="60" t="s">
@@ -31580,7 +31561,7 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="101" t="s">
+      <c r="A109" s="102" t="s">
         <v>744</v>
       </c>
       <c r="G109" s="22" t="s">
@@ -31588,7 +31569,7 @@
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="101" t="s">
+      <c r="A110" s="102" t="s">
         <v>744</v>
       </c>
       <c r="G110" s="22" t="s">
@@ -31596,7 +31577,7 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="101" t="s">
+      <c r="A111" s="102" t="s">
         <v>812</v>
       </c>
       <c r="B111" s="60" t="s">
@@ -31610,7 +31591,7 @@
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="101" t="s">
+      <c r="A112" s="102" t="s">
         <v>812</v>
       </c>
       <c r="B112" s="60" t="s">
@@ -31624,7 +31605,7 @@
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="101" t="s">
+      <c r="A113" s="102" t="s">
         <v>812</v>
       </c>
       <c r="B113" s="60" t="s">
@@ -31638,7 +31619,7 @@
       </c>
     </row>
     <row r="114" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="101" t="s">
+      <c r="A114" s="102" t="s">
         <v>812</v>
       </c>
       <c r="B114" s="22" t="s">
@@ -31652,7 +31633,7 @@
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="101" t="s">
+      <c r="A115" s="102" t="s">
         <v>812</v>
       </c>
       <c r="G115" s="22" t="s">
@@ -31660,7 +31641,7 @@
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="101" t="s">
+      <c r="A116" s="102" t="s">
         <v>812</v>
       </c>
       <c r="G116" s="22" t="s">
@@ -31668,7 +31649,7 @@
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="102" t="s">
+      <c r="A117" s="103" t="s">
         <v>322</v>
       </c>
       <c r="B117" s="60" t="s">
@@ -31682,7 +31663,7 @@
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="102" t="s">
+      <c r="A118" s="103" t="s">
         <v>322</v>
       </c>
       <c r="B118" s="29" t="s">
@@ -31696,7 +31677,7 @@
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="102" t="s">
+      <c r="A119" s="103" t="s">
         <v>322</v>
       </c>
       <c r="B119" s="60" t="s">
@@ -31710,7 +31691,7 @@
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="102" t="s">
+      <c r="A120" s="103" t="s">
         <v>322</v>
       </c>
       <c r="B120" s="60" t="s">
@@ -31724,7 +31705,7 @@
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="102" t="s">
+      <c r="A121" s="103" t="s">
         <v>322</v>
       </c>
       <c r="B121" s="60" t="s">
@@ -31738,7 +31719,7 @@
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="102" t="s">
+      <c r="A122" s="103" t="s">
         <v>322</v>
       </c>
       <c r="B122" s="60" t="s">
@@ -31752,7 +31733,7 @@
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="102" t="s">
+      <c r="A123" s="103" t="s">
         <v>322</v>
       </c>
       <c r="G123" s="22" t="s">
@@ -31760,7 +31741,7 @@
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="97" t="s">
+      <c r="A124" s="98" t="s">
         <v>2277</v>
       </c>
       <c r="B124" s="22" t="s">
@@ -31778,10 +31759,10 @@
       <c r="F124" s="22" t="s">
         <v>1806</v>
       </c>
-      <c r="G124" s="97"/>
+      <c r="G124" s="98"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A125" s="97" t="s">
+      <c r="A125" s="98" t="s">
         <v>2277</v>
       </c>
       <c r="B125" s="22" t="s">
@@ -31801,7 +31782,7 @@
       </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A126" s="97" t="s">
+      <c r="A126" s="98" t="s">
         <v>2277</v>
       </c>
       <c r="B126" s="22" t="s">
@@ -31821,7 +31802,7 @@
       </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A127" s="97" t="s">
+      <c r="A127" s="98" t="s">
         <v>2277</v>
       </c>
       <c r="B127" s="22" t="s">
@@ -31841,7 +31822,7 @@
       </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A128" s="97" t="s">
+      <c r="A128" s="98" t="s">
         <v>2277</v>
       </c>
       <c r="B128" s="22" t="s">
@@ -31887,7 +31868,7 @@
       <c r="D130" s="35" t="s">
         <v>2279</v>
       </c>
-      <c r="H130" s="103" t="s">
+      <c r="H130" s="104" t="s">
         <v>1210</v>
       </c>
     </row>
@@ -31904,7 +31885,7 @@
       <c r="D131" s="35" t="s">
         <v>2282</v>
       </c>
-      <c r="H131" s="104" t="s">
+      <c r="H131" s="105" t="s">
         <v>2283</v>
       </c>
     </row>
@@ -33105,7 +33086,7 @@
       <c r="E203" s="22"/>
       <c r="F203" s="22"/>
       <c r="G203" s="22"/>
-      <c r="H203" s="105"/>
+      <c r="H203" s="106"/>
       <c r="I203" s="22"/>
     </row>
     <row r="204" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33200,7 +33181,7 @@
       <c r="E208" s="22"/>
       <c r="F208" s="22"/>
       <c r="G208" s="22"/>
-      <c r="H208" s="105" t="s">
+      <c r="H208" s="106" t="s">
         <v>1198</v>
       </c>
       <c r="I208" s="22"/>
@@ -33499,7 +33480,7 @@
         <v>2450</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="29" t="s">
         <v>860</v>
       </c>
@@ -33512,6 +33493,11 @@
       <c r="D229" s="29" t="s">
         <v>2426</v>
       </c>
+      <c r="E229" s="29"/>
+      <c r="F229" s="29"/>
+      <c r="G229" s="29"/>
+      <c r="H229" s="29"/>
+      <c r="I229" s="29"/>
     </row>
     <row r="230" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="29" t="s">
@@ -33827,7 +33813,7 @@
       <c r="H245" s="29"/>
       <c r="I245" s="29"/>
     </row>
-    <row r="246" s="2" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="11" t="s">
         <v>1064</v>
       </c>
@@ -33840,21 +33826,21 @@
       <c r="D246" s="28" t="s">
         <v>2498</v>
       </c>
-      <c r="E246" s="29"/>
-      <c r="F246" s="29"/>
-      <c r="G246" s="29"/>
-      <c r="H246" s="29"/>
-      <c r="I246" s="29"/>
-    </row>
-    <row r="247" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="247" s="2" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="11" t="s">
         <v>1064</v>
       </c>
+      <c r="B247" s="29"/>
       <c r="C247" s="65"/>
       <c r="D247" s="65"/>
+      <c r="E247" s="29"/>
+      <c r="F247" s="29"/>
       <c r="G247" s="22" t="s">
         <v>2036</v>
       </c>
+      <c r="H247" s="29"/>
+      <c r="I247" s="29"/>
     </row>
     <row r="248" s="2" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="2" t="s">
@@ -34116,7 +34102,7 @@
       <c r="H262" s="29"/>
       <c r="I262" s="29"/>
     </row>
-    <row r="263" s="2" customFormat="true" ht="75.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="263" customFormat="false" ht="75.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="29" t="s">
         <v>986</v>
       </c>
@@ -34129,11 +34115,6 @@
       <c r="D263" s="28" t="s">
         <v>2534</v>
       </c>
-      <c r="E263" s="29"/>
-      <c r="F263" s="29"/>
-      <c r="G263" s="29"/>
-      <c r="H263" s="29"/>
-      <c r="I263" s="29"/>
     </row>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
commonTrip: Remplissage automatique des modes
part of #117

Les segments d'un déplacement commun sont pré-remplis lors du changement
de déplacement actif. Si on est dans l'échantillon partiel `commonTrip`
et que le déplacement n'a pas encore de segment, on regarde si c'est un
déplacement commun avec la personne (ie même heure de départ de
l'origine et d'arrivée à destination ET géographies des origines et
destinations à moins de 50 mètres de distance). Le mode est pré-remplie
seulement dans le cas d'un mode unique. `carDriver` et `carPassenger`
sont interverties si l'information du déplacement d'origine l'indique.

Ajout d'une note au texte de `segmentsIntro` si les données sont
pré-remplies d'un autre carnet de déplacements.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Choices" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Labels!$A$1:$F$259</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Labels!$A$1:$F$260</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Widgets!$A$1:$W$1048534</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4892" uniqueCount="2683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4896" uniqueCount="2686">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -2035,10 +2035,29 @@
     <t xml:space="preserve">segmentsIntro</t>
   </si>
   <si>
-    <t xml:space="preserve">Veuillez indiquer tous les modes de transport utilisés pour effectuer ce déplacement (de {{originName}} vers {{destinationName}}), dans l'ordre chronologique:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Please indicate all modes of transport used for this trip (from {{originName}} to {{destinationName}}), in chronological order:</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Veuillez indiquer tous les modes de transport utilisés pour effectuer ce déplacement (de {{originName}} vers {{destinationName}}), dans l'ordre chronologique:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">{{prefilledSegmentNote}}</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Please indicate all modes of transport used for this trip (from {{originName}} to {{destinationName}}), in chronological order:{{prefilledSegmentNote}}</t>
   </si>
   <si>
     <t xml:space="preserve">Mode de transport</t>
@@ -6948,6 +6967,17 @@
     <t xml:space="preserve">The transfer station(s) do not seem coherent for this trip</t>
   </si>
   <si>
+    <t xml:space="preserve">prefilledSegmentNote</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+__**Note:** Information pré-remplie en fonction de la déclaration de {{referenceNickname}}. Vérifier que les informations sont correctes et changer au besoin.__</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+__**Note:** Information prefilled from {{referenceNickname}}'s trip diary. Verify if the information is correct and change if needed.__</t>
+  </si>
+  <si>
     <t xml:space="preserve">personHasSchoolPlace_schoolchildcare</t>
   </si>
   <si>
@@ -8708,7 +8738,7 @@
     <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
     <numFmt numFmtId="167" formatCode="@"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -8792,6 +8822,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -9149,7 +9186,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9185,19 +9222,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9205,7 +9242,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9225,11 +9262,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9241,19 +9278,19 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9281,11 +9318,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9293,11 +9330,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9305,43 +9362,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9349,7 +9386,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9357,15 +9394,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9373,27 +9410,27 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -22854,7 +22891,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F264"/>
+  <dimension ref="A1:F265"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="53" width="16.73"/>
@@ -26683,117 +26720,117 @@
         <v>2110</v>
       </c>
     </row>
-    <row r="248" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A248" s="51" t="s">
-        <v>744</v>
-      </c>
-      <c r="B248" s="57" t="s">
+    <row r="248" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="53" t="s">
+        <v>548</v>
+      </c>
+      <c r="B248" s="8" t="s">
         <v>2111</v>
       </c>
       <c r="C248" s="8" t="s">
         <v>2112</v>
       </c>
-      <c r="D248" s="88" t="s">
+      <c r="D248" s="60" t="s">
         <v>2113</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A249" s="53" t="s">
+    <row r="249" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="51" t="s">
         <v>744</v>
       </c>
-      <c r="B249" s="89" t="s">
+      <c r="B249" s="57" t="s">
         <v>2114</v>
       </c>
-      <c r="C249" s="51" t="s">
-        <v>1361</v>
-      </c>
-      <c r="D249" s="54" t="s">
-        <v>1362</v>
-      </c>
-    </row>
-    <row r="250" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C249" s="8" t="s">
+        <v>2115</v>
+      </c>
+      <c r="D249" s="88" t="s">
+        <v>2116</v>
+      </c>
+    </row>
+    <row r="250" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="53" t="s">
         <v>744</v>
       </c>
       <c r="B250" s="89" t="s">
-        <v>2115</v>
-      </c>
-      <c r="C250" s="8" t="s">
-        <v>2116</v>
+        <v>2117</v>
+      </c>
+      <c r="C250" s="51" t="s">
+        <v>1361</v>
       </c>
       <c r="D250" s="54" t="s">
-        <v>2117</v>
-      </c>
-    </row>
-    <row r="251" customFormat="false" ht="285.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="53" t="s">
         <v>744</v>
       </c>
-      <c r="B251" s="56" t="s">
+      <c r="B251" s="89" t="s">
         <v>2118</v>
       </c>
-      <c r="C251" s="57" t="s">
+      <c r="C251" s="8" t="s">
         <v>2119</v>
       </c>
-      <c r="D251" s="57" t="s">
+      <c r="D251" s="54" t="s">
         <v>2120</v>
       </c>
-      <c r="E251" s="57" t="s">
-        <v>2121</v>
-      </c>
-      <c r="F251" s="57" t="s">
-        <v>2122</v>
-      </c>
-    </row>
-    <row r="252" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="252" customFormat="false" ht="285.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="53" t="s">
         <v>744</v>
       </c>
       <c r="B252" s="56" t="s">
+        <v>2121</v>
+      </c>
+      <c r="C252" s="57" t="s">
+        <v>2122</v>
+      </c>
+      <c r="D252" s="57" t="s">
         <v>2123</v>
       </c>
-      <c r="C252" s="57" t="s">
+      <c r="E252" s="57" t="s">
         <v>2124</v>
       </c>
-      <c r="D252" s="57" t="s">
+      <c r="F252" s="57" t="s">
         <v>2125</v>
       </c>
-      <c r="E252" s="57" t="s">
+    </row>
+    <row r="253" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="53" t="s">
+        <v>744</v>
+      </c>
+      <c r="B253" s="56" t="s">
         <v>2126</v>
       </c>
-      <c r="F252" s="57" t="s">
+      <c r="C253" s="57" t="s">
         <v>2127</v>
       </c>
-    </row>
-    <row r="253" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A253" s="53" t="s">
-        <v>823</v>
-      </c>
-      <c r="B253" s="53" t="s">
+      <c r="D253" s="57" t="s">
         <v>2128</v>
       </c>
-      <c r="C253" s="51" t="s">
-        <v>1361</v>
-      </c>
-      <c r="D253" s="54" t="s">
-        <v>1362</v>
-      </c>
-    </row>
-    <row r="254" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E253" s="57" t="s">
+        <v>2129</v>
+      </c>
+      <c r="F253" s="57" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="53" t="s">
         <v>823</v>
       </c>
       <c r="B254" s="53" t="s">
-        <v>2129</v>
-      </c>
-      <c r="C254" s="8" t="s">
-        <v>2130</v>
-      </c>
-      <c r="D254" s="8" t="s">
         <v>2131</v>
       </c>
-    </row>
-    <row r="255" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C254" s="51" t="s">
+        <v>1361</v>
+      </c>
+      <c r="D254" s="54" t="s">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="255" customFormat="false" ht="45.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="53" t="s">
         <v>823</v>
       </c>
@@ -26801,51 +26838,51 @@
         <v>2132</v>
       </c>
       <c r="C255" s="8" t="s">
-        <v>1419</v>
+        <v>2133</v>
       </c>
       <c r="D255" s="8" t="s">
-        <v>1420</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="53" t="s">
-        <v>1043</v>
+        <v>823</v>
       </c>
       <c r="B256" s="53" t="s">
-        <v>2133</v>
-      </c>
-      <c r="C256" s="51" t="s">
-        <v>1361</v>
-      </c>
-      <c r="D256" s="54" t="s">
-        <v>1362</v>
-      </c>
-    </row>
-    <row r="257" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2135</v>
+      </c>
+      <c r="C256" s="8" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D256" s="8" t="s">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="257" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="53" t="s">
         <v>1043</v>
       </c>
       <c r="B257" s="53" t="s">
-        <v>2134</v>
-      </c>
-      <c r="C257" s="8" t="s">
-        <v>2135</v>
+        <v>2136</v>
+      </c>
+      <c r="C257" s="51" t="s">
+        <v>1361</v>
       </c>
       <c r="D257" s="54" t="s">
-        <v>2136</v>
-      </c>
-    </row>
-    <row r="258" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="53" t="s">
-        <v>991</v>
-      </c>
-      <c r="B258" s="57" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B258" s="53" t="s">
         <v>2137</v>
       </c>
-      <c r="C258" s="57" t="s">
+      <c r="C258" s="8" t="s">
         <v>2138</v>
       </c>
-      <c r="D258" s="57" t="s">
+      <c r="D258" s="54" t="s">
         <v>2139</v>
       </c>
     </row>
@@ -26863,65 +26900,65 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="260" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="260" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="53" t="s">
-        <v>48</v>
-      </c>
-      <c r="B260" s="53" t="s">
+        <v>991</v>
+      </c>
+      <c r="B260" s="57" t="s">
         <v>2143</v>
       </c>
-      <c r="C260" s="51" t="s">
+      <c r="C260" s="57" t="s">
         <v>2144</v>
       </c>
-      <c r="D260" s="54" t="s">
+      <c r="D260" s="57" t="s">
         <v>2145</v>
       </c>
     </row>
-    <row r="261" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="261" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="53" t="s">
         <v>48</v>
       </c>
       <c r="B261" s="53" t="s">
         <v>2146</v>
       </c>
-      <c r="C261" s="8" t="s">
+      <c r="C261" s="51" t="s">
         <v>2147</v>
       </c>
       <c r="D261" s="54" t="s">
         <v>2148</v>
       </c>
     </row>
-    <row r="262" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="262" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="53" t="s">
         <v>48</v>
       </c>
       <c r="B262" s="53" t="s">
         <v>2149</v>
       </c>
-      <c r="C262" s="51" t="s">
-        <v>1361</v>
+      <c r="C262" s="8" t="s">
+        <v>2150</v>
       </c>
       <c r="D262" s="54" t="s">
-        <v>1362</v>
-      </c>
-    </row>
-    <row r="263" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2151</v>
+      </c>
+    </row>
+    <row r="263" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="53" t="s">
         <v>48</v>
       </c>
       <c r="B263" s="53" t="s">
-        <v>2150</v>
-      </c>
-      <c r="C263" s="8" t="s">
-        <v>2151</v>
+        <v>2152</v>
+      </c>
+      <c r="C263" s="51" t="s">
+        <v>1361</v>
       </c>
       <c r="D263" s="54" t="s">
-        <v>2152</v>
-      </c>
-    </row>
-    <row r="264" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="264" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="53" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="B264" s="53" t="s">
         <v>2153</v>
@@ -26929,12 +26966,26 @@
       <c r="C264" s="8" t="s">
         <v>2154</v>
       </c>
-      <c r="D264" s="8" t="s">
+      <c r="D264" s="54" t="s">
         <v>2155</v>
       </c>
     </row>
+    <row r="265" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="53" t="s">
+        <v>24</v>
+      </c>
+      <c r="B265" s="53" t="s">
+        <v>2156</v>
+      </c>
+      <c r="C265" s="8" t="s">
+        <v>2157</v>
+      </c>
+      <c r="D265" s="8" t="s">
+        <v>2158</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F259"/>
+  <autoFilter ref="A1:F260"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -26964,7 +27015,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="90" t="s">
-        <v>2156</v>
+        <v>2159</v>
       </c>
       <c r="B1" s="90" t="s">
         <v>1149</v>
@@ -26982,13 +27033,13 @@
         <v>9</v>
       </c>
       <c r="G1" s="90" t="s">
-        <v>2157</v>
+        <v>2160</v>
       </c>
       <c r="H1" s="90" t="s">
         <v>12</v>
       </c>
       <c r="I1" s="69" t="s">
-        <v>2158</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26999,10 +27050,10 @@
         <v>1157</v>
       </c>
       <c r="C2" s="56" t="s">
-        <v>2159</v>
+        <v>2162</v>
       </c>
       <c r="D2" s="56" t="s">
-        <v>2160</v>
+        <v>2163</v>
       </c>
       <c r="E2" s="56"/>
       <c r="F2" s="56"/>
@@ -27017,10 +27068,10 @@
         <v>1215</v>
       </c>
       <c r="C3" s="56" t="s">
-        <v>2161</v>
+        <v>2164</v>
       </c>
       <c r="D3" s="56" t="s">
-        <v>2162</v>
+        <v>2165</v>
       </c>
       <c r="E3" s="56"/>
       <c r="F3" s="56"/>
@@ -27035,10 +27086,10 @@
         <v>229</v>
       </c>
       <c r="C4" s="56" t="s">
-        <v>2163</v>
+        <v>2166</v>
       </c>
       <c r="D4" s="56" t="s">
-        <v>2164</v>
+        <v>2167</v>
       </c>
       <c r="E4" s="56"/>
       <c r="F4" s="56"/>
@@ -27047,7 +27098,7 @@
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
       <c r="B5" s="56" t="s">
         <v>229</v>
@@ -27065,16 +27116,16 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="C6" s="56" t="s">
-        <v>2167</v>
+        <v>2170</v>
       </c>
       <c r="D6" s="56" t="s">
-        <v>2168</v>
+        <v>2171</v>
       </c>
       <c r="E6" s="56"/>
       <c r="F6" s="56"/>
@@ -27089,10 +27140,10 @@
         <v>1161</v>
       </c>
       <c r="C7" s="56" t="s">
-        <v>2169</v>
+        <v>2172</v>
       </c>
       <c r="D7" s="56" t="s">
-        <v>2170</v>
+        <v>2173</v>
       </c>
       <c r="E7" s="56"/>
       <c r="F7" s="56"/>
@@ -27151,7 +27202,7 @@
       <c r="E11" s="56"/>
       <c r="F11" s="56"/>
       <c r="G11" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="H11" s="56"/>
     </row>
@@ -27205,10 +27256,10 @@
         <v>1157</v>
       </c>
       <c r="C15" s="54" t="s">
-        <v>2171</v>
+        <v>2174</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>2172</v>
+        <v>2175</v>
       </c>
       <c r="E15" s="54"/>
       <c r="F15" s="54"/>
@@ -27224,10 +27275,10 @@
         <v>1215</v>
       </c>
       <c r="C16" s="54" t="s">
-        <v>2173</v>
+        <v>2176</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>2174</v>
+        <v>2177</v>
       </c>
       <c r="E16" s="54"/>
       <c r="F16" s="54"/>
@@ -27237,16 +27288,16 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="92" t="s">
-        <v>2175</v>
+        <v>2178</v>
       </c>
       <c r="B17" s="56" t="s">
-        <v>2176</v>
+        <v>2179</v>
       </c>
       <c r="C17" s="56" t="s">
-        <v>2177</v>
+        <v>2180</v>
       </c>
       <c r="D17" s="56" t="s">
-        <v>2178</v>
+        <v>2181</v>
       </c>
       <c r="E17" s="56"/>
       <c r="F17" s="56"/>
@@ -27255,16 +27306,16 @@
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="92" t="s">
-        <v>2175</v>
+        <v>2178</v>
       </c>
       <c r="B18" s="56" t="s">
-        <v>2179</v>
+        <v>2182</v>
       </c>
       <c r="C18" s="56" t="s">
-        <v>2180</v>
+        <v>2183</v>
       </c>
       <c r="D18" s="56" t="s">
-        <v>2181</v>
+        <v>2184</v>
       </c>
       <c r="E18" s="56"/>
       <c r="F18" s="56"/>
@@ -27273,7 +27324,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="92" t="s">
-        <v>2175</v>
+        <v>2178</v>
       </c>
       <c r="B19" s="56"/>
       <c r="C19" s="56"/>
@@ -27290,13 +27341,13 @@
         <v>187</v>
       </c>
       <c r="B20" s="56" t="s">
-        <v>2176</v>
+        <v>2179</v>
       </c>
       <c r="C20" s="56" t="s">
-        <v>2177</v>
+        <v>2180</v>
       </c>
       <c r="D20" s="56" t="s">
-        <v>2182</v>
+        <v>2185</v>
       </c>
       <c r="E20" s="56"/>
       <c r="F20" s="56"/>
@@ -27308,13 +27359,13 @@
         <v>187</v>
       </c>
       <c r="B21" s="56" t="s">
-        <v>2179</v>
+        <v>2182</v>
       </c>
       <c r="C21" s="56" t="s">
-        <v>2180</v>
+        <v>2183</v>
       </c>
       <c r="D21" s="56" t="s">
-        <v>2183</v>
+        <v>2186</v>
       </c>
       <c r="E21" s="56"/>
       <c r="F21" s="56"/>
@@ -27329,10 +27380,10 @@
         <v>189</v>
       </c>
       <c r="C22" s="56" t="s">
-        <v>2184</v>
+        <v>2187</v>
       </c>
       <c r="D22" s="56" t="s">
-        <v>2185</v>
+        <v>2188</v>
       </c>
       <c r="E22" s="56"/>
       <c r="F22" s="56"/>
@@ -27358,13 +27409,13 @@
         <v>306</v>
       </c>
       <c r="B24" s="56" t="s">
-        <v>2186</v>
+        <v>2189</v>
       </c>
       <c r="C24" s="56" t="s">
-        <v>2187</v>
+        <v>2190</v>
       </c>
       <c r="D24" s="56" t="s">
-        <v>2188</v>
+        <v>2191</v>
       </c>
       <c r="E24" s="56"/>
       <c r="F24" s="56"/>
@@ -27376,13 +27427,13 @@
         <v>306</v>
       </c>
       <c r="B25" s="56" t="s">
-        <v>2189</v>
+        <v>2192</v>
       </c>
       <c r="C25" s="56" t="s">
-        <v>2190</v>
+        <v>2193</v>
       </c>
       <c r="D25" s="56" t="s">
-        <v>2191</v>
+        <v>2194</v>
       </c>
       <c r="E25" s="56"/>
       <c r="F25" s="56"/>
@@ -27408,13 +27459,13 @@
         <v>299</v>
       </c>
       <c r="B27" s="56" t="s">
-        <v>2186</v>
+        <v>2189</v>
       </c>
       <c r="C27" s="56" t="s">
-        <v>2192</v>
+        <v>2195</v>
       </c>
       <c r="D27" s="56" t="s">
-        <v>2193</v>
+        <v>2196</v>
       </c>
       <c r="E27" s="56"/>
       <c r="F27" s="56"/>
@@ -27426,13 +27477,13 @@
         <v>299</v>
       </c>
       <c r="B28" s="56" t="s">
-        <v>2189</v>
+        <v>2192</v>
       </c>
       <c r="C28" s="56" t="s">
-        <v>2194</v>
+        <v>2197</v>
       </c>
       <c r="D28" s="56" t="s">
-        <v>2195</v>
+        <v>2198</v>
       </c>
       <c r="E28" s="56"/>
       <c r="F28" s="56"/>
@@ -27461,10 +27512,10 @@
         <v>1181</v>
       </c>
       <c r="C30" s="56" t="s">
-        <v>2196</v>
+        <v>2199</v>
       </c>
       <c r="D30" s="56" t="s">
-        <v>2197</v>
+        <v>2200</v>
       </c>
       <c r="E30" s="56"/>
       <c r="F30" s="56"/>
@@ -27483,10 +27534,10 @@
         <v>1182</v>
       </c>
       <c r="C31" s="56" t="s">
-        <v>2198</v>
+        <v>2201</v>
       </c>
       <c r="D31" s="56" t="s">
-        <v>2199</v>
+        <v>2202</v>
       </c>
       <c r="E31" s="56"/>
       <c r="F31" s="56"/>
@@ -27505,10 +27556,10 @@
         <v>1183</v>
       </c>
       <c r="C32" s="56" t="s">
-        <v>2200</v>
+        <v>2203</v>
       </c>
       <c r="D32" s="56" t="s">
-        <v>2201</v>
+        <v>2204</v>
       </c>
       <c r="E32" s="56"/>
       <c r="F32" s="56"/>
@@ -27527,10 +27578,10 @@
         <v>1185</v>
       </c>
       <c r="C33" s="56" t="s">
-        <v>2202</v>
+        <v>2205</v>
       </c>
       <c r="D33" s="56" t="s">
-        <v>2203</v>
+        <v>2206</v>
       </c>
       <c r="E33" s="56"/>
       <c r="F33" s="56"/>
@@ -27549,10 +27600,10 @@
         <v>1186</v>
       </c>
       <c r="C34" s="56" t="s">
-        <v>2204</v>
+        <v>2207</v>
       </c>
       <c r="D34" s="56" t="s">
-        <v>2205</v>
+        <v>2208</v>
       </c>
       <c r="E34" s="56"/>
       <c r="F34" s="56"/>
@@ -27568,13 +27619,13 @@
         <v>340</v>
       </c>
       <c r="B35" s="56" t="s">
-        <v>2206</v>
+        <v>2209</v>
       </c>
       <c r="C35" s="56" t="s">
-        <v>2207</v>
+        <v>2210</v>
       </c>
       <c r="D35" s="56" t="s">
-        <v>2208</v>
+        <v>2211</v>
       </c>
       <c r="E35" s="56"/>
       <c r="F35" s="56"/>
@@ -27589,13 +27640,13 @@
         <v>340</v>
       </c>
       <c r="B36" s="56" t="s">
-        <v>2209</v>
+        <v>2212</v>
       </c>
       <c r="C36" s="56" t="s">
-        <v>2210</v>
+        <v>2213</v>
       </c>
       <c r="D36" s="56" t="s">
-        <v>2211</v>
+        <v>2214</v>
       </c>
       <c r="E36" s="56"/>
       <c r="F36" s="56"/>
@@ -27611,10 +27662,10 @@
         <v>1252</v>
       </c>
       <c r="C37" s="56" t="s">
-        <v>2212</v>
+        <v>2215</v>
       </c>
       <c r="D37" s="56" t="s">
-        <v>2213</v>
+        <v>2216</v>
       </c>
       <c r="E37" s="56"/>
       <c r="F37" s="56"/>
@@ -27630,10 +27681,10 @@
         <v>1253</v>
       </c>
       <c r="C38" s="56" t="s">
-        <v>2214</v>
+        <v>2217</v>
       </c>
       <c r="D38" s="56" t="s">
-        <v>2215</v>
+        <v>2218</v>
       </c>
       <c r="E38" s="56"/>
       <c r="F38" s="56"/>
@@ -27646,13 +27697,13 @@
         <v>340</v>
       </c>
       <c r="B39" s="56" t="s">
-        <v>2216</v>
+        <v>2219</v>
       </c>
       <c r="C39" s="56" t="s">
-        <v>2217</v>
+        <v>2220</v>
       </c>
       <c r="D39" s="56" t="s">
-        <v>2218</v>
+        <v>2221</v>
       </c>
       <c r="E39" s="56"/>
       <c r="F39" s="56"/>
@@ -27665,13 +27716,13 @@
         <v>340</v>
       </c>
       <c r="B40" s="56" t="s">
-        <v>2219</v>
+        <v>2222</v>
       </c>
       <c r="C40" s="56" t="s">
-        <v>2220</v>
+        <v>2223</v>
       </c>
       <c r="D40" s="56" t="s">
-        <v>2221</v>
+        <v>2224</v>
       </c>
       <c r="E40" s="56"/>
       <c r="F40" s="56"/>
@@ -27689,7 +27740,7 @@
       <c r="E41" s="56"/>
       <c r="F41" s="56"/>
       <c r="G41" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
       <c r="H41" s="56"/>
       <c r="I41" s="69"/>
@@ -27714,13 +27765,13 @@
         <v>315</v>
       </c>
       <c r="B43" s="56" t="s">
-        <v>2222</v>
+        <v>2225</v>
       </c>
       <c r="C43" s="51" t="s">
-        <v>2223</v>
+        <v>2226</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>2224</v>
+        <v>2227</v>
       </c>
       <c r="E43" s="56"/>
       <c r="F43" s="56"/>
@@ -27733,13 +27784,13 @@
         <v>315</v>
       </c>
       <c r="B44" s="56" t="s">
-        <v>2225</v>
+        <v>2228</v>
       </c>
       <c r="C44" s="51" t="s">
-        <v>2226</v>
+        <v>2229</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>2227</v>
+        <v>2230</v>
       </c>
       <c r="E44" s="56"/>
       <c r="F44" s="56"/>
@@ -27752,13 +27803,13 @@
         <v>315</v>
       </c>
       <c r="B45" s="56" t="s">
-        <v>2228</v>
+        <v>2231</v>
       </c>
       <c r="C45" s="51" t="s">
-        <v>2229</v>
+        <v>2232</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>2230</v>
+        <v>2233</v>
       </c>
       <c r="E45" s="56"/>
       <c r="F45" s="56"/>
@@ -27771,13 +27822,13 @@
         <v>315</v>
       </c>
       <c r="B46" s="56" t="s">
-        <v>2231</v>
+        <v>2234</v>
       </c>
       <c r="C46" s="51" t="s">
-        <v>2232</v>
+        <v>2235</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>2233</v>
+        <v>2236</v>
       </c>
       <c r="E46" s="56"/>
       <c r="F46" s="56"/>
@@ -27795,7 +27846,7 @@
       <c r="E47" s="56"/>
       <c r="F47" s="56"/>
       <c r="G47" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="H47" s="56"/>
       <c r="I47" s="56"/>
@@ -27808,10 +27859,10 @@
         <v>1246</v>
       </c>
       <c r="C48" s="54" t="s">
-        <v>2234</v>
+        <v>2237</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>2235</v>
+        <v>2238</v>
       </c>
       <c r="E48" s="56"/>
       <c r="F48" s="56"/>
@@ -27826,13 +27877,13 @@
         <v>220</v>
       </c>
       <c r="B49" s="56" t="s">
-        <v>2236</v>
+        <v>2239</v>
       </c>
       <c r="C49" s="54" t="s">
-        <v>2237</v>
+        <v>2240</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>2238</v>
+        <v>2241</v>
       </c>
       <c r="E49" s="56"/>
       <c r="F49" s="56"/>
@@ -27847,13 +27898,13 @@
         <v>220</v>
       </c>
       <c r="B50" s="56" t="s">
-        <v>2239</v>
+        <v>2242</v>
       </c>
       <c r="C50" s="54" t="s">
-        <v>2240</v>
+        <v>2243</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>2241</v>
+        <v>2244</v>
       </c>
       <c r="E50" s="56"/>
       <c r="F50" s="56"/>
@@ -27869,10 +27920,10 @@
         <v>229</v>
       </c>
       <c r="C51" s="54" t="s">
-        <v>2242</v>
+        <v>2245</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>2243</v>
+        <v>2246</v>
       </c>
       <c r="E51" s="56"/>
       <c r="F51" s="56"/>
@@ -27890,7 +27941,7 @@
       <c r="E52" s="56"/>
       <c r="F52" s="56"/>
       <c r="G52" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="H52" s="56"/>
       <c r="I52" s="56"/>
@@ -27900,13 +27951,13 @@
         <v>226</v>
       </c>
       <c r="B53" s="56" t="s">
-        <v>2244</v>
+        <v>2247</v>
       </c>
       <c r="C53" s="54" t="s">
-        <v>2245</v>
+        <v>2248</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>2246</v>
+        <v>2249</v>
       </c>
       <c r="E53" s="56"/>
       <c r="F53" s="56"/>
@@ -27919,13 +27970,13 @@
         <v>226</v>
       </c>
       <c r="B54" s="56" t="s">
-        <v>2247</v>
+        <v>2250</v>
       </c>
       <c r="C54" s="54" t="s">
-        <v>2248</v>
+        <v>2251</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>2249</v>
+        <v>2252</v>
       </c>
       <c r="E54" s="56"/>
       <c r="F54" s="56"/>
@@ -27938,13 +27989,13 @@
         <v>226</v>
       </c>
       <c r="B55" s="56" t="s">
-        <v>2250</v>
+        <v>2253</v>
       </c>
       <c r="C55" s="54" t="s">
-        <v>2251</v>
+        <v>2254</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>2252</v>
+        <v>2255</v>
       </c>
       <c r="E55" s="56"/>
       <c r="F55" s="56"/>
@@ -27957,13 +28008,13 @@
         <v>226</v>
       </c>
       <c r="B56" s="56" t="s">
-        <v>2253</v>
+        <v>2256</v>
       </c>
       <c r="C56" s="54" t="s">
-        <v>2254</v>
+        <v>2257</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>2255</v>
+        <v>2258</v>
       </c>
       <c r="E56" s="56"/>
       <c r="F56" s="56"/>
@@ -27976,13 +28027,13 @@
         <v>226</v>
       </c>
       <c r="B57" s="56" t="s">
-        <v>2256</v>
+        <v>2259</v>
       </c>
       <c r="C57" s="54" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>2257</v>
+        <v>2260</v>
       </c>
       <c r="E57" s="56"/>
       <c r="F57" s="56"/>
@@ -27995,13 +28046,13 @@
         <v>226</v>
       </c>
       <c r="B58" s="56" t="s">
-        <v>2258</v>
+        <v>2261</v>
       </c>
       <c r="C58" s="54" t="s">
-        <v>2259</v>
+        <v>2262</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>2260</v>
+        <v>2263</v>
       </c>
       <c r="E58" s="56"/>
       <c r="F58" s="56"/>
@@ -28014,13 +28065,13 @@
         <v>226</v>
       </c>
       <c r="B59" s="56" t="s">
-        <v>2261</v>
+        <v>2264</v>
       </c>
       <c r="C59" s="54" t="s">
-        <v>2262</v>
+        <v>2265</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>2263</v>
+        <v>2266</v>
       </c>
       <c r="E59" s="56"/>
       <c r="F59" s="56"/>
@@ -28033,13 +28084,13 @@
         <v>226</v>
       </c>
       <c r="B60" s="56" t="s">
-        <v>2264</v>
+        <v>2267</v>
       </c>
       <c r="C60" s="54" t="s">
-        <v>2265</v>
+        <v>2268</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>2266</v>
+        <v>2269</v>
       </c>
       <c r="E60" s="56"/>
       <c r="F60" s="56"/>
@@ -28067,13 +28118,13 @@
         <v>226</v>
       </c>
       <c r="B62" s="56" t="s">
-        <v>2267</v>
+        <v>2270</v>
       </c>
       <c r="C62" s="54" t="s">
-        <v>2268</v>
+        <v>2271</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>2269</v>
+        <v>2272</v>
       </c>
       <c r="E62" s="56"/>
       <c r="F62" s="56"/>
@@ -28091,7 +28142,7 @@
       <c r="E63" s="56"/>
       <c r="F63" s="56"/>
       <c r="G63" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="H63" s="56"/>
       <c r="I63" s="56"/>
@@ -28104,10 +28155,10 @@
         <v>1157</v>
       </c>
       <c r="C64" s="54" t="s">
-        <v>2270</v>
+        <v>2273</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>2271</v>
+        <v>2274</v>
       </c>
       <c r="E64" s="56"/>
       <c r="F64" s="56"/>
@@ -28123,14 +28174,14 @@
         <v>1189</v>
       </c>
       <c r="C65" s="56" t="s">
-        <v>2272</v>
+        <v>2275</v>
       </c>
       <c r="D65" s="56" t="s">
-        <v>2273</v>
+        <v>2276</v>
       </c>
       <c r="E65" s="56"/>
       <c r="F65" s="56" t="s">
-        <v>2274</v>
+        <v>2277</v>
       </c>
       <c r="G65" s="56"/>
       <c r="H65" s="56"/>
@@ -28144,14 +28195,14 @@
         <v>1190</v>
       </c>
       <c r="C66" s="56" t="s">
-        <v>2275</v>
+        <v>2278</v>
       </c>
       <c r="D66" s="56" t="s">
-        <v>2276</v>
+        <v>2279</v>
       </c>
       <c r="E66" s="56"/>
       <c r="F66" s="56" t="s">
-        <v>2277</v>
+        <v>2280</v>
       </c>
       <c r="G66" s="56"/>
       <c r="H66" s="56"/>
@@ -28162,17 +28213,17 @@
         <v>322</v>
       </c>
       <c r="B67" s="56" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="C67" s="56" t="s">
-        <v>2279</v>
+        <v>2282</v>
       </c>
       <c r="D67" s="56" t="s">
-        <v>2280</v>
+        <v>2283</v>
       </c>
       <c r="E67" s="56"/>
       <c r="F67" s="56" t="s">
-        <v>2281</v>
+        <v>2284</v>
       </c>
       <c r="G67" s="56"/>
       <c r="H67" s="56"/>
@@ -28186,14 +28237,14 @@
         <v>1191</v>
       </c>
       <c r="C68" s="56" t="s">
-        <v>2282</v>
+        <v>2285</v>
       </c>
       <c r="D68" s="56" t="s">
-        <v>2283</v>
+        <v>2286</v>
       </c>
       <c r="E68" s="56"/>
       <c r="F68" s="56" t="s">
-        <v>2284</v>
+        <v>2287</v>
       </c>
       <c r="G68" s="56"/>
       <c r="H68" s="56"/>
@@ -28207,14 +28258,14 @@
         <v>1205</v>
       </c>
       <c r="C69" s="56" t="s">
-        <v>2285</v>
+        <v>2288</v>
       </c>
       <c r="D69" s="56" t="s">
-        <v>2286</v>
+        <v>2289</v>
       </c>
       <c r="E69" s="56"/>
       <c r="F69" s="56" t="s">
-        <v>2287</v>
+        <v>2290</v>
       </c>
       <c r="G69" s="56"/>
       <c r="H69" s="56"/>
@@ -28225,13 +28276,13 @@
         <v>895</v>
       </c>
       <c r="B70" s="69" t="s">
-        <v>2288</v>
+        <v>2291</v>
       </c>
       <c r="C70" s="69" t="s">
-        <v>2289</v>
+        <v>2292</v>
       </c>
       <c r="D70" s="69" t="s">
-        <v>2290</v>
+        <v>2293</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28239,13 +28290,13 @@
         <v>895</v>
       </c>
       <c r="B71" s="69" t="s">
-        <v>2291</v>
+        <v>2294</v>
       </c>
       <c r="C71" s="69" t="s">
-        <v>2292</v>
+        <v>2295</v>
       </c>
       <c r="D71" s="69" t="s">
-        <v>2293</v>
+        <v>2296</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28253,13 +28304,13 @@
         <v>895</v>
       </c>
       <c r="B72" s="69" t="s">
-        <v>2294</v>
+        <v>2297</v>
       </c>
       <c r="C72" s="69" t="s">
-        <v>2295</v>
+        <v>2298</v>
       </c>
       <c r="D72" s="69" t="s">
-        <v>2296</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="73" s="53" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28267,13 +28318,13 @@
         <v>895</v>
       </c>
       <c r="B73" s="69" t="s">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="C73" s="69" t="s">
-        <v>2298</v>
+        <v>2301</v>
       </c>
       <c r="D73" s="69" t="s">
-        <v>2299</v>
+        <v>2302</v>
       </c>
       <c r="E73" s="69"/>
       <c r="F73" s="69"/>
@@ -28286,13 +28337,13 @@
         <v>1069</v>
       </c>
       <c r="B74" s="69" t="s">
-        <v>2300</v>
+        <v>2303</v>
       </c>
       <c r="C74" s="69" t="s">
-        <v>2301</v>
+        <v>2304</v>
       </c>
       <c r="D74" s="69" t="s">
-        <v>2302</v>
+        <v>2305</v>
       </c>
       <c r="E74" s="69"/>
       <c r="F74" s="69"/>
@@ -28305,13 +28356,13 @@
         <v>1069</v>
       </c>
       <c r="B75" s="53" t="s">
-        <v>2303</v>
+        <v>2306</v>
       </c>
       <c r="C75" s="53" t="s">
-        <v>2304</v>
+        <v>2307</v>
       </c>
       <c r="D75" s="53" t="s">
-        <v>2305</v>
+        <v>2308</v>
       </c>
       <c r="G75" s="69"/>
       <c r="H75" s="69"/>
@@ -28322,13 +28373,13 @@
         <v>1069</v>
       </c>
       <c r="B76" s="53" t="s">
-        <v>2306</v>
+        <v>2309</v>
       </c>
       <c r="C76" s="53" t="s">
-        <v>2307</v>
+        <v>2310</v>
       </c>
       <c r="D76" s="53" t="s">
-        <v>2308</v>
+        <v>2311</v>
       </c>
       <c r="G76" s="69"/>
       <c r="H76" s="69"/>
@@ -28339,13 +28390,13 @@
         <v>1069</v>
       </c>
       <c r="B77" s="53" t="s">
-        <v>2309</v>
+        <v>2312</v>
       </c>
       <c r="C77" s="53" t="s">
-        <v>2310</v>
+        <v>2313</v>
       </c>
       <c r="D77" s="53" t="s">
-        <v>2311</v>
+        <v>2314</v>
       </c>
       <c r="G77" s="69"/>
       <c r="H77" s="69"/>
@@ -28356,13 +28407,13 @@
         <v>1069</v>
       </c>
       <c r="B78" s="53" t="s">
-        <v>2312</v>
+        <v>2315</v>
       </c>
       <c r="C78" s="53" t="s">
-        <v>2313</v>
+        <v>2316</v>
       </c>
       <c r="D78" s="53" t="s">
-        <v>2314</v>
+        <v>2317</v>
       </c>
       <c r="G78" s="69"/>
       <c r="H78" s="69"/>
@@ -28373,13 +28424,13 @@
         <v>1069</v>
       </c>
       <c r="B79" s="53" t="s">
-        <v>2315</v>
+        <v>2318</v>
       </c>
       <c r="C79" s="53" t="s">
-        <v>2316</v>
+        <v>2319</v>
       </c>
       <c r="D79" s="53" t="s">
-        <v>2317</v>
+        <v>2320</v>
       </c>
       <c r="G79" s="69"/>
       <c r="H79" s="69"/>
@@ -28390,13 +28441,13 @@
         <v>1069</v>
       </c>
       <c r="B80" s="53" t="s">
-        <v>2318</v>
+        <v>2321</v>
       </c>
       <c r="C80" s="53" t="s">
-        <v>2319</v>
+        <v>2322</v>
       </c>
       <c r="D80" s="53" t="s">
-        <v>2320</v>
+        <v>2323</v>
       </c>
       <c r="G80" s="69"/>
       <c r="H80" s="69"/>
@@ -28407,13 +28458,13 @@
         <v>1069</v>
       </c>
       <c r="B81" s="53" t="s">
-        <v>2321</v>
+        <v>2324</v>
       </c>
       <c r="C81" s="53" t="s">
-        <v>2322</v>
+        <v>2325</v>
       </c>
       <c r="D81" s="53" t="s">
-        <v>2323</v>
+        <v>2326</v>
       </c>
       <c r="G81" s="69"/>
       <c r="H81" s="69"/>
@@ -28424,13 +28475,13 @@
         <v>1069</v>
       </c>
       <c r="B82" s="53" t="s">
-        <v>2324</v>
+        <v>2327</v>
       </c>
       <c r="C82" s="53" t="s">
-        <v>2325</v>
+        <v>2328</v>
       </c>
       <c r="D82" s="53" t="s">
-        <v>2326</v>
+        <v>2329</v>
       </c>
       <c r="G82" s="69"/>
       <c r="H82" s="69"/>
@@ -28441,13 +28492,13 @@
         <v>1069</v>
       </c>
       <c r="B83" s="53" t="s">
-        <v>2327</v>
+        <v>2330</v>
       </c>
       <c r="C83" s="53" t="s">
-        <v>2328</v>
+        <v>2331</v>
       </c>
       <c r="D83" s="53" t="s">
-        <v>2329</v>
+        <v>2332</v>
       </c>
       <c r="G83" s="69"/>
       <c r="H83" s="69"/>
@@ -28458,13 +28509,13 @@
         <v>1069</v>
       </c>
       <c r="B84" s="53" t="s">
-        <v>2330</v>
+        <v>2333</v>
       </c>
       <c r="C84" s="53" t="s">
-        <v>2331</v>
+        <v>2334</v>
       </c>
       <c r="D84" s="53" t="s">
-        <v>2332</v>
+        <v>2335</v>
       </c>
       <c r="G84" s="69"/>
       <c r="H84" s="69"/>
@@ -28475,13 +28526,13 @@
         <v>1069</v>
       </c>
       <c r="B85" s="53" t="s">
-        <v>2333</v>
+        <v>2336</v>
       </c>
       <c r="C85" s="53" t="s">
-        <v>2334</v>
+        <v>2337</v>
       </c>
       <c r="D85" s="53" t="s">
-        <v>2335</v>
+        <v>2338</v>
       </c>
       <c r="G85" s="69"/>
       <c r="H85" s="69"/>
@@ -28492,13 +28543,13 @@
         <v>1069</v>
       </c>
       <c r="B86" s="69" t="s">
-        <v>2336</v>
+        <v>2339</v>
       </c>
       <c r="C86" s="69" t="s">
-        <v>2337</v>
+        <v>2340</v>
       </c>
       <c r="D86" s="69" t="s">
-        <v>2338</v>
+        <v>2341</v>
       </c>
       <c r="E86" s="69"/>
       <c r="F86" s="69"/>
@@ -28511,13 +28562,13 @@
         <v>1069</v>
       </c>
       <c r="B87" s="69" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="C87" s="69" t="s">
-        <v>2167</v>
+        <v>2170</v>
       </c>
       <c r="D87" s="69" t="s">
-        <v>2168</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28525,13 +28576,13 @@
         <v>1069</v>
       </c>
       <c r="B88" s="69" t="s">
-        <v>2339</v>
+        <v>2342</v>
       </c>
       <c r="C88" s="69" t="s">
-        <v>2169</v>
+        <v>2172</v>
       </c>
       <c r="D88" s="69" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28539,13 +28590,13 @@
         <v>99</v>
       </c>
       <c r="B89" s="69" t="s">
-        <v>2341</v>
+        <v>2344</v>
       </c>
       <c r="C89" s="69" t="s">
-        <v>2342</v>
+        <v>2345</v>
       </c>
       <c r="D89" s="69" t="s">
-        <v>2343</v>
+        <v>2346</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28553,13 +28604,13 @@
         <v>99</v>
       </c>
       <c r="B90" s="69" t="s">
-        <v>2344</v>
+        <v>2347</v>
       </c>
       <c r="C90" s="69" t="s">
-        <v>2345</v>
+        <v>2348</v>
       </c>
       <c r="D90" s="69" t="s">
-        <v>2346</v>
+        <v>2349</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28584,10 +28635,10 @@
         <v>1161</v>
       </c>
       <c r="C92" s="69" t="s">
-        <v>2169</v>
+        <v>2172</v>
       </c>
       <c r="D92" s="69" t="s">
-        <v>2340</v>
+        <v>2343</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28595,13 +28646,13 @@
         <v>423</v>
       </c>
       <c r="B93" s="56" t="s">
-        <v>2347</v>
+        <v>2350</v>
       </c>
       <c r="C93" s="54" t="s">
-        <v>2348</v>
+        <v>2351</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>2349</v>
+        <v>2352</v>
       </c>
       <c r="E93" s="54"/>
       <c r="F93" s="54"/>
@@ -28616,13 +28667,13 @@
         <v>423</v>
       </c>
       <c r="B94" s="56" t="s">
-        <v>2350</v>
+        <v>2353</v>
       </c>
       <c r="C94" s="54" t="s">
-        <v>2351</v>
+        <v>2354</v>
       </c>
       <c r="D94" s="8" t="s">
-        <v>2352</v>
+        <v>2355</v>
       </c>
       <c r="E94" s="54"/>
       <c r="F94" s="54"/>
@@ -28637,13 +28688,13 @@
         <v>423</v>
       </c>
       <c r="B95" s="56" t="s">
-        <v>2353</v>
+        <v>2356</v>
       </c>
       <c r="C95" s="54" t="s">
-        <v>2354</v>
+        <v>2357</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>2355</v>
+        <v>2358</v>
       </c>
       <c r="E95" s="54"/>
       <c r="F95" s="54"/>
@@ -28656,13 +28707,13 @@
         <v>423</v>
       </c>
       <c r="B96" s="56" t="s">
-        <v>2356</v>
+        <v>2359</v>
       </c>
       <c r="C96" s="54" t="s">
-        <v>2357</v>
+        <v>2360</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>2358</v>
+        <v>2361</v>
       </c>
       <c r="E96" s="54"/>
       <c r="F96" s="54"/>
@@ -28675,13 +28726,13 @@
         <v>423</v>
       </c>
       <c r="B97" s="56" t="s">
-        <v>2359</v>
+        <v>2362</v>
       </c>
       <c r="C97" s="54" t="s">
-        <v>2360</v>
+        <v>2363</v>
       </c>
       <c r="D97" s="8" t="s">
-        <v>2361</v>
+        <v>2364</v>
       </c>
       <c r="E97" s="54"/>
       <c r="F97" s="54"/>
@@ -28697,10 +28748,10 @@
         <v>1222</v>
       </c>
       <c r="C98" s="54" t="s">
-        <v>2362</v>
+        <v>2365</v>
       </c>
       <c r="D98" s="8" t="s">
-        <v>2363</v>
+        <v>2366</v>
       </c>
       <c r="E98" s="54"/>
       <c r="F98" s="54"/>
@@ -28718,10 +28769,10 @@
         <v>1223</v>
       </c>
       <c r="C99" s="54" t="s">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="D99" s="8" t="s">
-        <v>2365</v>
+        <v>2368</v>
       </c>
       <c r="E99" s="54"/>
       <c r="F99" s="54"/>
@@ -28734,13 +28785,13 @@
         <v>423</v>
       </c>
       <c r="B100" s="56" t="s">
-        <v>2366</v>
+        <v>2369</v>
       </c>
       <c r="C100" s="54" t="s">
-        <v>2367</v>
+        <v>2370</v>
       </c>
       <c r="D100" s="8" t="s">
-        <v>2368</v>
+        <v>2371</v>
       </c>
       <c r="E100" s="54"/>
       <c r="F100" s="54"/>
@@ -28771,10 +28822,10 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="96" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="B102" s="69" t="s">
-        <v>2370</v>
+        <v>2373</v>
       </c>
       <c r="C102" s="69" t="s">
         <v>1742</v>
@@ -28791,10 +28842,10 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="96" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="B103" s="69" t="s">
-        <v>2371</v>
+        <v>2374</v>
       </c>
       <c r="C103" s="69" t="s">
         <v>1747</v>
@@ -28811,16 +28862,16 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="96" t="s">
-        <v>2369</v>
+        <v>2372</v>
       </c>
       <c r="B104" s="69" t="s">
         <v>1215</v>
       </c>
       <c r="C104" s="69" t="s">
-        <v>2161</v>
+        <v>2164</v>
       </c>
       <c r="D104" s="69" t="s">
-        <v>2162</v>
+        <v>2165</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28828,13 +28879,13 @@
         <v>759</v>
       </c>
       <c r="B105" s="69" t="s">
-        <v>2372</v>
+        <v>2375</v>
       </c>
       <c r="C105" s="69" t="s">
-        <v>2373</v>
+        <v>2376</v>
       </c>
       <c r="D105" s="69" t="s">
-        <v>2374</v>
+        <v>2377</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28842,13 +28893,13 @@
         <v>759</v>
       </c>
       <c r="B106" s="69" t="s">
-        <v>2375</v>
+        <v>2378</v>
       </c>
       <c r="C106" s="69" t="s">
-        <v>2376</v>
+        <v>2379</v>
       </c>
       <c r="D106" s="69" t="s">
-        <v>2377</v>
+        <v>2380</v>
       </c>
       <c r="I106" s="93" t="n">
         <f aca="false">TRUE()</f>
@@ -28860,13 +28911,13 @@
         <v>759</v>
       </c>
       <c r="B107" s="69" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="C107" s="69" t="s">
-        <v>2379</v>
+        <v>2382</v>
       </c>
       <c r="D107" s="69" t="s">
-        <v>2380</v>
+        <v>2383</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28874,13 +28925,13 @@
         <v>759</v>
       </c>
       <c r="B108" s="69" t="s">
-        <v>2381</v>
+        <v>2384</v>
       </c>
       <c r="C108" s="69" t="s">
-        <v>2382</v>
+        <v>2385</v>
       </c>
       <c r="D108" s="69" t="s">
-        <v>2383</v>
+        <v>2386</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28888,7 +28939,7 @@
         <v>759</v>
       </c>
       <c r="G109" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28896,7 +28947,7 @@
         <v>759</v>
       </c>
       <c r="G110" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28904,13 +28955,13 @@
         <v>819</v>
       </c>
       <c r="B111" s="69" t="s">
-        <v>2384</v>
+        <v>2387</v>
       </c>
       <c r="C111" s="69" t="s">
-        <v>2385</v>
+        <v>2388</v>
       </c>
       <c r="D111" s="69" t="s">
-        <v>2386</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28918,13 +28969,13 @@
         <v>819</v>
       </c>
       <c r="B112" s="69" t="s">
-        <v>2387</v>
+        <v>2390</v>
       </c>
       <c r="C112" s="69" t="s">
-        <v>2388</v>
+        <v>2391</v>
       </c>
       <c r="D112" s="69" t="s">
-        <v>2389</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28932,13 +28983,13 @@
         <v>819</v>
       </c>
       <c r="B113" s="69" t="s">
-        <v>2378</v>
+        <v>2381</v>
       </c>
       <c r="C113" s="69" t="s">
-        <v>2390</v>
+        <v>2393</v>
       </c>
       <c r="D113" s="69" t="s">
-        <v>2391</v>
+        <v>2394</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28946,13 +28997,13 @@
         <v>819</v>
       </c>
       <c r="B114" s="56" t="s">
-        <v>2392</v>
+        <v>2395</v>
       </c>
       <c r="C114" s="54" t="s">
-        <v>2393</v>
+        <v>2396</v>
       </c>
       <c r="D114" s="51" t="s">
-        <v>2394</v>
+        <v>2397</v>
       </c>
       <c r="I114" s="93" t="n">
         <f aca="false">TRUE()</f>
@@ -28964,7 +29015,7 @@
         <v>819</v>
       </c>
       <c r="G115" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28972,7 +29023,7 @@
         <v>819</v>
       </c>
       <c r="G116" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28980,13 +29031,13 @@
         <v>347</v>
       </c>
       <c r="B117" s="69" t="s">
-        <v>2395</v>
+        <v>2398</v>
       </c>
       <c r="C117" s="69" t="s">
-        <v>2396</v>
+        <v>2399</v>
       </c>
       <c r="D117" s="69" t="s">
-        <v>2397</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -28994,13 +29045,13 @@
         <v>347</v>
       </c>
       <c r="B118" s="69" t="s">
-        <v>2398</v>
+        <v>2401</v>
       </c>
       <c r="C118" s="69" t="s">
-        <v>2399</v>
+        <v>2402</v>
       </c>
       <c r="D118" s="69" t="s">
-        <v>2400</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29008,13 +29059,13 @@
         <v>347</v>
       </c>
       <c r="B119" s="69" t="s">
-        <v>2401</v>
+        <v>2404</v>
       </c>
       <c r="C119" s="69" t="s">
-        <v>2402</v>
+        <v>2405</v>
       </c>
       <c r="D119" s="69" t="s">
-        <v>2403</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29027,103 +29078,103 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="92" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B121" s="56" t="s">
         <v>1189</v>
       </c>
       <c r="C121" s="56" t="s">
-        <v>2405</v>
+        <v>2408</v>
       </c>
       <c r="D121" s="56" t="s">
-        <v>2406</v>
+        <v>2409</v>
       </c>
       <c r="E121" s="56" t="s">
-        <v>2407</v>
+        <v>2410</v>
       </c>
       <c r="F121" s="56" t="s">
-        <v>2408</v>
+        <v>2411</v>
       </c>
       <c r="G121" s="92"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="92" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B122" s="56" t="s">
         <v>1190</v>
       </c>
       <c r="C122" s="56" t="s">
-        <v>2409</v>
+        <v>2412</v>
       </c>
       <c r="D122" s="56" t="s">
-        <v>2410</v>
+        <v>2413</v>
       </c>
       <c r="E122" s="56" t="s">
-        <v>2411</v>
+        <v>2414</v>
       </c>
       <c r="F122" s="56" t="s">
-        <v>2412</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="92" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B123" s="56" t="s">
         <v>1191</v>
       </c>
       <c r="C123" s="56" t="s">
-        <v>2413</v>
+        <v>2416</v>
       </c>
       <c r="D123" s="56" t="s">
-        <v>2414</v>
+        <v>2417</v>
       </c>
       <c r="E123" s="56" t="s">
-        <v>2415</v>
+        <v>2418</v>
       </c>
       <c r="F123" s="56" t="s">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="92" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B124" s="56" t="s">
         <v>1205</v>
       </c>
       <c r="C124" s="56" t="s">
-        <v>2417</v>
+        <v>2420</v>
       </c>
       <c r="D124" s="56" t="s">
-        <v>2418</v>
+        <v>2421</v>
       </c>
       <c r="E124" s="56" t="s">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="F124" s="56" t="s">
-        <v>2420</v>
+        <v>2423</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="92" t="s">
-        <v>2404</v>
+        <v>2407</v>
       </c>
       <c r="B125" s="56" t="s">
-        <v>2278</v>
+        <v>2281</v>
       </c>
       <c r="C125" s="56" t="s">
-        <v>2421</v>
+        <v>2424</v>
       </c>
       <c r="D125" s="56" t="s">
-        <v>2422</v>
+        <v>2425</v>
       </c>
       <c r="E125" s="56" t="s">
-        <v>2423</v>
+        <v>2426</v>
       </c>
       <c r="F125" s="56" t="s">
-        <v>2424</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29131,7 +29182,7 @@
         <v>686</v>
       </c>
       <c r="B126" s="69" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="C126" s="8" t="s">
         <v>2011</v>
@@ -29148,10 +29199,10 @@
         <v>1227</v>
       </c>
       <c r="C127" s="8" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="D127" s="60" t="s">
-        <v>2426</v>
+        <v>2429</v>
       </c>
       <c r="H127" s="98" t="s">
         <v>1225</v>
@@ -29162,16 +29213,16 @@
         <v>686</v>
       </c>
       <c r="B128" s="69" t="s">
-        <v>2427</v>
+        <v>2430</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>2428</v>
+        <v>2431</v>
       </c>
       <c r="D128" s="60" t="s">
-        <v>2429</v>
+        <v>2432</v>
       </c>
       <c r="H128" s="99" t="s">
-        <v>2430</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29179,7 +29230,7 @@
         <v>686</v>
       </c>
       <c r="B129" s="69" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="C129" s="8" t="s">
         <v>2020</v>
@@ -29196,7 +29247,7 @@
         <v>686</v>
       </c>
       <c r="B130" s="69" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="C130" s="8" t="s">
         <v>2023</v>
@@ -29220,7 +29271,7 @@
         <v>692</v>
       </c>
       <c r="B132" s="69" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="C132" s="8" t="s">
         <v>2011</v>
@@ -29234,7 +29285,7 @@
         <v>692</v>
       </c>
       <c r="B133" s="69" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>2030</v>
@@ -29248,7 +29299,7 @@
         <v>692</v>
       </c>
       <c r="B134" s="69" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="C134" s="8" t="s">
         <v>2020</v>
@@ -29265,7 +29316,7 @@
         <v>692</v>
       </c>
       <c r="B135" s="69" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="C135" s="8" t="s">
         <v>2023</v>
@@ -29279,13 +29330,13 @@
         <v>692</v>
       </c>
       <c r="B136" s="69" t="s">
-        <v>2434</v>
+        <v>2437</v>
       </c>
       <c r="C136" s="8" t="s">
-        <v>2435</v>
+        <v>2438</v>
       </c>
       <c r="D136" s="60" t="s">
-        <v>2436</v>
+        <v>2439</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29293,7 +29344,7 @@
         <v>692</v>
       </c>
       <c r="B137" s="69" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="C137" s="8" t="s">
         <v>2026</v>
@@ -29309,7 +29360,7 @@
       <c r="C138" s="60"/>
       <c r="D138" s="60"/>
       <c r="G138" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29317,16 +29368,16 @@
         <v>582</v>
       </c>
       <c r="B139" s="69" t="s">
-        <v>2438</v>
+        <v>2441</v>
       </c>
       <c r="C139" s="60" t="s">
-        <v>2439</v>
+        <v>2442</v>
       </c>
       <c r="D139" s="60" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="H139" s="57" t="s">
-        <v>2441</v>
+        <v>2444</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29337,13 +29388,13 @@
         <v>1215</v>
       </c>
       <c r="C140" s="60" t="s">
-        <v>2442</v>
+        <v>2445</v>
       </c>
       <c r="D140" s="60" t="s">
-        <v>2443</v>
+        <v>2446</v>
       </c>
       <c r="H140" s="8" t="s">
-        <v>2444</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29354,10 +29405,10 @@
         <v>1157</v>
       </c>
       <c r="C141" s="60" t="s">
-        <v>2445</v>
+        <v>2448</v>
       </c>
       <c r="D141" s="60" t="s">
-        <v>2446</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29365,13 +29416,13 @@
         <v>582</v>
       </c>
       <c r="B142" s="69" t="s">
-        <v>2447</v>
+        <v>2450</v>
       </c>
       <c r="C142" s="60" t="s">
-        <v>2448</v>
+        <v>2451</v>
       </c>
       <c r="D142" s="60" t="s">
-        <v>2449</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29381,7 +29432,7 @@
       <c r="C143" s="60"/>
       <c r="D143" s="60"/>
       <c r="G143" s="69" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29389,13 +29440,13 @@
         <v>615</v>
       </c>
       <c r="B144" s="69" t="s">
-        <v>2450</v>
+        <v>2453</v>
       </c>
       <c r="C144" s="60" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
       <c r="D144" s="60" t="s">
-        <v>2451</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29403,13 +29454,13 @@
         <v>615</v>
       </c>
       <c r="B145" s="69" t="s">
-        <v>2452</v>
+        <v>2455</v>
       </c>
       <c r="C145" s="60" t="s">
-        <v>2453</v>
+        <v>2456</v>
       </c>
       <c r="D145" s="60" t="s">
-        <v>2454</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29419,7 +29470,7 @@
       <c r="C146" s="60"/>
       <c r="D146" s="60"/>
       <c r="G146" s="69" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29427,13 +29478,13 @@
         <v>639</v>
       </c>
       <c r="B147" s="69" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>2456</v>
+        <v>2459</v>
       </c>
       <c r="D147" s="60" t="s">
-        <v>2457</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29441,13 +29492,13 @@
         <v>639</v>
       </c>
       <c r="B148" s="69" t="s">
-        <v>2458</v>
+        <v>2461</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>2459</v>
+        <v>2462</v>
       </c>
       <c r="D148" s="60" t="s">
-        <v>2460</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29457,7 +29508,7 @@
       <c r="C149" s="60"/>
       <c r="D149" s="60"/>
       <c r="G149" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29467,7 +29518,7 @@
       <c r="C150" s="60"/>
       <c r="D150" s="60"/>
       <c r="G150" s="69" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29475,13 +29526,13 @@
         <v>646</v>
       </c>
       <c r="B151" s="69" t="s">
-        <v>2461</v>
+        <v>2464</v>
       </c>
       <c r="C151" s="8" t="s">
-        <v>2462</v>
+        <v>2465</v>
       </c>
       <c r="D151" s="60" t="s">
-        <v>2463</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29489,13 +29540,13 @@
         <v>646</v>
       </c>
       <c r="B152" s="69" t="s">
-        <v>2464</v>
+        <v>2467</v>
       </c>
       <c r="C152" s="8" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
       <c r="D152" s="60" t="s">
-        <v>2465</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29503,13 +29554,13 @@
         <v>646</v>
       </c>
       <c r="B153" s="69" t="s">
-        <v>2466</v>
+        <v>2469</v>
       </c>
       <c r="C153" s="8" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
       <c r="D153" s="8" t="s">
-        <v>2467</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29517,13 +29568,13 @@
         <v>646</v>
       </c>
       <c r="B154" s="69" t="s">
-        <v>2468</v>
+        <v>2471</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
       <c r="D154" s="8" t="s">
-        <v>2469</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29533,7 +29584,7 @@
       <c r="C155" s="60"/>
       <c r="D155" s="60"/>
       <c r="G155" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29543,7 +29594,7 @@
       <c r="C156" s="60"/>
       <c r="D156" s="60"/>
       <c r="G156" s="69" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29551,13 +29602,13 @@
         <v>651</v>
       </c>
       <c r="B157" s="69" t="s">
-        <v>2470</v>
+        <v>2473</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>2471</v>
+        <v>2474</v>
       </c>
       <c r="D157" s="60" t="s">
-        <v>2472</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29565,13 +29616,13 @@
         <v>651</v>
       </c>
       <c r="B158" s="69" t="s">
-        <v>2473</v>
+        <v>2476</v>
       </c>
       <c r="C158" s="8" t="s">
-        <v>2474</v>
+        <v>2477</v>
       </c>
       <c r="D158" s="60" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29579,13 +29630,13 @@
         <v>651</v>
       </c>
       <c r="B159" s="69" t="s">
-        <v>2455</v>
+        <v>2458</v>
       </c>
       <c r="C159" s="8" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="D159" s="60" t="s">
-        <v>2477</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29593,13 +29644,13 @@
         <v>651</v>
       </c>
       <c r="B160" s="69" t="s">
-        <v>2478</v>
+        <v>2481</v>
       </c>
       <c r="C160" s="8" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
       <c r="D160" s="8" t="s">
-        <v>2479</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29607,13 +29658,13 @@
         <v>651</v>
       </c>
       <c r="B161" s="69" t="s">
-        <v>2480</v>
+        <v>2483</v>
       </c>
       <c r="C161" s="8" t="s">
-        <v>2481</v>
+        <v>2484</v>
       </c>
       <c r="D161" s="60" t="s">
-        <v>2482</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29623,7 +29674,7 @@
       <c r="C162" s="60"/>
       <c r="D162" s="60"/>
       <c r="G162" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29633,7 +29684,7 @@
       <c r="C163" s="60"/>
       <c r="D163" s="60"/>
       <c r="G163" s="69" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29641,7 +29692,7 @@
         <v>783</v>
       </c>
       <c r="B164" s="56" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="C164" s="69" t="s">
         <v>1960</v>
@@ -29660,7 +29711,7 @@
         <v>783</v>
       </c>
       <c r="B165" s="56" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="C165" s="69" t="s">
         <v>1978</v>
@@ -29679,13 +29730,13 @@
         <v>783</v>
       </c>
       <c r="B166" s="56" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>2483</v>
+        <v>2486</v>
       </c>
       <c r="D166" s="60" t="s">
-        <v>2484</v>
+        <v>2487</v>
       </c>
       <c r="E166" s="56"/>
       <c r="F166" s="56"/>
@@ -29698,7 +29749,7 @@
         <v>783</v>
       </c>
       <c r="B167" s="56" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="C167" s="8" t="s">
         <v>1913</v>
@@ -29717,7 +29768,7 @@
         <v>783</v>
       </c>
       <c r="B168" s="56" t="s">
-        <v>2485</v>
+        <v>2488</v>
       </c>
       <c r="C168" s="8" t="s">
         <v>1916</v>
@@ -29739,10 +29790,10 @@
         <v>229</v>
       </c>
       <c r="C169" s="54" t="s">
-        <v>2486</v>
+        <v>2489</v>
       </c>
       <c r="D169" s="8" t="s">
-        <v>2487</v>
+        <v>2490</v>
       </c>
       <c r="E169" s="56"/>
       <c r="F169" s="56"/>
@@ -29757,13 +29808,13 @@
         <v>783</v>
       </c>
       <c r="B170" s="56" t="s">
-        <v>2488</v>
+        <v>2491</v>
       </c>
       <c r="C170" s="54" t="s">
-        <v>2489</v>
+        <v>2492</v>
       </c>
       <c r="D170" s="8" t="s">
-        <v>2490</v>
+        <v>2493</v>
       </c>
       <c r="E170" s="56"/>
       <c r="F170" s="56"/>
@@ -29778,13 +29829,13 @@
         <v>129</v>
       </c>
       <c r="B171" s="56" t="s">
-        <v>2491</v>
+        <v>2494</v>
       </c>
       <c r="C171" s="54" t="s">
-        <v>2492</v>
+        <v>2495</v>
       </c>
       <c r="D171" s="8" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
       <c r="E171" s="56"/>
       <c r="F171" s="56"/>
@@ -29797,13 +29848,13 @@
         <v>129</v>
       </c>
       <c r="B172" s="56" t="s">
-        <v>2494</v>
+        <v>2497</v>
       </c>
       <c r="C172" s="54" t="s">
-        <v>2495</v>
+        <v>2498</v>
       </c>
       <c r="D172" s="8" t="s">
-        <v>2496</v>
+        <v>2499</v>
       </c>
       <c r="E172" s="56"/>
       <c r="F172" s="56"/>
@@ -29857,10 +29908,10 @@
         <v>2</v>
       </c>
       <c r="C175" s="55" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="D175" s="55" t="s">
-        <v>2497</v>
+        <v>2500</v>
       </c>
       <c r="E175" s="56"/>
       <c r="F175" s="56"/>
@@ -29876,10 +29927,10 @@
         <v>1157</v>
       </c>
       <c r="C176" s="54" t="s">
-        <v>2498</v>
+        <v>2501</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
       <c r="E176" s="56"/>
       <c r="F176" s="56"/>
@@ -29895,10 +29946,10 @@
         <v>1215</v>
       </c>
       <c r="C177" s="54" t="s">
-        <v>2500</v>
+        <v>2503</v>
       </c>
       <c r="D177" s="8" t="s">
-        <v>2501</v>
+        <v>2504</v>
       </c>
       <c r="E177" s="56"/>
       <c r="F177" s="56"/>
@@ -29916,7 +29967,7 @@
       <c r="E178" s="56"/>
       <c r="F178" s="56"/>
       <c r="G178" s="56" t="s">
-        <v>2166</v>
+        <v>2169</v>
       </c>
       <c r="H178" s="56"/>
       <c r="I178" s="56"/>
@@ -29926,13 +29977,13 @@
         <v>246</v>
       </c>
       <c r="B179" s="56" t="s">
-        <v>2502</v>
+        <v>2505</v>
       </c>
       <c r="C179" s="51" t="s">
-        <v>2503</v>
+        <v>2506</v>
       </c>
       <c r="D179" s="8" t="s">
-        <v>2504</v>
+        <v>2507</v>
       </c>
       <c r="E179" s="56"/>
       <c r="F179" s="56"/>
@@ -29947,13 +29998,13 @@
         <v>246</v>
       </c>
       <c r="B180" s="56" t="s">
-        <v>2505</v>
+        <v>2508</v>
       </c>
       <c r="C180" s="51" t="s">
-        <v>2506</v>
+        <v>2509</v>
       </c>
       <c r="D180" s="8" t="s">
-        <v>2507</v>
+        <v>2510</v>
       </c>
       <c r="E180" s="56"/>
       <c r="F180" s="56"/>
@@ -29968,13 +30019,13 @@
         <v>246</v>
       </c>
       <c r="B181" s="56" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
       <c r="C181" s="51" t="s">
-        <v>2509</v>
+        <v>2512</v>
       </c>
       <c r="D181" s="8" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="E181" s="56"/>
       <c r="F181" s="56"/>
@@ -29989,13 +30040,13 @@
         <v>246</v>
       </c>
       <c r="B182" s="56" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="C182" s="51" t="s">
-        <v>2512</v>
+        <v>2515</v>
       </c>
       <c r="D182" s="8" t="s">
-        <v>2513</v>
+        <v>2516</v>
       </c>
       <c r="E182" s="56"/>
       <c r="F182" s="56"/>
@@ -30010,13 +30061,13 @@
         <v>246</v>
       </c>
       <c r="B183" s="56" t="s">
-        <v>2514</v>
+        <v>2517</v>
       </c>
       <c r="C183" s="51" t="s">
-        <v>2515</v>
+        <v>2518</v>
       </c>
       <c r="D183" s="8" t="s">
-        <v>2516</v>
+        <v>2519</v>
       </c>
       <c r="E183" s="56"/>
       <c r="F183" s="56"/>
@@ -30031,13 +30082,13 @@
         <v>246</v>
       </c>
       <c r="B184" s="56" t="s">
-        <v>2517</v>
+        <v>2520</v>
       </c>
       <c r="C184" s="51" t="s">
-        <v>2518</v>
+        <v>2521</v>
       </c>
       <c r="D184" s="8" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
       <c r="E184" s="56"/>
       <c r="F184" s="56"/>
@@ -30052,13 +30103,13 @@
         <v>246</v>
       </c>
       <c r="B185" s="56" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
       <c r="C185" s="51" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
       <c r="D185" s="8" t="s">
-        <v>2522</v>
+        <v>2525</v>
       </c>
       <c r="E185" s="56"/>
       <c r="F185" s="56"/>
@@ -30073,13 +30124,13 @@
         <v>246</v>
       </c>
       <c r="B186" s="56" t="s">
-        <v>2523</v>
+        <v>2526</v>
       </c>
       <c r="C186" s="51" t="s">
-        <v>2524</v>
+        <v>2527</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>2525</v>
+        <v>2528</v>
       </c>
       <c r="E186" s="56"/>
       <c r="F186" s="56"/>
@@ -30094,13 +30145,13 @@
         <v>246</v>
       </c>
       <c r="B187" s="56" t="s">
-        <v>2526</v>
+        <v>2529</v>
       </c>
       <c r="C187" s="51" t="s">
-        <v>2527</v>
+        <v>2530</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>2528</v>
+        <v>2531</v>
       </c>
       <c r="E187" s="56"/>
       <c r="F187" s="56"/>
@@ -30118,10 +30169,10 @@
         <v>229</v>
       </c>
       <c r="C188" s="51" t="s">
-        <v>2163</v>
+        <v>2166</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>2164</v>
+        <v>2167</v>
       </c>
       <c r="E188" s="56"/>
       <c r="F188" s="56"/>
@@ -30151,13 +30202,13 @@
         <v>258</v>
       </c>
       <c r="B190" s="56" t="s">
-        <v>2529</v>
+        <v>2532</v>
       </c>
       <c r="C190" s="51" t="s">
-        <v>2530</v>
+        <v>2533</v>
       </c>
       <c r="D190" s="8" t="s">
-        <v>2531</v>
+        <v>2534</v>
       </c>
       <c r="E190" s="56"/>
       <c r="F190" s="56"/>
@@ -30172,13 +30223,13 @@
         <v>258</v>
       </c>
       <c r="B191" s="56" t="s">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="C191" s="51" t="s">
-        <v>2533</v>
+        <v>2536</v>
       </c>
       <c r="D191" s="8" t="s">
-        <v>2534</v>
+        <v>2537</v>
       </c>
       <c r="E191" s="56"/>
       <c r="F191" s="56"/>
@@ -30193,13 +30244,13 @@
         <v>258</v>
       </c>
       <c r="B192" s="56" t="s">
-        <v>2535</v>
+        <v>2538</v>
       </c>
       <c r="C192" s="51" t="s">
-        <v>2536</v>
+        <v>2539</v>
       </c>
       <c r="D192" s="8" t="s">
-        <v>2537</v>
+        <v>2540</v>
       </c>
       <c r="E192" s="56"/>
       <c r="F192" s="56"/>
@@ -30214,13 +30265,13 @@
         <v>258</v>
       </c>
       <c r="B193" s="56" t="s">
-        <v>2538</v>
+        <v>2541</v>
       </c>
       <c r="C193" s="51" t="s">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="D193" s="8" t="s">
-        <v>2540</v>
+        <v>2543</v>
       </c>
       <c r="E193" s="56"/>
       <c r="F193" s="56"/>
@@ -30235,13 +30286,13 @@
         <v>258</v>
       </c>
       <c r="B194" s="56" t="s">
-        <v>2541</v>
+        <v>2544</v>
       </c>
       <c r="C194" s="51" t="s">
-        <v>2542</v>
+        <v>2545</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>2543</v>
+        <v>2546</v>
       </c>
       <c r="E194" s="56"/>
       <c r="F194" s="56"/>
@@ -30256,13 +30307,13 @@
         <v>258</v>
       </c>
       <c r="B195" s="56" t="s">
-        <v>2544</v>
+        <v>2547</v>
       </c>
       <c r="C195" s="51" t="s">
-        <v>2545</v>
+        <v>2548</v>
       </c>
       <c r="D195" s="8" t="s">
-        <v>2546</v>
+        <v>2549</v>
       </c>
       <c r="E195" s="56"/>
       <c r="F195" s="56"/>
@@ -30277,13 +30328,13 @@
         <v>258</v>
       </c>
       <c r="B196" s="56" t="s">
-        <v>2547</v>
+        <v>2550</v>
       </c>
       <c r="C196" s="51" t="s">
-        <v>2548</v>
+        <v>2551</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="E196" s="56"/>
       <c r="F196" s="56"/>
@@ -30301,10 +30352,10 @@
         <v>1197</v>
       </c>
       <c r="C197" s="51" t="s">
-        <v>2550</v>
+        <v>2553</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="E197" s="56"/>
       <c r="F197" s="56"/>
@@ -30321,10 +30372,10 @@
         <v>229</v>
       </c>
       <c r="C198" s="51" t="s">
-        <v>2163</v>
+        <v>2166</v>
       </c>
       <c r="D198" s="8" t="s">
-        <v>2164</v>
+        <v>2167</v>
       </c>
       <c r="E198" s="56"/>
       <c r="F198" s="56"/>
@@ -30342,10 +30393,10 @@
         <v>1161</v>
       </c>
       <c r="C199" s="56" t="s">
-        <v>2169</v>
+        <v>2172</v>
       </c>
       <c r="D199" s="56" t="s">
-        <v>2170</v>
+        <v>2173</v>
       </c>
       <c r="E199" s="56"/>
       <c r="F199" s="56"/>
@@ -30359,13 +30410,13 @@
         <v>287</v>
       </c>
       <c r="B200" s="56" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="C200" s="51" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="D200" s="8" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="E200" s="56"/>
       <c r="F200" s="56"/>
@@ -30378,13 +30429,13 @@
         <v>287</v>
       </c>
       <c r="B201" s="56" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="C201" s="51" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="D201" s="8" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="E201" s="56"/>
       <c r="F201" s="56"/>
@@ -30397,13 +30448,13 @@
         <v>287</v>
       </c>
       <c r="B202" s="56" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="C202" s="51" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="D202" s="8" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="E202" s="56"/>
       <c r="F202" s="56"/>
@@ -30416,13 +30467,13 @@
         <v>287</v>
       </c>
       <c r="B203" s="56" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="C203" s="51" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="D203" s="8" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="E203" s="56"/>
       <c r="F203" s="56"/>
@@ -30435,13 +30486,13 @@
         <v>287</v>
       </c>
       <c r="B204" s="56" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="C204" s="51" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="D204" s="8" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="E204" s="56"/>
       <c r="F204" s="56"/>
@@ -30454,13 +30505,13 @@
         <v>294</v>
       </c>
       <c r="B205" s="56" t="s">
-        <v>2552</v>
+        <v>2555</v>
       </c>
       <c r="C205" s="51" t="s">
-        <v>2553</v>
+        <v>2556</v>
       </c>
       <c r="D205" s="8" t="s">
-        <v>2554</v>
+        <v>2557</v>
       </c>
       <c r="E205" s="56"/>
       <c r="F205" s="56"/>
@@ -30475,13 +30526,13 @@
         <v>294</v>
       </c>
       <c r="B206" s="56" t="s">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="C206" s="51" t="s">
-        <v>2556</v>
+        <v>2559</v>
       </c>
       <c r="D206" s="8" t="s">
-        <v>2557</v>
+        <v>2560</v>
       </c>
       <c r="E206" s="56"/>
       <c r="F206" s="56"/>
@@ -30494,13 +30545,13 @@
         <v>294</v>
       </c>
       <c r="B207" s="56" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="C207" s="51" t="s">
-        <v>2559</v>
+        <v>2562</v>
       </c>
       <c r="D207" s="8" t="s">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="E207" s="56"/>
       <c r="F207" s="56"/>
@@ -30513,13 +30564,13 @@
         <v>294</v>
       </c>
       <c r="B208" s="56" t="s">
-        <v>2561</v>
+        <v>2564</v>
       </c>
       <c r="C208" s="51" t="s">
-        <v>2562</v>
+        <v>2565</v>
       </c>
       <c r="D208" s="8" t="s">
-        <v>2563</v>
+        <v>2566</v>
       </c>
       <c r="E208" s="56"/>
       <c r="F208" s="56"/>
@@ -30532,13 +30583,13 @@
         <v>294</v>
       </c>
       <c r="B209" s="56" t="s">
-        <v>2564</v>
+        <v>2567</v>
       </c>
       <c r="C209" s="51" t="s">
-        <v>2565</v>
+        <v>2568</v>
       </c>
       <c r="D209" s="8" t="s">
-        <v>2566</v>
+        <v>2569</v>
       </c>
       <c r="E209" s="56"/>
       <c r="F209" s="56"/>
@@ -30551,7 +30602,7 @@
         <v>847</v>
       </c>
       <c r="B210" s="69" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="C210" s="69" t="s">
         <v>2011</v>
@@ -30565,7 +30616,7 @@
         <v>847</v>
       </c>
       <c r="B211" s="69" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="C211" s="69" t="s">
         <v>2030</v>
@@ -30579,13 +30630,13 @@
         <v>847</v>
       </c>
       <c r="B212" s="69" t="s">
-        <v>2567</v>
+        <v>2570</v>
       </c>
       <c r="C212" s="69" t="s">
-        <v>2568</v>
+        <v>2571</v>
       </c>
       <c r="D212" s="69" t="s">
-        <v>2569</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30593,13 +30644,13 @@
         <v>847</v>
       </c>
       <c r="B213" s="69" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="C213" s="69" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="D213" s="69" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30607,7 +30658,7 @@
         <v>847</v>
       </c>
       <c r="G214" s="69" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30615,13 +30666,13 @@
         <v>872</v>
       </c>
       <c r="B215" s="69" t="s">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="C215" s="69" t="s">
-        <v>2573</v>
+        <v>2576</v>
       </c>
       <c r="D215" s="69" t="s">
-        <v>2574</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30629,13 +30680,13 @@
         <v>872</v>
       </c>
       <c r="B216" s="69" t="s">
-        <v>2575</v>
+        <v>2578</v>
       </c>
       <c r="C216" s="69" t="s">
-        <v>2576</v>
+        <v>2579</v>
       </c>
       <c r="D216" s="69" t="s">
-        <v>2577</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30643,13 +30694,13 @@
         <v>872</v>
       </c>
       <c r="B217" s="69" t="s">
-        <v>2578</v>
+        <v>2581</v>
       </c>
       <c r="C217" s="69" t="s">
-        <v>2579</v>
+        <v>2582</v>
       </c>
       <c r="D217" s="69" t="s">
-        <v>2580</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30657,13 +30708,13 @@
         <v>872</v>
       </c>
       <c r="B218" s="69" t="s">
-        <v>2581</v>
+        <v>2584</v>
       </c>
       <c r="C218" s="69" t="s">
-        <v>2582</v>
+        <v>2585</v>
       </c>
       <c r="D218" s="69" t="s">
-        <v>2583</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30671,13 +30722,13 @@
         <v>872</v>
       </c>
       <c r="B219" s="69" t="s">
-        <v>2584</v>
+        <v>2587</v>
       </c>
       <c r="C219" s="69" t="s">
-        <v>2585</v>
+        <v>2588</v>
       </c>
       <c r="D219" s="69" t="s">
-        <v>2586</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30685,13 +30736,13 @@
         <v>872</v>
       </c>
       <c r="B220" s="69" t="s">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="C220" s="69" t="s">
-        <v>2588</v>
+        <v>2591</v>
       </c>
       <c r="D220" s="69" t="s">
-        <v>2589</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30702,10 +30753,10 @@
         <v>229</v>
       </c>
       <c r="C221" s="69" t="s">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="D221" s="69" t="s">
-        <v>2591</v>
+        <v>2594</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30713,7 +30764,7 @@
         <v>877</v>
       </c>
       <c r="B222" s="69" t="s">
-        <v>2425</v>
+        <v>2428</v>
       </c>
       <c r="C222" s="69" t="s">
         <v>2011</v>
@@ -30727,7 +30778,7 @@
         <v>877</v>
       </c>
       <c r="B223" s="69" t="s">
-        <v>2433</v>
+        <v>2436</v>
       </c>
       <c r="C223" s="69" t="s">
         <v>2030</v>
@@ -30741,13 +30792,13 @@
         <v>877</v>
       </c>
       <c r="B224" s="69" t="s">
-        <v>2431</v>
+        <v>2434</v>
       </c>
       <c r="C224" s="69" t="s">
-        <v>2592</v>
+        <v>2595</v>
       </c>
       <c r="D224" s="69" t="s">
-        <v>2593</v>
+        <v>2596</v>
       </c>
     </row>
     <row r="225" s="53" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30755,13 +30806,13 @@
         <v>877</v>
       </c>
       <c r="B225" s="69" t="s">
-        <v>2432</v>
+        <v>2435</v>
       </c>
       <c r="C225" s="69" t="s">
-        <v>2594</v>
+        <v>2597</v>
       </c>
       <c r="D225" s="69" t="s">
-        <v>2595</v>
+        <v>2598</v>
       </c>
       <c r="E225" s="69"/>
       <c r="F225" s="69"/>
@@ -30774,13 +30825,13 @@
         <v>877</v>
       </c>
       <c r="B226" s="69" t="s">
-        <v>2437</v>
+        <v>2440</v>
       </c>
       <c r="C226" s="69" t="s">
-        <v>2570</v>
+        <v>2573</v>
       </c>
       <c r="D226" s="69" t="s">
-        <v>2571</v>
+        <v>2574</v>
       </c>
       <c r="E226" s="69"/>
       <c r="F226" s="69"/>
@@ -30796,10 +30847,10 @@
         <v>229</v>
       </c>
       <c r="C227" s="69" t="s">
-        <v>2596</v>
+        <v>2599</v>
       </c>
       <c r="D227" s="69" t="s">
-        <v>2597</v>
+        <v>2600</v>
       </c>
       <c r="E227" s="69"/>
       <c r="F227" s="69"/>
@@ -30815,10 +30866,10 @@
         <v>1248</v>
       </c>
       <c r="C228" s="8" t="s">
-        <v>2598</v>
+        <v>2601</v>
       </c>
       <c r="D228" s="8" t="s">
-        <v>2599</v>
+        <v>2602</v>
       </c>
       <c r="E228" s="69"/>
       <c r="F228" s="69"/>
@@ -30831,13 +30882,13 @@
         <v>1042</v>
       </c>
       <c r="B229" s="69" t="s">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="C229" s="8" t="s">
-        <v>2601</v>
+        <v>2604</v>
       </c>
       <c r="D229" s="8" t="s">
-        <v>2602</v>
+        <v>2605</v>
       </c>
       <c r="E229" s="69"/>
       <c r="F229" s="69"/>
@@ -30852,13 +30903,13 @@
         <v>1042</v>
       </c>
       <c r="B230" s="69" t="s">
-        <v>2603</v>
+        <v>2606</v>
       </c>
       <c r="C230" s="8" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
       <c r="D230" s="8" t="s">
-        <v>2605</v>
+        <v>2608</v>
       </c>
       <c r="E230" s="69"/>
       <c r="F230" s="69"/>
@@ -30873,13 +30924,13 @@
         <v>1042</v>
       </c>
       <c r="B231" s="69" t="s">
-        <v>2606</v>
+        <v>2609</v>
       </c>
       <c r="C231" s="8" t="s">
-        <v>2607</v>
+        <v>2610</v>
       </c>
       <c r="D231" s="54" t="s">
-        <v>2608</v>
+        <v>2611</v>
       </c>
       <c r="E231" s="69"/>
       <c r="F231" s="69"/>
@@ -30894,13 +30945,13 @@
         <v>1042</v>
       </c>
       <c r="B232" s="69" t="s">
-        <v>2609</v>
+        <v>2612</v>
       </c>
       <c r="C232" s="8" t="s">
-        <v>2610</v>
+        <v>2613</v>
       </c>
       <c r="D232" s="51" t="s">
-        <v>2611</v>
+        <v>2614</v>
       </c>
       <c r="E232" s="69"/>
       <c r="F232" s="69"/>
@@ -30913,13 +30964,13 @@
         <v>1048</v>
       </c>
       <c r="B233" s="69" t="s">
-        <v>2612</v>
+        <v>2615</v>
       </c>
       <c r="C233" s="8" t="s">
-        <v>2613</v>
+        <v>2616</v>
       </c>
       <c r="D233" s="8" t="s">
-        <v>2614</v>
+        <v>2617</v>
       </c>
       <c r="E233" s="69"/>
       <c r="F233" s="69"/>
@@ -30934,13 +30985,13 @@
         <v>1048</v>
       </c>
       <c r="B234" s="69" t="s">
-        <v>2615</v>
+        <v>2618</v>
       </c>
       <c r="C234" s="8" t="s">
-        <v>2616</v>
+        <v>2619</v>
       </c>
       <c r="D234" s="8" t="s">
-        <v>2617</v>
+        <v>2620</v>
       </c>
       <c r="E234" s="69"/>
       <c r="F234" s="69"/>
@@ -30955,13 +31006,13 @@
         <v>1048</v>
       </c>
       <c r="B235" s="69" t="s">
-        <v>2618</v>
+        <v>2621</v>
       </c>
       <c r="C235" s="8" t="s">
-        <v>2619</v>
+        <v>2622</v>
       </c>
       <c r="D235" s="8" t="s">
-        <v>2620</v>
+        <v>2623</v>
       </c>
       <c r="E235" s="69"/>
       <c r="F235" s="69"/>
@@ -30971,16 +31022,16 @@
     </row>
     <row r="236" s="53" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="57" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="B236" s="69" t="s">
         <v>1157</v>
       </c>
       <c r="C236" s="54" t="s">
-        <v>2622</v>
+        <v>2625</v>
       </c>
       <c r="D236" s="8" t="s">
-        <v>2623</v>
+        <v>2626</v>
       </c>
       <c r="E236" s="69"/>
       <c r="F236" s="69"/>
@@ -30990,16 +31041,16 @@
     </row>
     <row r="237" s="53" customFormat="true" ht="30.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="57" t="s">
-        <v>2621</v>
+        <v>2624</v>
       </c>
       <c r="B237" s="69" t="s">
         <v>1215</v>
       </c>
       <c r="C237" s="54" t="s">
-        <v>2624</v>
+        <v>2627</v>
       </c>
       <c r="D237" s="51" t="s">
-        <v>2625</v>
+        <v>2628</v>
       </c>
       <c r="E237" s="69"/>
       <c r="F237" s="69"/>
@@ -31012,13 +31063,13 @@
         <v>1078</v>
       </c>
       <c r="B238" s="69" t="s">
-        <v>2626</v>
+        <v>2629</v>
       </c>
       <c r="C238" s="8" t="s">
-        <v>2627</v>
+        <v>2630</v>
       </c>
       <c r="D238" s="54" t="s">
-        <v>2628</v>
+        <v>2631</v>
       </c>
       <c r="E238" s="69"/>
       <c r="F238" s="69"/>
@@ -31031,13 +31082,13 @@
         <v>1078</v>
       </c>
       <c r="B239" s="69" t="s">
-        <v>2629</v>
+        <v>2632</v>
       </c>
       <c r="C239" s="8" t="s">
-        <v>2630</v>
+        <v>2633</v>
       </c>
       <c r="D239" s="54" t="s">
-        <v>2631</v>
+        <v>2634</v>
       </c>
       <c r="E239" s="69"/>
       <c r="F239" s="69"/>
@@ -31050,13 +31101,13 @@
         <v>1078</v>
       </c>
       <c r="B240" s="69" t="s">
-        <v>2632</v>
+        <v>2635</v>
       </c>
       <c r="C240" s="8" t="s">
-        <v>2633</v>
+        <v>2636</v>
       </c>
       <c r="D240" s="54" t="s">
-        <v>2634</v>
+        <v>2637</v>
       </c>
       <c r="E240" s="69"/>
       <c r="F240" s="69"/>
@@ -31069,13 +31120,13 @@
         <v>1078</v>
       </c>
       <c r="B241" s="69" t="s">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="C241" s="8" t="s">
-        <v>2636</v>
+        <v>2639</v>
       </c>
       <c r="D241" s="54" t="s">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="E241" s="69"/>
       <c r="F241" s="69"/>
@@ -31088,13 +31139,13 @@
         <v>1078</v>
       </c>
       <c r="B242" s="69" t="s">
-        <v>2638</v>
+        <v>2641</v>
       </c>
       <c r="C242" s="8" t="s">
-        <v>2639</v>
+        <v>2642</v>
       </c>
       <c r="D242" s="54" t="s">
-        <v>2640</v>
+        <v>2643</v>
       </c>
     </row>
     <row r="243" s="53" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31102,13 +31153,13 @@
         <v>1078</v>
       </c>
       <c r="B243" s="69" t="s">
-        <v>2641</v>
+        <v>2644</v>
       </c>
       <c r="C243" s="8" t="s">
-        <v>2642</v>
+        <v>2645</v>
       </c>
       <c r="D243" s="54" t="s">
-        <v>2643</v>
+        <v>2646</v>
       </c>
       <c r="E243" s="69"/>
       <c r="F243" s="69"/>
@@ -31126,7 +31177,7 @@
       <c r="E244" s="69"/>
       <c r="F244" s="69"/>
       <c r="G244" s="56" t="s">
-        <v>2165</v>
+        <v>2168</v>
       </c>
       <c r="H244" s="69"/>
       <c r="I244" s="69"/>
@@ -31136,13 +31187,13 @@
         <v>936</v>
       </c>
       <c r="B245" s="53" t="s">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="C245" s="53" t="s">
-        <v>2645</v>
+        <v>2648</v>
       </c>
       <c r="D245" s="53" t="s">
-        <v>2646</v>
+        <v>2649</v>
       </c>
     </row>
     <row r="246" s="53" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31150,13 +31201,13 @@
         <v>936</v>
       </c>
       <c r="B246" s="53" t="s">
-        <v>2558</v>
+        <v>2561</v>
       </c>
       <c r="C246" s="53" t="s">
-        <v>2647</v>
+        <v>2650</v>
       </c>
       <c r="D246" s="53" t="s">
-        <v>2648</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="247" s="53" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31164,13 +31215,13 @@
         <v>936</v>
       </c>
       <c r="B247" s="53" t="s">
-        <v>2649</v>
+        <v>2652</v>
       </c>
       <c r="C247" s="53" t="s">
-        <v>2650</v>
+        <v>2653</v>
       </c>
       <c r="D247" s="53" t="s">
-        <v>2651</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="248" s="53" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31178,13 +31229,13 @@
         <v>936</v>
       </c>
       <c r="B248" s="53" t="s">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="C248" s="53" t="s">
-        <v>2653</v>
+        <v>2656</v>
       </c>
       <c r="D248" s="53" t="s">
-        <v>2654</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="249" s="53" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31192,13 +31243,13 @@
         <v>936</v>
       </c>
       <c r="B249" s="53" t="s">
-        <v>2655</v>
+        <v>2658</v>
       </c>
       <c r="C249" s="53" t="s">
-        <v>2656</v>
+        <v>2659</v>
       </c>
       <c r="D249" s="53" t="s">
-        <v>2657</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="250" s="53" customFormat="true" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31209,10 +31260,10 @@
         <v>-2</v>
       </c>
       <c r="C250" s="60" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="D250" s="60" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="E250" s="69"/>
       <c r="F250" s="69"/>
@@ -31228,10 +31279,10 @@
         <v>-1</v>
       </c>
       <c r="C251" s="60" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="D251" s="60" t="s">
-        <v>2661</v>
+        <v>2664</v>
       </c>
       <c r="E251" s="69"/>
       <c r="F251" s="69"/>
@@ -31247,10 +31298,10 @@
         <v>0</v>
       </c>
       <c r="C252" s="60" t="s">
-        <v>2662</v>
+        <v>2665</v>
       </c>
       <c r="D252" s="60" t="s">
-        <v>2663</v>
+        <v>2666</v>
       </c>
       <c r="E252" s="69"/>
       <c r="F252" s="69"/>
@@ -31266,10 +31317,10 @@
         <v>1</v>
       </c>
       <c r="C253" s="60" t="s">
-        <v>2664</v>
+        <v>2667</v>
       </c>
       <c r="D253" s="60" t="s">
-        <v>2665</v>
+        <v>2668</v>
       </c>
       <c r="E253" s="69"/>
       <c r="F253" s="69"/>
@@ -31285,10 +31336,10 @@
         <v>2</v>
       </c>
       <c r="C254" s="60" t="s">
-        <v>2666</v>
+        <v>2669</v>
       </c>
       <c r="D254" s="60" t="s">
-        <v>2667</v>
+        <v>2670</v>
       </c>
       <c r="E254" s="69"/>
       <c r="F254" s="69"/>
@@ -31304,10 +31355,10 @@
         <v>0</v>
       </c>
       <c r="C255" s="51" t="s">
-        <v>2668</v>
+        <v>2671</v>
       </c>
       <c r="D255" s="60" t="s">
-        <v>2669</v>
+        <v>2672</v>
       </c>
       <c r="E255" s="69"/>
       <c r="F255" s="69"/>
@@ -31323,10 +31374,10 @@
         <v>1</v>
       </c>
       <c r="C256" s="51" t="s">
-        <v>2670</v>
+        <v>2673</v>
       </c>
       <c r="D256" s="54" t="s">
-        <v>2671</v>
+        <v>2674</v>
       </c>
       <c r="E256" s="69"/>
       <c r="F256" s="69"/>
@@ -31342,10 +31393,10 @@
         <v>2</v>
       </c>
       <c r="C257" s="51" t="s">
-        <v>2672</v>
+        <v>2675</v>
       </c>
       <c r="D257" s="54" t="s">
-        <v>2673</v>
+        <v>2676</v>
       </c>
       <c r="E257" s="69"/>
       <c r="F257" s="69"/>
@@ -31361,10 +31412,10 @@
         <v>3</v>
       </c>
       <c r="C258" s="51" t="s">
-        <v>2674</v>
+        <v>2677</v>
       </c>
       <c r="D258" s="54" t="s">
-        <v>2675</v>
+        <v>2678</v>
       </c>
       <c r="E258" s="69"/>
       <c r="F258" s="69"/>
@@ -31380,10 +31431,10 @@
         <v>4</v>
       </c>
       <c r="C259" s="51" t="s">
-        <v>2676</v>
+        <v>2679</v>
       </c>
       <c r="D259" s="54" t="s">
-        <v>2677</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="15.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31394,10 +31445,10 @@
         <v>-1</v>
       </c>
       <c r="C260" s="51" t="s">
-        <v>2678</v>
+        <v>2681</v>
       </c>
       <c r="D260" s="54" t="s">
-        <v>2679</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31405,13 +31456,13 @@
         <v>39</v>
       </c>
       <c r="B261" s="69" t="s">
-        <v>2680</v>
+        <v>2683</v>
       </c>
       <c r="C261" s="69" t="s">
-        <v>2681</v>
+        <v>2684</v>
       </c>
       <c r="D261" s="69" t="s">
-        <v>2682</v>
+        <v>2685</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auth: mise à jour des textes pour l'authentification passwordless
fixes #206

Le texte auth est ajouté au fichier excel.

Les textes pour le courriel sont ajoutés manuellement au fichier
`customServer.yml` car la gestion des fichier de locales ne fonctionnent
pas de la même façon côté serveur et réécrire dans le fichier server.yml
n'écrase pas la version d'Evolution.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4895" uniqueCount="2683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4899" uniqueCount="2687">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -7173,6 +7173,18 @@
   </si>
   <si>
     <t xml:space="preserve">You must confirm that the access code is correctly typed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">auth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CheckMagicEmail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un lien de connexion a été envoyé à l’adresse courriel que vous avez fournie. Si vous ne le trouvez pas dans votre boîte de réception, vérifiez vos pourriels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A connection link has been sent to the email address you provided. If you do not see it in your inbox, check your spam folder.</t>
   </si>
   <si>
     <t xml:space="preserve">choicesName</t>
@@ -9036,7 +9048,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -9383,6 +9395,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -23234,7 +23250,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F265"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="16.66"/>
@@ -27327,6 +27343,22 @@
         <v>2168</v>
       </c>
     </row>
+    <row r="266" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="50" t="s">
+        <v>2169</v>
+      </c>
+      <c r="B266" s="87" t="s">
+        <v>2170</v>
+      </c>
+      <c r="C266" s="87" t="s">
+        <v>2171</v>
+      </c>
+      <c r="D266" s="87" t="s">
+        <v>2172</v>
+      </c>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A1:F260"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -27357,32 +27389,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="87" t="s">
-        <v>2169</v>
-      </c>
-      <c r="B1" s="87" t="s">
+      <c r="A1" s="88" t="s">
+        <v>2173</v>
+      </c>
+      <c r="B1" s="88" t="s">
         <v>1159</v>
       </c>
-      <c r="C1" s="87" t="s">
+      <c r="C1" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="87" t="s">
+      <c r="D1" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="88" t="s">
+      <c r="E1" s="89" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="88" t="s">
+      <c r="F1" s="89" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="87" t="s">
-        <v>2170</v>
-      </c>
-      <c r="H1" s="87" t="s">
+      <c r="G1" s="88" t="s">
+        <v>2174</v>
+      </c>
+      <c r="H1" s="88" t="s">
         <v>12</v>
       </c>
       <c r="I1" s="66" t="s">
-        <v>2171</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27393,10 +27425,10 @@
         <v>1167</v>
       </c>
       <c r="C2" s="53" t="s">
-        <v>2172</v>
+        <v>2176</v>
       </c>
       <c r="D2" s="53" t="s">
-        <v>2173</v>
+        <v>2177</v>
       </c>
       <c r="E2" s="53"/>
       <c r="F2" s="53"/>
@@ -27411,10 +27443,10 @@
         <v>1225</v>
       </c>
       <c r="C3" s="53" t="s">
-        <v>2174</v>
+        <v>2178</v>
       </c>
       <c r="D3" s="53" t="s">
-        <v>2175</v>
+        <v>2179</v>
       </c>
       <c r="E3" s="53"/>
       <c r="F3" s="53"/>
@@ -27429,10 +27461,10 @@
         <v>229</v>
       </c>
       <c r="C4" s="53" t="s">
-        <v>2176</v>
+        <v>2180</v>
       </c>
       <c r="D4" s="53" t="s">
-        <v>2177</v>
+        <v>2181</v>
       </c>
       <c r="E4" s="53"/>
       <c r="F4" s="53"/>
@@ -27441,7 +27473,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
       <c r="B5" s="53" t="s">
         <v>229</v>
@@ -27459,16 +27491,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="C6" s="53" t="s">
-        <v>2180</v>
+        <v>2184</v>
       </c>
       <c r="D6" s="53" t="s">
-        <v>2181</v>
+        <v>2185</v>
       </c>
       <c r="E6" s="53"/>
       <c r="F6" s="53"/>
@@ -27483,10 +27515,10 @@
         <v>1171</v>
       </c>
       <c r="C7" s="53" t="s">
-        <v>2182</v>
+        <v>2186</v>
       </c>
       <c r="D7" s="53" t="s">
-        <v>2183</v>
+        <v>2187</v>
       </c>
       <c r="E7" s="53"/>
       <c r="F7" s="53"/>
@@ -27545,7 +27577,7 @@
       <c r="E11" s="53"/>
       <c r="F11" s="53"/>
       <c r="G11" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="H11" s="53"/>
     </row>
@@ -27599,10 +27631,10 @@
         <v>1167</v>
       </c>
       <c r="C15" s="51" t="s">
-        <v>2184</v>
+        <v>2188</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>2185</v>
+        <v>2189</v>
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="51"/>
@@ -27618,10 +27650,10 @@
         <v>1225</v>
       </c>
       <c r="C16" s="51" t="s">
-        <v>2186</v>
+        <v>2190</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>2187</v>
+        <v>2191</v>
       </c>
       <c r="E16" s="51"/>
       <c r="F16" s="51"/>
@@ -27630,17 +27662,17 @@
       <c r="I16" s="53"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="89" t="s">
-        <v>2188</v>
+      <c r="A17" s="90" t="s">
+        <v>2192</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>2189</v>
+        <v>2193</v>
       </c>
       <c r="C17" s="53" t="s">
-        <v>2190</v>
+        <v>2194</v>
       </c>
       <c r="D17" s="53" t="s">
-        <v>2191</v>
+        <v>2195</v>
       </c>
       <c r="E17" s="53"/>
       <c r="F17" s="53"/>
@@ -27648,17 +27680,17 @@
       <c r="H17" s="53"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="89" t="s">
-        <v>2188</v>
+      <c r="A18" s="90" t="s">
+        <v>2192</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>2192</v>
+        <v>2196</v>
       </c>
       <c r="C18" s="53" t="s">
-        <v>2193</v>
+        <v>2197</v>
       </c>
       <c r="D18" s="53" t="s">
-        <v>2194</v>
+        <v>2198</v>
       </c>
       <c r="E18" s="53"/>
       <c r="F18" s="53"/>
@@ -27666,8 +27698,8 @@
       <c r="H18" s="53"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="89" t="s">
-        <v>2188</v>
+      <c r="A19" s="90" t="s">
+        <v>2192</v>
       </c>
       <c r="B19" s="53"/>
       <c r="C19" s="53"/>
@@ -27680,17 +27712,17 @@
       <c r="H19" s="53"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="89" t="s">
+      <c r="A20" s="90" t="s">
         <v>187</v>
       </c>
       <c r="B20" s="53" t="s">
-        <v>2189</v>
+        <v>2193</v>
       </c>
       <c r="C20" s="53" t="s">
-        <v>2190</v>
+        <v>2194</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>2195</v>
+        <v>2199</v>
       </c>
       <c r="E20" s="53"/>
       <c r="F20" s="53"/>
@@ -27698,17 +27730,17 @@
       <c r="H20" s="53"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="89" t="s">
+      <c r="A21" s="90" t="s">
         <v>187</v>
       </c>
       <c r="B21" s="53" t="s">
-        <v>2192</v>
+        <v>2196</v>
       </c>
       <c r="C21" s="53" t="s">
-        <v>2193</v>
+        <v>2197</v>
       </c>
       <c r="D21" s="53" t="s">
-        <v>2196</v>
+        <v>2200</v>
       </c>
       <c r="E21" s="53"/>
       <c r="F21" s="53"/>
@@ -27716,17 +27748,17 @@
       <c r="H21" s="53"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="89" t="s">
+      <c r="A22" s="90" t="s">
         <v>187</v>
       </c>
       <c r="B22" s="53" t="s">
         <v>189</v>
       </c>
       <c r="C22" s="53" t="s">
-        <v>2197</v>
+        <v>2201</v>
       </c>
       <c r="D22" s="53" t="s">
-        <v>2198</v>
+        <v>2202</v>
       </c>
       <c r="E22" s="53"/>
       <c r="F22" s="53"/>
@@ -27734,7 +27766,7 @@
       <c r="H22" s="53"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="89" t="s">
+      <c r="A23" s="90" t="s">
         <v>187</v>
       </c>
       <c r="B23" s="53"/>
@@ -27752,13 +27784,13 @@
         <v>306</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>2199</v>
+        <v>2203</v>
       </c>
       <c r="C24" s="53" t="s">
-        <v>2200</v>
+        <v>2204</v>
       </c>
       <c r="D24" s="53" t="s">
-        <v>2201</v>
+        <v>2205</v>
       </c>
       <c r="E24" s="53"/>
       <c r="F24" s="53"/>
@@ -27770,13 +27802,13 @@
         <v>306</v>
       </c>
       <c r="B25" s="53" t="s">
-        <v>2202</v>
+        <v>2206</v>
       </c>
       <c r="C25" s="53" t="s">
-        <v>2203</v>
+        <v>2207</v>
       </c>
       <c r="D25" s="53" t="s">
-        <v>2204</v>
+        <v>2208</v>
       </c>
       <c r="E25" s="53"/>
       <c r="F25" s="53"/>
@@ -27802,13 +27834,13 @@
         <v>299</v>
       </c>
       <c r="B27" s="53" t="s">
-        <v>2199</v>
+        <v>2203</v>
       </c>
       <c r="C27" s="53" t="s">
-        <v>2205</v>
+        <v>2209</v>
       </c>
       <c r="D27" s="53" t="s">
-        <v>2206</v>
+        <v>2210</v>
       </c>
       <c r="E27" s="53"/>
       <c r="F27" s="53"/>
@@ -27820,13 +27852,13 @@
         <v>299</v>
       </c>
       <c r="B28" s="53" t="s">
-        <v>2202</v>
+        <v>2206</v>
       </c>
       <c r="C28" s="53" t="s">
-        <v>2207</v>
+        <v>2211</v>
       </c>
       <c r="D28" s="53" t="s">
-        <v>2208</v>
+        <v>2212</v>
       </c>
       <c r="E28" s="53"/>
       <c r="F28" s="53"/>
@@ -27855,16 +27887,16 @@
         <v>1191</v>
       </c>
       <c r="C30" s="53" t="s">
-        <v>2209</v>
+        <v>2213</v>
       </c>
       <c r="D30" s="53" t="s">
-        <v>2210</v>
+        <v>2214</v>
       </c>
       <c r="E30" s="53"/>
       <c r="F30" s="53"/>
       <c r="G30" s="53"/>
       <c r="H30" s="53"/>
-      <c r="I30" s="90" t="n">
+      <c r="I30" s="91" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27877,16 +27909,16 @@
         <v>1192</v>
       </c>
       <c r="C31" s="53" t="s">
-        <v>2211</v>
+        <v>2215</v>
       </c>
       <c r="D31" s="53" t="s">
-        <v>2212</v>
+        <v>2216</v>
       </c>
       <c r="E31" s="53"/>
       <c r="F31" s="53"/>
       <c r="G31" s="53"/>
       <c r="H31" s="53"/>
-      <c r="I31" s="90" t="n">
+      <c r="I31" s="91" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27899,16 +27931,16 @@
         <v>1193</v>
       </c>
       <c r="C32" s="53" t="s">
-        <v>2213</v>
+        <v>2217</v>
       </c>
       <c r="D32" s="53" t="s">
-        <v>2214</v>
+        <v>2218</v>
       </c>
       <c r="E32" s="53"/>
       <c r="F32" s="53"/>
       <c r="G32" s="53"/>
       <c r="H32" s="53"/>
-      <c r="I32" s="90" t="n">
+      <c r="I32" s="91" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27921,16 +27953,16 @@
         <v>1195</v>
       </c>
       <c r="C33" s="53" t="s">
-        <v>2215</v>
+        <v>2219</v>
       </c>
       <c r="D33" s="53" t="s">
-        <v>2216</v>
+        <v>2220</v>
       </c>
       <c r="E33" s="53"/>
       <c r="F33" s="53"/>
       <c r="G33" s="53"/>
       <c r="H33" s="53"/>
-      <c r="I33" s="90" t="n">
+      <c r="I33" s="91" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27943,16 +27975,16 @@
         <v>1196</v>
       </c>
       <c r="C34" s="53" t="s">
-        <v>2217</v>
+        <v>2221</v>
       </c>
       <c r="D34" s="53" t="s">
-        <v>2218</v>
+        <v>2222</v>
       </c>
       <c r="E34" s="53"/>
       <c r="F34" s="53"/>
       <c r="G34" s="53"/>
       <c r="H34" s="53"/>
-      <c r="I34" s="90" t="n">
+      <c r="I34" s="91" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27962,13 +27994,13 @@
         <v>340</v>
       </c>
       <c r="B35" s="53" t="s">
-        <v>2219</v>
+        <v>2223</v>
       </c>
       <c r="C35" s="53" t="s">
-        <v>2220</v>
+        <v>2224</v>
       </c>
       <c r="D35" s="53" t="s">
-        <v>2221</v>
+        <v>2225</v>
       </c>
       <c r="E35" s="53"/>
       <c r="F35" s="53"/>
@@ -27983,13 +28015,13 @@
         <v>340</v>
       </c>
       <c r="B36" s="53" t="s">
-        <v>2222</v>
+        <v>2226</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>2223</v>
+        <v>2227</v>
       </c>
       <c r="D36" s="53" t="s">
-        <v>2224</v>
+        <v>2228</v>
       </c>
       <c r="E36" s="53"/>
       <c r="F36" s="53"/>
@@ -28005,10 +28037,10 @@
         <v>1262</v>
       </c>
       <c r="C37" s="53" t="s">
-        <v>2225</v>
+        <v>2229</v>
       </c>
       <c r="D37" s="53" t="s">
-        <v>2226</v>
+        <v>2230</v>
       </c>
       <c r="E37" s="53"/>
       <c r="F37" s="53"/>
@@ -28024,10 +28056,10 @@
         <v>1263</v>
       </c>
       <c r="C38" s="53" t="s">
-        <v>2227</v>
+        <v>2231</v>
       </c>
       <c r="D38" s="53" t="s">
-        <v>2228</v>
+        <v>2232</v>
       </c>
       <c r="E38" s="53"/>
       <c r="F38" s="53"/>
@@ -28040,13 +28072,13 @@
         <v>340</v>
       </c>
       <c r="B39" s="53" t="s">
-        <v>2229</v>
+        <v>2233</v>
       </c>
       <c r="C39" s="53" t="s">
-        <v>2230</v>
+        <v>2234</v>
       </c>
       <c r="D39" s="53" t="s">
-        <v>2231</v>
+        <v>2235</v>
       </c>
       <c r="E39" s="53"/>
       <c r="F39" s="53"/>
@@ -28059,13 +28091,13 @@
         <v>340</v>
       </c>
       <c r="B40" s="53" t="s">
-        <v>2232</v>
+        <v>2236</v>
       </c>
       <c r="C40" s="53" t="s">
-        <v>2233</v>
+        <v>2237</v>
       </c>
       <c r="D40" s="53" t="s">
-        <v>2234</v>
+        <v>2238</v>
       </c>
       <c r="E40" s="53"/>
       <c r="F40" s="53"/>
@@ -28083,7 +28115,7 @@
       <c r="E41" s="53"/>
       <c r="F41" s="53"/>
       <c r="G41" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
       <c r="H41" s="53"/>
       <c r="I41" s="66"/>
@@ -28108,13 +28140,13 @@
         <v>315</v>
       </c>
       <c r="B43" s="53" t="s">
-        <v>2235</v>
+        <v>2239</v>
       </c>
       <c r="C43" s="48" t="s">
-        <v>2236</v>
+        <v>2240</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>2237</v>
+        <v>2241</v>
       </c>
       <c r="E43" s="53"/>
       <c r="F43" s="53"/>
@@ -28127,13 +28159,13 @@
         <v>315</v>
       </c>
       <c r="B44" s="53" t="s">
-        <v>2238</v>
+        <v>2242</v>
       </c>
       <c r="C44" s="48" t="s">
-        <v>2239</v>
+        <v>2243</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>2240</v>
+        <v>2244</v>
       </c>
       <c r="E44" s="53"/>
       <c r="F44" s="53"/>
@@ -28146,13 +28178,13 @@
         <v>315</v>
       </c>
       <c r="B45" s="53" t="s">
-        <v>2241</v>
+        <v>2245</v>
       </c>
       <c r="C45" s="48" t="s">
-        <v>2242</v>
+        <v>2246</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>2243</v>
+        <v>2247</v>
       </c>
       <c r="E45" s="53"/>
       <c r="F45" s="53"/>
@@ -28165,13 +28197,13 @@
         <v>315</v>
       </c>
       <c r="B46" s="53" t="s">
-        <v>2244</v>
+        <v>2248</v>
       </c>
       <c r="C46" s="48" t="s">
-        <v>2245</v>
+        <v>2249</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>2246</v>
+        <v>2250</v>
       </c>
       <c r="E46" s="53"/>
       <c r="F46" s="53"/>
@@ -28189,7 +28221,7 @@
       <c r="E47" s="53"/>
       <c r="F47" s="53"/>
       <c r="G47" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="H47" s="53"/>
       <c r="I47" s="53"/>
@@ -28202,10 +28234,10 @@
         <v>1256</v>
       </c>
       <c r="C48" s="51" t="s">
-        <v>2247</v>
+        <v>2251</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>2248</v>
+        <v>2252</v>
       </c>
       <c r="E48" s="53"/>
       <c r="F48" s="53"/>
@@ -28220,13 +28252,13 @@
         <v>220</v>
       </c>
       <c r="B49" s="53" t="s">
-        <v>2249</v>
+        <v>2253</v>
       </c>
       <c r="C49" s="51" t="s">
-        <v>2250</v>
+        <v>2254</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>2251</v>
+        <v>2255</v>
       </c>
       <c r="E49" s="53"/>
       <c r="F49" s="53"/>
@@ -28241,13 +28273,13 @@
         <v>220</v>
       </c>
       <c r="B50" s="53" t="s">
-        <v>2252</v>
+        <v>2256</v>
       </c>
       <c r="C50" s="51" t="s">
-        <v>2253</v>
+        <v>2257</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>2254</v>
+        <v>2258</v>
       </c>
       <c r="E50" s="53"/>
       <c r="F50" s="53"/>
@@ -28263,10 +28295,10 @@
         <v>229</v>
       </c>
       <c r="C51" s="51" t="s">
-        <v>2255</v>
+        <v>2259</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>2256</v>
+        <v>2260</v>
       </c>
       <c r="E51" s="53"/>
       <c r="F51" s="53"/>
@@ -28284,7 +28316,7 @@
       <c r="E52" s="53"/>
       <c r="F52" s="53"/>
       <c r="G52" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="H52" s="53"/>
       <c r="I52" s="53"/>
@@ -28294,13 +28326,13 @@
         <v>226</v>
       </c>
       <c r="B53" s="53" t="s">
-        <v>2257</v>
+        <v>2261</v>
       </c>
       <c r="C53" s="51" t="s">
-        <v>2258</v>
+        <v>2262</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>2259</v>
+        <v>2263</v>
       </c>
       <c r="E53" s="53"/>
       <c r="F53" s="53"/>
@@ -28313,13 +28345,13 @@
         <v>226</v>
       </c>
       <c r="B54" s="53" t="s">
-        <v>2260</v>
+        <v>2264</v>
       </c>
       <c r="C54" s="51" t="s">
-        <v>2261</v>
+        <v>2265</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>2262</v>
+        <v>2266</v>
       </c>
       <c r="E54" s="53"/>
       <c r="F54" s="53"/>
@@ -28332,13 +28364,13 @@
         <v>226</v>
       </c>
       <c r="B55" s="53" t="s">
-        <v>2263</v>
+        <v>2267</v>
       </c>
       <c r="C55" s="51" t="s">
-        <v>2264</v>
+        <v>2268</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>2265</v>
+        <v>2269</v>
       </c>
       <c r="E55" s="53"/>
       <c r="F55" s="53"/>
@@ -28351,13 +28383,13 @@
         <v>226</v>
       </c>
       <c r="B56" s="53" t="s">
-        <v>2266</v>
+        <v>2270</v>
       </c>
       <c r="C56" s="51" t="s">
-        <v>2267</v>
+        <v>2271</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>2268</v>
+        <v>2272</v>
       </c>
       <c r="E56" s="53"/>
       <c r="F56" s="53"/>
@@ -28370,13 +28402,13 @@
         <v>226</v>
       </c>
       <c r="B57" s="53" t="s">
-        <v>2269</v>
+        <v>2273</v>
       </c>
       <c r="C57" s="51" t="s">
-        <v>2270</v>
+        <v>2274</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>2270</v>
+        <v>2274</v>
       </c>
       <c r="E57" s="53"/>
       <c r="F57" s="53"/>
@@ -28389,13 +28421,13 @@
         <v>226</v>
       </c>
       <c r="B58" s="53" t="s">
-        <v>2271</v>
+        <v>2275</v>
       </c>
       <c r="C58" s="51" t="s">
-        <v>2272</v>
+        <v>2276</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>2273</v>
+        <v>2277</v>
       </c>
       <c r="E58" s="53"/>
       <c r="F58" s="53"/>
@@ -28408,13 +28440,13 @@
         <v>226</v>
       </c>
       <c r="B59" s="53" t="s">
-        <v>2274</v>
+        <v>2278</v>
       </c>
       <c r="C59" s="51" t="s">
-        <v>2275</v>
+        <v>2279</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>2276</v>
+        <v>2280</v>
       </c>
       <c r="E59" s="53"/>
       <c r="F59" s="53"/>
@@ -28427,13 +28459,13 @@
         <v>226</v>
       </c>
       <c r="B60" s="53" t="s">
-        <v>2277</v>
+        <v>2281</v>
       </c>
       <c r="C60" s="51" t="s">
-        <v>2278</v>
+        <v>2282</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>2279</v>
+        <v>2283</v>
       </c>
       <c r="E60" s="53"/>
       <c r="F60" s="53"/>
@@ -28461,13 +28493,13 @@
         <v>226</v>
       </c>
       <c r="B62" s="53" t="s">
-        <v>2280</v>
+        <v>2284</v>
       </c>
       <c r="C62" s="51" t="s">
-        <v>2281</v>
+        <v>2285</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>2282</v>
+        <v>2286</v>
       </c>
       <c r="E62" s="53"/>
       <c r="F62" s="53"/>
@@ -28485,7 +28517,7 @@
       <c r="E63" s="53"/>
       <c r="F63" s="53"/>
       <c r="G63" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="H63" s="53"/>
       <c r="I63" s="53"/>
@@ -28498,10 +28530,10 @@
         <v>1167</v>
       </c>
       <c r="C64" s="51" t="s">
-        <v>2283</v>
+        <v>2287</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>2284</v>
+        <v>2288</v>
       </c>
       <c r="E64" s="53"/>
       <c r="F64" s="53"/>
@@ -28510,164 +28542,164 @@
       <c r="I64" s="53"/>
     </row>
     <row r="65" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="89" t="s">
+      <c r="A65" s="90" t="s">
         <v>322</v>
       </c>
       <c r="B65" s="53" t="s">
         <v>1199</v>
       </c>
       <c r="C65" s="53" t="s">
-        <v>2285</v>
+        <v>2289</v>
       </c>
       <c r="D65" s="53" t="s">
-        <v>2286</v>
+        <v>2290</v>
       </c>
       <c r="E65" s="53"/>
       <c r="F65" s="53" t="s">
-        <v>2287</v>
+        <v>2291</v>
       </c>
       <c r="G65" s="53"/>
       <c r="H65" s="53"/>
       <c r="I65" s="66"/>
     </row>
     <row r="66" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="89" t="s">
+      <c r="A66" s="90" t="s">
         <v>322</v>
       </c>
       <c r="B66" s="53" t="s">
         <v>1200</v>
       </c>
       <c r="C66" s="53" t="s">
-        <v>2288</v>
+        <v>2292</v>
       </c>
       <c r="D66" s="53" t="s">
-        <v>2289</v>
+        <v>2293</v>
       </c>
       <c r="E66" s="53"/>
       <c r="F66" s="53" t="s">
-        <v>2290</v>
+        <v>2294</v>
       </c>
       <c r="G66" s="53"/>
       <c r="H66" s="53"/>
       <c r="I66" s="66"/>
     </row>
     <row r="67" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="89" t="s">
+      <c r="A67" s="90" t="s">
         <v>322</v>
       </c>
       <c r="B67" s="53" t="s">
-        <v>2291</v>
+        <v>2295</v>
       </c>
       <c r="C67" s="53" t="s">
-        <v>2292</v>
+        <v>2296</v>
       </c>
       <c r="D67" s="53" t="s">
-        <v>2293</v>
+        <v>2297</v>
       </c>
       <c r="E67" s="53"/>
       <c r="F67" s="53" t="s">
-        <v>2294</v>
+        <v>2298</v>
       </c>
       <c r="G67" s="53"/>
       <c r="H67" s="53"/>
       <c r="I67" s="66"/>
     </row>
     <row r="68" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="89" t="s">
+      <c r="A68" s="90" t="s">
         <v>322</v>
       </c>
       <c r="B68" s="53" t="s">
         <v>1201</v>
       </c>
       <c r="C68" s="53" t="s">
-        <v>2295</v>
+        <v>2299</v>
       </c>
       <c r="D68" s="53" t="s">
-        <v>2296</v>
+        <v>2300</v>
       </c>
       <c r="E68" s="53"/>
       <c r="F68" s="53" t="s">
-        <v>2297</v>
+        <v>2301</v>
       </c>
       <c r="G68" s="53"/>
       <c r="H68" s="53"/>
       <c r="I68" s="66"/>
     </row>
     <row r="69" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="89" t="s">
+      <c r="A69" s="90" t="s">
         <v>322</v>
       </c>
       <c r="B69" s="53" t="s">
         <v>1215</v>
       </c>
       <c r="C69" s="53" t="s">
-        <v>2298</v>
+        <v>2302</v>
       </c>
       <c r="D69" s="53" t="s">
-        <v>2299</v>
+        <v>2303</v>
       </c>
       <c r="E69" s="53"/>
       <c r="F69" s="53" t="s">
-        <v>2300</v>
+        <v>2304</v>
       </c>
       <c r="G69" s="53"/>
       <c r="H69" s="53"/>
       <c r="I69" s="66"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="89" t="s">
+      <c r="A70" s="90" t="s">
         <v>905</v>
       </c>
       <c r="B70" s="66" t="s">
-        <v>2301</v>
+        <v>2305</v>
       </c>
       <c r="C70" s="66" t="s">
-        <v>2302</v>
+        <v>2306</v>
       </c>
       <c r="D70" s="66" t="s">
-        <v>2303</v>
+        <v>2307</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="89" t="s">
+      <c r="A71" s="90" t="s">
         <v>905</v>
       </c>
       <c r="B71" s="66" t="s">
-        <v>2304</v>
+        <v>2308</v>
       </c>
       <c r="C71" s="66" t="s">
-        <v>2305</v>
+        <v>2309</v>
       </c>
       <c r="D71" s="66" t="s">
-        <v>2306</v>
+        <v>2310</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="89" t="s">
+      <c r="A72" s="90" t="s">
         <v>905</v>
       </c>
       <c r="B72" s="66" t="s">
-        <v>2307</v>
+        <v>2311</v>
       </c>
       <c r="C72" s="66" t="s">
-        <v>2308</v>
+        <v>2312</v>
       </c>
       <c r="D72" s="66" t="s">
-        <v>2309</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="73" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="89" t="s">
+      <c r="A73" s="90" t="s">
         <v>905</v>
       </c>
       <c r="B73" s="66" t="s">
-        <v>2310</v>
+        <v>2314</v>
       </c>
       <c r="C73" s="66" t="s">
-        <v>2311</v>
+        <v>2315</v>
       </c>
       <c r="D73" s="66" t="s">
-        <v>2312</v>
+        <v>2316</v>
       </c>
       <c r="E73" s="66"/>
       <c r="F73" s="66"/>
@@ -28680,13 +28712,13 @@
         <v>1079</v>
       </c>
       <c r="B74" s="53" t="s">
-        <v>2313</v>
+        <v>2317</v>
       </c>
       <c r="C74" s="51" t="s">
-        <v>2314</v>
+        <v>2318</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>2315</v>
+        <v>2319</v>
       </c>
       <c r="E74" s="51"/>
       <c r="F74" s="51"/>
@@ -28699,13 +28731,13 @@
         <v>1079</v>
       </c>
       <c r="B75" s="53" t="s">
-        <v>2316</v>
+        <v>2320</v>
       </c>
       <c r="C75" s="51" t="s">
-        <v>2317</v>
+        <v>2321</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>2318</v>
+        <v>2322</v>
       </c>
       <c r="E75" s="51"/>
       <c r="F75" s="51"/>
@@ -28718,13 +28750,13 @@
         <v>1079</v>
       </c>
       <c r="B76" s="53" t="s">
-        <v>2319</v>
+        <v>2323</v>
       </c>
       <c r="C76" s="51" t="s">
-        <v>2320</v>
+        <v>2324</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>2321</v>
+        <v>2325</v>
       </c>
       <c r="E76" s="51"/>
       <c r="F76" s="51"/>
@@ -28737,13 +28769,13 @@
         <v>1079</v>
       </c>
       <c r="B77" s="53" t="s">
-        <v>2322</v>
+        <v>2326</v>
       </c>
       <c r="C77" s="51" t="s">
-        <v>2323</v>
+        <v>2327</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>2324</v>
+        <v>2328</v>
       </c>
       <c r="E77" s="51"/>
       <c r="F77" s="51"/>
@@ -28756,13 +28788,13 @@
         <v>1079</v>
       </c>
       <c r="B78" s="53" t="s">
-        <v>2325</v>
+        <v>2329</v>
       </c>
       <c r="C78" s="51" t="s">
-        <v>2326</v>
+        <v>2330</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>2327</v>
+        <v>2331</v>
       </c>
       <c r="E78" s="51"/>
       <c r="F78" s="51"/>
@@ -28775,13 +28807,13 @@
         <v>1079</v>
       </c>
       <c r="B79" s="53" t="s">
-        <v>2328</v>
+        <v>2332</v>
       </c>
       <c r="C79" s="51" t="s">
-        <v>2329</v>
+        <v>2333</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>2330</v>
+        <v>2334</v>
       </c>
       <c r="E79" s="51"/>
       <c r="F79" s="51"/>
@@ -28794,13 +28826,13 @@
         <v>1079</v>
       </c>
       <c r="B80" s="53" t="s">
-        <v>2331</v>
+        <v>2335</v>
       </c>
       <c r="C80" s="51" t="s">
-        <v>2332</v>
+        <v>2336</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>2333</v>
+        <v>2337</v>
       </c>
       <c r="E80" s="51"/>
       <c r="F80" s="51"/>
@@ -28813,13 +28845,13 @@
         <v>1079</v>
       </c>
       <c r="B81" s="53" t="s">
-        <v>2334</v>
+        <v>2338</v>
       </c>
       <c r="C81" s="51" t="s">
-        <v>2335</v>
+        <v>2339</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>2336</v>
+        <v>2340</v>
       </c>
       <c r="E81" s="51"/>
       <c r="F81" s="51"/>
@@ -28832,13 +28864,13 @@
         <v>1079</v>
       </c>
       <c r="B82" s="53" t="s">
-        <v>2337</v>
+        <v>2341</v>
       </c>
       <c r="C82" s="51" t="s">
-        <v>2338</v>
+        <v>2342</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>2339</v>
+        <v>2343</v>
       </c>
       <c r="E82" s="51"/>
       <c r="F82" s="51"/>
@@ -28851,13 +28883,13 @@
         <v>1079</v>
       </c>
       <c r="B83" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="C83" s="51" t="s">
-        <v>2180</v>
+        <v>2184</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>2181</v>
+        <v>2185</v>
       </c>
       <c r="E83" s="51"/>
       <c r="F83" s="51"/>
@@ -28870,13 +28902,13 @@
         <v>1079</v>
       </c>
       <c r="B84" s="53" t="s">
-        <v>2340</v>
+        <v>2344</v>
       </c>
       <c r="C84" s="51" t="s">
-        <v>2182</v>
+        <v>2186</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>2341</v>
+        <v>2345</v>
       </c>
       <c r="E84" s="51"/>
       <c r="F84" s="51"/>
@@ -28885,35 +28917,35 @@
       <c r="I84" s="53"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="91" t="s">
+      <c r="A85" s="92" t="s">
         <v>99</v>
       </c>
       <c r="B85" s="66" t="s">
-        <v>2342</v>
+        <v>2346</v>
       </c>
       <c r="C85" s="66" t="s">
-        <v>2343</v>
+        <v>2347</v>
       </c>
       <c r="D85" s="66" t="s">
-        <v>2344</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="91" t="s">
+      <c r="A86" s="92" t="s">
         <v>99</v>
       </c>
       <c r="B86" s="66" t="s">
-        <v>2345</v>
+        <v>2349</v>
       </c>
       <c r="C86" s="66" t="s">
-        <v>2346</v>
+        <v>2350</v>
       </c>
       <c r="D86" s="66" t="s">
-        <v>2347</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="91" t="s">
+      <c r="A87" s="92" t="s">
         <v>99</v>
       </c>
       <c r="B87" s="66" t="s">
@@ -28927,31 +28959,31 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="91" t="s">
+      <c r="A88" s="92" t="s">
         <v>99</v>
       </c>
       <c r="B88" s="66" t="s">
         <v>1171</v>
       </c>
       <c r="C88" s="66" t="s">
-        <v>2182</v>
+        <v>2186</v>
       </c>
       <c r="D88" s="66" t="s">
-        <v>2341</v>
+        <v>2345</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="92" t="s">
+      <c r="A89" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B89" s="53" t="s">
-        <v>2348</v>
+        <v>2352</v>
       </c>
       <c r="C89" s="51" t="s">
-        <v>2349</v>
+        <v>2353</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>2350</v>
+        <v>2354</v>
       </c>
       <c r="E89" s="51"/>
       <c r="F89" s="51"/>
@@ -28962,17 +28994,17 @@
       <c r="I89" s="53"/>
     </row>
     <row r="90" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="92" t="s">
+      <c r="A90" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B90" s="53" t="s">
-        <v>2351</v>
+        <v>2355</v>
       </c>
       <c r="C90" s="51" t="s">
-        <v>2352</v>
+        <v>2356</v>
       </c>
       <c r="D90" s="8" t="s">
-        <v>2353</v>
+        <v>2357</v>
       </c>
       <c r="E90" s="51"/>
       <c r="F90" s="51"/>
@@ -28983,17 +29015,17 @@
       <c r="I90" s="53"/>
     </row>
     <row r="91" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="92" t="s">
+      <c r="A91" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B91" s="53" t="s">
-        <v>2354</v>
+        <v>2358</v>
       </c>
       <c r="C91" s="51" t="s">
-        <v>2355</v>
+        <v>2359</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>2356</v>
+        <v>2360</v>
       </c>
       <c r="E91" s="51"/>
       <c r="F91" s="51"/>
@@ -29002,17 +29034,17 @@
       <c r="I91" s="53"/>
     </row>
     <row r="92" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="92" t="s">
+      <c r="A92" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B92" s="53" t="s">
-        <v>2357</v>
+        <v>2361</v>
       </c>
       <c r="C92" s="51" t="s">
-        <v>2358</v>
+        <v>2362</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>2359</v>
+        <v>2363</v>
       </c>
       <c r="E92" s="51"/>
       <c r="F92" s="51"/>
@@ -29021,17 +29053,17 @@
       <c r="I92" s="53"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="92" t="s">
+      <c r="A93" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B93" s="53" t="s">
-        <v>2360</v>
+        <v>2364</v>
       </c>
       <c r="C93" s="51" t="s">
-        <v>2361</v>
+        <v>2365</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>2362</v>
+        <v>2366</v>
       </c>
       <c r="E93" s="51"/>
       <c r="F93" s="51"/>
@@ -29040,17 +29072,17 @@
       <c r="I93" s="53"/>
     </row>
     <row r="94" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="92" t="s">
+      <c r="A94" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B94" s="53" t="s">
         <v>1232</v>
       </c>
       <c r="C94" s="51" t="s">
-        <v>2363</v>
+        <v>2367</v>
       </c>
       <c r="D94" s="8" t="s">
-        <v>2364</v>
+        <v>2368</v>
       </c>
       <c r="E94" s="51"/>
       <c r="F94" s="51"/>
@@ -29061,17 +29093,17 @@
       <c r="I94" s="53"/>
     </row>
     <row r="95" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="92" t="s">
+      <c r="A95" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B95" s="53" t="s">
         <v>1233</v>
       </c>
       <c r="C95" s="51" t="s">
-        <v>2365</v>
+        <v>2369</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>2366</v>
+        <v>2370</v>
       </c>
       <c r="E95" s="51"/>
       <c r="F95" s="51"/>
@@ -29080,17 +29112,17 @@
       <c r="I95" s="53"/>
     </row>
     <row r="96" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="92" t="s">
+      <c r="A96" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B96" s="53" t="s">
-        <v>2367</v>
+        <v>2371</v>
       </c>
       <c r="C96" s="51" t="s">
-        <v>2368</v>
+        <v>2372</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>2369</v>
+        <v>2373</v>
       </c>
       <c r="E96" s="51"/>
       <c r="F96" s="51"/>
@@ -29101,7 +29133,7 @@
       <c r="I96" s="53"/>
     </row>
     <row r="97" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="92" t="s">
+      <c r="A97" s="93" t="s">
         <v>423</v>
       </c>
       <c r="B97" s="53" t="s">
@@ -29120,11 +29152,11 @@
       <c r="I97" s="53"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="93" t="s">
-        <v>2370</v>
+      <c r="A98" s="94" t="s">
+        <v>2374</v>
       </c>
       <c r="B98" s="66" t="s">
-        <v>2371</v>
+        <v>2375</v>
       </c>
       <c r="C98" s="66" t="s">
         <v>1752</v>
@@ -29140,11 +29172,11 @@
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="93" t="s">
-        <v>2370</v>
+      <c r="A99" s="94" t="s">
+        <v>2374</v>
       </c>
       <c r="B99" s="66" t="s">
-        <v>2372</v>
+        <v>2376</v>
       </c>
       <c r="C99" s="66" t="s">
         <v>1757</v>
@@ -29160,215 +29192,215 @@
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="93" t="s">
-        <v>2370</v>
+      <c r="A100" s="94" t="s">
+        <v>2374</v>
       </c>
       <c r="B100" s="66" t="s">
         <v>1225</v>
       </c>
       <c r="C100" s="66" t="s">
-        <v>2174</v>
+        <v>2178</v>
       </c>
       <c r="D100" s="66" t="s">
-        <v>2175</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="93" t="s">
+      <c r="A101" s="94" t="s">
         <v>771</v>
       </c>
       <c r="B101" s="66" t="s">
-        <v>2373</v>
+        <v>2377</v>
       </c>
       <c r="C101" s="66" t="s">
-        <v>2374</v>
+        <v>2378</v>
       </c>
       <c r="D101" s="66" t="s">
-        <v>2375</v>
+        <v>2379</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="93" t="s">
+      <c r="A102" s="94" t="s">
         <v>771</v>
       </c>
       <c r="B102" s="66" t="s">
-        <v>2376</v>
+        <v>2380</v>
       </c>
       <c r="C102" s="66" t="s">
-        <v>2377</v>
+        <v>2381</v>
       </c>
       <c r="D102" s="66" t="s">
-        <v>2378</v>
-      </c>
-      <c r="I102" s="90" t="n">
+        <v>2382</v>
+      </c>
+      <c r="I102" s="91" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="93" t="s">
+      <c r="A103" s="94" t="s">
         <v>771</v>
       </c>
       <c r="B103" s="66" t="s">
-        <v>2379</v>
+        <v>2383</v>
       </c>
       <c r="C103" s="66" t="s">
-        <v>2380</v>
+        <v>2384</v>
       </c>
       <c r="D103" s="66" t="s">
-        <v>2381</v>
+        <v>2385</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="93" t="s">
+      <c r="A104" s="94" t="s">
         <v>771</v>
       </c>
       <c r="B104" s="66" t="s">
-        <v>2382</v>
+        <v>2386</v>
       </c>
       <c r="C104" s="66" t="s">
+        <v>2387</v>
+      </c>
+      <c r="D104" s="66" t="s">
+        <v>2388</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="94" t="s">
+        <v>771</v>
+      </c>
+      <c r="G105" s="53" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="94" t="s">
+        <v>771</v>
+      </c>
+      <c r="G106" s="53" t="s">
+        <v>2183</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="94" t="s">
+        <v>829</v>
+      </c>
+      <c r="B107" s="66" t="s">
+        <v>2389</v>
+      </c>
+      <c r="C107" s="66" t="s">
+        <v>2390</v>
+      </c>
+      <c r="D107" s="66" t="s">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="94" t="s">
+        <v>829</v>
+      </c>
+      <c r="B108" s="66" t="s">
+        <v>2392</v>
+      </c>
+      <c r="C108" s="66" t="s">
+        <v>2393</v>
+      </c>
+      <c r="D108" s="66" t="s">
+        <v>2394</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="94" t="s">
+        <v>829</v>
+      </c>
+      <c r="B109" s="66" t="s">
         <v>2383</v>
       </c>
-      <c r="D104" s="66" t="s">
-        <v>2384</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="93" t="s">
-        <v>771</v>
-      </c>
-      <c r="G105" s="53" t="s">
-        <v>2178</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="93" t="s">
-        <v>771</v>
-      </c>
-      <c r="G106" s="53" t="s">
-        <v>2179</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="93" t="s">
+      <c r="C109" s="66" t="s">
+        <v>2395</v>
+      </c>
+      <c r="D109" s="66" t="s">
+        <v>2396</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="94" t="s">
         <v>829</v>
       </c>
-      <c r="B107" s="66" t="s">
-        <v>2385</v>
-      </c>
-      <c r="C107" s="66" t="s">
-        <v>2386</v>
-      </c>
-      <c r="D107" s="66" t="s">
-        <v>2387</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="93" t="s">
+      <c r="B110" s="53" t="s">
+        <v>2397</v>
+      </c>
+      <c r="C110" s="51" t="s">
+        <v>2398</v>
+      </c>
+      <c r="D110" s="48" t="s">
+        <v>2399</v>
+      </c>
+      <c r="I110" s="91" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="94" t="s">
         <v>829</v>
       </c>
-      <c r="B108" s="66" t="s">
-        <v>2388</v>
-      </c>
-      <c r="C108" s="66" t="s">
-        <v>2389</v>
-      </c>
-      <c r="D108" s="66" t="s">
-        <v>2390</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="93" t="s">
+      <c r="G111" s="53" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="94" t="s">
         <v>829</v>
       </c>
-      <c r="B109" s="66" t="s">
-        <v>2379</v>
-      </c>
-      <c r="C109" s="66" t="s">
-        <v>2391</v>
-      </c>
-      <c r="D109" s="66" t="s">
-        <v>2392</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="93" t="s">
-        <v>829</v>
-      </c>
-      <c r="B110" s="53" t="s">
-        <v>2393</v>
-      </c>
-      <c r="C110" s="51" t="s">
-        <v>2394</v>
-      </c>
-      <c r="D110" s="48" t="s">
-        <v>2395</v>
-      </c>
-      <c r="I110" s="90" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="93" t="s">
-        <v>829</v>
-      </c>
-      <c r="G111" s="53" t="s">
-        <v>2178</v>
-      </c>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="93" t="s">
-        <v>829</v>
-      </c>
       <c r="G112" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="94" t="s">
+      <c r="A113" s="95" t="s">
         <v>347</v>
       </c>
       <c r="B113" s="66" t="s">
-        <v>2396</v>
+        <v>2400</v>
       </c>
       <c r="C113" s="66" t="s">
-        <v>2397</v>
+        <v>2401</v>
       </c>
       <c r="D113" s="66" t="s">
-        <v>2398</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="94" t="s">
+      <c r="A114" s="95" t="s">
         <v>347</v>
       </c>
       <c r="B114" s="66" t="s">
-        <v>2399</v>
+        <v>2403</v>
       </c>
       <c r="C114" s="66" t="s">
-        <v>2400</v>
+        <v>2404</v>
       </c>
       <c r="D114" s="66" t="s">
-        <v>2401</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="94" t="s">
+      <c r="A115" s="95" t="s">
         <v>347</v>
       </c>
       <c r="B115" s="66" t="s">
-        <v>2402</v>
+        <v>2406</v>
       </c>
       <c r="C115" s="66" t="s">
-        <v>2403</v>
+        <v>2407</v>
       </c>
       <c r="D115" s="66" t="s">
-        <v>2404</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="94" t="s">
+      <c r="A116" s="95" t="s">
         <v>347</v>
       </c>
       <c r="G116" s="53" t="s">
@@ -29376,104 +29408,104 @@
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="89" t="s">
-        <v>2405</v>
+      <c r="A117" s="90" t="s">
+        <v>2409</v>
       </c>
       <c r="B117" s="53" t="s">
         <v>1199</v>
       </c>
       <c r="C117" s="53" t="s">
-        <v>2406</v>
+        <v>2410</v>
       </c>
       <c r="D117" s="53" t="s">
-        <v>2407</v>
+        <v>2411</v>
       </c>
       <c r="E117" s="53" t="s">
-        <v>2408</v>
+        <v>2412</v>
       </c>
       <c r="F117" s="53" t="s">
+        <v>2413</v>
+      </c>
+      <c r="G117" s="90"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="90" t="s">
         <v>2409</v>
-      </c>
-      <c r="G117" s="89"/>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="89" t="s">
-        <v>2405</v>
       </c>
       <c r="B118" s="53" t="s">
         <v>1200</v>
       </c>
       <c r="C118" s="53" t="s">
-        <v>2410</v>
+        <v>2414</v>
       </c>
       <c r="D118" s="53" t="s">
-        <v>2411</v>
+        <v>2415</v>
       </c>
       <c r="E118" s="53" t="s">
-        <v>2412</v>
+        <v>2416</v>
       </c>
       <c r="F118" s="53" t="s">
-        <v>2413</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="89" t="s">
-        <v>2405</v>
+      <c r="A119" s="90" t="s">
+        <v>2409</v>
       </c>
       <c r="B119" s="53" t="s">
         <v>1201</v>
       </c>
       <c r="C119" s="53" t="s">
-        <v>2414</v>
+        <v>2418</v>
       </c>
       <c r="D119" s="53" t="s">
-        <v>2415</v>
+        <v>2419</v>
       </c>
       <c r="E119" s="53" t="s">
-        <v>2416</v>
+        <v>2420</v>
       </c>
       <c r="F119" s="53" t="s">
-        <v>2417</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="89" t="s">
-        <v>2405</v>
+      <c r="A120" s="90" t="s">
+        <v>2409</v>
       </c>
       <c r="B120" s="53" t="s">
         <v>1215</v>
       </c>
       <c r="C120" s="53" t="s">
-        <v>2418</v>
+        <v>2422</v>
       </c>
       <c r="D120" s="53" t="s">
-        <v>2419</v>
+        <v>2423</v>
       </c>
       <c r="E120" s="53" t="s">
-        <v>2420</v>
+        <v>2424</v>
       </c>
       <c r="F120" s="53" t="s">
-        <v>2421</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="89" t="s">
-        <v>2405</v>
+      <c r="A121" s="90" t="s">
+        <v>2409</v>
       </c>
       <c r="B121" s="53" t="s">
-        <v>2291</v>
+        <v>2295</v>
       </c>
       <c r="C121" s="53" t="s">
-        <v>2422</v>
+        <v>2426</v>
       </c>
       <c r="D121" s="53" t="s">
-        <v>2423</v>
+        <v>2427</v>
       </c>
       <c r="E121" s="53" t="s">
-        <v>2424</v>
+        <v>2428</v>
       </c>
       <c r="F121" s="53" t="s">
-        <v>2425</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29481,7 +29513,7 @@
         <v>698</v>
       </c>
       <c r="B122" s="66" t="s">
-        <v>2426</v>
+        <v>2430</v>
       </c>
       <c r="C122" s="8" t="s">
         <v>2021</v>
@@ -29498,12 +29530,12 @@
         <v>1237</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>2427</v>
+        <v>2431</v>
       </c>
       <c r="D123" s="57" t="s">
-        <v>2427</v>
-      </c>
-      <c r="H123" s="95" t="s">
+        <v>2431</v>
+      </c>
+      <c r="H123" s="96" t="s">
         <v>1235</v>
       </c>
     </row>
@@ -29512,16 +29544,16 @@
         <v>698</v>
       </c>
       <c r="B124" s="66" t="s">
-        <v>2428</v>
+        <v>2432</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>2429</v>
+        <v>2433</v>
       </c>
       <c r="D124" s="57" t="s">
-        <v>2430</v>
-      </c>
-      <c r="H124" s="96" t="s">
-        <v>2431</v>
+        <v>2434</v>
+      </c>
+      <c r="H124" s="97" t="s">
+        <v>2435</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29529,7 +29561,7 @@
         <v>698</v>
       </c>
       <c r="B125" s="66" t="s">
-        <v>2432</v>
+        <v>2436</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>2030</v>
@@ -29546,7 +29578,7 @@
         <v>698</v>
       </c>
       <c r="B126" s="66" t="s">
-        <v>2433</v>
+        <v>2437</v>
       </c>
       <c r="C126" s="8" t="s">
         <v>2033</v>
@@ -29570,7 +29602,7 @@
         <v>704</v>
       </c>
       <c r="B128" s="66" t="s">
-        <v>2426</v>
+        <v>2430</v>
       </c>
       <c r="C128" s="8" t="s">
         <v>2021</v>
@@ -29584,7 +29616,7 @@
         <v>704</v>
       </c>
       <c r="B129" s="66" t="s">
-        <v>2434</v>
+        <v>2438</v>
       </c>
       <c r="C129" s="8" t="s">
         <v>2040</v>
@@ -29598,7 +29630,7 @@
         <v>704</v>
       </c>
       <c r="B130" s="66" t="s">
-        <v>2432</v>
+        <v>2436</v>
       </c>
       <c r="C130" s="8" t="s">
         <v>2030</v>
@@ -29615,7 +29647,7 @@
         <v>704</v>
       </c>
       <c r="B131" s="66" t="s">
-        <v>2433</v>
+        <v>2437</v>
       </c>
       <c r="C131" s="8" t="s">
         <v>2033</v>
@@ -29629,13 +29661,13 @@
         <v>704</v>
       </c>
       <c r="B132" s="66" t="s">
-        <v>2435</v>
+        <v>2439</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>2436</v>
+        <v>2440</v>
       </c>
       <c r="D132" s="57" t="s">
-        <v>2437</v>
+        <v>2441</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29643,7 +29675,7 @@
         <v>704</v>
       </c>
       <c r="B133" s="66" t="s">
-        <v>2438</v>
+        <v>2442</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>2036</v>
@@ -29659,7 +29691,7 @@
       <c r="C134" s="57"/>
       <c r="D134" s="57"/>
       <c r="G134" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29667,16 +29699,16 @@
         <v>594</v>
       </c>
       <c r="B135" s="66" t="s">
-        <v>2439</v>
+        <v>2443</v>
       </c>
       <c r="C135" s="57" t="s">
-        <v>2440</v>
+        <v>2444</v>
       </c>
       <c r="D135" s="57" t="s">
-        <v>2441</v>
+        <v>2445</v>
       </c>
       <c r="H135" s="54" t="s">
-        <v>2442</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29687,13 +29719,13 @@
         <v>1225</v>
       </c>
       <c r="C136" s="57" t="s">
-        <v>2443</v>
+        <v>2447</v>
       </c>
       <c r="D136" s="57" t="s">
-        <v>2444</v>
+        <v>2448</v>
       </c>
       <c r="H136" s="8" t="s">
-        <v>2445</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29704,10 +29736,10 @@
         <v>1167</v>
       </c>
       <c r="C137" s="57" t="s">
-        <v>2446</v>
+        <v>2450</v>
       </c>
       <c r="D137" s="57" t="s">
-        <v>2447</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29715,13 +29747,13 @@
         <v>594</v>
       </c>
       <c r="B138" s="66" t="s">
-        <v>2448</v>
+        <v>2452</v>
       </c>
       <c r="C138" s="57" t="s">
-        <v>2449</v>
+        <v>2453</v>
       </c>
       <c r="D138" s="57" t="s">
-        <v>2450</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29731,7 +29763,7 @@
       <c r="C139" s="57"/>
       <c r="D139" s="57"/>
       <c r="G139" s="66" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29739,13 +29771,13 @@
         <v>627</v>
       </c>
       <c r="B140" s="66" t="s">
-        <v>2451</v>
+        <v>2455</v>
       </c>
       <c r="C140" s="57" t="s">
-        <v>2452</v>
+        <v>2456</v>
       </c>
       <c r="D140" s="57" t="s">
-        <v>2452</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29753,13 +29785,13 @@
         <v>627</v>
       </c>
       <c r="B141" s="66" t="s">
-        <v>2453</v>
+        <v>2457</v>
       </c>
       <c r="C141" s="57" t="s">
-        <v>2454</v>
+        <v>2458</v>
       </c>
       <c r="D141" s="57" t="s">
-        <v>2455</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29769,7 +29801,7 @@
       <c r="C142" s="57"/>
       <c r="D142" s="57"/>
       <c r="G142" s="66" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29777,13 +29809,13 @@
         <v>651</v>
       </c>
       <c r="B143" s="66" t="s">
-        <v>2456</v>
+        <v>2460</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>2457</v>
+        <v>2461</v>
       </c>
       <c r="D143" s="57" t="s">
-        <v>2458</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29791,13 +29823,13 @@
         <v>651</v>
       </c>
       <c r="B144" s="66" t="s">
-        <v>2459</v>
+        <v>2463</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>2460</v>
+        <v>2464</v>
       </c>
       <c r="D144" s="57" t="s">
-        <v>2461</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29807,7 +29839,7 @@
       <c r="C145" s="57"/>
       <c r="D145" s="57"/>
       <c r="G145" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29817,7 +29849,7 @@
       <c r="C146" s="57"/>
       <c r="D146" s="57"/>
       <c r="G146" s="66" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29825,13 +29857,13 @@
         <v>658</v>
       </c>
       <c r="B147" s="66" t="s">
-        <v>2462</v>
+        <v>2466</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>2463</v>
+        <v>2467</v>
       </c>
       <c r="D147" s="57" t="s">
-        <v>2464</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29839,13 +29871,13 @@
         <v>658</v>
       </c>
       <c r="B148" s="66" t="s">
-        <v>2465</v>
+        <v>2469</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>2466</v>
+        <v>2470</v>
       </c>
       <c r="D148" s="57" t="s">
-        <v>2466</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29853,13 +29885,13 @@
         <v>658</v>
       </c>
       <c r="B149" s="66" t="s">
-        <v>2467</v>
+        <v>2471</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>2468</v>
+        <v>2472</v>
       </c>
       <c r="D149" s="8" t="s">
-        <v>2468</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29867,13 +29899,13 @@
         <v>658</v>
       </c>
       <c r="B150" s="66" t="s">
-        <v>2469</v>
+        <v>2473</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>2470</v>
+        <v>2474</v>
       </c>
       <c r="D150" s="8" t="s">
-        <v>2470</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29883,7 +29915,7 @@
       <c r="C151" s="57"/>
       <c r="D151" s="57"/>
       <c r="G151" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29893,7 +29925,7 @@
       <c r="C152" s="57"/>
       <c r="D152" s="57"/>
       <c r="G152" s="66" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29901,13 +29933,13 @@
         <v>663</v>
       </c>
       <c r="B153" s="66" t="s">
-        <v>2471</v>
+        <v>2475</v>
       </c>
       <c r="C153" s="8" t="s">
-        <v>2472</v>
+        <v>2476</v>
       </c>
       <c r="D153" s="57" t="s">
-        <v>2473</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29915,13 +29947,13 @@
         <v>663</v>
       </c>
       <c r="B154" s="66" t="s">
-        <v>2474</v>
+        <v>2478</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>2475</v>
+        <v>2479</v>
       </c>
       <c r="D154" s="57" t="s">
-        <v>2476</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29929,13 +29961,13 @@
         <v>663</v>
       </c>
       <c r="B155" s="66" t="s">
-        <v>2456</v>
+        <v>2460</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>2477</v>
+        <v>2481</v>
       </c>
       <c r="D155" s="57" t="s">
-        <v>2478</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29943,13 +29975,13 @@
         <v>663</v>
       </c>
       <c r="B156" s="66" t="s">
-        <v>2479</v>
+        <v>2483</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>2480</v>
+        <v>2484</v>
       </c>
       <c r="D156" s="8" t="s">
-        <v>2480</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29957,13 +29989,13 @@
         <v>663</v>
       </c>
       <c r="B157" s="66" t="s">
-        <v>2481</v>
+        <v>2485</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>2482</v>
+        <v>2486</v>
       </c>
       <c r="D157" s="57" t="s">
-        <v>2483</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29973,7 +30005,7 @@
       <c r="C158" s="57"/>
       <c r="D158" s="57"/>
       <c r="G158" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29983,7 +30015,7 @@
       <c r="C159" s="57"/>
       <c r="D159" s="57"/>
       <c r="G159" s="66" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29991,7 +30023,7 @@
         <v>793</v>
       </c>
       <c r="B160" s="53" t="s">
-        <v>2432</v>
+        <v>2436</v>
       </c>
       <c r="C160" s="66" t="s">
         <v>1970</v>
@@ -30010,7 +30042,7 @@
         <v>793</v>
       </c>
       <c r="B161" s="53" t="s">
-        <v>2433</v>
+        <v>2437</v>
       </c>
       <c r="C161" s="66" t="s">
         <v>1988</v>
@@ -30029,13 +30061,13 @@
         <v>793</v>
       </c>
       <c r="B162" s="53" t="s">
-        <v>2438</v>
+        <v>2442</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>2484</v>
+        <v>2488</v>
       </c>
       <c r="D162" s="57" t="s">
-        <v>2485</v>
+        <v>2489</v>
       </c>
       <c r="E162" s="53"/>
       <c r="F162" s="53"/>
@@ -30048,7 +30080,7 @@
         <v>793</v>
       </c>
       <c r="B163" s="53" t="s">
-        <v>2426</v>
+        <v>2430</v>
       </c>
       <c r="C163" s="8" t="s">
         <v>1923</v>
@@ -30067,7 +30099,7 @@
         <v>793</v>
       </c>
       <c r="B164" s="53" t="s">
-        <v>2486</v>
+        <v>2490</v>
       </c>
       <c r="C164" s="8" t="s">
         <v>1926</v>
@@ -30089,10 +30121,10 @@
         <v>229</v>
       </c>
       <c r="C165" s="51" t="s">
-        <v>2487</v>
+        <v>2491</v>
       </c>
       <c r="D165" s="8" t="s">
-        <v>2488</v>
+        <v>2492</v>
       </c>
       <c r="E165" s="53"/>
       <c r="F165" s="53"/>
@@ -30107,13 +30139,13 @@
         <v>793</v>
       </c>
       <c r="B166" s="53" t="s">
-        <v>2489</v>
+        <v>2493</v>
       </c>
       <c r="C166" s="51" t="s">
-        <v>2490</v>
+        <v>2494</v>
       </c>
       <c r="D166" s="8" t="s">
-        <v>2491</v>
+        <v>2495</v>
       </c>
       <c r="E166" s="53"/>
       <c r="F166" s="53"/>
@@ -30128,13 +30160,13 @@
         <v>141</v>
       </c>
       <c r="B167" s="53" t="s">
-        <v>2492</v>
+        <v>2496</v>
       </c>
       <c r="C167" s="51" t="s">
-        <v>2493</v>
+        <v>2497</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>2494</v>
+        <v>2498</v>
       </c>
       <c r="E167" s="53"/>
       <c r="F167" s="53"/>
@@ -30147,13 +30179,13 @@
         <v>141</v>
       </c>
       <c r="B168" s="53" t="s">
-        <v>2495</v>
+        <v>2499</v>
       </c>
       <c r="C168" s="51" t="s">
-        <v>2496</v>
+        <v>2500</v>
       </c>
       <c r="D168" s="8" t="s">
-        <v>2497</v>
+        <v>2501</v>
       </c>
       <c r="E168" s="53"/>
       <c r="F168" s="53"/>
@@ -30169,10 +30201,10 @@
         <v>1167</v>
       </c>
       <c r="C169" s="51" t="s">
-        <v>2498</v>
+        <v>2502</v>
       </c>
       <c r="D169" s="8" t="s">
-        <v>2499</v>
+        <v>2503</v>
       </c>
       <c r="E169" s="53"/>
       <c r="F169" s="53"/>
@@ -30188,10 +30220,10 @@
         <v>1225</v>
       </c>
       <c r="C170" s="51" t="s">
-        <v>2500</v>
+        <v>2504</v>
       </c>
       <c r="D170" s="8" t="s">
-        <v>2501</v>
+        <v>2505</v>
       </c>
       <c r="E170" s="53"/>
       <c r="F170" s="53"/>
@@ -30209,7 +30241,7 @@
       <c r="E171" s="53"/>
       <c r="F171" s="53"/>
       <c r="G171" s="53" t="s">
-        <v>2179</v>
+        <v>2183</v>
       </c>
       <c r="H171" s="53"/>
       <c r="I171" s="53"/>
@@ -30219,13 +30251,13 @@
         <v>246</v>
       </c>
       <c r="B172" s="53" t="s">
-        <v>2502</v>
+        <v>2506</v>
       </c>
       <c r="C172" s="48" t="s">
-        <v>2503</v>
+        <v>2507</v>
       </c>
       <c r="D172" s="8" t="s">
-        <v>2504</v>
+        <v>2508</v>
       </c>
       <c r="E172" s="53"/>
       <c r="F172" s="53"/>
@@ -30240,13 +30272,13 @@
         <v>246</v>
       </c>
       <c r="B173" s="53" t="s">
-        <v>2505</v>
+        <v>2509</v>
       </c>
       <c r="C173" s="48" t="s">
-        <v>2506</v>
+        <v>2510</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>2507</v>
+        <v>2511</v>
       </c>
       <c r="E173" s="53"/>
       <c r="F173" s="53"/>
@@ -30261,13 +30293,13 @@
         <v>246</v>
       </c>
       <c r="B174" s="53" t="s">
-        <v>2508</v>
+        <v>2512</v>
       </c>
       <c r="C174" s="48" t="s">
-        <v>2509</v>
+        <v>2513</v>
       </c>
       <c r="D174" s="8" t="s">
-        <v>2510</v>
+        <v>2514</v>
       </c>
       <c r="E174" s="53"/>
       <c r="F174" s="53"/>
@@ -30282,13 +30314,13 @@
         <v>246</v>
       </c>
       <c r="B175" s="53" t="s">
-        <v>2511</v>
+        <v>2515</v>
       </c>
       <c r="C175" s="48" t="s">
-        <v>2512</v>
+        <v>2516</v>
       </c>
       <c r="D175" s="8" t="s">
-        <v>2513</v>
+        <v>2517</v>
       </c>
       <c r="E175" s="53"/>
       <c r="F175" s="53"/>
@@ -30303,13 +30335,13 @@
         <v>246</v>
       </c>
       <c r="B176" s="53" t="s">
-        <v>2514</v>
+        <v>2518</v>
       </c>
       <c r="C176" s="48" t="s">
-        <v>2515</v>
+        <v>2519</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>2516</v>
+        <v>2520</v>
       </c>
       <c r="E176" s="53"/>
       <c r="F176" s="53"/>
@@ -30324,13 +30356,13 @@
         <v>246</v>
       </c>
       <c r="B177" s="53" t="s">
-        <v>2517</v>
+        <v>2521</v>
       </c>
       <c r="C177" s="48" t="s">
-        <v>2518</v>
+        <v>2522</v>
       </c>
       <c r="D177" s="8" t="s">
-        <v>2519</v>
+        <v>2523</v>
       </c>
       <c r="E177" s="53"/>
       <c r="F177" s="53"/>
@@ -30345,13 +30377,13 @@
         <v>246</v>
       </c>
       <c r="B178" s="53" t="s">
-        <v>2520</v>
+        <v>2524</v>
       </c>
       <c r="C178" s="48" t="s">
-        <v>2521</v>
+        <v>2525</v>
       </c>
       <c r="D178" s="8" t="s">
-        <v>2522</v>
+        <v>2526</v>
       </c>
       <c r="E178" s="53"/>
       <c r="F178" s="53"/>
@@ -30366,13 +30398,13 @@
         <v>246</v>
       </c>
       <c r="B179" s="53" t="s">
-        <v>2523</v>
+        <v>2527</v>
       </c>
       <c r="C179" s="48" t="s">
-        <v>2524</v>
+        <v>2528</v>
       </c>
       <c r="D179" s="8" t="s">
-        <v>2525</v>
+        <v>2529</v>
       </c>
       <c r="E179" s="53"/>
       <c r="F179" s="53"/>
@@ -30387,13 +30419,13 @@
         <v>246</v>
       </c>
       <c r="B180" s="53" t="s">
-        <v>2526</v>
+        <v>2530</v>
       </c>
       <c r="C180" s="48" t="s">
-        <v>2527</v>
+        <v>2531</v>
       </c>
       <c r="D180" s="8" t="s">
-        <v>2528</v>
+        <v>2532</v>
       </c>
       <c r="E180" s="53"/>
       <c r="F180" s="53"/>
@@ -30411,10 +30443,10 @@
         <v>229</v>
       </c>
       <c r="C181" s="48" t="s">
-        <v>2176</v>
+        <v>2180</v>
       </c>
       <c r="D181" s="8" t="s">
-        <v>2177</v>
+        <v>2181</v>
       </c>
       <c r="E181" s="53"/>
       <c r="F181" s="53"/>
@@ -30444,13 +30476,13 @@
         <v>258</v>
       </c>
       <c r="B183" s="53" t="s">
-        <v>2529</v>
+        <v>2533</v>
       </c>
       <c r="C183" s="48" t="s">
-        <v>2530</v>
+        <v>2534</v>
       </c>
       <c r="D183" s="8" t="s">
-        <v>2531</v>
+        <v>2535</v>
       </c>
       <c r="E183" s="53"/>
       <c r="F183" s="53"/>
@@ -30465,13 +30497,13 @@
         <v>258</v>
       </c>
       <c r="B184" s="53" t="s">
-        <v>2532</v>
+        <v>2536</v>
       </c>
       <c r="C184" s="48" t="s">
-        <v>2533</v>
+        <v>2537</v>
       </c>
       <c r="D184" s="8" t="s">
-        <v>2534</v>
+        <v>2538</v>
       </c>
       <c r="E184" s="53"/>
       <c r="F184" s="53"/>
@@ -30486,13 +30518,13 @@
         <v>258</v>
       </c>
       <c r="B185" s="53" t="s">
-        <v>2535</v>
+        <v>2539</v>
       </c>
       <c r="C185" s="48" t="s">
-        <v>2536</v>
+        <v>2540</v>
       </c>
       <c r="D185" s="8" t="s">
-        <v>2537</v>
+        <v>2541</v>
       </c>
       <c r="E185" s="53"/>
       <c r="F185" s="53"/>
@@ -30507,13 +30539,13 @@
         <v>258</v>
       </c>
       <c r="B186" s="53" t="s">
-        <v>2538</v>
+        <v>2542</v>
       </c>
       <c r="C186" s="48" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>2540</v>
+        <v>2544</v>
       </c>
       <c r="E186" s="53"/>
       <c r="F186" s="53"/>
@@ -30528,13 +30560,13 @@
         <v>258</v>
       </c>
       <c r="B187" s="53" t="s">
-        <v>2541</v>
+        <v>2545</v>
       </c>
       <c r="C187" s="48" t="s">
-        <v>2542</v>
+        <v>2546</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>2543</v>
+        <v>2547</v>
       </c>
       <c r="E187" s="53"/>
       <c r="F187" s="53"/>
@@ -30549,13 +30581,13 @@
         <v>258</v>
       </c>
       <c r="B188" s="53" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
       <c r="C188" s="48" t="s">
-        <v>2545</v>
+        <v>2549</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>2546</v>
+        <v>2550</v>
       </c>
       <c r="E188" s="53"/>
       <c r="F188" s="53"/>
@@ -30570,13 +30602,13 @@
         <v>258</v>
       </c>
       <c r="B189" s="53" t="s">
-        <v>2547</v>
+        <v>2551</v>
       </c>
       <c r="C189" s="48" t="s">
-        <v>2548</v>
+        <v>2552</v>
       </c>
       <c r="D189" s="8" t="s">
-        <v>2549</v>
+        <v>2553</v>
       </c>
       <c r="E189" s="53"/>
       <c r="F189" s="53"/>
@@ -30594,10 +30626,10 @@
         <v>1207</v>
       </c>
       <c r="C190" s="48" t="s">
-        <v>2550</v>
+        <v>2554</v>
       </c>
       <c r="D190" s="8" t="s">
-        <v>2551</v>
+        <v>2555</v>
       </c>
       <c r="E190" s="53"/>
       <c r="F190" s="53"/>
@@ -30614,10 +30646,10 @@
         <v>229</v>
       </c>
       <c r="C191" s="48" t="s">
-        <v>2176</v>
+        <v>2180</v>
       </c>
       <c r="D191" s="8" t="s">
-        <v>2177</v>
+        <v>2181</v>
       </c>
       <c r="E191" s="53"/>
       <c r="F191" s="53"/>
@@ -30635,10 +30667,10 @@
         <v>1171</v>
       </c>
       <c r="C192" s="53" t="s">
-        <v>2182</v>
+        <v>2186</v>
       </c>
       <c r="D192" s="53" t="s">
-        <v>2183</v>
+        <v>2187</v>
       </c>
       <c r="E192" s="53"/>
       <c r="F192" s="53"/>
@@ -30652,18 +30684,18 @@
         <v>287</v>
       </c>
       <c r="B193" s="53" t="s">
-        <v>2552</v>
+        <v>2556</v>
       </c>
       <c r="C193" s="48" t="s">
-        <v>2553</v>
+        <v>2557</v>
       </c>
       <c r="D193" s="8" t="s">
-        <v>2554</v>
+        <v>2558</v>
       </c>
       <c r="E193" s="53"/>
       <c r="F193" s="53"/>
       <c r="G193" s="53"/>
-      <c r="H193" s="97"/>
+      <c r="H193" s="98"/>
       <c r="I193" s="53"/>
     </row>
     <row r="194" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30671,13 +30703,13 @@
         <v>287</v>
       </c>
       <c r="B194" s="53" t="s">
-        <v>2555</v>
+        <v>2559</v>
       </c>
       <c r="C194" s="48" t="s">
-        <v>2556</v>
+        <v>2560</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>2557</v>
+        <v>2561</v>
       </c>
       <c r="E194" s="53"/>
       <c r="F194" s="53"/>
@@ -30690,13 +30722,13 @@
         <v>287</v>
       </c>
       <c r="B195" s="53" t="s">
-        <v>2558</v>
+        <v>2562</v>
       </c>
       <c r="C195" s="48" t="s">
-        <v>2559</v>
+        <v>2563</v>
       </c>
       <c r="D195" s="8" t="s">
-        <v>2560</v>
+        <v>2564</v>
       </c>
       <c r="E195" s="53"/>
       <c r="F195" s="53"/>
@@ -30709,13 +30741,13 @@
         <v>287</v>
       </c>
       <c r="B196" s="53" t="s">
-        <v>2561</v>
+        <v>2565</v>
       </c>
       <c r="C196" s="48" t="s">
-        <v>2562</v>
+        <v>2566</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>2563</v>
+        <v>2567</v>
       </c>
       <c r="E196" s="53"/>
       <c r="F196" s="53"/>
@@ -30728,13 +30760,13 @@
         <v>287</v>
       </c>
       <c r="B197" s="53" t="s">
-        <v>2564</v>
+        <v>2568</v>
       </c>
       <c r="C197" s="48" t="s">
-        <v>2565</v>
+        <v>2569</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>2566</v>
+        <v>2570</v>
       </c>
       <c r="E197" s="53"/>
       <c r="F197" s="53"/>
@@ -30747,18 +30779,18 @@
         <v>294</v>
       </c>
       <c r="B198" s="53" t="s">
-        <v>2552</v>
+        <v>2556</v>
       </c>
       <c r="C198" s="48" t="s">
-        <v>2553</v>
+        <v>2557</v>
       </c>
       <c r="D198" s="8" t="s">
-        <v>2554</v>
+        <v>2558</v>
       </c>
       <c r="E198" s="53"/>
       <c r="F198" s="53"/>
       <c r="G198" s="53"/>
-      <c r="H198" s="97" t="s">
+      <c r="H198" s="98" t="s">
         <v>1223</v>
       </c>
       <c r="I198" s="53"/>
@@ -30768,13 +30800,13 @@
         <v>294</v>
       </c>
       <c r="B199" s="53" t="s">
-        <v>2555</v>
+        <v>2559</v>
       </c>
       <c r="C199" s="48" t="s">
-        <v>2556</v>
+        <v>2560</v>
       </c>
       <c r="D199" s="8" t="s">
-        <v>2557</v>
+        <v>2561</v>
       </c>
       <c r="E199" s="53"/>
       <c r="F199" s="53"/>
@@ -30787,13 +30819,13 @@
         <v>294</v>
       </c>
       <c r="B200" s="53" t="s">
-        <v>2558</v>
+        <v>2562</v>
       </c>
       <c r="C200" s="48" t="s">
-        <v>2559</v>
+        <v>2563</v>
       </c>
       <c r="D200" s="8" t="s">
-        <v>2560</v>
+        <v>2564</v>
       </c>
       <c r="E200" s="53"/>
       <c r="F200" s="53"/>
@@ -30806,13 +30838,13 @@
         <v>294</v>
       </c>
       <c r="B201" s="53" t="s">
-        <v>2561</v>
+        <v>2565</v>
       </c>
       <c r="C201" s="48" t="s">
-        <v>2562</v>
+        <v>2566</v>
       </c>
       <c r="D201" s="8" t="s">
-        <v>2563</v>
+        <v>2567</v>
       </c>
       <c r="E201" s="53"/>
       <c r="F201" s="53"/>
@@ -30825,13 +30857,13 @@
         <v>294</v>
       </c>
       <c r="B202" s="53" t="s">
-        <v>2564</v>
+        <v>2568</v>
       </c>
       <c r="C202" s="48" t="s">
-        <v>2565</v>
+        <v>2569</v>
       </c>
       <c r="D202" s="8" t="s">
-        <v>2566</v>
+        <v>2570</v>
       </c>
       <c r="E202" s="53"/>
       <c r="F202" s="53"/>
@@ -30844,7 +30876,7 @@
         <v>857</v>
       </c>
       <c r="B203" s="66" t="s">
-        <v>2426</v>
+        <v>2430</v>
       </c>
       <c r="C203" s="66" t="s">
         <v>2021</v>
@@ -30858,7 +30890,7 @@
         <v>857</v>
       </c>
       <c r="B204" s="66" t="s">
-        <v>2434</v>
+        <v>2438</v>
       </c>
       <c r="C204" s="66" t="s">
         <v>2040</v>
@@ -30872,13 +30904,13 @@
         <v>857</v>
       </c>
       <c r="B205" s="66" t="s">
-        <v>2567</v>
+        <v>2571</v>
       </c>
       <c r="C205" s="66" t="s">
-        <v>2568</v>
+        <v>2572</v>
       </c>
       <c r="D205" s="66" t="s">
-        <v>2569</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30886,13 +30918,13 @@
         <v>857</v>
       </c>
       <c r="B206" s="66" t="s">
-        <v>2438</v>
+        <v>2442</v>
       </c>
       <c r="C206" s="66" t="s">
-        <v>2570</v>
+        <v>2574</v>
       </c>
       <c r="D206" s="66" t="s">
-        <v>2571</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30900,7 +30932,7 @@
         <v>857</v>
       </c>
       <c r="G207" s="66" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30908,13 +30940,13 @@
         <v>882</v>
       </c>
       <c r="B208" s="66" t="s">
-        <v>2572</v>
+        <v>2576</v>
       </c>
       <c r="C208" s="66" t="s">
-        <v>2573</v>
+        <v>2577</v>
       </c>
       <c r="D208" s="66" t="s">
-        <v>2574</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30922,13 +30954,13 @@
         <v>882</v>
       </c>
       <c r="B209" s="66" t="s">
-        <v>2575</v>
+        <v>2579</v>
       </c>
       <c r="C209" s="66" t="s">
-        <v>2576</v>
+        <v>2580</v>
       </c>
       <c r="D209" s="66" t="s">
-        <v>2577</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30936,13 +30968,13 @@
         <v>882</v>
       </c>
       <c r="B210" s="66" t="s">
-        <v>2578</v>
+        <v>2582</v>
       </c>
       <c r="C210" s="66" t="s">
-        <v>2579</v>
+        <v>2583</v>
       </c>
       <c r="D210" s="66" t="s">
-        <v>2580</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30950,13 +30982,13 @@
         <v>882</v>
       </c>
       <c r="B211" s="66" t="s">
-        <v>2581</v>
+        <v>2585</v>
       </c>
       <c r="C211" s="66" t="s">
-        <v>2582</v>
+        <v>2586</v>
       </c>
       <c r="D211" s="66" t="s">
-        <v>2583</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30964,13 +30996,13 @@
         <v>882</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>2584</v>
+        <v>2588</v>
       </c>
       <c r="C212" s="66" t="s">
-        <v>2585</v>
+        <v>2589</v>
       </c>
       <c r="D212" s="66" t="s">
-        <v>2586</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30978,13 +31010,13 @@
         <v>882</v>
       </c>
       <c r="B213" s="66" t="s">
-        <v>2587</v>
+        <v>2591</v>
       </c>
       <c r="C213" s="66" t="s">
-        <v>2588</v>
+        <v>2592</v>
       </c>
       <c r="D213" s="66" t="s">
-        <v>2589</v>
+        <v>2593</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30995,10 +31027,10 @@
         <v>229</v>
       </c>
       <c r="C214" s="66" t="s">
-        <v>2590</v>
+        <v>2594</v>
       </c>
       <c r="D214" s="66" t="s">
-        <v>2591</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31006,7 +31038,7 @@
         <v>887</v>
       </c>
       <c r="B215" s="66" t="s">
-        <v>2426</v>
+        <v>2430</v>
       </c>
       <c r="C215" s="66" t="s">
         <v>2021</v>
@@ -31020,7 +31052,7 @@
         <v>887</v>
       </c>
       <c r="B216" s="66" t="s">
-        <v>2434</v>
+        <v>2438</v>
       </c>
       <c r="C216" s="66" t="s">
         <v>2040</v>
@@ -31034,13 +31066,13 @@
         <v>887</v>
       </c>
       <c r="B217" s="66" t="s">
-        <v>2432</v>
+        <v>2436</v>
       </c>
       <c r="C217" s="66" t="s">
-        <v>2592</v>
+        <v>2596</v>
       </c>
       <c r="D217" s="66" t="s">
-        <v>2593</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="218" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31048,13 +31080,13 @@
         <v>887</v>
       </c>
       <c r="B218" s="66" t="s">
-        <v>2433</v>
+        <v>2437</v>
       </c>
       <c r="C218" s="66" t="s">
-        <v>2594</v>
+        <v>2598</v>
       </c>
       <c r="D218" s="66" t="s">
-        <v>2595</v>
+        <v>2599</v>
       </c>
       <c r="E218" s="66"/>
       <c r="F218" s="66"/>
@@ -31067,13 +31099,13 @@
         <v>887</v>
       </c>
       <c r="B219" s="66" t="s">
-        <v>2438</v>
+        <v>2442</v>
       </c>
       <c r="C219" s="66" t="s">
-        <v>2570</v>
+        <v>2574</v>
       </c>
       <c r="D219" s="66" t="s">
-        <v>2571</v>
+        <v>2575</v>
       </c>
       <c r="E219" s="66"/>
       <c r="F219" s="66"/>
@@ -31089,10 +31121,10 @@
         <v>229</v>
       </c>
       <c r="C220" s="66" t="s">
-        <v>2596</v>
+        <v>2600</v>
       </c>
       <c r="D220" s="66" t="s">
-        <v>2597</v>
+        <v>2601</v>
       </c>
       <c r="E220" s="66"/>
       <c r="F220" s="66"/>
@@ -31108,10 +31140,10 @@
         <v>1258</v>
       </c>
       <c r="C221" s="8" t="s">
-        <v>2598</v>
+        <v>2602</v>
       </c>
       <c r="D221" s="8" t="s">
-        <v>2599</v>
+        <v>2603</v>
       </c>
       <c r="E221" s="66"/>
       <c r="F221" s="66"/>
@@ -31124,13 +31156,13 @@
         <v>1052</v>
       </c>
       <c r="B222" s="66" t="s">
-        <v>2600</v>
+        <v>2604</v>
       </c>
       <c r="C222" s="8" t="s">
-        <v>2601</v>
+        <v>2605</v>
       </c>
       <c r="D222" s="8" t="s">
-        <v>2602</v>
+        <v>2606</v>
       </c>
       <c r="E222" s="66"/>
       <c r="F222" s="66"/>
@@ -31145,13 +31177,13 @@
         <v>1052</v>
       </c>
       <c r="B223" s="66" t="s">
-        <v>2603</v>
+        <v>2607</v>
       </c>
       <c r="C223" s="8" t="s">
-        <v>2604</v>
+        <v>2608</v>
       </c>
       <c r="D223" s="8" t="s">
-        <v>2605</v>
+        <v>2609</v>
       </c>
       <c r="E223" s="66"/>
       <c r="F223" s="66"/>
@@ -31166,13 +31198,13 @@
         <v>1052</v>
       </c>
       <c r="B224" s="66" t="s">
-        <v>2606</v>
+        <v>2610</v>
       </c>
       <c r="C224" s="8" t="s">
-        <v>2607</v>
+        <v>2611</v>
       </c>
       <c r="D224" s="51" t="s">
-        <v>2608</v>
+        <v>2612</v>
       </c>
       <c r="E224" s="66"/>
       <c r="F224" s="66"/>
@@ -31187,13 +31219,13 @@
         <v>1052</v>
       </c>
       <c r="B225" s="66" t="s">
-        <v>2609</v>
+        <v>2613</v>
       </c>
       <c r="C225" s="8" t="s">
-        <v>2610</v>
+        <v>2614</v>
       </c>
       <c r="D225" s="48" t="s">
-        <v>2611</v>
+        <v>2615</v>
       </c>
       <c r="E225" s="66"/>
       <c r="F225" s="66"/>
@@ -31206,13 +31238,13 @@
         <v>1058</v>
       </c>
       <c r="B226" s="66" t="s">
-        <v>2612</v>
+        <v>2616</v>
       </c>
       <c r="C226" s="8" t="s">
-        <v>2613</v>
+        <v>2617</v>
       </c>
       <c r="D226" s="8" t="s">
-        <v>2614</v>
+        <v>2618</v>
       </c>
       <c r="E226" s="66"/>
       <c r="F226" s="66"/>
@@ -31227,13 +31259,13 @@
         <v>1058</v>
       </c>
       <c r="B227" s="66" t="s">
-        <v>2615</v>
+        <v>2619</v>
       </c>
       <c r="C227" s="8" t="s">
-        <v>2616</v>
+        <v>2620</v>
       </c>
       <c r="D227" s="8" t="s">
-        <v>2617</v>
+        <v>2621</v>
       </c>
       <c r="E227" s="66"/>
       <c r="F227" s="66"/>
@@ -31248,13 +31280,13 @@
         <v>1058</v>
       </c>
       <c r="B228" s="66" t="s">
-        <v>2618</v>
+        <v>2622</v>
       </c>
       <c r="C228" s="8" t="s">
-        <v>2619</v>
+        <v>2623</v>
       </c>
       <c r="D228" s="8" t="s">
-        <v>2620</v>
+        <v>2624</v>
       </c>
       <c r="E228" s="66"/>
       <c r="F228" s="66"/>
@@ -31264,16 +31296,16 @@
     </row>
     <row r="229" s="50" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="54" t="s">
-        <v>2621</v>
+        <v>2625</v>
       </c>
       <c r="B229" s="66" t="s">
         <v>1167</v>
       </c>
       <c r="C229" s="51" t="s">
-        <v>2622</v>
+        <v>2626</v>
       </c>
       <c r="D229" s="8" t="s">
-        <v>2623</v>
+        <v>2627</v>
       </c>
       <c r="E229" s="66"/>
       <c r="F229" s="66"/>
@@ -31283,16 +31315,16 @@
     </row>
     <row r="230" s="50" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="54" t="s">
-        <v>2621</v>
+        <v>2625</v>
       </c>
       <c r="B230" s="66" t="s">
         <v>1225</v>
       </c>
       <c r="C230" s="51" t="s">
-        <v>2624</v>
+        <v>2628</v>
       </c>
       <c r="D230" s="48" t="s">
-        <v>2625</v>
+        <v>2629</v>
       </c>
       <c r="E230" s="66"/>
       <c r="F230" s="66"/>
@@ -31305,13 +31337,13 @@
         <v>1088</v>
       </c>
       <c r="B231" s="66" t="s">
-        <v>2626</v>
+        <v>2630</v>
       </c>
       <c r="C231" s="8" t="s">
-        <v>2627</v>
+        <v>2631</v>
       </c>
       <c r="D231" s="51" t="s">
-        <v>2628</v>
+        <v>2632</v>
       </c>
       <c r="E231" s="66"/>
       <c r="F231" s="66"/>
@@ -31324,13 +31356,13 @@
         <v>1088</v>
       </c>
       <c r="B232" s="66" t="s">
-        <v>2629</v>
+        <v>2633</v>
       </c>
       <c r="C232" s="8" t="s">
-        <v>2630</v>
+        <v>2634</v>
       </c>
       <c r="D232" s="51" t="s">
-        <v>2631</v>
+        <v>2635</v>
       </c>
       <c r="E232" s="66"/>
       <c r="F232" s="66"/>
@@ -31343,13 +31375,13 @@
         <v>1088</v>
       </c>
       <c r="B233" s="66" t="s">
-        <v>2632</v>
+        <v>2636</v>
       </c>
       <c r="C233" s="8" t="s">
-        <v>2633</v>
+        <v>2637</v>
       </c>
       <c r="D233" s="51" t="s">
-        <v>2634</v>
+        <v>2638</v>
       </c>
       <c r="E233" s="66"/>
       <c r="F233" s="66"/>
@@ -31362,13 +31394,13 @@
         <v>1088</v>
       </c>
       <c r="B234" s="66" t="s">
-        <v>2635</v>
+        <v>2639</v>
       </c>
       <c r="C234" s="8" t="s">
-        <v>2636</v>
+        <v>2640</v>
       </c>
       <c r="D234" s="51" t="s">
-        <v>2637</v>
+        <v>2641</v>
       </c>
       <c r="E234" s="66"/>
       <c r="F234" s="66"/>
@@ -31381,13 +31413,13 @@
         <v>1088</v>
       </c>
       <c r="B235" s="66" t="s">
-        <v>2638</v>
+        <v>2642</v>
       </c>
       <c r="C235" s="8" t="s">
-        <v>2639</v>
+        <v>2643</v>
       </c>
       <c r="D235" s="51" t="s">
-        <v>2640</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="236" s="50" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31395,13 +31427,13 @@
         <v>1088</v>
       </c>
       <c r="B236" s="66" t="s">
-        <v>2641</v>
+        <v>2645</v>
       </c>
       <c r="C236" s="8" t="s">
-        <v>2642</v>
+        <v>2646</v>
       </c>
       <c r="D236" s="51" t="s">
-        <v>2643</v>
+        <v>2647</v>
       </c>
       <c r="E236" s="66"/>
       <c r="F236" s="66"/>
@@ -31419,7 +31451,7 @@
       <c r="E237" s="66"/>
       <c r="F237" s="66"/>
       <c r="G237" s="53" t="s">
-        <v>2178</v>
+        <v>2182</v>
       </c>
       <c r="H237" s="66"/>
       <c r="I237" s="66"/>
@@ -31429,13 +31461,13 @@
         <v>946</v>
       </c>
       <c r="B238" s="50" t="s">
-        <v>2644</v>
+        <v>2648</v>
       </c>
       <c r="C238" s="50" t="s">
-        <v>2645</v>
+        <v>2649</v>
       </c>
       <c r="D238" s="50" t="s">
-        <v>2646</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="239" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31443,13 +31475,13 @@
         <v>946</v>
       </c>
       <c r="B239" s="50" t="s">
-        <v>2558</v>
+        <v>2562</v>
       </c>
       <c r="C239" s="50" t="s">
-        <v>2647</v>
+        <v>2651</v>
       </c>
       <c r="D239" s="50" t="s">
-        <v>2648</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="240" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31457,13 +31489,13 @@
         <v>946</v>
       </c>
       <c r="B240" s="50" t="s">
-        <v>2649</v>
+        <v>2653</v>
       </c>
       <c r="C240" s="50" t="s">
-        <v>2650</v>
+        <v>2654</v>
       </c>
       <c r="D240" s="50" t="s">
-        <v>2651</v>
+        <v>2655</v>
       </c>
     </row>
     <row r="241" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31471,13 +31503,13 @@
         <v>946</v>
       </c>
       <c r="B241" s="50" t="s">
-        <v>2652</v>
+        <v>2656</v>
       </c>
       <c r="C241" s="50" t="s">
-        <v>2653</v>
+        <v>2657</v>
       </c>
       <c r="D241" s="50" t="s">
-        <v>2654</v>
+        <v>2658</v>
       </c>
     </row>
     <row r="242" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31485,13 +31517,13 @@
         <v>946</v>
       </c>
       <c r="B242" s="50" t="s">
-        <v>2655</v>
+        <v>2659</v>
       </c>
       <c r="C242" s="50" t="s">
-        <v>2656</v>
+        <v>2660</v>
       </c>
       <c r="D242" s="50" t="s">
-        <v>2657</v>
+        <v>2661</v>
       </c>
     </row>
     <row r="243" s="50" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31502,10 +31534,10 @@
         <v>-2</v>
       </c>
       <c r="C243" s="57" t="s">
-        <v>2658</v>
+        <v>2662</v>
       </c>
       <c r="D243" s="57" t="s">
-        <v>2659</v>
+        <v>2663</v>
       </c>
       <c r="E243" s="66"/>
       <c r="F243" s="66"/>
@@ -31521,10 +31553,10 @@
         <v>-1</v>
       </c>
       <c r="C244" s="57" t="s">
-        <v>2660</v>
+        <v>2664</v>
       </c>
       <c r="D244" s="57" t="s">
-        <v>2661</v>
+        <v>2665</v>
       </c>
       <c r="E244" s="66"/>
       <c r="F244" s="66"/>
@@ -31540,10 +31572,10 @@
         <v>0</v>
       </c>
       <c r="C245" s="57" t="s">
-        <v>2662</v>
+        <v>2666</v>
       </c>
       <c r="D245" s="57" t="s">
-        <v>2663</v>
+        <v>2667</v>
       </c>
       <c r="E245" s="66"/>
       <c r="F245" s="66"/>
@@ -31559,10 +31591,10 @@
         <v>1</v>
       </c>
       <c r="C246" s="57" t="s">
-        <v>2664</v>
+        <v>2668</v>
       </c>
       <c r="D246" s="57" t="s">
-        <v>2665</v>
+        <v>2669</v>
       </c>
       <c r="E246" s="66"/>
       <c r="F246" s="66"/>
@@ -31578,10 +31610,10 @@
         <v>2</v>
       </c>
       <c r="C247" s="57" t="s">
-        <v>2666</v>
+        <v>2670</v>
       </c>
       <c r="D247" s="57" t="s">
-        <v>2667</v>
+        <v>2671</v>
       </c>
       <c r="E247" s="66"/>
       <c r="F247" s="66"/>
@@ -31597,10 +31629,10 @@
         <v>0</v>
       </c>
       <c r="C248" s="48" t="s">
-        <v>2668</v>
+        <v>2672</v>
       </c>
       <c r="D248" s="57" t="s">
-        <v>2669</v>
+        <v>2673</v>
       </c>
       <c r="E248" s="66"/>
       <c r="F248" s="66"/>
@@ -31616,10 +31648,10 @@
         <v>1</v>
       </c>
       <c r="C249" s="48" t="s">
-        <v>2670</v>
+        <v>2674</v>
       </c>
       <c r="D249" s="51" t="s">
-        <v>2671</v>
+        <v>2675</v>
       </c>
       <c r="E249" s="66"/>
       <c r="F249" s="66"/>
@@ -31635,10 +31667,10 @@
         <v>2</v>
       </c>
       <c r="C250" s="48" t="s">
-        <v>2672</v>
+        <v>2676</v>
       </c>
       <c r="D250" s="51" t="s">
-        <v>2673</v>
+        <v>2677</v>
       </c>
       <c r="E250" s="66"/>
       <c r="F250" s="66"/>
@@ -31654,10 +31686,10 @@
         <v>3</v>
       </c>
       <c r="C251" s="48" t="s">
-        <v>2674</v>
+        <v>2678</v>
       </c>
       <c r="D251" s="51" t="s">
-        <v>2675</v>
+        <v>2679</v>
       </c>
       <c r="E251" s="66"/>
       <c r="F251" s="66"/>
@@ -31673,10 +31705,10 @@
         <v>4</v>
       </c>
       <c r="C252" s="48" t="s">
-        <v>2676</v>
+        <v>2680</v>
       </c>
       <c r="D252" s="51" t="s">
-        <v>2677</v>
+        <v>2681</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31687,10 +31719,10 @@
         <v>-1</v>
       </c>
       <c r="C253" s="48" t="s">
-        <v>2678</v>
+        <v>2682</v>
       </c>
       <c r="D253" s="51" t="s">
-        <v>2679</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31698,13 +31730,13 @@
         <v>39</v>
       </c>
       <c r="B254" s="66" t="s">
-        <v>2680</v>
+        <v>2684</v>
       </c>
       <c r="C254" s="66" t="s">
-        <v>2681</v>
+        <v>2685</v>
       </c>
       <c r="D254" s="66" t="s">
-        <v>2682</v>
+        <v>2686</v>
       </c>
     </row>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
tripsIntro: rename `outOfTerritory` to `returnedHome`
fixes #192

The question and field are renamed to better represent the response,
with `yes` meaning that the person returned home and `no` the person
stayed out of territory all day.

Also fix the conditional for the `outOfTerritoryMembers` question to be
displayed only if `returnedHome` is `no`.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -1549,10 +1549,10 @@
     <t xml:space="preserve">departurePlaceOtherChoices</t>
   </si>
   <si>
-    <t xml:space="preserve">personOutOfTerritory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">household.persons.{_activePersonId}.journeys.{_activeJourneyId}.outOfTerritory</t>
+    <t xml:space="preserve">personReturnedHome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">household.persons.{_activePersonId}.journeys.{_activeJourneyId}.returnedHome</t>
   </si>
   <si>
     <t xml:space="preserve">Est-ce que {{nickname}} est retourn{{gender:é/ée/é(e)}} au domicile ({{address}}) la journée du {{journeyDate}}?</t>
@@ -1621,13 +1621,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">customLabels={{personOutOfTerritoryCustomLabel}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">outOfTerritoryConditional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">outOfTerritoryCustomChoices</t>
+    <t xml:space="preserve">customLabels={{personReturnedHomeCustomLabel}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">returnedHomeConditional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">returnedHomeCustomChoices</t>
   </si>
   <si>
     <t xml:space="preserve">Custom choices because it has the departure place type in the labels
@@ -4202,7 +4202,7 @@
     <t xml:space="preserve">hotelForVacation</t>
   </si>
   <si>
-    <t xml:space="preserve">${currentJourney}.outOfTerritory</t>
+    <t xml:space="preserve">${currentJourney}.returnedHome</t>
   </si>
   <si>
     <t xml:space="preserve">isCurrentSegmentNotTransitBusConditional</t>
@@ -6304,7 +6304,7 @@
     <t xml:space="preserve">I did make at least one trip on {{journeyDate}}</t>
   </si>
   <si>
-    <t xml:space="preserve">outOfTerritoryChoiceNo</t>
+    <t xml:space="preserve">returnedHomeChoiceNo</t>
   </si>
   <si>
     <t xml:space="preserve">Non, {{nickname}} est rest{{gender:é/ée/é(e)}} à cet endroit jusqu’au lendemain</t>
@@ -6319,7 +6319,7 @@
     <t xml:space="preserve">No, I stayed at this place until the next day</t>
   </si>
   <si>
-    <t xml:space="preserve">outOfTerritoryChoiceNo_hotelForWork</t>
+    <t xml:space="preserve">returnedHomeChoiceNo_hotelForWork</t>
   </si>
   <si>
     <t xml:space="preserve">Non, {{nickname}} est rest{{gender:é/ée/é(e)}} en voyage pour le travail jusqu’au lendemain</t>
@@ -6334,7 +6334,7 @@
     <t xml:space="preserve">No, I stayed away for work until the next day</t>
   </si>
   <si>
-    <t xml:space="preserve">outOfTerritoryChoiceNo_hotelForVacation</t>
+    <t xml:space="preserve">returnedHomeChoiceNo_hotelForVacation</t>
   </si>
   <si>
     <t xml:space="preserve">Non, {{nickname}} est rest{{gender:é/ée/é(e)}} en vacances jusqu’au lendemain</t>
@@ -6349,7 +6349,7 @@
     <t xml:space="preserve">No, I stayed on vacation until the next day</t>
   </si>
   <si>
-    <t xml:space="preserve">outOfTerritoryChoiceYes</t>
+    <t xml:space="preserve">returnedHomeChoiceYes</t>
   </si>
   <si>
     <t xml:space="preserve">Oui, {{nickname}} est reven{{gender:u/ue/u(e)}} au domicile avant le lendemain</t>
@@ -9397,8 +9397,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -21315,7 +21315,7 @@
         <v>1163</v>
       </c>
       <c r="E82" s="57" t="s">
-        <v>1167</v>
+        <v>1225</v>
       </c>
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
@@ -23250,7 +23250,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1048576"/>
+  <dimension ref="A1:F266"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="16.66"/>
@@ -27343,8 +27343,8 @@
         <v>2168</v>
       </c>
     </row>
-    <row r="266" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A266" s="50" t="s">
+    <row r="266" s="87" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="87" t="s">
         <v>2169</v>
       </c>
       <c r="B266" s="87" t="s">
@@ -27357,8 +27357,6 @@
         <v>2172</v>
       </c>
     </row>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A1:F260"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
RA and zat: centralize calculation on server
part of #262

Add a server helper function `updatePathsWithZonesIntersectingPoint`,
which adds the updated paths to calculate the intersecting zones (zat
and RA for now). It adds the corresponding zones to the geography's
properties, so if the geography is deleted, there are no stale values.

This helper function is called everywhere a geography is set (home,
visited place, prefilled home geography)

Update the zat matrix validation, as well as the home RA conditionals,
to match the new approach with the values in the geography's properties.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -4250,7 +4250,7 @@
     <t xml:space="preserve">${currentPerson}.hasSchoolPlace</t>
   </si>
   <si>
-    <t xml:space="preserve">home.RA</t>
+    <t xml:space="preserve">home.geography.properties.RA</t>
   </si>
   <si>
     <t xml:space="preserve">freqAttitudinal</t>
@@ -9048,7 +9048,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="98">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -9394,10 +9394,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -27343,17 +27339,17 @@
         <v>2168</v>
       </c>
     </row>
-    <row r="266" s="87" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A266" s="87" t="s">
+    <row r="266" s="74" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="74" t="s">
         <v>2169</v>
       </c>
-      <c r="B266" s="87" t="s">
+      <c r="B266" s="74" t="s">
         <v>2170</v>
       </c>
-      <c r="C266" s="87" t="s">
+      <c r="C266" s="74" t="s">
         <v>2171</v>
       </c>
-      <c r="D266" s="87" t="s">
+      <c r="D266" s="74" t="s">
         <v>2172</v>
       </c>
     </row>
@@ -27387,28 +27383,28 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="87" t="s">
         <v>2173</v>
       </c>
-      <c r="B1" s="88" t="s">
+      <c r="B1" s="87" t="s">
         <v>1159</v>
       </c>
-      <c r="C1" s="88" t="s">
+      <c r="C1" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="88" t="s">
+      <c r="D1" s="87" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="89" t="s">
+      <c r="E1" s="88" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="89" t="s">
+      <c r="F1" s="88" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="88" t="s">
+      <c r="G1" s="87" t="s">
         <v>2174</v>
       </c>
-      <c r="H1" s="88" t="s">
+      <c r="H1" s="87" t="s">
         <v>12</v>
       </c>
       <c r="I1" s="66" t="s">
@@ -27660,7 +27656,7 @@
       <c r="I16" s="53"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="90" t="s">
+      <c r="A17" s="89" t="s">
         <v>2192</v>
       </c>
       <c r="B17" s="53" t="s">
@@ -27678,7 +27674,7 @@
       <c r="H17" s="53"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="89" t="s">
         <v>2192</v>
       </c>
       <c r="B18" s="53" t="s">
@@ -27696,7 +27692,7 @@
       <c r="H18" s="53"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="90" t="s">
+      <c r="A19" s="89" t="s">
         <v>2192</v>
       </c>
       <c r="B19" s="53"/>
@@ -27710,7 +27706,7 @@
       <c r="H19" s="53"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="90" t="s">
+      <c r="A20" s="89" t="s">
         <v>187</v>
       </c>
       <c r="B20" s="53" t="s">
@@ -27728,7 +27724,7 @@
       <c r="H20" s="53"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="89" t="s">
         <v>187</v>
       </c>
       <c r="B21" s="53" t="s">
@@ -27746,7 +27742,7 @@
       <c r="H21" s="53"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="90" t="s">
+      <c r="A22" s="89" t="s">
         <v>187</v>
       </c>
       <c r="B22" s="53" t="s">
@@ -27764,7 +27760,7 @@
       <c r="H22" s="53"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="90" t="s">
+      <c r="A23" s="89" t="s">
         <v>187</v>
       </c>
       <c r="B23" s="53"/>
@@ -27894,7 +27890,7 @@
       <c r="F30" s="53"/>
       <c r="G30" s="53"/>
       <c r="H30" s="53"/>
-      <c r="I30" s="91" t="n">
+      <c r="I30" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27916,7 +27912,7 @@
       <c r="F31" s="53"/>
       <c r="G31" s="53"/>
       <c r="H31" s="53"/>
-      <c r="I31" s="91" t="n">
+      <c r="I31" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27938,7 +27934,7 @@
       <c r="F32" s="53"/>
       <c r="G32" s="53"/>
       <c r="H32" s="53"/>
-      <c r="I32" s="91" t="n">
+      <c r="I32" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27960,7 +27956,7 @@
       <c r="F33" s="53"/>
       <c r="G33" s="53"/>
       <c r="H33" s="53"/>
-      <c r="I33" s="91" t="n">
+      <c r="I33" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -27982,7 +27978,7 @@
       <c r="F34" s="53"/>
       <c r="G34" s="53"/>
       <c r="H34" s="53"/>
-      <c r="I34" s="91" t="n">
+      <c r="I34" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -28540,7 +28536,7 @@
       <c r="I64" s="53"/>
     </row>
     <row r="65" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="90" t="s">
+      <c r="A65" s="89" t="s">
         <v>322</v>
       </c>
       <c r="B65" s="53" t="s">
@@ -28561,7 +28557,7 @@
       <c r="I65" s="66"/>
     </row>
     <row r="66" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="90" t="s">
+      <c r="A66" s="89" t="s">
         <v>322</v>
       </c>
       <c r="B66" s="53" t="s">
@@ -28582,7 +28578,7 @@
       <c r="I66" s="66"/>
     </row>
     <row r="67" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="90" t="s">
+      <c r="A67" s="89" t="s">
         <v>322</v>
       </c>
       <c r="B67" s="53" t="s">
@@ -28603,7 +28599,7 @@
       <c r="I67" s="66"/>
     </row>
     <row r="68" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="90" t="s">
+      <c r="A68" s="89" t="s">
         <v>322</v>
       </c>
       <c r="B68" s="53" t="s">
@@ -28624,7 +28620,7 @@
       <c r="I68" s="66"/>
     </row>
     <row r="69" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="90" t="s">
+      <c r="A69" s="89" t="s">
         <v>322</v>
       </c>
       <c r="B69" s="53" t="s">
@@ -28645,7 +28641,7 @@
       <c r="I69" s="66"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="90" t="s">
+      <c r="A70" s="89" t="s">
         <v>905</v>
       </c>
       <c r="B70" s="66" t="s">
@@ -28659,7 +28655,7 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="90" t="s">
+      <c r="A71" s="89" t="s">
         <v>905</v>
       </c>
       <c r="B71" s="66" t="s">
@@ -28673,7 +28669,7 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="90" t="s">
+      <c r="A72" s="89" t="s">
         <v>905</v>
       </c>
       <c r="B72" s="66" t="s">
@@ -28687,7 +28683,7 @@
       </c>
     </row>
     <row r="73" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="90" t="s">
+      <c r="A73" s="89" t="s">
         <v>905</v>
       </c>
       <c r="B73" s="66" t="s">
@@ -28915,7 +28911,7 @@
       <c r="I84" s="53"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="92" t="s">
+      <c r="A85" s="91" t="s">
         <v>99</v>
       </c>
       <c r="B85" s="66" t="s">
@@ -28929,7 +28925,7 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="92" t="s">
+      <c r="A86" s="91" t="s">
         <v>99</v>
       </c>
       <c r="B86" s="66" t="s">
@@ -28943,7 +28939,7 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="92" t="s">
+      <c r="A87" s="91" t="s">
         <v>99</v>
       </c>
       <c r="B87" s="66" t="s">
@@ -28957,7 +28953,7 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="92" t="s">
+      <c r="A88" s="91" t="s">
         <v>99</v>
       </c>
       <c r="B88" s="66" t="s">
@@ -28971,7 +28967,7 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="93" t="s">
+      <c r="A89" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B89" s="53" t="s">
@@ -28992,7 +28988,7 @@
       <c r="I89" s="53"/>
     </row>
     <row r="90" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="93" t="s">
+      <c r="A90" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B90" s="53" t="s">
@@ -29013,7 +29009,7 @@
       <c r="I90" s="53"/>
     </row>
     <row r="91" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="93" t="s">
+      <c r="A91" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B91" s="53" t="s">
@@ -29032,7 +29028,7 @@
       <c r="I91" s="53"/>
     </row>
     <row r="92" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="93" t="s">
+      <c r="A92" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B92" s="53" t="s">
@@ -29051,7 +29047,7 @@
       <c r="I92" s="53"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="93" t="s">
+      <c r="A93" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B93" s="53" t="s">
@@ -29070,7 +29066,7 @@
       <c r="I93" s="53"/>
     </row>
     <row r="94" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="93" t="s">
+      <c r="A94" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B94" s="53" t="s">
@@ -29091,7 +29087,7 @@
       <c r="I94" s="53"/>
     </row>
     <row r="95" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="93" t="s">
+      <c r="A95" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B95" s="53" t="s">
@@ -29110,7 +29106,7 @@
       <c r="I95" s="53"/>
     </row>
     <row r="96" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="93" t="s">
+      <c r="A96" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B96" s="53" t="s">
@@ -29131,7 +29127,7 @@
       <c r="I96" s="53"/>
     </row>
     <row r="97" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="93" t="s">
+      <c r="A97" s="92" t="s">
         <v>423</v>
       </c>
       <c r="B97" s="53" t="s">
@@ -29150,7 +29146,7 @@
       <c r="I97" s="53"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="94" t="s">
+      <c r="A98" s="93" t="s">
         <v>2374</v>
       </c>
       <c r="B98" s="66" t="s">
@@ -29170,7 +29166,7 @@
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="94" t="s">
+      <c r="A99" s="93" t="s">
         <v>2374</v>
       </c>
       <c r="B99" s="66" t="s">
@@ -29190,7 +29186,7 @@
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="94" t="s">
+      <c r="A100" s="93" t="s">
         <v>2374</v>
       </c>
       <c r="B100" s="66" t="s">
@@ -29204,7 +29200,7 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="94" t="s">
+      <c r="A101" s="93" t="s">
         <v>771</v>
       </c>
       <c r="B101" s="66" t="s">
@@ -29218,7 +29214,7 @@
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="94" t="s">
+      <c r="A102" s="93" t="s">
         <v>771</v>
       </c>
       <c r="B102" s="66" t="s">
@@ -29230,13 +29226,13 @@
       <c r="D102" s="66" t="s">
         <v>2382</v>
       </c>
-      <c r="I102" s="91" t="n">
+      <c r="I102" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="94" t="s">
+      <c r="A103" s="93" t="s">
         <v>771</v>
       </c>
       <c r="B103" s="66" t="s">
@@ -29250,7 +29246,7 @@
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="94" t="s">
+      <c r="A104" s="93" t="s">
         <v>771</v>
       </c>
       <c r="B104" s="66" t="s">
@@ -29264,7 +29260,7 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="94" t="s">
+      <c r="A105" s="93" t="s">
         <v>771</v>
       </c>
       <c r="G105" s="53" t="s">
@@ -29272,7 +29268,7 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="94" t="s">
+      <c r="A106" s="93" t="s">
         <v>771</v>
       </c>
       <c r="G106" s="53" t="s">
@@ -29280,7 +29276,7 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="94" t="s">
+      <c r="A107" s="93" t="s">
         <v>829</v>
       </c>
       <c r="B107" s="66" t="s">
@@ -29294,7 +29290,7 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="94" t="s">
+      <c r="A108" s="93" t="s">
         <v>829</v>
       </c>
       <c r="B108" s="66" t="s">
@@ -29308,7 +29304,7 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="94" t="s">
+      <c r="A109" s="93" t="s">
         <v>829</v>
       </c>
       <c r="B109" s="66" t="s">
@@ -29322,7 +29318,7 @@
       </c>
     </row>
     <row r="110" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="94" t="s">
+      <c r="A110" s="93" t="s">
         <v>829</v>
       </c>
       <c r="B110" s="53" t="s">
@@ -29334,13 +29330,13 @@
       <c r="D110" s="48" t="s">
         <v>2399</v>
       </c>
-      <c r="I110" s="91" t="n">
+      <c r="I110" s="90" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="94" t="s">
+      <c r="A111" s="93" t="s">
         <v>829</v>
       </c>
       <c r="G111" s="53" t="s">
@@ -29348,7 +29344,7 @@
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="94" t="s">
+      <c r="A112" s="93" t="s">
         <v>829</v>
       </c>
       <c r="G112" s="53" t="s">
@@ -29356,7 +29352,7 @@
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="95" t="s">
+      <c r="A113" s="94" t="s">
         <v>347</v>
       </c>
       <c r="B113" s="66" t="s">
@@ -29370,7 +29366,7 @@
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="95" t="s">
+      <c r="A114" s="94" t="s">
         <v>347</v>
       </c>
       <c r="B114" s="66" t="s">
@@ -29384,7 +29380,7 @@
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="95" t="s">
+      <c r="A115" s="94" t="s">
         <v>347</v>
       </c>
       <c r="B115" s="66" t="s">
@@ -29398,7 +29394,7 @@
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="95" t="s">
+      <c r="A116" s="94" t="s">
         <v>347</v>
       </c>
       <c r="G116" s="53" t="s">
@@ -29406,7 +29402,7 @@
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="90" t="s">
+      <c r="A117" s="89" t="s">
         <v>2409</v>
       </c>
       <c r="B117" s="53" t="s">
@@ -29424,10 +29420,10 @@
       <c r="F117" s="53" t="s">
         <v>2413</v>
       </c>
-      <c r="G117" s="90"/>
+      <c r="G117" s="89"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="90" t="s">
+      <c r="A118" s="89" t="s">
         <v>2409</v>
       </c>
       <c r="B118" s="53" t="s">
@@ -29447,7 +29443,7 @@
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="90" t="s">
+      <c r="A119" s="89" t="s">
         <v>2409</v>
       </c>
       <c r="B119" s="53" t="s">
@@ -29467,7 +29463,7 @@
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="90" t="s">
+      <c r="A120" s="89" t="s">
         <v>2409</v>
       </c>
       <c r="B120" s="53" t="s">
@@ -29487,7 +29483,7 @@
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="90" t="s">
+      <c r="A121" s="89" t="s">
         <v>2409</v>
       </c>
       <c r="B121" s="53" t="s">
@@ -29533,7 +29529,7 @@
       <c r="D123" s="57" t="s">
         <v>2431</v>
       </c>
-      <c r="H123" s="96" t="s">
+      <c r="H123" s="95" t="s">
         <v>1235</v>
       </c>
     </row>
@@ -29550,7 +29546,7 @@
       <c r="D124" s="57" t="s">
         <v>2434</v>
       </c>
-      <c r="H124" s="97" t="s">
+      <c r="H124" s="96" t="s">
         <v>2435</v>
       </c>
     </row>
@@ -30693,7 +30689,7 @@
       <c r="E193" s="53"/>
       <c r="F193" s="53"/>
       <c r="G193" s="53"/>
-      <c r="H193" s="98"/>
+      <c r="H193" s="97"/>
       <c r="I193" s="53"/>
     </row>
     <row r="194" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30788,7 +30784,7 @@
       <c r="E198" s="53"/>
       <c r="F198" s="53"/>
       <c r="G198" s="53"/>
-      <c r="H198" s="98" t="s">
+      <c r="H198" s="97" t="s">
         <v>1223</v>
       </c>
       <c r="I198" s="53"/>

</xml_diff>

<commit_message>
home: ajout du lien vers les règlements du tirage
fixes #115

Le lien est ajouté vers le cms de l'artm
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -194,35 +194,8 @@
     <t xml:space="preserve">wantToParticipateToDraw</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Je souhaite participer au **tirage au sort**
-__Seuls les gagnants seront contactés. Il est nécessaire de terminer le questionnaire pour être retenu (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[Voir règlement](lien)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">).__</t>
-    </r>
+    <t xml:space="preserve">Je souhaite participer au **tirage au sort**
+__Seuls les gagnants seront contactés. Il est nécessaire de terminer le questionnaire pour être retenu (&lt;a href="https://www.artm.quebec/wp-content/uploads/2026/07/Reglement-concours_Enquete-2026-Pm_FR.pdf" target="_blank"&gt;Voir règlement&lt;/a&gt;).__</t>
   </si>
   <si>
     <r>
@@ -243,7 +216,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">[View rules](lien)</t>
+      <t xml:space="preserve">&lt;a href="https://www.artm.quebec/wp-content/uploads/2026/08/Contest-Rules_2026-Pm_EN.pdf" target="_blank"&gt;View rules&lt;/a&gt;</t>
     </r>
     <r>
       <rPr>
@@ -10191,7 +10164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
         <v>52</v>
       </c>
@@ -26130,13 +26103,13 @@
       <c r="A177" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B177" s="0" t="s">
+      <c r="B177" s="50" t="s">
         <v>1922</v>
       </c>
-      <c r="C177" s="0" t="s">
+      <c r="C177" s="50" t="s">
         <v>1923</v>
       </c>
-      <c r="D177" s="0" t="s">
+      <c r="D177" s="50" t="s">
         <v>1924</v>
       </c>
     </row>
@@ -26144,13 +26117,13 @@
       <c r="A178" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B178" s="0" t="s">
+      <c r="B178" s="50" t="s">
         <v>1925</v>
       </c>
-      <c r="C178" s="0" t="s">
+      <c r="C178" s="50" t="s">
         <v>1926</v>
       </c>
-      <c r="D178" s="0" t="s">
+      <c r="D178" s="50" t="s">
         <v>1927</v>
       </c>
     </row>
@@ -26158,13 +26131,13 @@
       <c r="A179" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B179" s="0" t="s">
+      <c r="B179" s="50" t="s">
         <v>1928</v>
       </c>
-      <c r="C179" s="0" t="s">
+      <c r="C179" s="50" t="s">
         <v>1929</v>
       </c>
-      <c r="D179" s="0" t="s">
+      <c r="D179" s="50" t="s">
         <v>1929</v>
       </c>
     </row>
@@ -26172,13 +26145,13 @@
       <c r="A180" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B180" s="0" t="s">
+      <c r="B180" s="50" t="s">
         <v>1930</v>
       </c>
-      <c r="C180" s="0" t="s">
+      <c r="C180" s="50" t="s">
         <v>1931</v>
       </c>
-      <c r="D180" s="0" t="s">
+      <c r="D180" s="50" t="s">
         <v>1932</v>
       </c>
     </row>
@@ -26186,13 +26159,13 @@
       <c r="A181" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B181" s="0" t="s">
+      <c r="B181" s="50" t="s">
         <v>1933</v>
       </c>
-      <c r="C181" s="0" t="s">
+      <c r="C181" s="50" t="s">
         <v>1934</v>
       </c>
-      <c r="D181" s="0" t="s">
+      <c r="D181" s="50" t="s">
         <v>1935</v>
       </c>
     </row>
@@ -26200,13 +26173,13 @@
       <c r="A182" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B182" s="0" t="s">
+      <c r="B182" s="50" t="s">
         <v>1936</v>
       </c>
-      <c r="C182" s="0" t="s">
+      <c r="C182" s="50" t="s">
         <v>1937</v>
       </c>
-      <c r="D182" s="0" t="s">
+      <c r="D182" s="50" t="s">
         <v>1938</v>
       </c>
     </row>
@@ -26214,13 +26187,13 @@
       <c r="A183" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B183" s="0" t="s">
+      <c r="B183" s="50" t="s">
         <v>1939</v>
       </c>
-      <c r="C183" s="0" t="s">
+      <c r="C183" s="50" t="s">
         <v>1940</v>
       </c>
-      <c r="D183" s="0" t="s">
+      <c r="D183" s="50" t="s">
         <v>1941</v>
       </c>
     </row>
@@ -26228,13 +26201,13 @@
       <c r="A184" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B184" s="0" t="s">
+      <c r="B184" s="50" t="s">
         <v>1942</v>
       </c>
-      <c r="C184" s="0" t="s">
+      <c r="C184" s="50" t="s">
         <v>1943</v>
       </c>
-      <c r="D184" s="0" t="s">
+      <c r="D184" s="50" t="s">
         <v>1944</v>
       </c>
     </row>
@@ -26242,13 +26215,13 @@
       <c r="A185" s="50" t="s">
         <v>560</v>
       </c>
-      <c r="B185" s="0" t="s">
+      <c r="B185" s="50" t="s">
         <v>1945</v>
       </c>
-      <c r="C185" s="0" t="s">
+      <c r="C185" s="50" t="s">
         <v>1601</v>
       </c>
-      <c r="D185" s="0" t="s">
+      <c r="D185" s="50" t="s">
         <v>1602</v>
       </c>
     </row>

</xml_diff>

<commit_message>
segments: ajouter les boutons 'Autre' et 'Je ne sais pas'
fixes #176

Pour les questions de station d'entrée/sorties de la liste déroulante,
un choix 'autre' est ajouté dans tous les cas et 'dontknow' si la
personne n'est pas auto-répondante.

Ces valeurs sont aussi ajoutées en raccourcis au bas du widget.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -16,7 +16,7 @@
     <sheet name="Choices" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Labels!$A$1:$F$269</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Labels!$A$1:$F$271</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Widgets!$A$1:$W$1048536</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4935" uniqueCount="2702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4943" uniqueCount="2704">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -7030,6 +7030,12 @@
   <si>
     <t xml:space="preserve">
 __**Note:** Information prefilled from {{referenceNickname}}'s trip diary. Verify if the information is correct and change if needed.__</t>
+  </si>
+  <si>
+    <t xml:space="preserve">featureSelect.other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">featureSelect.dontKnow</t>
   </si>
   <si>
     <t xml:space="preserve">personHasSchoolPlace_schoolchildcare</t>
@@ -23264,7 +23270,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F275"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="50" width="16.66"/>
@@ -27233,114 +27239,114 @@
         <v>2138</v>
       </c>
     </row>
-    <row r="258" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A258" s="48" t="s">
+    <row r="258" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="50" t="s">
+        <v>560</v>
+      </c>
+      <c r="B258" s="8" t="s">
+        <v>2139</v>
+      </c>
+      <c r="C258" s="8" t="s">
+        <v>1601</v>
+      </c>
+      <c r="D258" s="57" t="s">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="50" t="s">
+        <v>560</v>
+      </c>
+      <c r="B259" s="8" t="s">
+        <v>2140</v>
+      </c>
+      <c r="C259" s="8" t="s">
+        <v>1432</v>
+      </c>
+      <c r="D259" s="57" t="s">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="48" t="s">
         <v>756</v>
       </c>
-      <c r="B258" s="54" t="s">
-        <v>2139</v>
-      </c>
-      <c r="C258" s="8" t="s">
-        <v>2140</v>
-      </c>
-      <c r="D258" s="85" t="s">
+      <c r="B260" s="54" t="s">
         <v>2141</v>
       </c>
-    </row>
-    <row r="259" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A259" s="50" t="s">
-        <v>756</v>
-      </c>
-      <c r="B259" s="86" t="s">
+      <c r="C260" s="8" t="s">
         <v>2142</v>
       </c>
-      <c r="C259" s="48" t="s">
-        <v>1371</v>
-      </c>
-      <c r="D259" s="51" t="s">
-        <v>1372</v>
-      </c>
-    </row>
-    <row r="260" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A260" s="50" t="s">
-        <v>756</v>
-      </c>
-      <c r="B260" s="86" t="s">
+      <c r="D260" s="85" t="s">
         <v>2143</v>
       </c>
-      <c r="C260" s="8" t="s">
-        <v>2144</v>
-      </c>
-      <c r="D260" s="51" t="s">
-        <v>2145</v>
-      </c>
-    </row>
-    <row r="261" customFormat="false" ht="285.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="261" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="50" t="s">
         <v>756</v>
       </c>
-      <c r="B261" s="53" t="s">
-        <v>2146</v>
-      </c>
-      <c r="C261" s="54" t="s">
-        <v>2147</v>
-      </c>
-      <c r="D261" s="54" t="s">
-        <v>2148</v>
-      </c>
-      <c r="E261" s="54" t="s">
-        <v>2149</v>
-      </c>
-      <c r="F261" s="54" t="s">
-        <v>2150</v>
-      </c>
-    </row>
-    <row r="262" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B261" s="86" t="s">
+        <v>2144</v>
+      </c>
+      <c r="C261" s="48" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D261" s="51" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="50" t="s">
         <v>756</v>
       </c>
-      <c r="B262" s="53" t="s">
+      <c r="B262" s="86" t="s">
+        <v>2145</v>
+      </c>
+      <c r="C262" s="8" t="s">
+        <v>2146</v>
+      </c>
+      <c r="D262" s="51" t="s">
+        <v>2147</v>
+      </c>
+    </row>
+    <row r="263" customFormat="false" ht="285.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="50" t="s">
+        <v>756</v>
+      </c>
+      <c r="B263" s="53" t="s">
+        <v>2148</v>
+      </c>
+      <c r="C263" s="54" t="s">
+        <v>2149</v>
+      </c>
+      <c r="D263" s="54" t="s">
+        <v>2150</v>
+      </c>
+      <c r="E263" s="54" t="s">
         <v>2151</v>
       </c>
-      <c r="C262" s="54" t="s">
+      <c r="F263" s="54" t="s">
         <v>2152</v>
       </c>
-      <c r="D262" s="54" t="s">
+    </row>
+    <row r="264" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="50" t="s">
+        <v>756</v>
+      </c>
+      <c r="B264" s="53" t="s">
         <v>2153</v>
       </c>
-      <c r="E262" s="54" t="s">
+      <c r="C264" s="54" t="s">
         <v>2154</v>
       </c>
-      <c r="F262" s="54" t="s">
+      <c r="D264" s="54" t="s">
         <v>2155</v>
       </c>
-    </row>
-    <row r="263" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A263" s="50" t="s">
-        <v>833</v>
-      </c>
-      <c r="B263" s="50" t="s">
+      <c r="E264" s="54" t="s">
         <v>2156</v>
       </c>
-      <c r="C263" s="48" t="s">
-        <v>1371</v>
-      </c>
-      <c r="D263" s="51" t="s">
-        <v>1372</v>
-      </c>
-    </row>
-    <row r="264" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A264" s="50" t="s">
-        <v>833</v>
-      </c>
-      <c r="B264" s="50" t="s">
+      <c r="F264" s="54" t="s">
         <v>2157</v>
-      </c>
-      <c r="C264" s="8" t="s">
-        <v>2158</v>
-      </c>
-      <c r="D264" s="8" t="s">
-        <v>2159</v>
       </c>
     </row>
     <row r="265" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27348,97 +27354,97 @@
         <v>833</v>
       </c>
       <c r="B265" s="50" t="s">
+        <v>2158</v>
+      </c>
+      <c r="C265" s="48" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D265" s="51" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="266" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A266" s="50" t="s">
+        <v>833</v>
+      </c>
+      <c r="B266" s="50" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C266" s="8" t="s">
         <v>2160</v>
       </c>
-      <c r="C265" s="8" t="s">
-        <v>1429</v>
-      </c>
-      <c r="D265" s="8" t="s">
-        <v>1430</v>
-      </c>
-    </row>
-    <row r="266" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A266" s="50" t="s">
-        <v>1053</v>
-      </c>
-      <c r="B266" s="50" t="s">
+      <c r="D266" s="8" t="s">
         <v>2161</v>
       </c>
-      <c r="C266" s="48" t="s">
-        <v>1371</v>
-      </c>
-      <c r="D266" s="51" t="s">
-        <v>1372</v>
-      </c>
-    </row>
-    <row r="267" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="267" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="50" t="s">
-        <v>1053</v>
+        <v>833</v>
       </c>
       <c r="B267" s="50" t="s">
         <v>2162</v>
       </c>
       <c r="C267" s="8" t="s">
+        <v>1429</v>
+      </c>
+      <c r="D267" s="8" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="268" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A268" s="50" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B268" s="50" t="s">
         <v>2163</v>
       </c>
-      <c r="D267" s="51" t="s">
+      <c r="C268" s="48" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D268" s="51" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="269" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A269" s="50" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B269" s="50" t="s">
         <v>2164</v>
       </c>
-    </row>
-    <row r="268" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A268" s="50" t="s">
+      <c r="C269" s="8" t="s">
+        <v>2165</v>
+      </c>
+      <c r="D269" s="51" t="s">
+        <v>2166</v>
+      </c>
+    </row>
+    <row r="270" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A270" s="50" t="s">
         <v>1001</v>
       </c>
-      <c r="B268" s="54" t="s">
-        <v>2165</v>
-      </c>
-      <c r="C268" s="54" t="s">
-        <v>2166</v>
-      </c>
-      <c r="D268" s="54" t="s">
+      <c r="B270" s="54" t="s">
         <v>2167</v>
       </c>
-    </row>
-    <row r="269" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A269" s="50" t="s">
+      <c r="C270" s="54" t="s">
+        <v>2168</v>
+      </c>
+      <c r="D270" s="54" t="s">
+        <v>2169</v>
+      </c>
+    </row>
+    <row r="271" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A271" s="50" t="s">
         <v>1001</v>
       </c>
-      <c r="B269" s="54" t="s">
-        <v>2168</v>
-      </c>
-      <c r="C269" s="54" t="s">
-        <v>2169</v>
-      </c>
-      <c r="D269" s="54" t="s">
+      <c r="B271" s="54" t="s">
         <v>2170</v>
       </c>
-    </row>
-    <row r="270" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A270" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="B270" s="50" t="s">
+      <c r="C271" s="54" t="s">
         <v>2171</v>
       </c>
-      <c r="C270" s="48" t="s">
+      <c r="D271" s="54" t="s">
         <v>2172</v>
-      </c>
-      <c r="D270" s="51" t="s">
-        <v>2173</v>
-      </c>
-    </row>
-    <row r="271" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A271" s="50" t="s">
-        <v>48</v>
-      </c>
-      <c r="B271" s="50" t="s">
-        <v>2174</v>
-      </c>
-      <c r="C271" s="8" t="s">
-        <v>2175</v>
-      </c>
-      <c r="D271" s="51" t="s">
-        <v>2176</v>
       </c>
     </row>
     <row r="272" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27446,59 +27452,87 @@
         <v>48</v>
       </c>
       <c r="B272" s="50" t="s">
-        <v>2177</v>
+        <v>2173</v>
       </c>
       <c r="C272" s="48" t="s">
-        <v>1371</v>
+        <v>2174</v>
       </c>
       <c r="D272" s="51" t="s">
-        <v>1372</v>
-      </c>
-    </row>
-    <row r="273" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2175</v>
+      </c>
+    </row>
+    <row r="273" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="50" t="s">
         <v>48</v>
       </c>
       <c r="B273" s="50" t="s">
+        <v>2176</v>
+      </c>
+      <c r="C273" s="8" t="s">
+        <v>2177</v>
+      </c>
+      <c r="D273" s="51" t="s">
         <v>2178</v>
       </c>
-      <c r="C273" s="8" t="s">
+    </row>
+    <row r="274" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A274" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="B274" s="50" t="s">
         <v>2179</v>
       </c>
-      <c r="D273" s="51" t="s">
+      <c r="C274" s="48" t="s">
+        <v>1371</v>
+      </c>
+      <c r="D274" s="51" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="275" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A275" s="50" t="s">
+        <v>48</v>
+      </c>
+      <c r="B275" s="50" t="s">
         <v>2180</v>
       </c>
-    </row>
-    <row r="274" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A274" s="50" t="s">
+      <c r="C275" s="8" t="s">
+        <v>2181</v>
+      </c>
+      <c r="D275" s="51" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="276" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A276" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="B274" s="50" t="s">
-        <v>2181</v>
-      </c>
-      <c r="C274" s="8" t="s">
-        <v>2182</v>
-      </c>
-      <c r="D274" s="8" t="s">
+      <c r="B276" s="50" t="s">
         <v>2183</v>
       </c>
-    </row>
-    <row r="275" s="74" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A275" s="74" t="s">
+      <c r="C276" s="8" t="s">
         <v>2184</v>
       </c>
-      <c r="B275" s="74" t="s">
+      <c r="D276" s="8" t="s">
         <v>2185</v>
       </c>
-      <c r="C275" s="74" t="s">
+    </row>
+    <row r="277" s="74" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A277" s="74" t="s">
         <v>2186</v>
       </c>
-      <c r="D275" s="74" t="s">
+      <c r="B277" s="74" t="s">
         <v>2187</v>
       </c>
+      <c r="C277" s="74" t="s">
+        <v>2188</v>
+      </c>
+      <c r="D277" s="74" t="s">
+        <v>2189</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F269"/>
+  <autoFilter ref="A1:F271"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -27528,7 +27562,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="87" t="s">
-        <v>2188</v>
+        <v>2190</v>
       </c>
       <c r="B1" s="87" t="s">
         <v>1159</v>
@@ -27546,13 +27580,13 @@
         <v>9</v>
       </c>
       <c r="G1" s="87" t="s">
-        <v>2189</v>
+        <v>2191</v>
       </c>
       <c r="H1" s="87" t="s">
         <v>12</v>
       </c>
       <c r="I1" s="66" t="s">
-        <v>2190</v>
+        <v>2192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27563,10 +27597,10 @@
         <v>1167</v>
       </c>
       <c r="C2" s="53" t="s">
-        <v>2191</v>
+        <v>2193</v>
       </c>
       <c r="D2" s="53" t="s">
-        <v>2192</v>
+        <v>2194</v>
       </c>
       <c r="E2" s="53"/>
       <c r="F2" s="53"/>
@@ -27581,10 +27615,10 @@
         <v>1225</v>
       </c>
       <c r="C3" s="53" t="s">
-        <v>2193</v>
+        <v>2195</v>
       </c>
       <c r="D3" s="53" t="s">
-        <v>2194</v>
+        <v>2196</v>
       </c>
       <c r="E3" s="53"/>
       <c r="F3" s="53"/>
@@ -27599,10 +27633,10 @@
         <v>229</v>
       </c>
       <c r="C4" s="53" t="s">
-        <v>2195</v>
+        <v>2197</v>
       </c>
       <c r="D4" s="53" t="s">
-        <v>2196</v>
+        <v>2198</v>
       </c>
       <c r="E4" s="53"/>
       <c r="F4" s="53"/>
@@ -27611,7 +27645,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
       <c r="B5" s="53" t="s">
         <v>229</v>
@@ -27629,16 +27663,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="C6" s="53" t="s">
-        <v>2199</v>
+        <v>2201</v>
       </c>
       <c r="D6" s="53" t="s">
-        <v>2200</v>
+        <v>2202</v>
       </c>
       <c r="E6" s="53"/>
       <c r="F6" s="53"/>
@@ -27653,10 +27687,10 @@
         <v>1171</v>
       </c>
       <c r="C7" s="53" t="s">
-        <v>2201</v>
+        <v>2203</v>
       </c>
       <c r="D7" s="53" t="s">
-        <v>2202</v>
+        <v>2204</v>
       </c>
       <c r="E7" s="53"/>
       <c r="F7" s="53"/>
@@ -27715,7 +27749,7 @@
       <c r="E11" s="53"/>
       <c r="F11" s="53"/>
       <c r="G11" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="H11" s="53"/>
     </row>
@@ -27769,10 +27803,10 @@
         <v>1167</v>
       </c>
       <c r="C15" s="51" t="s">
-        <v>2203</v>
+        <v>2205</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>2204</v>
+        <v>2206</v>
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="51"/>
@@ -27788,10 +27822,10 @@
         <v>1225</v>
       </c>
       <c r="C16" s="51" t="s">
-        <v>2205</v>
+        <v>2207</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>2206</v>
+        <v>2208</v>
       </c>
       <c r="E16" s="51"/>
       <c r="F16" s="51"/>
@@ -27801,16 +27835,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="89" t="s">
-        <v>2207</v>
+        <v>2209</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>2208</v>
+        <v>2210</v>
       </c>
       <c r="C17" s="53" t="s">
-        <v>2209</v>
+        <v>2211</v>
       </c>
       <c r="D17" s="53" t="s">
-        <v>2210</v>
+        <v>2212</v>
       </c>
       <c r="E17" s="53"/>
       <c r="F17" s="53"/>
@@ -27819,16 +27853,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="89" t="s">
-        <v>2207</v>
+        <v>2209</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>2211</v>
+        <v>2213</v>
       </c>
       <c r="C18" s="53" t="s">
-        <v>2212</v>
+        <v>2214</v>
       </c>
       <c r="D18" s="53" t="s">
-        <v>2213</v>
+        <v>2215</v>
       </c>
       <c r="E18" s="53"/>
       <c r="F18" s="53"/>
@@ -27837,7 +27871,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="89" t="s">
-        <v>2207</v>
+        <v>2209</v>
       </c>
       <c r="B19" s="53"/>
       <c r="C19" s="53"/>
@@ -27854,13 +27888,13 @@
         <v>187</v>
       </c>
       <c r="B20" s="53" t="s">
-        <v>2208</v>
+        <v>2210</v>
       </c>
       <c r="C20" s="53" t="s">
-        <v>2209</v>
+        <v>2211</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>2214</v>
+        <v>2216</v>
       </c>
       <c r="E20" s="53"/>
       <c r="F20" s="53"/>
@@ -27872,13 +27906,13 @@
         <v>187</v>
       </c>
       <c r="B21" s="53" t="s">
-        <v>2211</v>
+        <v>2213</v>
       </c>
       <c r="C21" s="53" t="s">
-        <v>2212</v>
+        <v>2214</v>
       </c>
       <c r="D21" s="53" t="s">
-        <v>2215</v>
+        <v>2217</v>
       </c>
       <c r="E21" s="53"/>
       <c r="F21" s="53"/>
@@ -27893,10 +27927,10 @@
         <v>189</v>
       </c>
       <c r="C22" s="53" t="s">
-        <v>2216</v>
+        <v>2218</v>
       </c>
       <c r="D22" s="53" t="s">
-        <v>2217</v>
+        <v>2219</v>
       </c>
       <c r="E22" s="53"/>
       <c r="F22" s="53"/>
@@ -27922,13 +27956,13 @@
         <v>306</v>
       </c>
       <c r="B24" s="53" t="s">
-        <v>2218</v>
+        <v>2220</v>
       </c>
       <c r="C24" s="53" t="s">
-        <v>2219</v>
+        <v>2221</v>
       </c>
       <c r="D24" s="53" t="s">
-        <v>2220</v>
+        <v>2222</v>
       </c>
       <c r="E24" s="53"/>
       <c r="F24" s="53"/>
@@ -27940,13 +27974,13 @@
         <v>306</v>
       </c>
       <c r="B25" s="53" t="s">
-        <v>2221</v>
+        <v>2223</v>
       </c>
       <c r="C25" s="53" t="s">
-        <v>2222</v>
+        <v>2224</v>
       </c>
       <c r="D25" s="53" t="s">
-        <v>2223</v>
+        <v>2225</v>
       </c>
       <c r="E25" s="53"/>
       <c r="F25" s="53"/>
@@ -27972,13 +28006,13 @@
         <v>299</v>
       </c>
       <c r="B27" s="53" t="s">
-        <v>2218</v>
+        <v>2220</v>
       </c>
       <c r="C27" s="53" t="s">
-        <v>2224</v>
+        <v>2226</v>
       </c>
       <c r="D27" s="53" t="s">
-        <v>2225</v>
+        <v>2227</v>
       </c>
       <c r="E27" s="53"/>
       <c r="F27" s="53"/>
@@ -27990,13 +28024,13 @@
         <v>299</v>
       </c>
       <c r="B28" s="53" t="s">
-        <v>2221</v>
+        <v>2223</v>
       </c>
       <c r="C28" s="53" t="s">
-        <v>2226</v>
+        <v>2228</v>
       </c>
       <c r="D28" s="53" t="s">
-        <v>2227</v>
+        <v>2229</v>
       </c>
       <c r="E28" s="53"/>
       <c r="F28" s="53"/>
@@ -28025,10 +28059,10 @@
         <v>1191</v>
       </c>
       <c r="C30" s="53" t="s">
-        <v>2228</v>
+        <v>2230</v>
       </c>
       <c r="D30" s="53" t="s">
-        <v>2229</v>
+        <v>2231</v>
       </c>
       <c r="E30" s="53"/>
       <c r="F30" s="53"/>
@@ -28047,10 +28081,10 @@
         <v>1192</v>
       </c>
       <c r="C31" s="53" t="s">
-        <v>2230</v>
+        <v>2232</v>
       </c>
       <c r="D31" s="53" t="s">
-        <v>2231</v>
+        <v>2233</v>
       </c>
       <c r="E31" s="53"/>
       <c r="F31" s="53"/>
@@ -28069,10 +28103,10 @@
         <v>1193</v>
       </c>
       <c r="C32" s="53" t="s">
-        <v>2232</v>
+        <v>2234</v>
       </c>
       <c r="D32" s="53" t="s">
-        <v>2233</v>
+        <v>2235</v>
       </c>
       <c r="E32" s="53"/>
       <c r="F32" s="53"/>
@@ -28091,10 +28125,10 @@
         <v>1195</v>
       </c>
       <c r="C33" s="53" t="s">
-        <v>2234</v>
+        <v>2236</v>
       </c>
       <c r="D33" s="53" t="s">
-        <v>2235</v>
+        <v>2237</v>
       </c>
       <c r="E33" s="53"/>
       <c r="F33" s="53"/>
@@ -28113,10 +28147,10 @@
         <v>1196</v>
       </c>
       <c r="C34" s="53" t="s">
-        <v>2236</v>
+        <v>2238</v>
       </c>
       <c r="D34" s="53" t="s">
-        <v>2237</v>
+        <v>2239</v>
       </c>
       <c r="E34" s="53"/>
       <c r="F34" s="53"/>
@@ -28132,13 +28166,13 @@
         <v>340</v>
       </c>
       <c r="B35" s="53" t="s">
-        <v>2238</v>
+        <v>2240</v>
       </c>
       <c r="C35" s="53" t="s">
-        <v>2239</v>
+        <v>2241</v>
       </c>
       <c r="D35" s="53" t="s">
-        <v>2240</v>
+        <v>2242</v>
       </c>
       <c r="E35" s="53"/>
       <c r="F35" s="53"/>
@@ -28153,13 +28187,13 @@
         <v>340</v>
       </c>
       <c r="B36" s="53" t="s">
-        <v>2241</v>
+        <v>2243</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>2242</v>
+        <v>2244</v>
       </c>
       <c r="D36" s="53" t="s">
-        <v>2243</v>
+        <v>2245</v>
       </c>
       <c r="E36" s="53"/>
       <c r="F36" s="53"/>
@@ -28175,10 +28209,10 @@
         <v>1262</v>
       </c>
       <c r="C37" s="53" t="s">
-        <v>2244</v>
+        <v>2246</v>
       </c>
       <c r="D37" s="53" t="s">
-        <v>2245</v>
+        <v>2247</v>
       </c>
       <c r="E37" s="53"/>
       <c r="F37" s="53"/>
@@ -28194,10 +28228,10 @@
         <v>1263</v>
       </c>
       <c r="C38" s="53" t="s">
-        <v>2246</v>
+        <v>2248</v>
       </c>
       <c r="D38" s="53" t="s">
-        <v>2247</v>
+        <v>2249</v>
       </c>
       <c r="E38" s="53"/>
       <c r="F38" s="53"/>
@@ -28210,13 +28244,13 @@
         <v>340</v>
       </c>
       <c r="B39" s="53" t="s">
-        <v>2248</v>
+        <v>2250</v>
       </c>
       <c r="C39" s="53" t="s">
-        <v>2249</v>
+        <v>2251</v>
       </c>
       <c r="D39" s="53" t="s">
-        <v>2250</v>
+        <v>2252</v>
       </c>
       <c r="E39" s="53"/>
       <c r="F39" s="53"/>
@@ -28229,13 +28263,13 @@
         <v>340</v>
       </c>
       <c r="B40" s="53" t="s">
-        <v>2251</v>
+        <v>2253</v>
       </c>
       <c r="C40" s="53" t="s">
-        <v>2252</v>
+        <v>2254</v>
       </c>
       <c r="D40" s="53" t="s">
-        <v>2253</v>
+        <v>2255</v>
       </c>
       <c r="E40" s="53"/>
       <c r="F40" s="53"/>
@@ -28253,7 +28287,7 @@
       <c r="E41" s="53"/>
       <c r="F41" s="53"/>
       <c r="G41" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
       <c r="H41" s="53"/>
       <c r="I41" s="66"/>
@@ -28278,13 +28312,13 @@
         <v>315</v>
       </c>
       <c r="B43" s="53" t="s">
-        <v>2254</v>
+        <v>2256</v>
       </c>
       <c r="C43" s="48" t="s">
-        <v>2255</v>
+        <v>2257</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>2256</v>
+        <v>2258</v>
       </c>
       <c r="E43" s="53"/>
       <c r="F43" s="53"/>
@@ -28297,13 +28331,13 @@
         <v>315</v>
       </c>
       <c r="B44" s="53" t="s">
-        <v>2257</v>
+        <v>2259</v>
       </c>
       <c r="C44" s="48" t="s">
-        <v>2258</v>
+        <v>2260</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>2259</v>
+        <v>2261</v>
       </c>
       <c r="E44" s="53"/>
       <c r="F44" s="53"/>
@@ -28316,13 +28350,13 @@
         <v>315</v>
       </c>
       <c r="B45" s="53" t="s">
-        <v>2260</v>
+        <v>2262</v>
       </c>
       <c r="C45" s="48" t="s">
-        <v>2261</v>
+        <v>2263</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>2262</v>
+        <v>2264</v>
       </c>
       <c r="E45" s="53"/>
       <c r="F45" s="53"/>
@@ -28335,13 +28369,13 @@
         <v>315</v>
       </c>
       <c r="B46" s="53" t="s">
-        <v>2263</v>
+        <v>2265</v>
       </c>
       <c r="C46" s="48" t="s">
-        <v>2264</v>
+        <v>2266</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>2265</v>
+        <v>2267</v>
       </c>
       <c r="E46" s="53"/>
       <c r="F46" s="53"/>
@@ -28359,7 +28393,7 @@
       <c r="E47" s="53"/>
       <c r="F47" s="53"/>
       <c r="G47" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="H47" s="53"/>
       <c r="I47" s="53"/>
@@ -28372,10 +28406,10 @@
         <v>1256</v>
       </c>
       <c r="C48" s="51" t="s">
-        <v>2266</v>
+        <v>2268</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>2267</v>
+        <v>2269</v>
       </c>
       <c r="E48" s="53"/>
       <c r="F48" s="53"/>
@@ -28390,13 +28424,13 @@
         <v>220</v>
       </c>
       <c r="B49" s="53" t="s">
-        <v>2268</v>
+        <v>2270</v>
       </c>
       <c r="C49" s="51" t="s">
-        <v>2269</v>
+        <v>2271</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>2270</v>
+        <v>2272</v>
       </c>
       <c r="E49" s="53"/>
       <c r="F49" s="53"/>
@@ -28411,13 +28445,13 @@
         <v>220</v>
       </c>
       <c r="B50" s="53" t="s">
-        <v>2271</v>
+        <v>2273</v>
       </c>
       <c r="C50" s="51" t="s">
-        <v>2272</v>
+        <v>2274</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>2273</v>
+        <v>2275</v>
       </c>
       <c r="E50" s="53"/>
       <c r="F50" s="53"/>
@@ -28433,10 +28467,10 @@
         <v>229</v>
       </c>
       <c r="C51" s="51" t="s">
-        <v>2274</v>
+        <v>2276</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>2275</v>
+        <v>2277</v>
       </c>
       <c r="E51" s="53"/>
       <c r="F51" s="53"/>
@@ -28454,7 +28488,7 @@
       <c r="E52" s="53"/>
       <c r="F52" s="53"/>
       <c r="G52" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="H52" s="53"/>
       <c r="I52" s="53"/>
@@ -28464,13 +28498,13 @@
         <v>226</v>
       </c>
       <c r="B53" s="53" t="s">
-        <v>2276</v>
+        <v>2278</v>
       </c>
       <c r="C53" s="51" t="s">
-        <v>2277</v>
+        <v>2279</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>2278</v>
+        <v>2280</v>
       </c>
       <c r="E53" s="53"/>
       <c r="F53" s="53"/>
@@ -28483,13 +28517,13 @@
         <v>226</v>
       </c>
       <c r="B54" s="53" t="s">
-        <v>2279</v>
+        <v>2281</v>
       </c>
       <c r="C54" s="51" t="s">
-        <v>2280</v>
+        <v>2282</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>2281</v>
+        <v>2283</v>
       </c>
       <c r="E54" s="53"/>
       <c r="F54" s="53"/>
@@ -28502,13 +28536,13 @@
         <v>226</v>
       </c>
       <c r="B55" s="53" t="s">
-        <v>2282</v>
+        <v>2284</v>
       </c>
       <c r="C55" s="51" t="s">
-        <v>2283</v>
+        <v>2285</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>2284</v>
+        <v>2286</v>
       </c>
       <c r="E55" s="53"/>
       <c r="F55" s="53"/>
@@ -28521,13 +28555,13 @@
         <v>226</v>
       </c>
       <c r="B56" s="53" t="s">
-        <v>2285</v>
+        <v>2287</v>
       </c>
       <c r="C56" s="51" t="s">
-        <v>2286</v>
+        <v>2288</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>2287</v>
+        <v>2289</v>
       </c>
       <c r="E56" s="53"/>
       <c r="F56" s="53"/>
@@ -28540,13 +28574,13 @@
         <v>226</v>
       </c>
       <c r="B57" s="53" t="s">
-        <v>2288</v>
+        <v>2290</v>
       </c>
       <c r="C57" s="51" t="s">
-        <v>2289</v>
+        <v>2291</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>2289</v>
+        <v>2291</v>
       </c>
       <c r="E57" s="53"/>
       <c r="F57" s="53"/>
@@ -28559,13 +28593,13 @@
         <v>226</v>
       </c>
       <c r="B58" s="53" t="s">
-        <v>2290</v>
+        <v>2292</v>
       </c>
       <c r="C58" s="51" t="s">
-        <v>2291</v>
+        <v>2293</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>2292</v>
+        <v>2294</v>
       </c>
       <c r="E58" s="53"/>
       <c r="F58" s="53"/>
@@ -28578,13 +28612,13 @@
         <v>226</v>
       </c>
       <c r="B59" s="53" t="s">
-        <v>2293</v>
+        <v>2295</v>
       </c>
       <c r="C59" s="51" t="s">
-        <v>2294</v>
+        <v>2296</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>2295</v>
+        <v>2297</v>
       </c>
       <c r="E59" s="53"/>
       <c r="F59" s="53"/>
@@ -28597,13 +28631,13 @@
         <v>226</v>
       </c>
       <c r="B60" s="53" t="s">
-        <v>2296</v>
+        <v>2298</v>
       </c>
       <c r="C60" s="51" t="s">
-        <v>2297</v>
+        <v>2299</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>2298</v>
+        <v>2300</v>
       </c>
       <c r="E60" s="53"/>
       <c r="F60" s="53"/>
@@ -28631,13 +28665,13 @@
         <v>226</v>
       </c>
       <c r="B62" s="53" t="s">
-        <v>2299</v>
+        <v>2301</v>
       </c>
       <c r="C62" s="51" t="s">
-        <v>2300</v>
+        <v>2302</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>2301</v>
+        <v>2303</v>
       </c>
       <c r="E62" s="53"/>
       <c r="F62" s="53"/>
@@ -28655,7 +28689,7 @@
       <c r="E63" s="53"/>
       <c r="F63" s="53"/>
       <c r="G63" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="H63" s="53"/>
       <c r="I63" s="53"/>
@@ -28668,10 +28702,10 @@
         <v>1167</v>
       </c>
       <c r="C64" s="51" t="s">
-        <v>2302</v>
+        <v>2304</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>2303</v>
+        <v>2305</v>
       </c>
       <c r="E64" s="53"/>
       <c r="F64" s="53"/>
@@ -28687,14 +28721,14 @@
         <v>1199</v>
       </c>
       <c r="C65" s="53" t="s">
-        <v>2304</v>
+        <v>2306</v>
       </c>
       <c r="D65" s="53" t="s">
-        <v>2305</v>
+        <v>2307</v>
       </c>
       <c r="E65" s="53"/>
       <c r="F65" s="53" t="s">
-        <v>2306</v>
+        <v>2308</v>
       </c>
       <c r="G65" s="53"/>
       <c r="H65" s="53"/>
@@ -28708,14 +28742,14 @@
         <v>1200</v>
       </c>
       <c r="C66" s="53" t="s">
-        <v>2307</v>
+        <v>2309</v>
       </c>
       <c r="D66" s="53" t="s">
-        <v>2308</v>
+        <v>2310</v>
       </c>
       <c r="E66" s="53"/>
       <c r="F66" s="53" t="s">
-        <v>2309</v>
+        <v>2311</v>
       </c>
       <c r="G66" s="53"/>
       <c r="H66" s="53"/>
@@ -28726,17 +28760,17 @@
         <v>322</v>
       </c>
       <c r="B67" s="53" t="s">
-        <v>2310</v>
+        <v>2312</v>
       </c>
       <c r="C67" s="53" t="s">
-        <v>2311</v>
+        <v>2313</v>
       </c>
       <c r="D67" s="53" t="s">
-        <v>2312</v>
+        <v>2314</v>
       </c>
       <c r="E67" s="53"/>
       <c r="F67" s="53" t="s">
-        <v>2313</v>
+        <v>2315</v>
       </c>
       <c r="G67" s="53"/>
       <c r="H67" s="53"/>
@@ -28750,14 +28784,14 @@
         <v>1201</v>
       </c>
       <c r="C68" s="53" t="s">
-        <v>2314</v>
+        <v>2316</v>
       </c>
       <c r="D68" s="53" t="s">
-        <v>2315</v>
+        <v>2317</v>
       </c>
       <c r="E68" s="53"/>
       <c r="F68" s="53" t="s">
-        <v>2316</v>
+        <v>2318</v>
       </c>
       <c r="G68" s="53"/>
       <c r="H68" s="53"/>
@@ -28771,14 +28805,14 @@
         <v>1215</v>
       </c>
       <c r="C69" s="53" t="s">
-        <v>2317</v>
+        <v>2319</v>
       </c>
       <c r="D69" s="53" t="s">
-        <v>2318</v>
+        <v>2320</v>
       </c>
       <c r="E69" s="53"/>
       <c r="F69" s="53" t="s">
-        <v>2319</v>
+        <v>2321</v>
       </c>
       <c r="G69" s="53"/>
       <c r="H69" s="53"/>
@@ -28789,13 +28823,13 @@
         <v>905</v>
       </c>
       <c r="B70" s="66" t="s">
-        <v>2320</v>
+        <v>2322</v>
       </c>
       <c r="C70" s="66" t="s">
-        <v>2321</v>
+        <v>2323</v>
       </c>
       <c r="D70" s="66" t="s">
-        <v>2322</v>
+        <v>2324</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28803,13 +28837,13 @@
         <v>905</v>
       </c>
       <c r="B71" s="66" t="s">
-        <v>2323</v>
+        <v>2325</v>
       </c>
       <c r="C71" s="66" t="s">
-        <v>2324</v>
+        <v>2326</v>
       </c>
       <c r="D71" s="66" t="s">
-        <v>2325</v>
+        <v>2327</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28817,13 +28851,13 @@
         <v>905</v>
       </c>
       <c r="B72" s="66" t="s">
-        <v>2326</v>
+        <v>2328</v>
       </c>
       <c r="C72" s="66" t="s">
-        <v>2327</v>
+        <v>2329</v>
       </c>
       <c r="D72" s="66" t="s">
-        <v>2328</v>
+        <v>2330</v>
       </c>
     </row>
     <row r="73" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28831,13 +28865,13 @@
         <v>905</v>
       </c>
       <c r="B73" s="66" t="s">
-        <v>2329</v>
+        <v>2331</v>
       </c>
       <c r="C73" s="66" t="s">
-        <v>2330</v>
+        <v>2332</v>
       </c>
       <c r="D73" s="66" t="s">
-        <v>2331</v>
+        <v>2333</v>
       </c>
       <c r="E73" s="66"/>
       <c r="F73" s="66"/>
@@ -28850,13 +28884,13 @@
         <v>1079</v>
       </c>
       <c r="B74" s="53" t="s">
-        <v>2332</v>
+        <v>2334</v>
       </c>
       <c r="C74" s="51" t="s">
-        <v>2333</v>
+        <v>2335</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>2334</v>
+        <v>2336</v>
       </c>
       <c r="E74" s="51"/>
       <c r="F74" s="51"/>
@@ -28869,13 +28903,13 @@
         <v>1079</v>
       </c>
       <c r="B75" s="53" t="s">
-        <v>2335</v>
+        <v>2337</v>
       </c>
       <c r="C75" s="51" t="s">
-        <v>2336</v>
+        <v>2338</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>2337</v>
+        <v>2339</v>
       </c>
       <c r="E75" s="51"/>
       <c r="F75" s="51"/>
@@ -28888,13 +28922,13 @@
         <v>1079</v>
       </c>
       <c r="B76" s="53" t="s">
-        <v>2338</v>
+        <v>2340</v>
       </c>
       <c r="C76" s="51" t="s">
-        <v>2339</v>
+        <v>2341</v>
       </c>
       <c r="D76" s="8" t="s">
-        <v>2340</v>
+        <v>2342</v>
       </c>
       <c r="E76" s="51"/>
       <c r="F76" s="51"/>
@@ -28907,13 +28941,13 @@
         <v>1079</v>
       </c>
       <c r="B77" s="53" t="s">
-        <v>2341</v>
+        <v>2343</v>
       </c>
       <c r="C77" s="51" t="s">
-        <v>2342</v>
+        <v>2344</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>2343</v>
+        <v>2345</v>
       </c>
       <c r="E77" s="51"/>
       <c r="F77" s="51"/>
@@ -28926,13 +28960,13 @@
         <v>1079</v>
       </c>
       <c r="B78" s="53" t="s">
-        <v>2344</v>
+        <v>2346</v>
       </c>
       <c r="C78" s="51" t="s">
-        <v>2345</v>
+        <v>2347</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>2346</v>
+        <v>2348</v>
       </c>
       <c r="E78" s="51"/>
       <c r="F78" s="51"/>
@@ -28945,13 +28979,13 @@
         <v>1079</v>
       </c>
       <c r="B79" s="53" t="s">
-        <v>2347</v>
+        <v>2349</v>
       </c>
       <c r="C79" s="51" t="s">
-        <v>2348</v>
+        <v>2350</v>
       </c>
       <c r="D79" s="8" t="s">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="E79" s="51"/>
       <c r="F79" s="51"/>
@@ -28964,13 +28998,13 @@
         <v>1079</v>
       </c>
       <c r="B80" s="53" t="s">
-        <v>2350</v>
+        <v>2352</v>
       </c>
       <c r="C80" s="51" t="s">
-        <v>2351</v>
+        <v>2353</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>2352</v>
+        <v>2354</v>
       </c>
       <c r="E80" s="51"/>
       <c r="F80" s="51"/>
@@ -28983,13 +29017,13 @@
         <v>1079</v>
       </c>
       <c r="B81" s="53" t="s">
-        <v>2353</v>
+        <v>2355</v>
       </c>
       <c r="C81" s="51" t="s">
-        <v>2354</v>
+        <v>2356</v>
       </c>
       <c r="D81" s="8" t="s">
-        <v>2355</v>
+        <v>2357</v>
       </c>
       <c r="E81" s="51"/>
       <c r="F81" s="51"/>
@@ -29002,13 +29036,13 @@
         <v>1079</v>
       </c>
       <c r="B82" s="53" t="s">
-        <v>2356</v>
+        <v>2358</v>
       </c>
       <c r="C82" s="51" t="s">
-        <v>2357</v>
+        <v>2359</v>
       </c>
       <c r="D82" s="8" t="s">
-        <v>2358</v>
+        <v>2360</v>
       </c>
       <c r="E82" s="51"/>
       <c r="F82" s="51"/>
@@ -29021,13 +29055,13 @@
         <v>1079</v>
       </c>
       <c r="B83" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="C83" s="51" t="s">
-        <v>2199</v>
+        <v>2201</v>
       </c>
       <c r="D83" s="8" t="s">
-        <v>2200</v>
+        <v>2202</v>
       </c>
       <c r="E83" s="51"/>
       <c r="F83" s="51"/>
@@ -29040,13 +29074,13 @@
         <v>1079</v>
       </c>
       <c r="B84" s="53" t="s">
-        <v>2359</v>
+        <v>2361</v>
       </c>
       <c r="C84" s="51" t="s">
-        <v>2201</v>
+        <v>2203</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>2360</v>
+        <v>2362</v>
       </c>
       <c r="E84" s="51"/>
       <c r="F84" s="51"/>
@@ -29059,13 +29093,13 @@
         <v>99</v>
       </c>
       <c r="B85" s="66" t="s">
-        <v>2361</v>
+        <v>2363</v>
       </c>
       <c r="C85" s="66" t="s">
-        <v>2362</v>
+        <v>2364</v>
       </c>
       <c r="D85" s="66" t="s">
-        <v>2363</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29073,13 +29107,13 @@
         <v>99</v>
       </c>
       <c r="B86" s="66" t="s">
-        <v>2364</v>
+        <v>2366</v>
       </c>
       <c r="C86" s="66" t="s">
-        <v>2365</v>
+        <v>2367</v>
       </c>
       <c r="D86" s="66" t="s">
-        <v>2366</v>
+        <v>2368</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29104,10 +29138,10 @@
         <v>1171</v>
       </c>
       <c r="C88" s="66" t="s">
-        <v>2201</v>
+        <v>2203</v>
       </c>
       <c r="D88" s="66" t="s">
-        <v>2360</v>
+        <v>2362</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29115,13 +29149,13 @@
         <v>423</v>
       </c>
       <c r="B89" s="53" t="s">
-        <v>2367</v>
+        <v>2369</v>
       </c>
       <c r="C89" s="51" t="s">
-        <v>2368</v>
+        <v>2370</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>2369</v>
+        <v>2371</v>
       </c>
       <c r="E89" s="51"/>
       <c r="F89" s="51"/>
@@ -29136,13 +29170,13 @@
         <v>423</v>
       </c>
       <c r="B90" s="53" t="s">
-        <v>2370</v>
+        <v>2372</v>
       </c>
       <c r="C90" s="51" t="s">
-        <v>2371</v>
+        <v>2373</v>
       </c>
       <c r="D90" s="8" t="s">
-        <v>2372</v>
+        <v>2374</v>
       </c>
       <c r="E90" s="51"/>
       <c r="F90" s="51"/>
@@ -29157,13 +29191,13 @@
         <v>423</v>
       </c>
       <c r="B91" s="53" t="s">
-        <v>2373</v>
+        <v>2375</v>
       </c>
       <c r="C91" s="51" t="s">
-        <v>2374</v>
+        <v>2376</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>2375</v>
+        <v>2377</v>
       </c>
       <c r="E91" s="51"/>
       <c r="F91" s="51"/>
@@ -29176,13 +29210,13 @@
         <v>423</v>
       </c>
       <c r="B92" s="53" t="s">
-        <v>2376</v>
+        <v>2378</v>
       </c>
       <c r="C92" s="51" t="s">
-        <v>2377</v>
+        <v>2379</v>
       </c>
       <c r="D92" s="8" t="s">
-        <v>2378</v>
+        <v>2380</v>
       </c>
       <c r="E92" s="51"/>
       <c r="F92" s="51"/>
@@ -29195,13 +29229,13 @@
         <v>423</v>
       </c>
       <c r="B93" s="53" t="s">
-        <v>2379</v>
+        <v>2381</v>
       </c>
       <c r="C93" s="51" t="s">
-        <v>2380</v>
+        <v>2382</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>2381</v>
+        <v>2383</v>
       </c>
       <c r="E93" s="51"/>
       <c r="F93" s="51"/>
@@ -29217,10 +29251,10 @@
         <v>1232</v>
       </c>
       <c r="C94" s="51" t="s">
-        <v>2382</v>
+        <v>2384</v>
       </c>
       <c r="D94" s="8" t="s">
-        <v>2383</v>
+        <v>2385</v>
       </c>
       <c r="E94" s="51"/>
       <c r="F94" s="51"/>
@@ -29238,10 +29272,10 @@
         <v>1233</v>
       </c>
       <c r="C95" s="51" t="s">
-        <v>2384</v>
+        <v>2386</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>2385</v>
+        <v>2387</v>
       </c>
       <c r="E95" s="51"/>
       <c r="F95" s="51"/>
@@ -29254,13 +29288,13 @@
         <v>423</v>
       </c>
       <c r="B96" s="53" t="s">
-        <v>2386</v>
+        <v>2388</v>
       </c>
       <c r="C96" s="51" t="s">
-        <v>2387</v>
+        <v>2389</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>2388</v>
+        <v>2390</v>
       </c>
       <c r="E96" s="51"/>
       <c r="F96" s="51"/>
@@ -29291,10 +29325,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="93" t="s">
-        <v>2389</v>
+        <v>2391</v>
       </c>
       <c r="B98" s="66" t="s">
-        <v>2390</v>
+        <v>2392</v>
       </c>
       <c r="C98" s="66" t="s">
         <v>1752</v>
@@ -29311,10 +29345,10 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="93" t="s">
-        <v>2389</v>
+        <v>2391</v>
       </c>
       <c r="B99" s="66" t="s">
-        <v>2391</v>
+        <v>2393</v>
       </c>
       <c r="C99" s="66" t="s">
         <v>1757</v>
@@ -29331,16 +29365,16 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="93" t="s">
-        <v>2389</v>
+        <v>2391</v>
       </c>
       <c r="B100" s="66" t="s">
         <v>1225</v>
       </c>
       <c r="C100" s="66" t="s">
-        <v>2193</v>
+        <v>2195</v>
       </c>
       <c r="D100" s="66" t="s">
-        <v>2194</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29348,13 +29382,13 @@
         <v>771</v>
       </c>
       <c r="B101" s="66" t="s">
-        <v>2392</v>
+        <v>2394</v>
       </c>
       <c r="C101" s="66" t="s">
-        <v>2393</v>
+        <v>2395</v>
       </c>
       <c r="D101" s="66" t="s">
-        <v>2394</v>
+        <v>2396</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29362,13 +29396,13 @@
         <v>771</v>
       </c>
       <c r="B102" s="66" t="s">
-        <v>2395</v>
+        <v>2397</v>
       </c>
       <c r="C102" s="66" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="D102" s="66" t="s">
-        <v>2397</v>
+        <v>2399</v>
       </c>
       <c r="I102" s="90" t="n">
         <f aca="false">TRUE()</f>
@@ -29380,13 +29414,13 @@
         <v>771</v>
       </c>
       <c r="B103" s="66" t="s">
-        <v>2398</v>
+        <v>2400</v>
       </c>
       <c r="C103" s="66" t="s">
-        <v>2399</v>
+        <v>2401</v>
       </c>
       <c r="D103" s="66" t="s">
-        <v>2400</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29394,13 +29428,13 @@
         <v>771</v>
       </c>
       <c r="B104" s="66" t="s">
-        <v>2401</v>
+        <v>2403</v>
       </c>
       <c r="C104" s="66" t="s">
-        <v>2402</v>
+        <v>2404</v>
       </c>
       <c r="D104" s="66" t="s">
-        <v>2403</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29408,7 +29442,7 @@
         <v>771</v>
       </c>
       <c r="G105" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29416,7 +29450,7 @@
         <v>771</v>
       </c>
       <c r="G106" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29424,13 +29458,13 @@
         <v>829</v>
       </c>
       <c r="B107" s="66" t="s">
-        <v>2404</v>
+        <v>2406</v>
       </c>
       <c r="C107" s="66" t="s">
-        <v>2405</v>
+        <v>2407</v>
       </c>
       <c r="D107" s="66" t="s">
-        <v>2406</v>
+        <v>2408</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29438,13 +29472,13 @@
         <v>829</v>
       </c>
       <c r="B108" s="66" t="s">
-        <v>2407</v>
+        <v>2409</v>
       </c>
       <c r="C108" s="66" t="s">
-        <v>2408</v>
+        <v>2410</v>
       </c>
       <c r="D108" s="66" t="s">
-        <v>2409</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29452,13 +29486,13 @@
         <v>829</v>
       </c>
       <c r="B109" s="66" t="s">
-        <v>2398</v>
+        <v>2400</v>
       </c>
       <c r="C109" s="66" t="s">
-        <v>2410</v>
+        <v>2412</v>
       </c>
       <c r="D109" s="66" t="s">
-        <v>2411</v>
+        <v>2413</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29466,13 +29500,13 @@
         <v>829</v>
       </c>
       <c r="B110" s="53" t="s">
-        <v>2412</v>
+        <v>2414</v>
       </c>
       <c r="C110" s="51" t="s">
-        <v>2413</v>
+        <v>2415</v>
       </c>
       <c r="D110" s="48" t="s">
-        <v>2414</v>
+        <v>2416</v>
       </c>
       <c r="I110" s="90" t="n">
         <f aca="false">TRUE()</f>
@@ -29484,7 +29518,7 @@
         <v>829</v>
       </c>
       <c r="G111" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29492,7 +29526,7 @@
         <v>829</v>
       </c>
       <c r="G112" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29500,13 +29534,13 @@
         <v>347</v>
       </c>
       <c r="B113" s="66" t="s">
-        <v>2415</v>
+        <v>2417</v>
       </c>
       <c r="C113" s="66" t="s">
-        <v>2416</v>
+        <v>2418</v>
       </c>
       <c r="D113" s="66" t="s">
-        <v>2417</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29514,13 +29548,13 @@
         <v>347</v>
       </c>
       <c r="B114" s="66" t="s">
-        <v>2418</v>
+        <v>2420</v>
       </c>
       <c r="C114" s="66" t="s">
-        <v>2419</v>
+        <v>2421</v>
       </c>
       <c r="D114" s="66" t="s">
-        <v>2420</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29528,13 +29562,13 @@
         <v>347</v>
       </c>
       <c r="B115" s="66" t="s">
-        <v>2421</v>
+        <v>2423</v>
       </c>
       <c r="C115" s="66" t="s">
-        <v>2422</v>
+        <v>2424</v>
       </c>
       <c r="D115" s="66" t="s">
-        <v>2423</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29547,103 +29581,103 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="89" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="B117" s="53" t="s">
         <v>1199</v>
       </c>
       <c r="C117" s="53" t="s">
-        <v>2425</v>
+        <v>2427</v>
       </c>
       <c r="D117" s="53" t="s">
-        <v>2426</v>
+        <v>2428</v>
       </c>
       <c r="E117" s="53" t="s">
-        <v>2427</v>
+        <v>2429</v>
       </c>
       <c r="F117" s="53" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
       <c r="G117" s="89"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="89" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="B118" s="53" t="s">
         <v>1200</v>
       </c>
       <c r="C118" s="53" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
       <c r="D118" s="53" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
       <c r="E118" s="53" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
       <c r="F118" s="53" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="89" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="B119" s="53" t="s">
         <v>1201</v>
       </c>
       <c r="C119" s="53" t="s">
-        <v>2433</v>
+        <v>2435</v>
       </c>
       <c r="D119" s="53" t="s">
-        <v>2434</v>
+        <v>2436</v>
       </c>
       <c r="E119" s="53" t="s">
-        <v>2435</v>
+        <v>2437</v>
       </c>
       <c r="F119" s="53" t="s">
-        <v>2436</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="89" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="B120" s="53" t="s">
         <v>1215</v>
       </c>
       <c r="C120" s="53" t="s">
-        <v>2437</v>
+        <v>2439</v>
       </c>
       <c r="D120" s="53" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
       <c r="E120" s="53" t="s">
-        <v>2439</v>
+        <v>2441</v>
       </c>
       <c r="F120" s="53" t="s">
-        <v>2440</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="89" t="s">
-        <v>2424</v>
+        <v>2426</v>
       </c>
       <c r="B121" s="53" t="s">
-        <v>2310</v>
+        <v>2312</v>
       </c>
       <c r="C121" s="53" t="s">
-        <v>2441</v>
+        <v>2443</v>
       </c>
       <c r="D121" s="53" t="s">
-        <v>2442</v>
+        <v>2444</v>
       </c>
       <c r="E121" s="53" t="s">
-        <v>2443</v>
+        <v>2445</v>
       </c>
       <c r="F121" s="53" t="s">
-        <v>2444</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29651,7 +29685,7 @@
         <v>698</v>
       </c>
       <c r="B122" s="66" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="C122" s="8" t="s">
         <v>1923</v>
@@ -29668,10 +29702,10 @@
         <v>1237</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="D123" s="57" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="H123" s="95" t="s">
         <v>1235</v>
@@ -29682,16 +29716,16 @@
         <v>698</v>
       </c>
       <c r="B124" s="66" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
       <c r="D124" s="57" t="s">
-        <v>2449</v>
+        <v>2451</v>
       </c>
       <c r="H124" s="96" t="s">
-        <v>2450</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29699,7 +29733,7 @@
         <v>698</v>
       </c>
       <c r="B125" s="66" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>1940</v>
@@ -29716,7 +29750,7 @@
         <v>698</v>
       </c>
       <c r="B126" s="66" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="C126" s="8" t="s">
         <v>1937</v>
@@ -29740,7 +29774,7 @@
         <v>704</v>
       </c>
       <c r="B128" s="66" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="C128" s="8" t="s">
         <v>1923</v>
@@ -29754,7 +29788,7 @@
         <v>704</v>
       </c>
       <c r="B129" s="66" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="C129" s="8" t="s">
         <v>1926</v>
@@ -29768,7 +29802,7 @@
         <v>704</v>
       </c>
       <c r="B130" s="66" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="C130" s="8" t="s">
         <v>1940</v>
@@ -29785,7 +29819,7 @@
         <v>704</v>
       </c>
       <c r="B131" s="66" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="C131" s="8" t="s">
         <v>1937</v>
@@ -29799,13 +29833,13 @@
         <v>704</v>
       </c>
       <c r="B132" s="66" t="s">
-        <v>2454</v>
+        <v>2456</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>2455</v>
+        <v>2457</v>
       </c>
       <c r="D132" s="57" t="s">
-        <v>2456</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29813,7 +29847,7 @@
         <v>704</v>
       </c>
       <c r="B133" s="66" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="C133" s="8" t="s">
         <v>2055</v>
@@ -29829,7 +29863,7 @@
       <c r="C134" s="57"/>
       <c r="D134" s="57"/>
       <c r="G134" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29837,16 +29871,16 @@
         <v>594</v>
       </c>
       <c r="B135" s="66" t="s">
-        <v>2458</v>
+        <v>2460</v>
       </c>
       <c r="C135" s="57" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="D135" s="57" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="H135" s="54" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29857,13 +29891,13 @@
         <v>1225</v>
       </c>
       <c r="C136" s="57" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="D136" s="57" t="s">
-        <v>2463</v>
+        <v>2465</v>
       </c>
       <c r="H136" s="8" t="s">
-        <v>2464</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29874,10 +29908,10 @@
         <v>1167</v>
       </c>
       <c r="C137" s="57" t="s">
-        <v>2465</v>
+        <v>2467</v>
       </c>
       <c r="D137" s="57" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29885,13 +29919,13 @@
         <v>594</v>
       </c>
       <c r="B138" s="66" t="s">
-        <v>2467</v>
+        <v>2469</v>
       </c>
       <c r="C138" s="57" t="s">
-        <v>2468</v>
+        <v>2470</v>
       </c>
       <c r="D138" s="57" t="s">
-        <v>2469</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29901,7 +29935,7 @@
       <c r="C139" s="57"/>
       <c r="D139" s="57"/>
       <c r="G139" s="66" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29909,13 +29943,13 @@
         <v>627</v>
       </c>
       <c r="B140" s="66" t="s">
-        <v>2470</v>
+        <v>2472</v>
       </c>
       <c r="C140" s="57" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="D140" s="57" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29923,13 +29957,13 @@
         <v>627</v>
       </c>
       <c r="B141" s="66" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="C141" s="57" t="s">
-        <v>2473</v>
+        <v>2475</v>
       </c>
       <c r="D141" s="57" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29939,7 +29973,7 @@
       <c r="C142" s="57"/>
       <c r="D142" s="57"/>
       <c r="G142" s="66" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29947,13 +29981,13 @@
         <v>651</v>
       </c>
       <c r="B143" s="66" t="s">
-        <v>2475</v>
+        <v>2477</v>
       </c>
       <c r="C143" s="8" t="s">
-        <v>2476</v>
+        <v>2478</v>
       </c>
       <c r="D143" s="57" t="s">
-        <v>2477</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29961,13 +29995,13 @@
         <v>651</v>
       </c>
       <c r="B144" s="66" t="s">
-        <v>2478</v>
+        <v>2480</v>
       </c>
       <c r="C144" s="8" t="s">
-        <v>2479</v>
+        <v>2481</v>
       </c>
       <c r="D144" s="57" t="s">
-        <v>2480</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29977,7 +30011,7 @@
       <c r="C145" s="57"/>
       <c r="D145" s="57"/>
       <c r="G145" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29987,7 +30021,7 @@
       <c r="C146" s="57"/>
       <c r="D146" s="57"/>
       <c r="G146" s="66" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29995,13 +30029,13 @@
         <v>658</v>
       </c>
       <c r="B147" s="66" t="s">
-        <v>2481</v>
+        <v>2483</v>
       </c>
       <c r="C147" s="8" t="s">
-        <v>2482</v>
+        <v>2484</v>
       </c>
       <c r="D147" s="57" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30009,13 +30043,13 @@
         <v>658</v>
       </c>
       <c r="B148" s="66" t="s">
-        <v>2484</v>
+        <v>2486</v>
       </c>
       <c r="C148" s="8" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
       <c r="D148" s="57" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30023,13 +30057,13 @@
         <v>658</v>
       </c>
       <c r="B149" s="66" t="s">
-        <v>2486</v>
+        <v>2488</v>
       </c>
       <c r="C149" s="8" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
       <c r="D149" s="8" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30037,13 +30071,13 @@
         <v>658</v>
       </c>
       <c r="B150" s="66" t="s">
-        <v>2488</v>
+        <v>2490</v>
       </c>
       <c r="C150" s="8" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
       <c r="D150" s="8" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30053,7 +30087,7 @@
       <c r="C151" s="57"/>
       <c r="D151" s="57"/>
       <c r="G151" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30063,7 +30097,7 @@
       <c r="C152" s="57"/>
       <c r="D152" s="57"/>
       <c r="G152" s="66" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30071,13 +30105,13 @@
         <v>663</v>
       </c>
       <c r="B153" s="66" t="s">
-        <v>2490</v>
+        <v>2492</v>
       </c>
       <c r="C153" s="8" t="s">
-        <v>2491</v>
+        <v>2493</v>
       </c>
       <c r="D153" s="57" t="s">
-        <v>2492</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30085,13 +30119,13 @@
         <v>663</v>
       </c>
       <c r="B154" s="66" t="s">
-        <v>2493</v>
+        <v>2495</v>
       </c>
       <c r="C154" s="8" t="s">
-        <v>2494</v>
+        <v>2496</v>
       </c>
       <c r="D154" s="57" t="s">
-        <v>2495</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30099,13 +30133,13 @@
         <v>663</v>
       </c>
       <c r="B155" s="66" t="s">
-        <v>2475</v>
+        <v>2477</v>
       </c>
       <c r="C155" s="8" t="s">
-        <v>2496</v>
+        <v>2498</v>
       </c>
       <c r="D155" s="57" t="s">
-        <v>2497</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30113,13 +30147,13 @@
         <v>663</v>
       </c>
       <c r="B156" s="66" t="s">
-        <v>2498</v>
+        <v>2500</v>
       </c>
       <c r="C156" s="8" t="s">
-        <v>2499</v>
+        <v>2501</v>
       </c>
       <c r="D156" s="8" t="s">
-        <v>2499</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30127,13 +30161,13 @@
         <v>663</v>
       </c>
       <c r="B157" s="66" t="s">
-        <v>2500</v>
+        <v>2502</v>
       </c>
       <c r="C157" s="8" t="s">
-        <v>2501</v>
+        <v>2503</v>
       </c>
       <c r="D157" s="57" t="s">
-        <v>2502</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30143,7 +30177,7 @@
       <c r="C158" s="57"/>
       <c r="D158" s="57"/>
       <c r="G158" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30153,7 +30187,7 @@
       <c r="C159" s="57"/>
       <c r="D159" s="57"/>
       <c r="G159" s="66" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30161,7 +30195,7 @@
         <v>793</v>
       </c>
       <c r="B160" s="53" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="C160" s="66" t="s">
         <v>1994</v>
@@ -30180,7 +30214,7 @@
         <v>793</v>
       </c>
       <c r="B161" s="53" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="C161" s="66" t="s">
         <v>2012</v>
@@ -30199,13 +30233,13 @@
         <v>793</v>
       </c>
       <c r="B162" s="53" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>2503</v>
+        <v>2505</v>
       </c>
       <c r="D162" s="57" t="s">
-        <v>2504</v>
+        <v>2506</v>
       </c>
       <c r="E162" s="53"/>
       <c r="F162" s="53"/>
@@ -30218,7 +30252,7 @@
         <v>793</v>
       </c>
       <c r="B163" s="53" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="C163" s="8" t="s">
         <v>1947</v>
@@ -30237,7 +30271,7 @@
         <v>793</v>
       </c>
       <c r="B164" s="53" t="s">
-        <v>2505</v>
+        <v>2507</v>
       </c>
       <c r="C164" s="8" t="s">
         <v>1950</v>
@@ -30259,10 +30293,10 @@
         <v>229</v>
       </c>
       <c r="C165" s="51" t="s">
-        <v>2506</v>
+        <v>2508</v>
       </c>
       <c r="D165" s="8" t="s">
-        <v>2507</v>
+        <v>2509</v>
       </c>
       <c r="E165" s="53"/>
       <c r="F165" s="53"/>
@@ -30277,13 +30311,13 @@
         <v>793</v>
       </c>
       <c r="B166" s="53" t="s">
-        <v>2508</v>
+        <v>2510</v>
       </c>
       <c r="C166" s="51" t="s">
-        <v>2509</v>
+        <v>2511</v>
       </c>
       <c r="D166" s="8" t="s">
-        <v>2510</v>
+        <v>2512</v>
       </c>
       <c r="E166" s="53"/>
       <c r="F166" s="53"/>
@@ -30298,13 +30332,13 @@
         <v>141</v>
       </c>
       <c r="B167" s="53" t="s">
-        <v>2511</v>
+        <v>2513</v>
       </c>
       <c r="C167" s="51" t="s">
-        <v>2512</v>
+        <v>2514</v>
       </c>
       <c r="D167" s="8" t="s">
-        <v>2513</v>
+        <v>2515</v>
       </c>
       <c r="E167" s="53"/>
       <c r="F167" s="53"/>
@@ -30317,13 +30351,13 @@
         <v>141</v>
       </c>
       <c r="B168" s="53" t="s">
-        <v>2514</v>
+        <v>2516</v>
       </c>
       <c r="C168" s="51" t="s">
-        <v>2515</v>
+        <v>2517</v>
       </c>
       <c r="D168" s="8" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
       <c r="E168" s="53"/>
       <c r="F168" s="53"/>
@@ -30339,10 +30373,10 @@
         <v>1167</v>
       </c>
       <c r="C169" s="51" t="s">
-        <v>2517</v>
+        <v>2519</v>
       </c>
       <c r="D169" s="8" t="s">
-        <v>2518</v>
+        <v>2520</v>
       </c>
       <c r="E169" s="53"/>
       <c r="F169" s="53"/>
@@ -30358,10 +30392,10 @@
         <v>1225</v>
       </c>
       <c r="C170" s="51" t="s">
-        <v>2519</v>
+        <v>2521</v>
       </c>
       <c r="D170" s="8" t="s">
-        <v>2520</v>
+        <v>2522</v>
       </c>
       <c r="E170" s="53"/>
       <c r="F170" s="53"/>
@@ -30379,7 +30413,7 @@
       <c r="E171" s="53"/>
       <c r="F171" s="53"/>
       <c r="G171" s="53" t="s">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="H171" s="53"/>
       <c r="I171" s="53"/>
@@ -30389,13 +30423,13 @@
         <v>246</v>
       </c>
       <c r="B172" s="53" t="s">
-        <v>2521</v>
+        <v>2523</v>
       </c>
       <c r="C172" s="48" t="s">
-        <v>2522</v>
+        <v>2524</v>
       </c>
       <c r="D172" s="8" t="s">
-        <v>2523</v>
+        <v>2525</v>
       </c>
       <c r="E172" s="53"/>
       <c r="F172" s="53"/>
@@ -30410,13 +30444,13 @@
         <v>246</v>
       </c>
       <c r="B173" s="53" t="s">
-        <v>2524</v>
+        <v>2526</v>
       </c>
       <c r="C173" s="48" t="s">
-        <v>2525</v>
+        <v>2527</v>
       </c>
       <c r="D173" s="8" t="s">
-        <v>2526</v>
+        <v>2528</v>
       </c>
       <c r="E173" s="53"/>
       <c r="F173" s="53"/>
@@ -30431,13 +30465,13 @@
         <v>246</v>
       </c>
       <c r="B174" s="53" t="s">
-        <v>2527</v>
+        <v>2529</v>
       </c>
       <c r="C174" s="48" t="s">
-        <v>2528</v>
+        <v>2530</v>
       </c>
       <c r="D174" s="8" t="s">
-        <v>2529</v>
+        <v>2531</v>
       </c>
       <c r="E174" s="53"/>
       <c r="F174" s="53"/>
@@ -30452,13 +30486,13 @@
         <v>246</v>
       </c>
       <c r="B175" s="53" t="s">
-        <v>2530</v>
+        <v>2532</v>
       </c>
       <c r="C175" s="48" t="s">
-        <v>2531</v>
+        <v>2533</v>
       </c>
       <c r="D175" s="8" t="s">
-        <v>2532</v>
+        <v>2534</v>
       </c>
       <c r="E175" s="53"/>
       <c r="F175" s="53"/>
@@ -30473,13 +30507,13 @@
         <v>246</v>
       </c>
       <c r="B176" s="53" t="s">
-        <v>2533</v>
+        <v>2535</v>
       </c>
       <c r="C176" s="48" t="s">
-        <v>2534</v>
+        <v>2536</v>
       </c>
       <c r="D176" s="8" t="s">
-        <v>2535</v>
+        <v>2537</v>
       </c>
       <c r="E176" s="53"/>
       <c r="F176" s="53"/>
@@ -30494,13 +30528,13 @@
         <v>246</v>
       </c>
       <c r="B177" s="53" t="s">
-        <v>2536</v>
+        <v>2538</v>
       </c>
       <c r="C177" s="48" t="s">
-        <v>2537</v>
+        <v>2539</v>
       </c>
       <c r="D177" s="8" t="s">
-        <v>2538</v>
+        <v>2540</v>
       </c>
       <c r="E177" s="53"/>
       <c r="F177" s="53"/>
@@ -30515,13 +30549,13 @@
         <v>246</v>
       </c>
       <c r="B178" s="53" t="s">
-        <v>2539</v>
+        <v>2541</v>
       </c>
       <c r="C178" s="48" t="s">
-        <v>2540</v>
+        <v>2542</v>
       </c>
       <c r="D178" s="8" t="s">
-        <v>2541</v>
+        <v>2543</v>
       </c>
       <c r="E178" s="53"/>
       <c r="F178" s="53"/>
@@ -30536,13 +30570,13 @@
         <v>246</v>
       </c>
       <c r="B179" s="53" t="s">
-        <v>2542</v>
+        <v>2544</v>
       </c>
       <c r="C179" s="48" t="s">
-        <v>2543</v>
+        <v>2545</v>
       </c>
       <c r="D179" s="8" t="s">
-        <v>2544</v>
+        <v>2546</v>
       </c>
       <c r="E179" s="53"/>
       <c r="F179" s="53"/>
@@ -30557,13 +30591,13 @@
         <v>246</v>
       </c>
       <c r="B180" s="53" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="C180" s="48" t="s">
-        <v>2546</v>
+        <v>2548</v>
       </c>
       <c r="D180" s="8" t="s">
-        <v>2547</v>
+        <v>2549</v>
       </c>
       <c r="E180" s="53"/>
       <c r="F180" s="53"/>
@@ -30581,10 +30615,10 @@
         <v>229</v>
       </c>
       <c r="C181" s="48" t="s">
-        <v>2195</v>
+        <v>2197</v>
       </c>
       <c r="D181" s="8" t="s">
-        <v>2196</v>
+        <v>2198</v>
       </c>
       <c r="E181" s="53"/>
       <c r="F181" s="53"/>
@@ -30614,13 +30648,13 @@
         <v>258</v>
       </c>
       <c r="B183" s="53" t="s">
-        <v>2548</v>
+        <v>2550</v>
       </c>
       <c r="C183" s="48" t="s">
-        <v>2549</v>
+        <v>2551</v>
       </c>
       <c r="D183" s="8" t="s">
-        <v>2550</v>
+        <v>2552</v>
       </c>
       <c r="E183" s="53"/>
       <c r="F183" s="53"/>
@@ -30635,13 +30669,13 @@
         <v>258</v>
       </c>
       <c r="B184" s="53" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
       <c r="C184" s="48" t="s">
-        <v>2552</v>
+        <v>2554</v>
       </c>
       <c r="D184" s="8" t="s">
-        <v>2553</v>
+        <v>2555</v>
       </c>
       <c r="E184" s="53"/>
       <c r="F184" s="53"/>
@@ -30656,13 +30690,13 @@
         <v>258</v>
       </c>
       <c r="B185" s="53" t="s">
-        <v>2554</v>
+        <v>2556</v>
       </c>
       <c r="C185" s="48" t="s">
-        <v>2555</v>
+        <v>2557</v>
       </c>
       <c r="D185" s="8" t="s">
-        <v>2556</v>
+        <v>2558</v>
       </c>
       <c r="E185" s="53"/>
       <c r="F185" s="53"/>
@@ -30677,13 +30711,13 @@
         <v>258</v>
       </c>
       <c r="B186" s="53" t="s">
-        <v>2557</v>
+        <v>2559</v>
       </c>
       <c r="C186" s="48" t="s">
-        <v>2558</v>
+        <v>2560</v>
       </c>
       <c r="D186" s="8" t="s">
-        <v>2559</v>
+        <v>2561</v>
       </c>
       <c r="E186" s="53"/>
       <c r="F186" s="53"/>
@@ -30698,13 +30732,13 @@
         <v>258</v>
       </c>
       <c r="B187" s="53" t="s">
-        <v>2560</v>
+        <v>2562</v>
       </c>
       <c r="C187" s="48" t="s">
-        <v>2561</v>
+        <v>2563</v>
       </c>
       <c r="D187" s="8" t="s">
-        <v>2562</v>
+        <v>2564</v>
       </c>
       <c r="E187" s="53"/>
       <c r="F187" s="53"/>
@@ -30719,13 +30753,13 @@
         <v>258</v>
       </c>
       <c r="B188" s="53" t="s">
-        <v>2563</v>
+        <v>2565</v>
       </c>
       <c r="C188" s="48" t="s">
-        <v>2564</v>
+        <v>2566</v>
       </c>
       <c r="D188" s="8" t="s">
-        <v>2565</v>
+        <v>2567</v>
       </c>
       <c r="E188" s="53"/>
       <c r="F188" s="53"/>
@@ -30740,13 +30774,13 @@
         <v>258</v>
       </c>
       <c r="B189" s="53" t="s">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="C189" s="48" t="s">
-        <v>2567</v>
+        <v>2569</v>
       </c>
       <c r="D189" s="8" t="s">
-        <v>2568</v>
+        <v>2570</v>
       </c>
       <c r="E189" s="53"/>
       <c r="F189" s="53"/>
@@ -30764,10 +30798,10 @@
         <v>1207</v>
       </c>
       <c r="C190" s="48" t="s">
-        <v>2569</v>
+        <v>2571</v>
       </c>
       <c r="D190" s="8" t="s">
-        <v>2570</v>
+        <v>2572</v>
       </c>
       <c r="E190" s="53"/>
       <c r="F190" s="53"/>
@@ -30784,10 +30818,10 @@
         <v>229</v>
       </c>
       <c r="C191" s="48" t="s">
-        <v>2195</v>
+        <v>2197</v>
       </c>
       <c r="D191" s="8" t="s">
-        <v>2196</v>
+        <v>2198</v>
       </c>
       <c r="E191" s="53"/>
       <c r="F191" s="53"/>
@@ -30805,10 +30839,10 @@
         <v>1171</v>
       </c>
       <c r="C192" s="53" t="s">
-        <v>2201</v>
+        <v>2203</v>
       </c>
       <c r="D192" s="53" t="s">
-        <v>2202</v>
+        <v>2204</v>
       </c>
       <c r="E192" s="53"/>
       <c r="F192" s="53"/>
@@ -30822,13 +30856,13 @@
         <v>287</v>
       </c>
       <c r="B193" s="53" t="s">
-        <v>2571</v>
+        <v>2573</v>
       </c>
       <c r="C193" s="48" t="s">
-        <v>2572</v>
+        <v>2574</v>
       </c>
       <c r="D193" s="8" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="E193" s="53"/>
       <c r="F193" s="53"/>
@@ -30841,13 +30875,13 @@
         <v>287</v>
       </c>
       <c r="B194" s="53" t="s">
-        <v>2574</v>
+        <v>2576</v>
       </c>
       <c r="C194" s="48" t="s">
-        <v>2575</v>
+        <v>2577</v>
       </c>
       <c r="D194" s="8" t="s">
-        <v>2576</v>
+        <v>2578</v>
       </c>
       <c r="E194" s="53"/>
       <c r="F194" s="53"/>
@@ -30860,13 +30894,13 @@
         <v>287</v>
       </c>
       <c r="B195" s="53" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="C195" s="48" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
       <c r="D195" s="8" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
       <c r="E195" s="53"/>
       <c r="F195" s="53"/>
@@ -30879,13 +30913,13 @@
         <v>287</v>
       </c>
       <c r="B196" s="53" t="s">
-        <v>2580</v>
+        <v>2582</v>
       </c>
       <c r="C196" s="48" t="s">
-        <v>2581</v>
+        <v>2583</v>
       </c>
       <c r="D196" s="8" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
       <c r="E196" s="53"/>
       <c r="F196" s="53"/>
@@ -30898,13 +30932,13 @@
         <v>287</v>
       </c>
       <c r="B197" s="53" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
       <c r="C197" s="48" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
       <c r="D197" s="8" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
       <c r="E197" s="53"/>
       <c r="F197" s="53"/>
@@ -30917,13 +30951,13 @@
         <v>294</v>
       </c>
       <c r="B198" s="53" t="s">
-        <v>2571</v>
+        <v>2573</v>
       </c>
       <c r="C198" s="48" t="s">
-        <v>2572</v>
+        <v>2574</v>
       </c>
       <c r="D198" s="8" t="s">
-        <v>2573</v>
+        <v>2575</v>
       </c>
       <c r="E198" s="53"/>
       <c r="F198" s="53"/>
@@ -30938,13 +30972,13 @@
         <v>294</v>
       </c>
       <c r="B199" s="53" t="s">
-        <v>2574</v>
+        <v>2576</v>
       </c>
       <c r="C199" s="48" t="s">
-        <v>2575</v>
+        <v>2577</v>
       </c>
       <c r="D199" s="8" t="s">
-        <v>2576</v>
+        <v>2578</v>
       </c>
       <c r="E199" s="53"/>
       <c r="F199" s="53"/>
@@ -30957,13 +30991,13 @@
         <v>294</v>
       </c>
       <c r="B200" s="53" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="C200" s="48" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
       <c r="D200" s="8" t="s">
-        <v>2579</v>
+        <v>2581</v>
       </c>
       <c r="E200" s="53"/>
       <c r="F200" s="53"/>
@@ -30976,13 +31010,13 @@
         <v>294</v>
       </c>
       <c r="B201" s="53" t="s">
-        <v>2580</v>
+        <v>2582</v>
       </c>
       <c r="C201" s="48" t="s">
-        <v>2581</v>
+        <v>2583</v>
       </c>
       <c r="D201" s="8" t="s">
-        <v>2582</v>
+        <v>2584</v>
       </c>
       <c r="E201" s="53"/>
       <c r="F201" s="53"/>
@@ -30995,13 +31029,13 @@
         <v>294</v>
       </c>
       <c r="B202" s="53" t="s">
-        <v>2583</v>
+        <v>2585</v>
       </c>
       <c r="C202" s="48" t="s">
-        <v>2584</v>
+        <v>2586</v>
       </c>
       <c r="D202" s="8" t="s">
-        <v>2585</v>
+        <v>2587</v>
       </c>
       <c r="E202" s="53"/>
       <c r="F202" s="53"/>
@@ -31014,7 +31048,7 @@
         <v>857</v>
       </c>
       <c r="B203" s="66" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="C203" s="66" t="s">
         <v>1923</v>
@@ -31028,7 +31062,7 @@
         <v>857</v>
       </c>
       <c r="B204" s="66" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="C204" s="66" t="s">
         <v>1926</v>
@@ -31042,13 +31076,13 @@
         <v>857</v>
       </c>
       <c r="B205" s="66" t="s">
-        <v>2586</v>
+        <v>2588</v>
       </c>
       <c r="C205" s="66" t="s">
-        <v>2587</v>
+        <v>2589</v>
       </c>
       <c r="D205" s="66" t="s">
-        <v>2588</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31056,13 +31090,13 @@
         <v>857</v>
       </c>
       <c r="B206" s="66" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="C206" s="66" t="s">
-        <v>2589</v>
+        <v>2591</v>
       </c>
       <c r="D206" s="66" t="s">
-        <v>2590</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31070,7 +31104,7 @@
         <v>857</v>
       </c>
       <c r="G207" s="66" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31078,13 +31112,13 @@
         <v>882</v>
       </c>
       <c r="B208" s="66" t="s">
-        <v>2591</v>
+        <v>2593</v>
       </c>
       <c r="C208" s="66" t="s">
-        <v>2592</v>
+        <v>2594</v>
       </c>
       <c r="D208" s="66" t="s">
-        <v>2593</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31092,13 +31126,13 @@
         <v>882</v>
       </c>
       <c r="B209" s="66" t="s">
-        <v>2594</v>
+        <v>2596</v>
       </c>
       <c r="C209" s="66" t="s">
-        <v>2595</v>
+        <v>2597</v>
       </c>
       <c r="D209" s="66" t="s">
-        <v>2596</v>
+        <v>2598</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31106,13 +31140,13 @@
         <v>882</v>
       </c>
       <c r="B210" s="66" t="s">
-        <v>2597</v>
+        <v>2599</v>
       </c>
       <c r="C210" s="66" t="s">
-        <v>2598</v>
+        <v>2600</v>
       </c>
       <c r="D210" s="66" t="s">
-        <v>2599</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31120,13 +31154,13 @@
         <v>882</v>
       </c>
       <c r="B211" s="66" t="s">
-        <v>2600</v>
+        <v>2602</v>
       </c>
       <c r="C211" s="66" t="s">
-        <v>2601</v>
+        <v>2603</v>
       </c>
       <c r="D211" s="66" t="s">
-        <v>2602</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31134,13 +31168,13 @@
         <v>882</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>2603</v>
+        <v>2605</v>
       </c>
       <c r="C212" s="66" t="s">
-        <v>2604</v>
+        <v>2606</v>
       </c>
       <c r="D212" s="66" t="s">
-        <v>2605</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31148,13 +31182,13 @@
         <v>882</v>
       </c>
       <c r="B213" s="66" t="s">
-        <v>2606</v>
+        <v>2608</v>
       </c>
       <c r="C213" s="66" t="s">
-        <v>2607</v>
+        <v>2609</v>
       </c>
       <c r="D213" s="66" t="s">
-        <v>2608</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31165,10 +31199,10 @@
         <v>229</v>
       </c>
       <c r="C214" s="66" t="s">
-        <v>2609</v>
+        <v>2611</v>
       </c>
       <c r="D214" s="66" t="s">
-        <v>2610</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31176,7 +31210,7 @@
         <v>887</v>
       </c>
       <c r="B215" s="66" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="C215" s="66" t="s">
         <v>1923</v>
@@ -31190,7 +31224,7 @@
         <v>887</v>
       </c>
       <c r="B216" s="66" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="C216" s="66" t="s">
         <v>1926</v>
@@ -31204,13 +31238,13 @@
         <v>887</v>
       </c>
       <c r="B217" s="66" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="C217" s="66" t="s">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="D217" s="66" t="s">
-        <v>2612</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="218" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31218,13 +31252,13 @@
         <v>887</v>
       </c>
       <c r="B218" s="66" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="C218" s="66" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="D218" s="66" t="s">
-        <v>2614</v>
+        <v>2616</v>
       </c>
       <c r="E218" s="66"/>
       <c r="F218" s="66"/>
@@ -31237,13 +31271,13 @@
         <v>887</v>
       </c>
       <c r="B219" s="66" t="s">
-        <v>2457</v>
+        <v>2459</v>
       </c>
       <c r="C219" s="66" t="s">
-        <v>2589</v>
+        <v>2591</v>
       </c>
       <c r="D219" s="66" t="s">
-        <v>2590</v>
+        <v>2592</v>
       </c>
       <c r="E219" s="66"/>
       <c r="F219" s="66"/>
@@ -31259,10 +31293,10 @@
         <v>229</v>
       </c>
       <c r="C220" s="66" t="s">
-        <v>2615</v>
+        <v>2617</v>
       </c>
       <c r="D220" s="66" t="s">
-        <v>2616</v>
+        <v>2618</v>
       </c>
       <c r="E220" s="66"/>
       <c r="F220" s="66"/>
@@ -31278,10 +31312,10 @@
         <v>1258</v>
       </c>
       <c r="C221" s="8" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
       <c r="D221" s="8" t="s">
-        <v>2618</v>
+        <v>2620</v>
       </c>
       <c r="E221" s="66"/>
       <c r="F221" s="66"/>
@@ -31294,13 +31328,13 @@
         <v>1052</v>
       </c>
       <c r="B222" s="66" t="s">
-        <v>2619</v>
+        <v>2621</v>
       </c>
       <c r="C222" s="8" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="D222" s="8" t="s">
-        <v>2621</v>
+        <v>2623</v>
       </c>
       <c r="E222" s="66"/>
       <c r="F222" s="66"/>
@@ -31315,13 +31349,13 @@
         <v>1052</v>
       </c>
       <c r="B223" s="66" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C223" s="8" t="s">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="D223" s="8" t="s">
-        <v>2624</v>
+        <v>2626</v>
       </c>
       <c r="E223" s="66"/>
       <c r="F223" s="66"/>
@@ -31336,13 +31370,13 @@
         <v>1052</v>
       </c>
       <c r="B224" s="66" t="s">
-        <v>2625</v>
+        <v>2627</v>
       </c>
       <c r="C224" s="8" t="s">
-        <v>2626</v>
+        <v>2628</v>
       </c>
       <c r="D224" s="51" t="s">
-        <v>2627</v>
+        <v>2629</v>
       </c>
       <c r="E224" s="66"/>
       <c r="F224" s="66"/>
@@ -31357,13 +31391,13 @@
         <v>1052</v>
       </c>
       <c r="B225" s="66" t="s">
-        <v>2628</v>
+        <v>2630</v>
       </c>
       <c r="C225" s="8" t="s">
-        <v>2629</v>
+        <v>2631</v>
       </c>
       <c r="D225" s="48" t="s">
-        <v>2630</v>
+        <v>2632</v>
       </c>
       <c r="E225" s="66"/>
       <c r="F225" s="66"/>
@@ -31376,13 +31410,13 @@
         <v>1058</v>
       </c>
       <c r="B226" s="66" t="s">
-        <v>2631</v>
+        <v>2633</v>
       </c>
       <c r="C226" s="8" t="s">
-        <v>2632</v>
+        <v>2634</v>
       </c>
       <c r="D226" s="8" t="s">
-        <v>2633</v>
+        <v>2635</v>
       </c>
       <c r="E226" s="66"/>
       <c r="F226" s="66"/>
@@ -31397,13 +31431,13 @@
         <v>1058</v>
       </c>
       <c r="B227" s="66" t="s">
-        <v>2634</v>
+        <v>2636</v>
       </c>
       <c r="C227" s="8" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="D227" s="8" t="s">
-        <v>2636</v>
+        <v>2638</v>
       </c>
       <c r="E227" s="66"/>
       <c r="F227" s="66"/>
@@ -31418,13 +31452,13 @@
         <v>1058</v>
       </c>
       <c r="B228" s="66" t="s">
-        <v>2637</v>
+        <v>2639</v>
       </c>
       <c r="C228" s="8" t="s">
-        <v>2638</v>
+        <v>2640</v>
       </c>
       <c r="D228" s="8" t="s">
-        <v>2639</v>
+        <v>2641</v>
       </c>
       <c r="E228" s="66"/>
       <c r="F228" s="66"/>
@@ -31434,16 +31468,16 @@
     </row>
     <row r="229" s="50" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="54" t="s">
-        <v>2640</v>
+        <v>2642</v>
       </c>
       <c r="B229" s="66" t="s">
         <v>1167</v>
       </c>
       <c r="C229" s="51" t="s">
-        <v>2641</v>
+        <v>2643</v>
       </c>
       <c r="D229" s="8" t="s">
-        <v>2642</v>
+        <v>2644</v>
       </c>
       <c r="E229" s="66"/>
       <c r="F229" s="66"/>
@@ -31453,16 +31487,16 @@
     </row>
     <row r="230" s="50" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="54" t="s">
-        <v>2640</v>
+        <v>2642</v>
       </c>
       <c r="B230" s="66" t="s">
         <v>1225</v>
       </c>
       <c r="C230" s="51" t="s">
-        <v>2643</v>
+        <v>2645</v>
       </c>
       <c r="D230" s="48" t="s">
-        <v>2644</v>
+        <v>2646</v>
       </c>
       <c r="E230" s="66"/>
       <c r="F230" s="66"/>
@@ -31475,13 +31509,13 @@
         <v>1088</v>
       </c>
       <c r="B231" s="66" t="s">
-        <v>2645</v>
+        <v>2647</v>
       </c>
       <c r="C231" s="8" t="s">
-        <v>2646</v>
+        <v>2648</v>
       </c>
       <c r="D231" s="51" t="s">
-        <v>2647</v>
+        <v>2649</v>
       </c>
       <c r="E231" s="66"/>
       <c r="F231" s="66"/>
@@ -31494,13 +31528,13 @@
         <v>1088</v>
       </c>
       <c r="B232" s="66" t="s">
-        <v>2648</v>
+        <v>2650</v>
       </c>
       <c r="C232" s="8" t="s">
-        <v>2649</v>
+        <v>2651</v>
       </c>
       <c r="D232" s="51" t="s">
-        <v>2650</v>
+        <v>2652</v>
       </c>
       <c r="E232" s="66"/>
       <c r="F232" s="66"/>
@@ -31513,13 +31547,13 @@
         <v>1088</v>
       </c>
       <c r="B233" s="66" t="s">
-        <v>2651</v>
+        <v>2653</v>
       </c>
       <c r="C233" s="8" t="s">
-        <v>2652</v>
+        <v>2654</v>
       </c>
       <c r="D233" s="51" t="s">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="E233" s="66"/>
       <c r="F233" s="66"/>
@@ -31532,13 +31566,13 @@
         <v>1088</v>
       </c>
       <c r="B234" s="66" t="s">
-        <v>2654</v>
+        <v>2656</v>
       </c>
       <c r="C234" s="8" t="s">
-        <v>2655</v>
+        <v>2657</v>
       </c>
       <c r="D234" s="51" t="s">
-        <v>2656</v>
+        <v>2658</v>
       </c>
       <c r="E234" s="66"/>
       <c r="F234" s="66"/>
@@ -31551,13 +31585,13 @@
         <v>1088</v>
       </c>
       <c r="B235" s="66" t="s">
-        <v>2657</v>
+        <v>2659</v>
       </c>
       <c r="C235" s="8" t="s">
-        <v>2658</v>
+        <v>2660</v>
       </c>
       <c r="D235" s="51" t="s">
-        <v>2659</v>
+        <v>2661</v>
       </c>
     </row>
     <row r="236" s="50" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31565,13 +31599,13 @@
         <v>1088</v>
       </c>
       <c r="B236" s="66" t="s">
-        <v>2660</v>
+        <v>2662</v>
       </c>
       <c r="C236" s="8" t="s">
-        <v>2661</v>
+        <v>2663</v>
       </c>
       <c r="D236" s="51" t="s">
-        <v>2662</v>
+        <v>2664</v>
       </c>
       <c r="E236" s="66"/>
       <c r="F236" s="66"/>
@@ -31589,7 +31623,7 @@
       <c r="E237" s="66"/>
       <c r="F237" s="66"/>
       <c r="G237" s="53" t="s">
-        <v>2197</v>
+        <v>2199</v>
       </c>
       <c r="H237" s="66"/>
       <c r="I237" s="66"/>
@@ -31599,13 +31633,13 @@
         <v>946</v>
       </c>
       <c r="B238" s="50" t="s">
-        <v>2663</v>
+        <v>2665</v>
       </c>
       <c r="C238" s="50" t="s">
-        <v>2664</v>
+        <v>2666</v>
       </c>
       <c r="D238" s="50" t="s">
-        <v>2665</v>
+        <v>2667</v>
       </c>
     </row>
     <row r="239" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31613,13 +31647,13 @@
         <v>946</v>
       </c>
       <c r="B239" s="50" t="s">
-        <v>2577</v>
+        <v>2579</v>
       </c>
       <c r="C239" s="50" t="s">
-        <v>2666</v>
+        <v>2668</v>
       </c>
       <c r="D239" s="50" t="s">
-        <v>2667</v>
+        <v>2669</v>
       </c>
     </row>
     <row r="240" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31627,13 +31661,13 @@
         <v>946</v>
       </c>
       <c r="B240" s="50" t="s">
-        <v>2668</v>
+        <v>2670</v>
       </c>
       <c r="C240" s="50" t="s">
-        <v>2669</v>
+        <v>2671</v>
       </c>
       <c r="D240" s="50" t="s">
-        <v>2670</v>
+        <v>2672</v>
       </c>
     </row>
     <row r="241" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31641,13 +31675,13 @@
         <v>946</v>
       </c>
       <c r="B241" s="50" t="s">
-        <v>2671</v>
+        <v>2673</v>
       </c>
       <c r="C241" s="50" t="s">
-        <v>2672</v>
+        <v>2674</v>
       </c>
       <c r="D241" s="50" t="s">
-        <v>2673</v>
+        <v>2675</v>
       </c>
     </row>
     <row r="242" s="50" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31655,13 +31689,13 @@
         <v>946</v>
       </c>
       <c r="B242" s="50" t="s">
-        <v>2674</v>
+        <v>2676</v>
       </c>
       <c r="C242" s="50" t="s">
-        <v>2675</v>
+        <v>2677</v>
       </c>
       <c r="D242" s="50" t="s">
-        <v>2676</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="243" s="50" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31672,10 +31706,10 @@
         <v>-2</v>
       </c>
       <c r="C243" s="57" t="s">
-        <v>2677</v>
+        <v>2679</v>
       </c>
       <c r="D243" s="57" t="s">
-        <v>2678</v>
+        <v>2680</v>
       </c>
       <c r="E243" s="66"/>
       <c r="F243" s="66"/>
@@ -31691,10 +31725,10 @@
         <v>-1</v>
       </c>
       <c r="C244" s="57" t="s">
-        <v>2679</v>
+        <v>2681</v>
       </c>
       <c r="D244" s="57" t="s">
-        <v>2680</v>
+        <v>2682</v>
       </c>
       <c r="E244" s="66"/>
       <c r="F244" s="66"/>
@@ -31710,10 +31744,10 @@
         <v>0</v>
       </c>
       <c r="C245" s="57" t="s">
-        <v>2681</v>
+        <v>2683</v>
       </c>
       <c r="D245" s="57" t="s">
-        <v>2682</v>
+        <v>2684</v>
       </c>
       <c r="E245" s="66"/>
       <c r="F245" s="66"/>
@@ -31729,10 +31763,10 @@
         <v>1</v>
       </c>
       <c r="C246" s="57" t="s">
-        <v>2683</v>
+        <v>2685</v>
       </c>
       <c r="D246" s="57" t="s">
-        <v>2684</v>
+        <v>2686</v>
       </c>
       <c r="E246" s="66"/>
       <c r="F246" s="66"/>
@@ -31748,10 +31782,10 @@
         <v>2</v>
       </c>
       <c r="C247" s="57" t="s">
-        <v>2685</v>
+        <v>2687</v>
       </c>
       <c r="D247" s="57" t="s">
-        <v>2686</v>
+        <v>2688</v>
       </c>
       <c r="E247" s="66"/>
       <c r="F247" s="66"/>
@@ -31767,10 +31801,10 @@
         <v>0</v>
       </c>
       <c r="C248" s="48" t="s">
-        <v>2687</v>
+        <v>2689</v>
       </c>
       <c r="D248" s="57" t="s">
-        <v>2688</v>
+        <v>2690</v>
       </c>
       <c r="E248" s="66"/>
       <c r="F248" s="66"/>
@@ -31786,10 +31820,10 @@
         <v>1</v>
       </c>
       <c r="C249" s="48" t="s">
-        <v>2689</v>
+        <v>2691</v>
       </c>
       <c r="D249" s="51" t="s">
-        <v>2690</v>
+        <v>2692</v>
       </c>
       <c r="E249" s="66"/>
       <c r="F249" s="66"/>
@@ -31805,10 +31839,10 @@
         <v>2</v>
       </c>
       <c r="C250" s="48" t="s">
-        <v>2691</v>
+        <v>2693</v>
       </c>
       <c r="D250" s="51" t="s">
-        <v>2692</v>
+        <v>2694</v>
       </c>
       <c r="E250" s="66"/>
       <c r="F250" s="66"/>
@@ -31824,10 +31858,10 @@
         <v>3</v>
       </c>
       <c r="C251" s="48" t="s">
-        <v>2693</v>
+        <v>2695</v>
       </c>
       <c r="D251" s="51" t="s">
-        <v>2694</v>
+        <v>2696</v>
       </c>
       <c r="E251" s="66"/>
       <c r="F251" s="66"/>
@@ -31843,10 +31877,10 @@
         <v>4</v>
       </c>
       <c r="C252" s="48" t="s">
-        <v>2695</v>
+        <v>2697</v>
       </c>
       <c r="D252" s="51" t="s">
-        <v>2696</v>
+        <v>2698</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31857,10 +31891,10 @@
         <v>-1</v>
       </c>
       <c r="C253" s="48" t="s">
-        <v>2697</v>
+        <v>2699</v>
       </c>
       <c r="D253" s="51" t="s">
-        <v>2698</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31868,13 +31902,13 @@
         <v>39</v>
       </c>
       <c r="B254" s="66" t="s">
-        <v>2699</v>
+        <v>2701</v>
       </c>
       <c r="C254" s="66" t="s">
-        <v>2700</v>
+        <v>2702</v>
       </c>
       <c r="D254" s="66" t="s">
-        <v>2701</v>
+        <v>2703</v>
       </c>
     </row>
     <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
visitedPlaces: fix étiquette de libellé `journeyDate`
fixes #205

Avec la mise à jour d'Évolution, le placeholder est maintenant
`journeyDates` pour les question builtin concernant une journey. L'excel
a donc été mis à jour en conséquence.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -1658,19 +1658,19 @@
     <t xml:space="preserve">personVisitedPlacesTitle</t>
   </si>
   <si>
-    <t xml:space="preserve">Lieux où {{nickname}} est allé{{gender:/e/(e)/(e)}} le {{journeyDate}} :
+    <t xml:space="preserve">Lieux où {{nickname}} est allé{{gender:/e/(e)/(e)}} le {{journeyDates}} :
 L'ordre chronologique doit être respecté.</t>
   </si>
   <si>
-    <t xml:space="preserve">Places {{nickname}} went on {{journeyDate}}:
+    <t xml:space="preserve">Places {{nickname}} went on {{journeyDates}}:
 Chronological order must be respected (i.e. sequence matters).</t>
   </si>
   <si>
-    <t xml:space="preserve">Lieux où vous êtes allé{{gender:/e/(e)/(e)}} le {{journeyDate}} :
+    <t xml:space="preserve">Lieux où vous êtes allé{{gender:/e/(e)/(e)}} le {{journeyDates}} :
 L'ordre chronologique doit être respecté.</t>
   </si>
   <si>
-    <t xml:space="preserve">Places you went on {{journeyDate}}:
+    <t xml:space="preserve">Places you went on {{journeyDates}}:
 Chronological order must be respected (i.e. sequence matters).</t>
   </si>
   <si>

</xml_diff>

<commit_message>
labels: mise à jour des textes des modes de commuting
Aussi ajout du hint pour les déplacements en automne.

fixes #308, fixes #307
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5000" uniqueCount="2732">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5000" uniqueCount="2736">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -2696,22 +2696,22 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Quel moyen de transport utilise habituellement {{nickname}} pour** se rendre à son lieu de travail?** 
+    <t xml:space="preserve">Quel moyen de transport utilise habituellement {{nickname}} pour** se rendre à son lieu de travail**, en automne?
 __Si plusieurs modes sont utilisés, indiquer le mode qui représente la plus grande partie de la distance parcourue.
 Si {{nickname}} fréquente plusieurs lieux, répondre en fonction du lieu déclaré ci-dessus.__</t>
   </si>
   <si>
-    <t xml:space="preserve">What mode of transportation does {{nickname}} usually use **to travel to their workplace?**
+    <t xml:space="preserve">What mode of transportation does {{nickname}} usually use **to travel to their workplace**, in automn?
 __If multiple modes are used, indicate the one that represents the largest share of distance traveled.
 If {{nickname}} works at multiple locations, respond based on the location identified above.__</t>
   </si>
   <si>
-    <t xml:space="preserve">Quel moyen de transport utilisez-vous habituellement pour** vous rendre à votre lieu de travail?** 
+    <t xml:space="preserve">Quel moyen de transport utilisez-vous habituellement pour** vous rendre à votre lieu de travail**, en automne? 
 __Si plusieurs modes sont utilisés, indiquer le mode qui représente la plus grande partie de la distance parcourue.
 Si vous fréquentez plusieurs lieux, répondre en fonction du lieu déclaré ci-dessus.__</t>
   </si>
   <si>
-    <t xml:space="preserve">What mode of transportation do you usually use **to travel to your workplace?**
+    <t xml:space="preserve">What mode of transportation do you usually use **to travel to your workplace**, in automn?
 __If multiple modes are used, indicate the one that represents the largest share of distance traveled.
 If you work at multiple locations, respond based on the location identified above.__</t>
   </si>
@@ -8122,6 +8122,18 @@
   </si>
   <si>
     <t xml:space="preserve">Longueuil Intermodal Terminal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto en tant que **conducteur**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Car as **driver**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto en tant que **passager**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Car as **passenger**</t>
   </si>
   <si>
     <t xml:space="preserve">**Transport en commun**</t>
@@ -16288,7 +16300,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="150.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="165.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="9" t="s">
         <v>786</v>
       </c>
@@ -30492,10 +30504,10 @@
         <v>2481</v>
       </c>
       <c r="C161" s="11" t="s">
-        <v>2024</v>
+        <v>2533</v>
       </c>
       <c r="D161" s="11" t="s">
-        <v>2025</v>
+        <v>2534</v>
       </c>
       <c r="G161" s="56"/>
       <c r="H161" s="56"/>
@@ -30509,10 +30521,10 @@
         <v>2482</v>
       </c>
       <c r="C162" s="11" t="s">
-        <v>2042</v>
+        <v>2535</v>
       </c>
       <c r="D162" s="11" t="s">
-        <v>2043</v>
+        <v>2536</v>
       </c>
       <c r="G162" s="56"/>
       <c r="H162" s="56"/>
@@ -30526,10 +30538,10 @@
         <v>2487</v>
       </c>
       <c r="C163" s="11" t="s">
-        <v>2533</v>
+        <v>2537</v>
       </c>
       <c r="D163" s="11" t="s">
-        <v>2534</v>
+        <v>2538</v>
       </c>
       <c r="G163" s="56"/>
       <c r="H163" s="56"/>
@@ -30557,7 +30569,7 @@
         <v>793</v>
       </c>
       <c r="B165" s="56" t="s">
-        <v>2535</v>
+        <v>2539</v>
       </c>
       <c r="C165" s="11" t="s">
         <v>1980</v>
@@ -30577,10 +30589,10 @@
         <v>232</v>
       </c>
       <c r="C166" s="11" t="s">
-        <v>2536</v>
+        <v>2540</v>
       </c>
       <c r="D166" s="11" t="s">
-        <v>2537</v>
+        <v>2541</v>
       </c>
       <c r="G166" s="56"/>
       <c r="H166" s="52" t="s">
@@ -30593,13 +30605,13 @@
         <v>793</v>
       </c>
       <c r="B167" s="56" t="s">
-        <v>2538</v>
+        <v>2542</v>
       </c>
       <c r="C167" s="11" t="s">
-        <v>2539</v>
+        <v>2543</v>
       </c>
       <c r="D167" s="11" t="s">
-        <v>2540</v>
+        <v>2544</v>
       </c>
       <c r="G167" s="56"/>
       <c r="H167" s="52" t="s">
@@ -30612,13 +30624,13 @@
         <v>141</v>
       </c>
       <c r="B168" s="56" t="s">
-        <v>2541</v>
+        <v>2545</v>
       </c>
       <c r="C168" s="11" t="s">
-        <v>2542</v>
+        <v>2546</v>
       </c>
       <c r="D168" s="11" t="s">
-        <v>2543</v>
+        <v>2547</v>
       </c>
       <c r="G168" s="56"/>
       <c r="H168" s="56"/>
@@ -30629,13 +30641,13 @@
         <v>141</v>
       </c>
       <c r="B169" s="56" t="s">
-        <v>2544</v>
+        <v>2548</v>
       </c>
       <c r="C169" s="11" t="s">
-        <v>2545</v>
+        <v>2549</v>
       </c>
       <c r="D169" s="11" t="s">
-        <v>2546</v>
+        <v>2550</v>
       </c>
       <c r="G169" s="56"/>
       <c r="H169" s="56"/>
@@ -30649,10 +30661,10 @@
         <v>1212</v>
       </c>
       <c r="C170" s="11" t="s">
-        <v>2547</v>
+        <v>2551</v>
       </c>
       <c r="D170" s="11" t="s">
-        <v>2548</v>
+        <v>2552</v>
       </c>
       <c r="G170" s="56"/>
       <c r="H170" s="56"/>
@@ -30666,10 +30678,10 @@
         <v>1248</v>
       </c>
       <c r="C171" s="11" t="s">
-        <v>2549</v>
+        <v>2553</v>
       </c>
       <c r="D171" s="11" t="s">
-        <v>2550</v>
+        <v>2554</v>
       </c>
       <c r="G171" s="56"/>
       <c r="H171" s="56"/>
@@ -30691,13 +30703,13 @@
         <v>248</v>
       </c>
       <c r="B173" s="56" t="s">
-        <v>2551</v>
+        <v>2555</v>
       </c>
       <c r="C173" s="11" t="s">
-        <v>2552</v>
+        <v>2556</v>
       </c>
       <c r="D173" s="11" t="s">
-        <v>2553</v>
+        <v>2557</v>
       </c>
       <c r="G173" s="56"/>
       <c r="H173" s="56" t="s">
@@ -30710,13 +30722,13 @@
         <v>248</v>
       </c>
       <c r="B174" s="56" t="s">
-        <v>2554</v>
+        <v>2558</v>
       </c>
       <c r="C174" s="11" t="s">
-        <v>2555</v>
+        <v>2559</v>
       </c>
       <c r="D174" s="11" t="s">
-        <v>2556</v>
+        <v>2560</v>
       </c>
       <c r="G174" s="56"/>
       <c r="H174" s="56" t="s">
@@ -30729,13 +30741,13 @@
         <v>248</v>
       </c>
       <c r="B175" s="56" t="s">
-        <v>2557</v>
+        <v>2561</v>
       </c>
       <c r="C175" s="11" t="s">
-        <v>2558</v>
+        <v>2562</v>
       </c>
       <c r="D175" s="11" t="s">
-        <v>2559</v>
+        <v>2563</v>
       </c>
       <c r="G175" s="56"/>
       <c r="H175" s="56" t="s">
@@ -30748,13 +30760,13 @@
         <v>248</v>
       </c>
       <c r="B176" s="56" t="s">
-        <v>2560</v>
+        <v>2564</v>
       </c>
       <c r="C176" s="11" t="s">
-        <v>2561</v>
+        <v>2565</v>
       </c>
       <c r="D176" s="11" t="s">
-        <v>2562</v>
+        <v>2566</v>
       </c>
       <c r="G176" s="56"/>
       <c r="H176" s="56" t="s">
@@ -30767,13 +30779,13 @@
         <v>248</v>
       </c>
       <c r="B177" s="56" t="s">
-        <v>2563</v>
+        <v>2567</v>
       </c>
       <c r="C177" s="11" t="s">
-        <v>2564</v>
+        <v>2568</v>
       </c>
       <c r="D177" s="11" t="s">
-        <v>2565</v>
+        <v>2569</v>
       </c>
       <c r="G177" s="56"/>
       <c r="H177" s="56" t="s">
@@ -30786,13 +30798,13 @@
         <v>248</v>
       </c>
       <c r="B178" s="56" t="s">
-        <v>2566</v>
+        <v>2570</v>
       </c>
       <c r="C178" s="11" t="s">
-        <v>2567</v>
+        <v>2571</v>
       </c>
       <c r="D178" s="11" t="s">
-        <v>2568</v>
+        <v>2572</v>
       </c>
       <c r="G178" s="56"/>
       <c r="H178" s="56" t="s">
@@ -30805,13 +30817,13 @@
         <v>248</v>
       </c>
       <c r="B179" s="56" t="s">
-        <v>2569</v>
+        <v>2573</v>
       </c>
       <c r="C179" s="11" t="s">
-        <v>2570</v>
+        <v>2574</v>
       </c>
       <c r="D179" s="11" t="s">
-        <v>2571</v>
+        <v>2575</v>
       </c>
       <c r="G179" s="56"/>
       <c r="H179" s="56" t="s">
@@ -30824,13 +30836,13 @@
         <v>248</v>
       </c>
       <c r="B180" s="56" t="s">
-        <v>2572</v>
+        <v>2576</v>
       </c>
       <c r="C180" s="11" t="s">
-        <v>2573</v>
+        <v>2577</v>
       </c>
       <c r="D180" s="11" t="s">
-        <v>2574</v>
+        <v>2578</v>
       </c>
       <c r="G180" s="56"/>
       <c r="H180" s="56" t="s">
@@ -30843,13 +30855,13 @@
         <v>248</v>
       </c>
       <c r="B181" s="56" t="s">
-        <v>2575</v>
+        <v>2579</v>
       </c>
       <c r="C181" s="11" t="s">
-        <v>2576</v>
+        <v>2580</v>
       </c>
       <c r="D181" s="11" t="s">
-        <v>2577</v>
+        <v>2581</v>
       </c>
       <c r="G181" s="56"/>
       <c r="H181" s="56" t="s">
@@ -30892,13 +30904,13 @@
         <v>260</v>
       </c>
       <c r="B184" s="56" t="s">
-        <v>2578</v>
+        <v>2582</v>
       </c>
       <c r="C184" s="11" t="s">
-        <v>2579</v>
+        <v>2583</v>
       </c>
       <c r="D184" s="11" t="s">
-        <v>2580</v>
+        <v>2584</v>
       </c>
       <c r="G184" s="56"/>
       <c r="H184" s="56" t="s">
@@ -30911,13 +30923,13 @@
         <v>260</v>
       </c>
       <c r="B185" s="56" t="s">
-        <v>2581</v>
+        <v>2585</v>
       </c>
       <c r="C185" s="11" t="s">
-        <v>2582</v>
+        <v>2586</v>
       </c>
       <c r="D185" s="11" t="s">
-        <v>2583</v>
+        <v>2587</v>
       </c>
       <c r="G185" s="56"/>
       <c r="H185" s="56" t="s">
@@ -30930,13 +30942,13 @@
         <v>260</v>
       </c>
       <c r="B186" s="56" t="s">
-        <v>2584</v>
+        <v>2588</v>
       </c>
       <c r="C186" s="11" t="s">
-        <v>2585</v>
+        <v>2589</v>
       </c>
       <c r="D186" s="11" t="s">
-        <v>2586</v>
+        <v>2590</v>
       </c>
       <c r="G186" s="56"/>
       <c r="H186" s="56" t="s">
@@ -30949,13 +30961,13 @@
         <v>260</v>
       </c>
       <c r="B187" s="56" t="s">
-        <v>2587</v>
+        <v>2591</v>
       </c>
       <c r="C187" s="11" t="s">
-        <v>2588</v>
+        <v>2592</v>
       </c>
       <c r="D187" s="11" t="s">
-        <v>2589</v>
+        <v>2593</v>
       </c>
       <c r="G187" s="56"/>
       <c r="H187" s="56" t="s">
@@ -30968,13 +30980,13 @@
         <v>260</v>
       </c>
       <c r="B188" s="56" t="s">
-        <v>2590</v>
+        <v>2594</v>
       </c>
       <c r="C188" s="11" t="s">
-        <v>2591</v>
+        <v>2595</v>
       </c>
       <c r="D188" s="11" t="s">
-        <v>2592</v>
+        <v>2596</v>
       </c>
       <c r="G188" s="56"/>
       <c r="H188" s="56" t="s">
@@ -30987,13 +30999,13 @@
         <v>260</v>
       </c>
       <c r="B189" s="56" t="s">
-        <v>2593</v>
+        <v>2597</v>
       </c>
       <c r="C189" s="11" t="s">
-        <v>2594</v>
+        <v>2598</v>
       </c>
       <c r="D189" s="11" t="s">
-        <v>2595</v>
+        <v>2599</v>
       </c>
       <c r="G189" s="56"/>
       <c r="H189" s="56" t="s">
@@ -31006,13 +31018,13 @@
         <v>260</v>
       </c>
       <c r="B190" s="56" t="s">
-        <v>2596</v>
+        <v>2600</v>
       </c>
       <c r="C190" s="11" t="s">
-        <v>2597</v>
+        <v>2601</v>
       </c>
       <c r="D190" s="11" t="s">
-        <v>2598</v>
+        <v>2602</v>
       </c>
       <c r="G190" s="56"/>
       <c r="H190" s="56" t="s">
@@ -31028,10 +31040,10 @@
         <v>1230</v>
       </c>
       <c r="C191" s="11" t="s">
-        <v>2599</v>
+        <v>2603</v>
       </c>
       <c r="D191" s="11" t="s">
-        <v>2600</v>
+        <v>2604</v>
       </c>
       <c r="G191" s="70"/>
       <c r="H191" s="56" t="s">
@@ -31082,13 +31094,13 @@
         <v>288</v>
       </c>
       <c r="B194" s="56" t="s">
-        <v>2601</v>
+        <v>2605</v>
       </c>
       <c r="C194" s="11" t="s">
-        <v>2602</v>
+        <v>2606</v>
       </c>
       <c r="D194" s="11" t="s">
-        <v>2603</v>
+        <v>2607</v>
       </c>
       <c r="G194" s="56"/>
       <c r="H194" s="95"/>
@@ -31099,13 +31111,13 @@
         <v>288</v>
       </c>
       <c r="B195" s="56" t="s">
-        <v>2604</v>
+        <v>2608</v>
       </c>
       <c r="C195" s="11" t="s">
-        <v>2605</v>
+        <v>2609</v>
       </c>
       <c r="D195" s="11" t="s">
-        <v>2606</v>
+        <v>2610</v>
       </c>
       <c r="G195" s="56"/>
       <c r="H195" s="56"/>
@@ -31116,13 +31128,13 @@
         <v>288</v>
       </c>
       <c r="B196" s="56" t="s">
-        <v>2607</v>
+        <v>2611</v>
       </c>
       <c r="C196" s="11" t="s">
-        <v>2608</v>
+        <v>2612</v>
       </c>
       <c r="D196" s="11" t="s">
-        <v>2609</v>
+        <v>2613</v>
       </c>
       <c r="G196" s="56"/>
       <c r="H196" s="56"/>
@@ -31133,13 +31145,13 @@
         <v>288</v>
       </c>
       <c r="B197" s="56" t="s">
-        <v>2610</v>
+        <v>2614</v>
       </c>
       <c r="C197" s="11" t="s">
-        <v>2611</v>
+        <v>2615</v>
       </c>
       <c r="D197" s="11" t="s">
-        <v>2612</v>
+        <v>2616</v>
       </c>
       <c r="G197" s="56"/>
       <c r="H197" s="56"/>
@@ -31150,13 +31162,13 @@
         <v>288</v>
       </c>
       <c r="B198" s="56" t="s">
-        <v>2613</v>
+        <v>2617</v>
       </c>
       <c r="C198" s="11" t="s">
-        <v>2614</v>
+        <v>2618</v>
       </c>
       <c r="D198" s="11" t="s">
-        <v>2615</v>
+        <v>2619</v>
       </c>
       <c r="G198" s="56"/>
       <c r="H198" s="56"/>
@@ -31167,13 +31179,13 @@
         <v>295</v>
       </c>
       <c r="B199" s="56" t="s">
-        <v>2601</v>
+        <v>2605</v>
       </c>
       <c r="C199" s="11" t="s">
-        <v>2602</v>
+        <v>2606</v>
       </c>
       <c r="D199" s="11" t="s">
-        <v>2603</v>
+        <v>2607</v>
       </c>
       <c r="G199" s="56"/>
       <c r="H199" s="95" t="s">
@@ -31186,13 +31198,13 @@
         <v>295</v>
       </c>
       <c r="B200" s="56" t="s">
-        <v>2604</v>
+        <v>2608</v>
       </c>
       <c r="C200" s="11" t="s">
-        <v>2605</v>
+        <v>2609</v>
       </c>
       <c r="D200" s="11" t="s">
-        <v>2606</v>
+        <v>2610</v>
       </c>
       <c r="G200" s="56"/>
       <c r="H200" s="56"/>
@@ -31203,13 +31215,13 @@
         <v>295</v>
       </c>
       <c r="B201" s="56" t="s">
-        <v>2607</v>
+        <v>2611</v>
       </c>
       <c r="C201" s="11" t="s">
-        <v>2608</v>
+        <v>2612</v>
       </c>
       <c r="D201" s="11" t="s">
-        <v>2609</v>
+        <v>2613</v>
       </c>
       <c r="G201" s="56"/>
       <c r="H201" s="56"/>
@@ -31220,13 +31232,13 @@
         <v>295</v>
       </c>
       <c r="B202" s="56" t="s">
-        <v>2610</v>
+        <v>2614</v>
       </c>
       <c r="C202" s="11" t="s">
-        <v>2611</v>
+        <v>2615</v>
       </c>
       <c r="D202" s="11" t="s">
-        <v>2612</v>
+        <v>2616</v>
       </c>
       <c r="G202" s="56"/>
       <c r="H202" s="56"/>
@@ -31237,13 +31249,13 @@
         <v>295</v>
       </c>
       <c r="B203" s="56" t="s">
-        <v>2613</v>
+        <v>2617</v>
       </c>
       <c r="C203" s="11" t="s">
-        <v>2614</v>
+        <v>2618</v>
       </c>
       <c r="D203" s="11" t="s">
-        <v>2615</v>
+        <v>2619</v>
       </c>
       <c r="G203" s="56"/>
       <c r="H203" s="56"/>
@@ -31282,13 +31294,13 @@
         <v>857</v>
       </c>
       <c r="B206" s="70" t="s">
-        <v>2616</v>
+        <v>2620</v>
       </c>
       <c r="C206" s="11" t="s">
-        <v>2617</v>
+        <v>2621</v>
       </c>
       <c r="D206" s="11" t="s">
-        <v>2618</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31299,10 +31311,10 @@
         <v>2487</v>
       </c>
       <c r="C207" s="11" t="s">
-        <v>2619</v>
+        <v>2623</v>
       </c>
       <c r="D207" s="11" t="s">
-        <v>2620</v>
+        <v>2624</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31318,13 +31330,13 @@
         <v>882</v>
       </c>
       <c r="B209" s="70" t="s">
-        <v>2621</v>
+        <v>2625</v>
       </c>
       <c r="C209" s="11" t="s">
-        <v>2622</v>
+        <v>2626</v>
       </c>
       <c r="D209" s="11" t="s">
-        <v>2623</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31332,13 +31344,13 @@
         <v>882</v>
       </c>
       <c r="B210" s="70" t="s">
-        <v>2624</v>
+        <v>2628</v>
       </c>
       <c r="C210" s="11" t="s">
-        <v>2625</v>
+        <v>2629</v>
       </c>
       <c r="D210" s="11" t="s">
-        <v>2626</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31346,13 +31358,13 @@
         <v>882</v>
       </c>
       <c r="B211" s="70" t="s">
-        <v>2627</v>
+        <v>2631</v>
       </c>
       <c r="C211" s="11" t="s">
-        <v>2628</v>
+        <v>2632</v>
       </c>
       <c r="D211" s="11" t="s">
-        <v>2629</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31360,13 +31372,13 @@
         <v>882</v>
       </c>
       <c r="B212" s="70" t="s">
-        <v>2630</v>
+        <v>2634</v>
       </c>
       <c r="C212" s="11" t="s">
-        <v>2631</v>
+        <v>2635</v>
       </c>
       <c r="D212" s="11" t="s">
-        <v>2632</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31374,13 +31386,13 @@
         <v>882</v>
       </c>
       <c r="B213" s="70" t="s">
-        <v>2633</v>
+        <v>2637</v>
       </c>
       <c r="C213" s="11" t="s">
-        <v>2634</v>
+        <v>2638</v>
       </c>
       <c r="D213" s="11" t="s">
-        <v>2635</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31388,13 +31400,13 @@
         <v>882</v>
       </c>
       <c r="B214" s="70" t="s">
-        <v>2636</v>
+        <v>2640</v>
       </c>
       <c r="C214" s="11" t="s">
-        <v>2637</v>
+        <v>2641</v>
       </c>
       <c r="D214" s="11" t="s">
-        <v>2638</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31405,10 +31417,10 @@
         <v>232</v>
       </c>
       <c r="C215" s="11" t="s">
-        <v>2639</v>
+        <v>2643</v>
       </c>
       <c r="D215" s="11" t="s">
-        <v>2640</v>
+        <v>2644</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31447,10 +31459,10 @@
         <v>2481</v>
       </c>
       <c r="C218" s="11" t="s">
-        <v>2641</v>
+        <v>2645</v>
       </c>
       <c r="D218" s="11" t="s">
-        <v>2642</v>
+        <v>2646</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31461,10 +31473,10 @@
         <v>2482</v>
       </c>
       <c r="C219" s="11" t="s">
-        <v>2643</v>
+        <v>2647</v>
       </c>
       <c r="D219" s="11" t="s">
-        <v>2644</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31475,10 +31487,10 @@
         <v>2487</v>
       </c>
       <c r="C220" s="11" t="s">
-        <v>2619</v>
+        <v>2623</v>
       </c>
       <c r="D220" s="11" t="s">
-        <v>2620</v>
+        <v>2624</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31489,10 +31501,10 @@
         <v>232</v>
       </c>
       <c r="C221" s="11" t="s">
-        <v>2645</v>
+        <v>2649</v>
       </c>
       <c r="D221" s="11" t="s">
-        <v>2646</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31503,10 +31515,10 @@
         <v>1282</v>
       </c>
       <c r="C222" s="11" t="s">
-        <v>2647</v>
+        <v>2651</v>
       </c>
       <c r="D222" s="11" t="s">
-        <v>2648</v>
+        <v>2652</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31514,13 +31526,13 @@
         <v>1075</v>
       </c>
       <c r="B223" s="70" t="s">
-        <v>2649</v>
+        <v>2653</v>
       </c>
       <c r="C223" s="11" t="s">
-        <v>2650</v>
+        <v>2654</v>
       </c>
       <c r="D223" s="11" t="s">
-        <v>2651</v>
+        <v>2655</v>
       </c>
       <c r="H223" s="54" t="s">
         <v>1189</v>
@@ -31531,13 +31543,13 @@
         <v>1075</v>
       </c>
       <c r="B224" s="70" t="s">
-        <v>2652</v>
+        <v>2656</v>
       </c>
       <c r="C224" s="11" t="s">
-        <v>2653</v>
+        <v>2657</v>
       </c>
       <c r="D224" s="11" t="s">
-        <v>2654</v>
+        <v>2658</v>
       </c>
       <c r="H224" s="54" t="s">
         <v>1189</v>
@@ -31548,13 +31560,13 @@
         <v>1075</v>
       </c>
       <c r="B225" s="70" t="s">
-        <v>2655</v>
+        <v>2659</v>
       </c>
       <c r="C225" s="11" t="s">
-        <v>2656</v>
+        <v>2660</v>
       </c>
       <c r="D225" s="11" t="s">
-        <v>2657</v>
+        <v>2661</v>
       </c>
       <c r="H225" s="54" t="s">
         <v>1189</v>
@@ -31565,13 +31577,13 @@
         <v>1075</v>
       </c>
       <c r="B226" s="70" t="s">
-        <v>2658</v>
+        <v>2662</v>
       </c>
       <c r="C226" s="11" t="s">
-        <v>2659</v>
+        <v>2663</v>
       </c>
       <c r="D226" s="11" t="s">
-        <v>2660</v>
+        <v>2664</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31579,13 +31591,13 @@
         <v>1081</v>
       </c>
       <c r="B227" s="70" t="s">
-        <v>2661</v>
+        <v>2665</v>
       </c>
       <c r="C227" s="11" t="s">
-        <v>2662</v>
+        <v>2666</v>
       </c>
       <c r="D227" s="11" t="s">
-        <v>2663</v>
+        <v>2667</v>
       </c>
       <c r="H227" s="54" t="s">
         <v>1189</v>
@@ -31596,13 +31608,13 @@
         <v>1081</v>
       </c>
       <c r="B228" s="70" t="s">
-        <v>2664</v>
+        <v>2668</v>
       </c>
       <c r="C228" s="11" t="s">
-        <v>2665</v>
+        <v>2669</v>
       </c>
       <c r="D228" s="11" t="s">
-        <v>2666</v>
+        <v>2670</v>
       </c>
       <c r="H228" s="54" t="s">
         <v>1188</v>
@@ -31613,41 +31625,41 @@
         <v>1081</v>
       </c>
       <c r="B229" s="70" t="s">
-        <v>2667</v>
+        <v>2671</v>
       </c>
       <c r="C229" s="11" t="s">
-        <v>2668</v>
+        <v>2672</v>
       </c>
       <c r="D229" s="11" t="s">
-        <v>2669</v>
+        <v>2673</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="57" t="s">
-        <v>2670</v>
+        <v>2674</v>
       </c>
       <c r="B230" s="70" t="s">
         <v>1212</v>
       </c>
       <c r="C230" s="11" t="s">
-        <v>2671</v>
+        <v>2675</v>
       </c>
       <c r="D230" s="11" t="s">
-        <v>2672</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="57" t="s">
-        <v>2670</v>
+        <v>2674</v>
       </c>
       <c r="B231" s="70" t="s">
         <v>1248</v>
       </c>
       <c r="C231" s="11" t="s">
-        <v>2673</v>
+        <v>2677</v>
       </c>
       <c r="D231" s="11" t="s">
-        <v>2674</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31655,13 +31667,13 @@
         <v>1111</v>
       </c>
       <c r="B232" s="70" t="s">
-        <v>2675</v>
+        <v>2679</v>
       </c>
       <c r="C232" s="11" t="s">
-        <v>2676</v>
+        <v>2680</v>
       </c>
       <c r="D232" s="11" t="s">
-        <v>2677</v>
+        <v>2681</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31669,13 +31681,13 @@
         <v>1111</v>
       </c>
       <c r="B233" s="70" t="s">
-        <v>2678</v>
+        <v>2682</v>
       </c>
       <c r="C233" s="11" t="s">
-        <v>2679</v>
+        <v>2683</v>
       </c>
       <c r="D233" s="11" t="s">
-        <v>2680</v>
+        <v>2684</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31683,13 +31695,13 @@
         <v>1111</v>
       </c>
       <c r="B234" s="70" t="s">
-        <v>2681</v>
+        <v>2685</v>
       </c>
       <c r="C234" s="11" t="s">
-        <v>2682</v>
+        <v>2686</v>
       </c>
       <c r="D234" s="11" t="s">
-        <v>2683</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="235" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31697,13 +31709,13 @@
         <v>1111</v>
       </c>
       <c r="B235" s="70" t="s">
-        <v>2684</v>
+        <v>2688</v>
       </c>
       <c r="C235" s="11" t="s">
-        <v>2685</v>
+        <v>2689</v>
       </c>
       <c r="D235" s="11" t="s">
-        <v>2686</v>
+        <v>2690</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31711,13 +31723,13 @@
         <v>1111</v>
       </c>
       <c r="B236" s="70" t="s">
-        <v>2687</v>
+        <v>2691</v>
       </c>
       <c r="C236" s="11" t="s">
-        <v>2688</v>
+        <v>2692</v>
       </c>
       <c r="D236" s="11" t="s">
-        <v>2689</v>
+        <v>2693</v>
       </c>
     </row>
     <row r="237" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31725,13 +31737,13 @@
         <v>1111</v>
       </c>
       <c r="B237" s="70" t="s">
-        <v>2690</v>
+        <v>2694</v>
       </c>
       <c r="C237" s="11" t="s">
-        <v>2691</v>
+        <v>2695</v>
       </c>
       <c r="D237" s="11" t="s">
-        <v>2692</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="238" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31747,13 +31759,13 @@
         <v>999</v>
       </c>
       <c r="B239" s="11" t="s">
-        <v>2693</v>
+        <v>2697</v>
       </c>
       <c r="C239" s="11" t="s">
-        <v>2694</v>
+        <v>2698</v>
       </c>
       <c r="D239" s="11" t="s">
-        <v>2695</v>
+        <v>2699</v>
       </c>
       <c r="G239" s="11"/>
       <c r="H239" s="11"/>
@@ -31764,13 +31776,13 @@
         <v>999</v>
       </c>
       <c r="B240" s="11" t="s">
-        <v>2607</v>
+        <v>2611</v>
       </c>
       <c r="C240" s="11" t="s">
-        <v>2696</v>
+        <v>2700</v>
       </c>
       <c r="D240" s="11" t="s">
-        <v>2697</v>
+        <v>2701</v>
       </c>
       <c r="G240" s="11"/>
       <c r="H240" s="11"/>
@@ -31781,13 +31793,13 @@
         <v>999</v>
       </c>
       <c r="B241" s="11" t="s">
-        <v>2698</v>
+        <v>2702</v>
       </c>
       <c r="C241" s="11" t="s">
-        <v>2699</v>
+        <v>2703</v>
       </c>
       <c r="D241" s="11" t="s">
-        <v>2700</v>
+        <v>2704</v>
       </c>
       <c r="G241" s="11"/>
       <c r="H241" s="11"/>
@@ -31798,13 +31810,13 @@
         <v>999</v>
       </c>
       <c r="B242" s="11" t="s">
-        <v>2701</v>
+        <v>2705</v>
       </c>
       <c r="C242" s="11" t="s">
-        <v>2702</v>
+        <v>2706</v>
       </c>
       <c r="D242" s="11" t="s">
-        <v>2703</v>
+        <v>2707</v>
       </c>
       <c r="G242" s="11"/>
       <c r="H242" s="11"/>
@@ -31815,13 +31827,13 @@
         <v>999</v>
       </c>
       <c r="B243" s="11" t="s">
-        <v>2704</v>
+        <v>2708</v>
       </c>
       <c r="C243" s="11" t="s">
-        <v>2705</v>
+        <v>2709</v>
       </c>
       <c r="D243" s="11" t="s">
-        <v>2706</v>
+        <v>2710</v>
       </c>
       <c r="G243" s="11"/>
       <c r="H243" s="11"/>
@@ -31835,10 +31847,10 @@
         <v>-2</v>
       </c>
       <c r="C244" s="11" t="s">
-        <v>2707</v>
+        <v>2711</v>
       </c>
       <c r="D244" s="11" t="s">
-        <v>2708</v>
+        <v>2712</v>
       </c>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31849,10 +31861,10 @@
         <v>-1</v>
       </c>
       <c r="C245" s="11" t="s">
-        <v>2709</v>
+        <v>2713</v>
       </c>
       <c r="D245" s="11" t="s">
-        <v>2710</v>
+        <v>2714</v>
       </c>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31863,10 +31875,10 @@
         <v>0</v>
       </c>
       <c r="C246" s="11" t="s">
-        <v>2711</v>
+        <v>2715</v>
       </c>
       <c r="D246" s="11" t="s">
-        <v>2712</v>
+        <v>2716</v>
       </c>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31877,10 +31889,10 @@
         <v>1</v>
       </c>
       <c r="C247" s="11" t="s">
-        <v>2713</v>
+        <v>2717</v>
       </c>
       <c r="D247" s="11" t="s">
-        <v>2714</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31891,10 +31903,10 @@
         <v>2</v>
       </c>
       <c r="C248" s="11" t="s">
-        <v>2715</v>
+        <v>2719</v>
       </c>
       <c r="D248" s="11" t="s">
-        <v>2716</v>
+        <v>2720</v>
       </c>
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31905,10 +31917,10 @@
         <v>0</v>
       </c>
       <c r="C249" s="11" t="s">
-        <v>2717</v>
+        <v>2721</v>
       </c>
       <c r="D249" s="11" t="s">
-        <v>2718</v>
+        <v>2722</v>
       </c>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31919,10 +31931,10 @@
         <v>1</v>
       </c>
       <c r="C250" s="11" t="s">
-        <v>2719</v>
+        <v>2723</v>
       </c>
       <c r="D250" s="11" t="s">
-        <v>2720</v>
+        <v>2724</v>
       </c>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31933,10 +31945,10 @@
         <v>2</v>
       </c>
       <c r="C251" s="11" t="s">
-        <v>2721</v>
+        <v>2725</v>
       </c>
       <c r="D251" s="11" t="s">
-        <v>2722</v>
+        <v>2726</v>
       </c>
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31947,10 +31959,10 @@
         <v>3</v>
       </c>
       <c r="C252" s="11" t="s">
-        <v>2723</v>
+        <v>2727</v>
       </c>
       <c r="D252" s="11" t="s">
-        <v>2724</v>
+        <v>2728</v>
       </c>
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31961,10 +31973,10 @@
         <v>4</v>
       </c>
       <c r="C253" s="11" t="s">
-        <v>2725</v>
+        <v>2729</v>
       </c>
       <c r="D253" s="11" t="s">
-        <v>2726</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31975,10 +31987,10 @@
         <v>-1</v>
       </c>
       <c r="C254" s="11" t="s">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="D254" s="11" t="s">
-        <v>2728</v>
+        <v>2732</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31986,13 +31998,13 @@
         <v>39</v>
       </c>
       <c r="B255" s="70" t="s">
-        <v>2729</v>
+        <v>2733</v>
       </c>
       <c r="C255" s="11" t="s">
-        <v>2730</v>
+        <v>2734</v>
       </c>
       <c r="D255" s="11" t="s">
-        <v>2731</v>
+        <v>2735</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
labels: mise à jour du libellé pour bachelorOrHigher en français
fixes #306
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -7884,7 +7884,7 @@
     <t xml:space="preserve">bachelorOrHigher</t>
   </si>
   <si>
-    <t xml:space="preserve">Certificat ou diplôme universitaire niveau baccalauréat ou supérieur</t>
+    <t xml:space="preserve">Baccalauréat ou supérieur</t>
   </si>
   <si>
     <t xml:space="preserve">Bachelor's degree or higher</t>

</xml_diff>

<commit_message>
labels: ajout d'un espace au texte anglais de subwayStationStart
fixes #315
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -2108,7 +2108,7 @@
     <t xml:space="preserve">**Station d'embarquement** (au départ) : </t>
   </si>
   <si>
-    <t xml:space="preserve">**Boarding station**(when entering the metro):</t>
+    <t xml:space="preserve">**Boarding station** (when entering the metro):</t>
   </si>
   <si>
     <t xml:space="preserve">subwayConditional</t>

</xml_diff>

<commit_message>
labels: mise à jour du texte pour membres du ménage hors domicile
fixes #324
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -1571,10 +1571,10 @@
     <t xml:space="preserve">household.persons.{_activePersonId}.journeys.{_activeJourneyId}.outOfTerritoryMembers</t>
   </si>
   <si>
-    <t xml:space="preserve">D’autres membres du ménage étaient aussi en dehors du domicile toute la journée?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Were other household members also outside home all day?</t>
+    <t xml:space="preserve">Quels autres membres du ménage étaient eux-aussi absents du domicile toute la journée ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which other household members were also away from home all day?</t>
   </si>
   <si>
     <t xml:space="preserve">outOfTerritoryMembersConditional</t>
@@ -9159,6 +9159,10 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -9193,10 +9197,6 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -13250,10 +13250,10 @@
       <c r="F70" s="9" t="s">
         <v>441</v>
       </c>
-      <c r="G70" s="9" t="s">
+      <c r="G70" s="30" t="s">
         <v>442</v>
       </c>
-      <c r="H70" s="9" t="s">
+      <c r="H70" s="30" t="s">
         <v>443</v>
       </c>
       <c r="I70" s="9"/>
@@ -13338,10 +13338,10 @@
       <c r="F72" s="18" t="s">
         <v>452</v>
       </c>
-      <c r="G72" s="30" t="s">
+      <c r="G72" s="31" t="s">
         <v>453</v>
       </c>
-      <c r="H72" s="30" t="s">
+      <c r="H72" s="31" t="s">
         <v>454</v>
       </c>
       <c r="I72" s="18"/>
@@ -13451,16 +13451,16 @@
       <c r="F75" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="G75" s="31" t="s">
+      <c r="G75" s="32" t="s">
         <v>457</v>
       </c>
-      <c r="H75" s="31" t="s">
+      <c r="H75" s="32" t="s">
         <v>458</v>
       </c>
-      <c r="I75" s="31" t="s">
+      <c r="I75" s="32" t="s">
         <v>459</v>
       </c>
-      <c r="J75" s="31" t="s">
+      <c r="J75" s="32" t="s">
         <v>460</v>
       </c>
       <c r="S75" s="1" t="b">
@@ -13577,7 +13577,7 @@
       <c r="B80" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="C80" s="32" t="n">
+      <c r="C80" s="33" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -13633,16 +13633,16 @@
       <c r="F81" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="G81" s="33" t="s">
+      <c r="G81" s="34" t="s">
         <v>485</v>
       </c>
-      <c r="H81" s="33" t="s">
+      <c r="H81" s="34" t="s">
         <v>486</v>
       </c>
-      <c r="I81" s="33" t="s">
+      <c r="I81" s="34" t="s">
         <v>487</v>
       </c>
-      <c r="J81" s="33" t="s">
+      <c r="J81" s="34" t="s">
         <v>488</v>
       </c>
       <c r="K81" s="9"/>
@@ -13676,16 +13676,16 @@
       <c r="F82" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="G82" s="33" t="s">
+      <c r="G82" s="34" t="s">
         <v>491</v>
       </c>
-      <c r="H82" s="33" t="s">
+      <c r="H82" s="34" t="s">
         <v>492</v>
       </c>
-      <c r="I82" s="33" t="s">
+      <c r="I82" s="34" t="s">
         <v>493</v>
       </c>
-      <c r="J82" s="33" t="s">
+      <c r="J82" s="34" t="s">
         <v>494</v>
       </c>
       <c r="K82" s="9"/>
@@ -14143,7 +14143,7 @@
       <c r="B97" s="17" t="s">
         <v>367</v>
       </c>
-      <c r="C97" s="34" t="n">
+      <c r="C97" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -14183,23 +14183,23 @@
       <c r="A98" s="19" t="s">
         <v>366</v>
       </c>
-      <c r="B98" s="35" t="s">
+      <c r="B98" s="36" t="s">
         <v>367</v>
       </c>
-      <c r="C98" s="36" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D98" s="35" t="s">
+      <c r="C98" s="37" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D98" s="36" t="s">
         <v>566</v>
       </c>
       <c r="E98" s="19"/>
       <c r="F98" s="19"/>
       <c r="G98" s="19"/>
       <c r="H98" s="19"/>
-      <c r="I98" s="35"/>
-      <c r="J98" s="35"/>
-      <c r="K98" s="35"/>
+      <c r="I98" s="36"/>
+      <c r="J98" s="36"/>
+      <c r="K98" s="36"/>
       <c r="L98" s="19"/>
       <c r="M98" s="19"/>
       <c r="N98" s="19"/>
@@ -14207,7 +14207,7 @@
       <c r="P98" s="19"/>
       <c r="Q98" s="19"/>
       <c r="R98" s="19"/>
-      <c r="S98" s="35" t="b">
+      <c r="S98" s="36" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -14221,42 +14221,42 @@
       <c r="A99" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="B99" s="31" t="s">
+      <c r="B99" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C99" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D99" s="31" t="s">
+      <c r="C99" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D99" s="32" t="s">
         <v>566</v>
       </c>
       <c r="F99" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="G99" s="31" t="s">
+      <c r="G99" s="32" t="s">
         <v>372</v>
       </c>
-      <c r="H99" s="31" t="s">
+      <c r="H99" s="32" t="s">
         <v>373</v>
       </c>
-      <c r="I99" s="31"/>
-      <c r="J99" s="31"/>
-      <c r="K99" s="31"/>
-      <c r="S99" s="31"/>
+      <c r="I99" s="32"/>
+      <c r="J99" s="32"/>
+      <c r="K99" s="32"/>
+      <c r="S99" s="32"/>
     </row>
     <row r="100" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="B100" s="31" t="s">
+      <c r="B100" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C100" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D100" s="31" t="s">
+      <c r="C100" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D100" s="32" t="s">
         <v>566</v>
       </c>
       <c r="F100" s="1" t="s">
@@ -14274,8 +14274,8 @@
       <c r="J100" s="9" t="s">
         <v>571</v>
       </c>
-      <c r="K100" s="31"/>
-      <c r="S100" s="31" t="b">
+      <c r="K100" s="32"/>
+      <c r="S100" s="32" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -14284,14 +14284,14 @@
       <c r="A101" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="B101" s="31" t="s">
+      <c r="B101" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C101" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D101" s="31" t="s">
+      <c r="C101" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D101" s="32" t="s">
         <v>566</v>
       </c>
       <c r="F101" s="1" t="s">
@@ -14309,44 +14309,44 @@
       <c r="J101" s="1" t="s">
         <v>576</v>
       </c>
-      <c r="K101" s="31"/>
-      <c r="S101" s="31"/>
+      <c r="K101" s="32"/>
+      <c r="S101" s="32"/>
     </row>
     <row r="102" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="B102" s="31" t="s">
+      <c r="B102" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C102" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D102" s="31" t="s">
+      <c r="C102" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D102" s="32" t="s">
         <v>566</v>
       </c>
       <c r="F102" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="H102" s="31"/>
-      <c r="I102" s="31"/>
-      <c r="J102" s="31"/>
-      <c r="K102" s="31"/>
-      <c r="S102" s="31"/>
+      <c r="H102" s="32"/>
+      <c r="I102" s="32"/>
+      <c r="J102" s="32"/>
+      <c r="K102" s="32"/>
+      <c r="S102" s="32"/>
     </row>
     <row r="103" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="B103" s="31" t="s">
+      <c r="B103" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C103" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D103" s="31" t="s">
+      <c r="C103" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D103" s="32" t="s">
         <v>566</v>
       </c>
       <c r="E103" s="1" t="s">
@@ -14363,21 +14363,21 @@
       </c>
       <c r="I103" s="11"/>
       <c r="J103" s="11"/>
-      <c r="K103" s="31"/>
-      <c r="S103" s="31"/>
+      <c r="K103" s="32"/>
+      <c r="S103" s="32"/>
     </row>
     <row r="104" s="12" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="B104" s="31" t="s">
+      <c r="B104" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C104" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D104" s="31" t="s">
+      <c r="C104" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D104" s="32" t="s">
         <v>566</v>
       </c>
       <c r="E104" s="1" t="s">
@@ -14389,12 +14389,12 @@
       <c r="G104" s="1" t="s">
         <v>583</v>
       </c>
-      <c r="H104" s="31" t="s">
+      <c r="H104" s="32" t="s">
         <v>584</v>
       </c>
-      <c r="I104" s="31"/>
-      <c r="J104" s="31"/>
-      <c r="K104" s="31"/>
+      <c r="I104" s="32"/>
+      <c r="J104" s="32"/>
+      <c r="K104" s="32"/>
       <c r="L104" s="1"/>
       <c r="M104" s="1"/>
       <c r="N104" s="1"/>
@@ -14402,7 +14402,7 @@
       <c r="P104" s="1"/>
       <c r="Q104" s="1"/>
       <c r="R104" s="1"/>
-      <c r="S104" s="31"/>
+      <c r="S104" s="32"/>
       <c r="T104" s="1"/>
       <c r="U104" s="1"/>
       <c r="V104" s="1"/>
@@ -14413,14 +14413,14 @@
       <c r="A105" s="1" t="s">
         <v>585</v>
       </c>
-      <c r="B105" s="31" t="s">
+      <c r="B105" s="32" t="s">
         <v>367</v>
       </c>
-      <c r="C105" s="37" t="n">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D105" s="31" t="s">
+      <c r="C105" s="38" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D105" s="32" t="s">
         <v>566</v>
       </c>
       <c r="E105" s="1" t="s">
@@ -14435,9 +14435,9 @@
       <c r="H105" s="9" t="s">
         <v>588</v>
       </c>
-      <c r="I105" s="31"/>
-      <c r="J105" s="31"/>
-      <c r="K105" s="31"/>
+      <c r="I105" s="32"/>
+      <c r="J105" s="32"/>
+      <c r="K105" s="32"/>
       <c r="L105" s="1"/>
       <c r="M105" s="1"/>
       <c r="N105" s="1"/>
@@ -14445,7 +14445,7 @@
       <c r="P105" s="1"/>
       <c r="Q105" s="1"/>
       <c r="R105" s="1"/>
-      <c r="S105" s="31"/>
+      <c r="S105" s="32"/>
       <c r="T105" s="1"/>
       <c r="U105" s="1"/>
       <c r="V105" s="1"/>
@@ -14720,7 +14720,7 @@
       <c r="U111" s="1"/>
       <c r="V111" s="1"/>
       <c r="W111" s="1"/>
-      <c r="X111" s="38" t="s">
+      <c r="X111" s="39" t="s">
         <v>615</v>
       </c>
     </row>
@@ -14770,7 +14770,7 @@
       <c r="U112" s="1"/>
       <c r="V112" s="1"/>
       <c r="W112" s="1"/>
-      <c r="X112" s="38" t="s">
+      <c r="X112" s="39" t="s">
         <v>615</v>
       </c>
     </row>
@@ -14822,7 +14822,7 @@
       <c r="U113" s="1"/>
       <c r="V113" s="1"/>
       <c r="W113" s="1"/>
-      <c r="X113" s="38"/>
+      <c r="X113" s="39"/>
     </row>
     <row r="114" s="12" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="9" t="s">
@@ -14920,7 +14920,7 @@
       <c r="U115" s="9"/>
       <c r="V115" s="9"/>
       <c r="W115" s="9"/>
-      <c r="X115" s="38" t="s">
+      <c r="X115" s="39" t="s">
         <v>615</v>
       </c>
     </row>
@@ -14972,7 +14972,7 @@
       <c r="U116" s="9"/>
       <c r="V116" s="9"/>
       <c r="W116" s="9"/>
-      <c r="X116" s="38" t="s">
+      <c r="X116" s="39" t="s">
         <v>642</v>
       </c>
     </row>
@@ -15022,7 +15022,7 @@
       <c r="U117" s="9"/>
       <c r="V117" s="9"/>
       <c r="W117" s="9"/>
-      <c r="X117" s="38" t="s">
+      <c r="X117" s="39" t="s">
         <v>615</v>
       </c>
     </row>
@@ -15072,7 +15072,7 @@
       <c r="U118" s="9"/>
       <c r="V118" s="9"/>
       <c r="W118" s="9"/>
-      <c r="X118" s="38" t="s">
+      <c r="X118" s="39" t="s">
         <v>615</v>
       </c>
     </row>
@@ -15957,7 +15957,7 @@
       <c r="B137" s="17" t="s">
         <v>367</v>
       </c>
-      <c r="C137" s="34" t="n">
+      <c r="C137" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -15971,7 +15971,7 @@
       <c r="G137" s="17" t="s">
         <v>754</v>
       </c>
-      <c r="H137" s="39" t="s">
+      <c r="H137" s="8" t="s">
         <v>755</v>
       </c>
       <c r="I137" s="17"/>
@@ -16600,7 +16600,7 @@
       <c r="B151" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="C151" s="34" t="n">
+      <c r="C151" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -17154,13 +17154,13 @@
       <c r="G164" s="1" t="s">
         <v>900</v>
       </c>
-      <c r="H164" s="31" t="s">
+      <c r="H164" s="32" t="s">
         <v>901</v>
       </c>
-      <c r="I164" s="31" t="s">
+      <c r="I164" s="32" t="s">
         <v>902</v>
       </c>
-      <c r="J164" s="31" t="s">
+      <c r="J164" s="32" t="s">
         <v>903</v>
       </c>
       <c r="M164" s="1" t="s">
@@ -17195,13 +17195,13 @@
       <c r="G165" s="1" t="s">
         <v>908</v>
       </c>
-      <c r="H165" s="31" t="s">
+      <c r="H165" s="32" t="s">
         <v>909</v>
       </c>
-      <c r="I165" s="31" t="s">
+      <c r="I165" s="32" t="s">
         <v>910</v>
       </c>
-      <c r="J165" s="31" t="s">
+      <c r="J165" s="32" t="s">
         <v>911</v>
       </c>
       <c r="K165" s="1"/>
@@ -17250,7 +17250,7 @@
       <c r="H166" s="1" t="s">
         <v>915</v>
       </c>
-      <c r="I166" s="31" t="s">
+      <c r="I166" s="32" t="s">
         <v>916</v>
       </c>
       <c r="J166" s="1" t="s">
@@ -18066,7 +18066,7 @@
       <c r="B184" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="C184" s="34" t="n">
+      <c r="C184" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -18197,7 +18197,7 @@
       <c r="B187" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="C187" s="34" t="n">
+      <c r="C187" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -18957,7 +18957,7 @@
       <c r="B203" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="C203" s="34" t="n">
+      <c r="C203" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -19444,7 +19444,7 @@
       <c r="B213" s="17" t="s">
         <v>165</v>
       </c>
-      <c r="C213" s="34" t="n">
+      <c r="C213" s="35" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -19906,7 +19906,7 @@
       <c r="F223" s="1" t="s">
         <v>1128</v>
       </c>
-      <c r="G223" s="31" t="s">
+      <c r="G223" s="32" t="s">
         <v>1129</v>
       </c>
       <c r="H223" s="1" t="s">
@@ -19934,7 +19934,7 @@
       <c r="D224" s="1" t="s">
         <v>1076</v>
       </c>
-      <c r="F224" s="31" t="s">
+      <c r="F224" s="32" t="s">
         <v>1132</v>
       </c>
       <c r="G224" s="1" t="s">
@@ -19967,7 +19967,7 @@
       <c r="F225" s="1" t="s">
         <v>1138</v>
       </c>
-      <c r="G225" s="31" t="s">
+      <c r="G225" s="32" t="s">
         <v>1139</v>
       </c>
       <c r="H225" s="1" t="s">
@@ -20004,7 +20004,7 @@
       <c r="F226" s="1" t="s">
         <v>1144</v>
       </c>
-      <c r="G226" s="31" t="s">
+      <c r="G226" s="32" t="s">
         <v>1145</v>
       </c>
       <c r="H226" s="1" t="s">
@@ -20038,7 +20038,7 @@
       <c r="F227" s="1" t="s">
         <v>1148</v>
       </c>
-      <c r="G227" s="31" t="s">
+      <c r="G227" s="32" t="s">
         <v>1149</v>
       </c>
       <c r="H227" s="1" t="s">
@@ -20075,7 +20075,7 @@
       <c r="F228" s="1" t="s">
         <v>1153</v>
       </c>
-      <c r="G228" s="31" t="s">
+      <c r="G228" s="32" t="s">
         <v>1154</v>
       </c>
       <c r="H228" s="1" t="s">
@@ -20112,7 +20112,7 @@
       <c r="F229" s="1" t="s">
         <v>1158</v>
       </c>
-      <c r="G229" s="31" t="s">
+      <c r="G229" s="32" t="s">
         <v>1159</v>
       </c>
       <c r="H229" s="1" t="s">
@@ -20149,7 +20149,7 @@
       <c r="F230" s="1" t="s">
         <v>1163</v>
       </c>
-      <c r="G230" s="31" t="s">
+      <c r="G230" s="32" t="s">
         <v>1164</v>
       </c>
       <c r="H230" s="1" t="s">
@@ -20217,7 +20217,7 @@
       <c r="B232" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C232" s="32" t="n">
+      <c r="C232" s="33" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -20247,7 +20247,7 @@
       <c r="B233" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C233" s="32" t="n">
+      <c r="C233" s="33" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -20273,7 +20273,7 @@
       <c r="B234" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C234" s="32" t="n">
+      <c r="C234" s="33" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
modes access/egress: ajout du champ texte pour 'other'
fixes #346

Le champ n'est toutefois pas obligatoire, dû à un bug sur cet élément
dans Evolution.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4984" uniqueCount="2721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4986" uniqueCount="2721">
   <si>
     <t xml:space="preserve">questionName</t>
   </si>
@@ -15455,6 +15455,9 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
+      <c r="U126" s="1" t="s">
+        <v>232</v>
+      </c>
       <c r="X126" s="1" t="s">
         <v>690</v>
       </c>
@@ -15793,6 +15796,9 @@
       <c r="S133" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
+      </c>
+      <c r="U133" s="1" t="s">
+        <v>232</v>
       </c>
       <c r="X133" s="1" t="s">
         <v>690</v>

</xml_diff>